<commit_message>
Release 2.8.0: version bump and regenerated examples
Publisher/policy/analyzer/optimizer/estimator/bundle/reviewer/decision versions
2.7.1 -> 2.8.0 (MODEL_VERSION and contract versions unchanged). Examples,
demo run, test results and workbook audit regenerated once.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo_output/workbook.xlsx
+++ b/examples/demo_output/workbook.xlsx
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="8" t="n">
-        <v>-176826.67</v>
+        <v>0</v>
       </c>
       <c r="N14" s="8" t="n">
         <v>0</v>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>-446946.29</v>
+        <v>-270119.62</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2778,7 +2778,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="AH5" s="14" t="inlineStr">
         <is>
-          <t>SCN-F6C96142718566E6610757F4</t>
+          <t>SCN-E1D619112BE62AFA050EA71A</t>
         </is>
       </c>
       <c r="AI5" s="15" t="inlineStr">
@@ -2994,12 +2994,12 @@
       </c>
       <c r="BC5" s="22" t="inlineStr">
         <is>
-          <t>["SCN-F6C96142718566E6610757F4","SCN-4CE208EB461A228615816740"]</t>
+          <t>["SCN-E1D619112BE62AFA050EA71A","SCN-B49B73B0344B4AF52B454990"]</t>
         </is>
       </c>
       <c r="BD5" s="22" t="inlineStr">
         <is>
-          <t>["CAND-7228133F8C9DCD58D5450164","CAND-CDC9DD7E27E8CA6ED23E9CEB","CAND-4CD23256DB0CA20822638058","CAND-F7CD1FD114943EA1AAB92DF2","CAND-1EB011ABA71F8CF380C298A8","CAND-78762B303EA11AF80300E2C3"]</t>
+          <t>["CAND-2FF10B6D104A88133435FFC9","CAND-DAC9E910F2A94A05B67B302A","CAND-567E1FFD79E2F9A61A59510F","CAND-585D0C22F7A86D37CE5BCDE5","CAND-B72E480BD8ADA0BAAADDB594","CAND-D7C2183B68BBD711C74005C7"]</t>
         </is>
       </c>
       <c r="BE5" s="22" t="inlineStr">
@@ -3009,14 +3009,14 @@
       </c>
       <c r="BF5" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-032D2043227CEDC95604F643":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-06FF9A63969D378F8BA1F07C":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":8},"EVID-08FF9FEB1B0F5DD025C7139B":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-0C186B67BBA35BE5E67FC5B4":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":400.0},"EVID-14B9E1F21FB6239C1605B425":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-1AD100E505AE1F8331626BFC":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":960},"EVID-24051B9A42F0A0296E9942FB":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-276F66B0ED2BE9C1F9FB7F7D":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9000},"EVID-2AD1BDE448603EA994275416":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2667},"EVID-34B06F602B3B350E40C7FB2F":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-379FF5C04A904D87A2DE5C67":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-37B58153FD21C4097D6839AF":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":11725.1},"EVID-43AC520BEDF28B837AD5491F":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-4D3C96F560A56E7EC4E79822":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-4E2C10D0BEF65086F73BD1BB":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-671AEFC2D527CBB61D748323":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":27000.0},"EVID-6A39CCAC873FB9B1E4CBD8F0":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-6EA74D3474DEBD48A2D18AA3":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2500},"EVID-6ED4860D13BF644A666A35DC":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-758B77C00654A7C0ADB79FEF":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":80.0},"EVID-76C886F1C575094A206B1C98":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-816032E26FD5D0505D12B7B5":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":23760.0},"EVID-832712B10A432503BA1E0ADE":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-844D3CCD8E1426B8521EC841":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-8B53A706B88503957283FBAF":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":480},"EVID-8C9114054238A654DB9B7C17":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-8D64B1C2140B8113E92CB584":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-8FDC7E9818FEE739EB1C3E96":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-9123C82F00FD3E06C4EC1397":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-9475F7B85538B16451EA1C33":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-9CDDE8E0C8CE33998BB2989D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-A1C75CA0E3C954E8451A24A9":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-A8636AD7291DF641B4479F73":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-A86EAA13EE5082AEC4DF0A44":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":10000},"EVID-B2362D5F32380977A933F401":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-B2F3556302DC172A975B5E1D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-B907494F116961DE176B0D84":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-B97068E09275EE196C280B20":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-C257109E096D0ECC02DBF878":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3000},"EVID-CB69D69A29C6EA7DB46849D4":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-CD8BAC81B5726CC8B4111349":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-CEBECE0D400BCC63E7372BA4":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-D0979C303C3ECC7B43215C4E":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-D6A8913E1EEDE597C6DE13D7":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-D6C1A66CD6414FC0530CD64D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E64F7F42523DB02D3B0CFEAB":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-F070BBED6A139F6AC2DDC3AB":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-F321D01534023722070D55FC":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-F3407AFA2008FBBDD9A22AB0":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-FBF33D9F734E4A15AC59AA04":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-FDBFFBC774D23EA471B31E96":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0}}</t>
+          <t>{"EVID-032D2043227CEDC95604F643":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-06FF9A63969D378F8BA1F07C":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":8},"EVID-08FF9FEB1B0F5DD025C7139B":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-0C186B67BBA35BE5E67FC5B4":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":400.0},"EVID-14B9E1F21FB6239C1605B425":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-1AD100E505AE1F8331626BFC":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":960},"EVID-24051B9A42F0A0296E9942FB":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-276F66B0ED2BE9C1F9FB7F7D":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9000},"EVID-2AD1BDE448603EA994275416":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2667},"EVID-34B06F602B3B350E40C7FB2F":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-379FF5C04A904D87A2DE5C67":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-37B58153FD21C4097D6839AF":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":11725.1},"EVID-43AC520BEDF28B837AD5491F":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-4D3C96F560A56E7EC4E79822":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-4E2C10D0BEF65086F73BD1BB":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-671AEFC2D527CBB61D748323":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":27000.0},"EVID-6A39CCAC873FB9B1E4CBD8F0":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-6EA74D3474DEBD48A2D18AA3":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2500},"EVID-6ED4860D13BF644A666A35DC":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-756332815C5D1223CA4A8740":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-758B77C00654A7C0ADB79FEF":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":80.0},"EVID-76C886F1C575094A206B1C98":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-816032E26FD5D0505D12B7B5":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":23760.0},"EVID-832712B10A432503BA1E0ADE":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-844D3CCD8E1426B8521EC841":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-8B53A706B88503957283FBAF":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":480},"EVID-8C9114054238A654DB9B7C17":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-8D64B1C2140B8113E92CB584":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-8FDC7E9818FEE739EB1C3E96":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-9123C82F00FD3E06C4EC1397":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-9475F7B85538B16451EA1C33":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-9CDDE8E0C8CE33998BB2989D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-A1C75CA0E3C954E8451A24A9":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-A8636AD7291DF641B4479F73":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-A86EAA13EE5082AEC4DF0A44":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":10000},"EVID-B2362D5F32380977A933F401":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-B2F3556302DC172A975B5E1D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-B907494F116961DE176B0D84":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-B97068E09275EE196C280B20":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-C257109E096D0ECC02DBF878":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3000},"EVID-CB69D69A29C6EA7DB46849D4":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-CD8BAC81B5726CC8B4111349":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-CEBECE0D400BCC63E7372BA4":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-D0979C303C3ECC7B43215C4E":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-D6A8913E1EEDE597C6DE13D7":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-D6C1A66CD6414FC0530CD64D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E64F7F42523DB02D3B0CFEAB":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-F070BBED6A139F6AC2DDC3AB":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-F321D01534023722070D55FC":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-F3407AFA2008FBBDD9A22AB0":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-FBF33D9F734E4A15AC59AA04":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-FDBFFBC774D23EA471B31E96":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0}}</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="AH6" s="14" t="inlineStr">
         <is>
-          <t>SCN-CB5E8798D5A13F523639541D</t>
+          <t>SCN-2EEA487274E8B4C2D2A00C65</t>
         </is>
       </c>
       <c r="AI6" s="15" t="inlineStr">
@@ -3232,12 +3232,12 @@
       </c>
       <c r="BC6" s="22" t="inlineStr">
         <is>
-          <t>["SCN-CB5E8798D5A13F523639541D","SCN-AF126D31FABFB5905E6640A4"]</t>
+          <t>["SCN-2EEA487274E8B4C2D2A00C65","SCN-69AD699F056B046156191604"]</t>
         </is>
       </c>
       <c r="BD6" s="22" t="inlineStr">
         <is>
-          <t>["CAND-BB5D8BD2733924BAA2A2BB82","CAND-F6DA76343C4F0EEC6747DD79","CAND-19E6151216E0827A2A6FA085","CAND-CF1FEEFF3DB94CBE4A3A7DCC","CAND-A122082B3BB2FB0568C91BF4","CAND-335D8BD4AAC3CB041A5DB0CB"]</t>
+          <t>["CAND-BBCE77B209F653D5A121588C","CAND-3107EA199EA58282439B64F2","CAND-59AA68AE5112DDA5910F67FF","CAND-EBBDB2090AA5F8307AFCB223","CAND-CDA61DCEC36313DD1885DFD7","CAND-5FD3D0884B03CB55AFDD5092"]</t>
         </is>
       </c>
       <c r="BE6" s="22" t="inlineStr">
@@ -3247,14 +3247,14 @@
       </c>
       <c r="BF6" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-008E22AC1569A178FD5BB0BB":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-011A7F44ED59741E3113CF84":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.8},"EVID-023EC964F3B265506A960264":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0A7D5DF3B5E2F45BE27DFD19":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":422},"EVID-10635B972051ED8C2A7BEF9D":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":264},"EVID-11111D2C5475DC38E61DFA06":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-2DB66798C05363656D798225":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-2E3E084CE9E030F23CDF5C69":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-31544533FEDFC669EB9E511D":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":64000.0},"EVID-3476CE9B58C832413C9CDD86":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3C8A3CCC5CABDA8C40603603":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-42CBBF164E0D9C6045421154":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-44DE1AAFD8BD8101A789E6D3":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-4732E4D4468FD04336EAA389":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-47D3DCEFC38B6037DA2C3C66":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-4AA93F65650373D3FBE29C04":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-4ABB2B728EAFAC6FBE30DB98":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":4875},"EVID-54D50055FE0A3E96237477FE":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-5975B1FAAF8D55B8BE39B16A":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-5DF889A28B3C24819F832003":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.8},"EVID-5E15646755CA81DC480F12E3":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-60346EE4CD6A756F88C9A889":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":74769.7},"EVID-61A44CDFF8B383C5ABB509D9":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-6E6FA15129845B3E6AA53F0D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-823A180D36962C7150FEB320":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":56320.0},"EVID-8686A768FBB341A60EA85745":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"X_LARGE"},"EVID-878FBB5F95499DF6B2898334":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-88AEFDEA380CDAD006F80001":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":6.5},"EVID-9DEB51B75BB99243343010BD":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-9FFE6B7A17D42D283F900800":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":48000},"EVID-ADB79C6C27705809054C828E":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":260},"EVID-B0B89C04931F9EF778B52C38":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-B6644BF4C662B07A42FBCE9B":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":25.0},"EVID-BA1E532B2C41577B6EE086D9":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":52},"EVID-BB7DFD2862AB2ADD1FA0CF31":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":3221225472},"EVID-C01955F26C5D765DE5852F5C":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-C5492D968DBE0CBA760D384E":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-D1E857F4F27E1D721E697232":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-D20432463AC399D3560B9BC0":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-D875C0624A470AC0E77CBF38":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":12.0},"EVID-DA03D70120DE2B052CB67DE3":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":216.67},"EVID-DD1C35D1D57DDC4796710BDC":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-DEFA78DE669DA4D64347ED77":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":12.0},"EVID-E237AFE39A08B3673A0DF2DC":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-E6918924A28E2011799B7FCB":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-E76BD458403FECA264E0C895":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":520},"EVID-EA733691C9BFE7B18FA8EE7E":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.8},"EVID-F596821EABB66977C5570861":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-F606E713FACB0671C4DF6405":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-F96600E8808D60DFD7238304":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":14000},"EVID-FEE2FD24549E680CEC9BF082":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0}}</t>
+          <t>{"EVID-008E22AC1569A178FD5BB0BB":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-011A7F44ED59741E3113CF84":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.8},"EVID-023EC964F3B265506A960264":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0A7D5DF3B5E2F45BE27DFD19":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":422},"EVID-10635B972051ED8C2A7BEF9D":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":264},"EVID-11111D2C5475DC38E61DFA06":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-2DB66798C05363656D798225":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-2E3E084CE9E030F23CDF5C69":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-31544533FEDFC669EB9E511D":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":64000.0},"EVID-3476CE9B58C832413C9CDD86":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3C8A3CCC5CABDA8C40603603":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-42CBBF164E0D9C6045421154":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-44DE1AAFD8BD8101A789E6D3":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-4732E4D4468FD04336EAA389":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-47D3DCEFC38B6037DA2C3C66":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-4AA93F65650373D3FBE29C04":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-4ABB2B728EAFAC6FBE30DB98":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":4875},"EVID-54D50055FE0A3E96237477FE":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-5975B1FAAF8D55B8BE39B16A":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-5DF889A28B3C24819F832003":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.8},"EVID-5E15646755CA81DC480F12E3":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-60346EE4CD6A756F88C9A889":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":74769.7},"EVID-61A44CDFF8B383C5ABB509D9":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-6E6FA15129845B3E6AA53F0D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-823A180D36962C7150FEB320":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":56320.0},"EVID-8686A768FBB341A60EA85745":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"X_LARGE"},"EVID-878FBB5F95499DF6B2898334":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-88AEFDEA380CDAD006F80001":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":6.5},"EVID-9DEB51B75BB99243343010BD":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-9FFE6B7A17D42D283F900800":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":48000},"EVID-ADB79C6C27705809054C828E":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":260},"EVID-B0B89C04931F9EF778B52C38":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-B6644BF4C662B07A42FBCE9B":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":25.0},"EVID-BA1E532B2C41577B6EE086D9":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":52},"EVID-BB7DFD2862AB2ADD1FA0CF31":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":3221225472},"EVID-C01955F26C5D765DE5852F5C":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-C5492D968DBE0CBA760D384E":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-D1E857F4F27E1D721E697232":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-D20432463AC399D3560B9BC0":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-D875C0624A470AC0E77CBF38":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":12.0},"EVID-DA03D70120DE2B052CB67DE3":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":216.67},"EVID-DD1C35D1D57DDC4796710BDC":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-DEFA78DE669DA4D64347ED77":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":12.0},"EVID-E237AFE39A08B3673A0DF2DC":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-E6918924A28E2011799B7FCB":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-E76BD458403FECA264E0C895":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":520},"EVID-EA733691C9BFE7B18FA8EE7E":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.8},"EVID-EC04540FF7292F7272B822B1":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-F596821EABB66977C5570861":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-F606E713FACB0671C4DF6405":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-F96600E8808D60DFD7238304":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":14000},"EVID-FEE2FD24549E680CEC9BF082":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0}}</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="AH7" s="14" t="inlineStr">
         <is>
-          <t>SCN-CE4B0C3CDE2534722A4AAADE</t>
+          <t>SCN-F7FD9602740588A931526FB1</t>
         </is>
       </c>
       <c r="AI7" s="15" t="inlineStr">
@@ -3470,12 +3470,12 @@
       </c>
       <c r="BC7" s="22" t="inlineStr">
         <is>
-          <t>["SCN-CE4B0C3CDE2534722A4AAADE","SCN-68F9545F52E814CE6E2CDC73"]</t>
+          <t>["SCN-F7FD9602740588A931526FB1","SCN-260783C9E116C39D21DA207C"]</t>
         </is>
       </c>
       <c r="BD7" s="22" t="inlineStr">
         <is>
-          <t>["CAND-B2CDD1956666E75CF94834A6","CAND-C86EF28A42FC56DB5AD00959","CAND-0B0E829222AD5BA2CA4E7612","CAND-E2B81BBFEB2D221645C6CC57","CAND-028FA513EA788FFB1FAADF4E","CAND-B994ABE33118C0EA458EFC1D"]</t>
+          <t>["CAND-5D7C7CA2D483F31C69008B3F","CAND-FF852A8F55F23A58470A0F50","CAND-6A370586BC9EDB6A5FE47F5D","CAND-6F350B226F959664414114EB","CAND-99A7041317161930A14478B9","CAND-99EF846309D3820B9095938B"]</t>
         </is>
       </c>
       <c r="BE7" s="22" t="inlineStr">
@@ -3485,14 +3485,14 @@
       </c>
       <c r="BF7" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-069E575F07ED5D3F026FFD84":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-07855EEDB66F6649A9D64E54":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-1614F9F08839318F3E399E84":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6500},"EVID-1805CF7D4543EFA78447DECE":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":60000.0},"EVID-1A6A8DE3CE8B9EC7EB08FD23":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-1D3DC4ADB1D13DC74AC5E8BA":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-1E19B5180CDF11B79E5F6827":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-256B2F425547D69D3B72A3A1":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-2774AF84EAE8D6AA54B380CA":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":214},"EVID-3301D8D217A4AF84708C338B":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-35340FC00083C675D1843DD6":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-3574F2628778A67585EA0BA6":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":600},"EVID-3DE1D1B65EC8D6C5C825F4CD":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":48000.0},"EVID-3E447650DBBC19DE5DC50006":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":3},"EVID-41B376CD33B233A60C984B5E":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":88.0},"EVID-441757A3E1AFD5C28DD3B5A6":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-4B10F42F3076E3A2C99D1E07":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":500.0},"EVID-5081D66C44958CDE25B84E14":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1200},"EVID-5257C5DF3373073974DA58CB":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-5377620EA4B90F62C3412859":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-5B97CD1773C12505CBA9E9E0":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-5F24A6CA88EA07B7E10EA266":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-686136A0CB3D558076E8814F":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-6D282145D7EDDBB713F4D360":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-6EF3D166591630B3C50D2BE2":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-75681E00F1AFFAE2ED2A7EE6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-7DE4C6A55F99666E0EA5E572":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-7EE079F6E39AE969EB70AD13":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-8709603247A35A8909AA6811":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-895BAEEB75D06CB18730FA3E":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1900},"EVID-972F35B29D44CBCD58534B38":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-990E7C65C9A55CFB360EA05A":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":42240.0},"EVID-A03A50B0A17A58F8B66899A5":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3750},"EVID-A1A5198F8F5C91C64ADA9CB8":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":6},"EVID-A5222E97CA81F6CAE91BF10A":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":21285.98},"EVID-A79643C41CABC592572377D2":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-AAE9AAC833B24F5DAC8690C9":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-B10D381B0DF19402AF720873":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-B3A1C76A1256AB7EA8739C31":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-C20E3596861AD2FFE5AC3C02":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":5500.0},"EVID-CC00770AFFDC1E9E926E98F8":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DC8E2B483D3DE477A9E63AD2":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-E0B79AC286DD69D55BD4D1D0":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-E1C905461AC9721CD8B685A6":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-E6596ABFC4A7555BB31D7835":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-E845955777C16A5CC8D7B84C":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-EAFB05CA0AE5AFF8B3549A43":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":3},"EVID-F27A7E33A3F59F365A5F2A13":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":11250},"EVID-F716D2784AE7839470A5204E":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-F9172897F8EA5E1460F7AED3":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-FDB65766E0DDA49AC4DD5518":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0}}</t>
+          <t>{"EVID-069E575F07ED5D3F026FFD84":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-07855EEDB66F6649A9D64E54":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-1614F9F08839318F3E399E84":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6500},"EVID-1805CF7D4543EFA78447DECE":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":60000.0},"EVID-1A6A8DE3CE8B9EC7EB08FD23":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-1D3DC4ADB1D13DC74AC5E8BA":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-1E19B5180CDF11B79E5F6827":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-256B2F425547D69D3B72A3A1":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-2774AF84EAE8D6AA54B380CA":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":214},"EVID-3301D8D217A4AF84708C338B":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-35340FC00083C675D1843DD6":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-3574F2628778A67585EA0BA6":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":600},"EVID-3DE1D1B65EC8D6C5C825F4CD":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":48000.0},"EVID-3E447650DBBC19DE5DC50006":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":3},"EVID-41B376CD33B233A60C984B5E":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":88.0},"EVID-441757A3E1AFD5C28DD3B5A6":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-4B10F42F3076E3A2C99D1E07":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":500.0},"EVID-5081D66C44958CDE25B84E14":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1200},"EVID-5257C5DF3373073974DA58CB":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-5377620EA4B90F62C3412859":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-5B97CD1773C12505CBA9E9E0":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-5F24A6CA88EA07B7E10EA266":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-686136A0CB3D558076E8814F":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-6D282145D7EDDBB713F4D360":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-6EF3D166591630B3C50D2BE2":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-75681E00F1AFFAE2ED2A7EE6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-7DE4C6A55F99666E0EA5E572":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-7EE079F6E39AE969EB70AD13":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-8709603247A35A8909AA6811":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-895BAEEB75D06CB18730FA3E":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1900},"EVID-972F35B29D44CBCD58534B38":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-990E7C65C9A55CFB360EA05A":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":42240.0},"EVID-A03A50B0A17A58F8B66899A5":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3750},"EVID-A1A5198F8F5C91C64ADA9CB8":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":6},"EVID-A5222E97CA81F6CAE91BF10A":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":21285.98},"EVID-A79643C41CABC592572377D2":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-AAE9AAC833B24F5DAC8690C9":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-B10D381B0DF19402AF720873":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-B3A1C76A1256AB7EA8739C31":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-C20E3596861AD2FFE5AC3C02":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":5500.0},"EVID-CC00770AFFDC1E9E926E98F8":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DC8E2B483D3DE477A9E63AD2":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-E0B79AC286DD69D55BD4D1D0":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-E1C905461AC9721CD8B685A6":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-E6596ABFC4A7555BB31D7835":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-E845955777C16A5CC8D7B84C":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-EAFB05CA0AE5AFF8B3549A43":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":3},"EVID-F27A7E33A3F59F365A5F2A13":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":11250},"EVID-F597D49E500FDB24F9B8434F":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-F716D2784AE7839470A5204E":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-F9172897F8EA5E1460F7AED3":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-FDB65766E0DDA49AC4DD5518":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0}}</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="AH8" s="14" t="inlineStr">
         <is>
-          <t>SCN-CC786000B1366D95D0796012</t>
+          <t>SCN-11A38429F99045CFB20CD972</t>
         </is>
       </c>
       <c r="AI8" s="15" t="inlineStr">
@@ -3708,12 +3708,12 @@
       </c>
       <c r="BC8" s="22" t="inlineStr">
         <is>
-          <t>["SCN-CC786000B1366D95D0796012","SCN-AE1383D5FC2C30D7B1E8A625"]</t>
+          <t>["SCN-11A38429F99045CFB20CD972","SCN-38846EB94CC8C77FF71512AF"]</t>
         </is>
       </c>
       <c r="BD8" s="22" t="inlineStr">
         <is>
-          <t>["CAND-377F9ED8A2D81DF0AEB07C32","CAND-F183F7D1929B7C7CD565A918","CAND-80AFEAAC17B90B6740091CD3","CAND-0EF3E4718784E98BA23D5C7D","CAND-CEA5FCCDA651DD76B15D02CA","CAND-02A4A2C622C961DA8C1E29A5"]</t>
+          <t>["CAND-E9365F5C153DFAA7DE67E118","CAND-594FA1A7DB150BCEAACADDBB","CAND-0076DB22E0A75900B6DEDFC0","CAND-3E445C7CDDA306563C04C796","CAND-05ACDA7D28A13AAFDF7F3D64","CAND-778A29A01C5B19EC469FD4F6"]</t>
         </is>
       </c>
       <c r="BE8" s="22" t="inlineStr">
@@ -3723,14 +3723,14 @@
       </c>
       <c r="BF8" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-02AC31FADD3A46DDE9AC8672":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":13500},"EVID-038E46D416CD216AAD824440":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":31680.0},"EVID-0464732E6A42CA0F844B4087":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-08768924F23A35F26342A6B5":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":36000.0},"EVID-0E02597D3213CE7CBA74C86C":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5380.16},"EVID-176A781FEEBE5770F9DAEF37":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-18FDAEBFE536A4B00BCC943B":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1200.0},"EVID-1AAD84553C8E637E76730749":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-21D4F887C9029EA0F56850FB":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-243A648173EECA82637526A2":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-32195F4EE7C22EE0A76A24DF":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-324212F35A7011A80C6A6BA3":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-40A178BD1DF4D54686AD685B":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-48F91F49DD6218451135C617":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-4E3921D0FBAE677EEECAE0EB":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-5555686F19810CB742AB7A40":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-5B6C5E71AB278ACD11F995EE":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-5F06B3FDD7ACBB245E6698BA":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-67D867B3C4DDC384C88CCEAC":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-6D9D8B05140A58FCCCC6B21D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-713EACCA2F8126A799E1FE36":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-7708133043264A423E91FC30":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":45.0},"EVID-79435A3C5E9A4B51CF52CEF1":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-801493CED8B276A53FB4E7EB":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-8179BFDB090DED8598025B95":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-82A3C2CACC14A589F634297C":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-8B4057F5428E31CC6A4E717E":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":4500},"EVID-92F3FA13732786DAEE01C242":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-9A22CE6B242B310D6790D2A6":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-A49976C5217F3BD58CB83CF6":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-ACF2755A20123E6FB62F422E":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-AD3A9EEEC8C5F309C7BFFEAA":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AEBBA0A1312EED28C3E7FF6C":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":12.0},"EVID-AED7559DAC9F0BC32BE18F62":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":30.0},"EVID-B568E4C752C9E441A2D4C225":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":12.0},"EVID-B60E91AD0D5EE1DCCDF5E814":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":45.0},"EVID-C0019743301EE0386725FF2D":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1440},"EVID-C39CBA43019A7E2E41D52699":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":15000},"EVID-C773DF3C6AB6E0020A078BA0":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":2160},"EVID-C84D5599AED99E6E15B53363":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-C95E6B1BC4B38F67DDC1C8A3":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":720},"EVID-CC8D27FB8F173BF573F8611E":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-CF2F6C72A37105641E360F0A":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":12.0},"EVID-D5F8E470729DAE096060C377":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-DD117FC3F483E6BEAABBAD0D":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":600.0},"EVID-DE39AAE7BF440BBDEED43AE7":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-E16CE8C168D9485757EF1951":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-EE9A980D23EE91DC1253C3A7":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":254},"EVID-F09C4FC7C53BF57EE512E078":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-F20E29ECD3DB17388D13ADC7":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-F711CDE22C38E70F8CB18F5F":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3600}}</t>
+          <t>{"EVID-02AC31FADD3A46DDE9AC8672":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":13500},"EVID-038E46D416CD216AAD824440":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":31680.0},"EVID-0464732E6A42CA0F844B4087":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-08768924F23A35F26342A6B5":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":36000.0},"EVID-0E02597D3213CE7CBA74C86C":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5380.16},"EVID-176A781FEEBE5770F9DAEF37":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-18FDAEBFE536A4B00BCC943B":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1200.0},"EVID-1AAD84553C8E637E76730749":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-21D4F887C9029EA0F56850FB":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-243A648173EECA82637526A2":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-2EBC5B132CA40C28109BD66A":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-32195F4EE7C22EE0A76A24DF":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-324212F35A7011A80C6A6BA3":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-40A178BD1DF4D54686AD685B":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-48F91F49DD6218451135C617":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-4E3921D0FBAE677EEECAE0EB":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-5555686F19810CB742AB7A40":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-5B6C5E71AB278ACD11F995EE":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-5F06B3FDD7ACBB245E6698BA":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-67D867B3C4DDC384C88CCEAC":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-6D9D8B05140A58FCCCC6B21D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-713EACCA2F8126A799E1FE36":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-7708133043264A423E91FC30":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":45.0},"EVID-79435A3C5E9A4B51CF52CEF1":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-801493CED8B276A53FB4E7EB":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-8179BFDB090DED8598025B95":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-82A3C2CACC14A589F634297C":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-8B4057F5428E31CC6A4E717E":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":4500},"EVID-92F3FA13732786DAEE01C242":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-9A22CE6B242B310D6790D2A6":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-A49976C5217F3BD58CB83CF6":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-ACF2755A20123E6FB62F422E":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-AD3A9EEEC8C5F309C7BFFEAA":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AEBBA0A1312EED28C3E7FF6C":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":12.0},"EVID-AED7559DAC9F0BC32BE18F62":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":30.0},"EVID-B568E4C752C9E441A2D4C225":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":12.0},"EVID-B60E91AD0D5EE1DCCDF5E814":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":45.0},"EVID-C0019743301EE0386725FF2D":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1440},"EVID-C39CBA43019A7E2E41D52699":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":15000},"EVID-C773DF3C6AB6E0020A078BA0":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":2160},"EVID-C84D5599AED99E6E15B53363":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-C95E6B1BC4B38F67DDC1C8A3":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":720},"EVID-CC8D27FB8F173BF573F8611E":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-CF2F6C72A37105641E360F0A":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":12.0},"EVID-D5F8E470729DAE096060C377":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-DD117FC3F483E6BEAABBAD0D":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":600.0},"EVID-DE39AAE7BF440BBDEED43AE7":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-E16CE8C168D9485757EF1951":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-EE9A980D23EE91DC1253C3A7":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":254},"EVID-F09C4FC7C53BF57EE512E078":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-F20E29ECD3DB17388D13ADC7":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-F711CDE22C38E70F8CB18F5F":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3600}}</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="AH9" s="14" t="inlineStr">
         <is>
-          <t>SCN-1B656E36C1F436B2D31FEE71</t>
+          <t>SCN-7B8535F47F089440D4CC3A6C</t>
         </is>
       </c>
       <c r="AI9" s="15" t="inlineStr">
@@ -3946,12 +3946,12 @@
       </c>
       <c r="BC9" s="22" t="inlineStr">
         <is>
-          <t>["SCN-1B656E36C1F436B2D31FEE71","SCN-562458A34AA20834D8E26D00"]</t>
+          <t>["SCN-7B8535F47F089440D4CC3A6C","SCN-ACAFEDE99BA9CDD0084D6217"]</t>
         </is>
       </c>
       <c r="BD9" s="22" t="inlineStr">
         <is>
-          <t>["CAND-8E9FD2A57101E24DC21989E6","CAND-54F63D00E2EFC9427B7F8293","CAND-E0276ED21AF1CA6ABDA3685B","CAND-C84C3FCC5EB73EA428D9DCED","CAND-E390311B2EF9D01C3C6F7D26","CAND-6E8B69CCEE3CE8F4973519A4"]</t>
+          <t>["CAND-1A583E97BA46A3119E6BC8BB","CAND-5BDB30FEB9889EFB8854DA36","CAND-7EAB4FCCBC7AFDB42AB9A6AD","CAND-95461AE6689D3B91CFE81AB8","CAND-161D0B44D8BDFBCB35A95C44","CAND-F9500B9F40B865363F195297"]</t>
         </is>
       </c>
       <c r="BE9" s="22" t="inlineStr">
@@ -3961,14 +3961,14 @@
       </c>
       <c r="BF9" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03E8FAF1FDB44202845A18D1":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0820CEB54C0C9FB6B9F22852":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":1.0},"EVID-1B192ACCE952B9BA66BB97FB":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-2DD59C451FE966A9147AB2F2":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-32A21389C39140EA33B86E25":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-330FF1973264E6F5B82457C4":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-361CBF305B9F3C7406789ACF":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":6750},"EVID-3DC605E1CCF1F51DFFAE7996":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-40DC3FEE74AE4DDCC6F181D7":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":720},"EVID-46C83E93199765E6A01DF9CD":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-4AD9BFC520F810E375C9F267":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-55950F406DCC975F644FF58E":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-565A318F59FE2D81C60059DB":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-5CAA18B018EFF8F0DDE6F929":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-5E83882E9CB63D27C16F478D":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2200},"EVID-5FB552A4A794A6CFE7CAB1F3":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-6B9164B56B380B7F848687D4":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-712DA15CD33F4E642FC88977":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-736AEF23E7ED9DFBA2AA3EED":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":15840.0},"EVID-792B427D8A8CD35CE856A2F0":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-7A91A2021AA57C5F33FA42C6":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-81523112C9E873756ADB144D":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":18000.0},"EVID-82A2364471F4A6799601E11B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":2250},"EVID-8337939F0AFF21D2C6FE2977":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-876511EC79C9ECE935F8ED00":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":360},"EVID-8C8337FFD7A78BAC7F921D11":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-903B0F4B759CBBBEEB13B613":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2333},"EVID-91B0650858728DBD33B126CD":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.2},"EVID-94793DBCDE4FA75AC3E4A69F":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-9B7C8E52FAACFD57E925E970":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-9DB540AB86F707F22A62FCA1":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-A75501B0489D683DBC75D3A9":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":242},"EVID-A7F458AC52E3BD6A823E5DB5":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-AA78D7495831C5BF3781E5B9":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":1.0},"EVID-B20B311CF63DDB084A77C558":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-B22219BB82949C3249DE631C":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-B25114965730FF7335477B28":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-B536175E2D40055600E398E5":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-BCFB1FB057779155A6A6149B":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.2},"EVID-CD0CA3D3B4B2BC5566C1D1F9":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-CE93052A4088BD04DDDFC0B4":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-D05F11599AD06F29F9E033F1":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-D558D8F42F4A30017D8B68C1":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":7},"EVID-D5EF658C7F2298FAC4A62844":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":18},"EVID-D75BC7CEF9C5E360F50654AF":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5646.94},"EVID-E5A742070F6622EF00822E7C":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":62.0},"EVID-F1FF5E3A4AF36A7D16C2F773":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.2},"EVID-F887625EFA3AE63183C78DF3":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-FAA816B37A09EEEF7686D7A7":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7000},"EVID-FCA9DE9BECCD4E0E057474C8":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-FFDE708589B4FB1A37CF7552":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":300.0}}</t>
+          <t>{"EVID-03E8FAF1FDB44202845A18D1":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0820CEB54C0C9FB6B9F22852":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":1.0},"EVID-1B192ACCE952B9BA66BB97FB":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-2DD59C451FE966A9147AB2F2":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-32A21389C39140EA33B86E25":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-32A60495C6A356B84CEDB62C":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-330FF1973264E6F5B82457C4":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-361CBF305B9F3C7406789ACF":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":6750},"EVID-3DC605E1CCF1F51DFFAE7996":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-40DC3FEE74AE4DDCC6F181D7":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":720},"EVID-46C83E93199765E6A01DF9CD":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-4AD9BFC520F810E375C9F267":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-55950F406DCC975F644FF58E":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-565A318F59FE2D81C60059DB":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-5CAA18B018EFF8F0DDE6F929":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-5E83882E9CB63D27C16F478D":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2200},"EVID-5FB552A4A794A6CFE7CAB1F3":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-6B9164B56B380B7F848687D4":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-712DA15CD33F4E642FC88977":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-736AEF23E7ED9DFBA2AA3EED":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":15840.0},"EVID-792B427D8A8CD35CE856A2F0":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-7A91A2021AA57C5F33FA42C6":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-81523112C9E873756ADB144D":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":18000.0},"EVID-82A2364471F4A6799601E11B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":2250},"EVID-8337939F0AFF21D2C6FE2977":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-876511EC79C9ECE935F8ED00":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":360},"EVID-8C8337FFD7A78BAC7F921D11":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-903B0F4B759CBBBEEB13B613":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2333},"EVID-91B0650858728DBD33B126CD":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.2},"EVID-94793DBCDE4FA75AC3E4A69F":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-9B7C8E52FAACFD57E925E970":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-9DB540AB86F707F22A62FCA1":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-A75501B0489D683DBC75D3A9":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":242},"EVID-A7F458AC52E3BD6A823E5DB5":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-AA78D7495831C5BF3781E5B9":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":1.0},"EVID-B20B311CF63DDB084A77C558":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-B22219BB82949C3249DE631C":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-B25114965730FF7335477B28":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-B536175E2D40055600E398E5":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-BCFB1FB057779155A6A6149B":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.2},"EVID-CD0CA3D3B4B2BC5566C1D1F9":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-CE93052A4088BD04DDDFC0B4":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-D05F11599AD06F29F9E033F1":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-D558D8F42F4A30017D8B68C1":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":7},"EVID-D5EF658C7F2298FAC4A62844":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":18},"EVID-D75BC7CEF9C5E360F50654AF":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5646.94},"EVID-E5A742070F6622EF00822E7C":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":62.0},"EVID-F1FF5E3A4AF36A7D16C2F773":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.2},"EVID-F887625EFA3AE63183C78DF3":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-FAA816B37A09EEEF7686D7A7":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7000},"EVID-FCA9DE9BECCD4E0E057474C8":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-FFDE708589B4FB1A37CF7552":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":300.0}}</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="AH10" s="14" t="inlineStr">
         <is>
-          <t>SCN-D7CBE49F5C50DE0E816A9CD2</t>
+          <t>SCN-3F6C04F0A9ED249FBC064295</t>
         </is>
       </c>
       <c r="AI10" s="15" t="inlineStr">
@@ -4184,12 +4184,12 @@
       </c>
       <c r="BC10" s="22" t="inlineStr">
         <is>
-          <t>["SCN-D7CBE49F5C50DE0E816A9CD2","SCN-509F0B84125F5B7EFD41B34F"]</t>
+          <t>["SCN-3F6C04F0A9ED249FBC064295","SCN-B39CD91F38AECF06C4899822"]</t>
         </is>
       </c>
       <c r="BD10" s="22" t="inlineStr">
         <is>
-          <t>["CAND-6B9EEF223CD62A0B0720714A","CAND-F878D946224283BA589FD98A","CAND-8931F3BE78641A385D65130D","CAND-1D1B4EC16ED60AB22768C5E8","CAND-2B65CE34434D627E7C4E7D0B","CAND-5D8E6A15050D0BC21F82DB67"]</t>
+          <t>["CAND-D1C4FA26B6E3600A9A21AC88","CAND-1DF24738E803FAC91A3628A9","CAND-79B0BE87400A9CFA38C8B82A","CAND-61DB2D99CF2B5F9EA7BB61F6","CAND-F05F1CA9672C73FA7DBC8109","CAND-BC13A971B047ACEFA8054A4E"]</t>
         </is>
       </c>
       <c r="BE10" s="22" t="inlineStr">
@@ -4199,14 +4199,14 @@
       </c>
       <c r="BF10" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03C8B5312C5FE9830BDCFF27":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-0FB34E16D22C0DC5D9782A12":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-11AF4398307CE0F6B2C95839":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":36},"EVID-12922A19AF92CAB3AA9714DD":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-12B133BC158CB307238E760D":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-238156F042195E83CB1D7BFD":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":30.0},"EVID-24B0F4C844E49CC0BBF290ED":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-29BAC5FF64717D55401618A4":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2800},"EVID-3169F24E668515676CDAEC06":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-338FBC5F582A0343A81D5D35":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":228},"EVID-34D2BE323D88FEFBD52BC157":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-3B28A16644A2A57DA7060FEB":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-48F5313AC3181ACA7638598F":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-496E780302F53950272CD89F":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-4DBA88B2BC78EFFDE0289BF2":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-4E3B3CFBE454C52D06E172D9":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":72},"EVID-573AE828EB0C16FFBDF39D89":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-5BAB9AE2F58AF32F2026C26F":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-5C6906863C57EB98A8D88F66":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-5F2D4AB39AABF5BAADEEEC14":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-683B1AE13834CF7A72976437":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":14500.0},"EVID-6A828E733BFBF0C431954454":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":12760.0},"EVID-6CDFF811B60AA588BA20E158":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-71FFD313D781A7EB30D0E021":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":3},"EVID-754094313E68ACA0FA861C99":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":11000},"EVID-79E52EE17204D63C325353E3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":6659.65},"EVID-7A0828DFF3D741851110137B":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-7C48F59A969F6B4129C6A6F7":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-84E8ACC912EFD5A45DC90F5F":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-8AF8AB5698F5F3CBA88B0794":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-9BFCB9789587DE8B131F843F":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-9C0887EA9BBD5DE729F8D5C2":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-A0D653C7E7295C8A6FCCA24B":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-A15E47B73E05ED02C3C19CD2":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-A3B4AC4B648CA9BA139F8C4F":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-A41BC0C2030EB101CE85B820":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-A8EFF5F2B461614CF5DBAA12":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-AC454960F83731A41C18B2E6":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-B5C6E9BC8D6DB4E66C7DEC14":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-C0E81BB6EA014B400613A97D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-C3766CBA9521FE51088A3D5D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-C57BD8997AEF9DA09175FE80":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-D279C5B2E8AE57BAA1C94081":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-D563A904AF61289F7E0D5BFE":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-D828BA2B7CE2902D2014DD21":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-D9C2F551D19A9FB621D5851F":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-E22A43BF0CCBA0DC7437C8CC":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-E42C4D645EC2B254E217C4BD":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-F8B206CAB99AC6B2BBEEEB53":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-FBBD7CA62DAF0F3CE7D41AA7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-FCE8F183005B58ACEF7C85B4":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":675}}</t>
+          <t>{"EVID-03C8B5312C5FE9830BDCFF27":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-0FB34E16D22C0DC5D9782A12":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-11AF4398307CE0F6B2C95839":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":36},"EVID-12922A19AF92CAB3AA9714DD":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-12B133BC158CB307238E760D":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-238156F042195E83CB1D7BFD":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":30.0},"EVID-24B0F4C844E49CC0BBF290ED":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-29BAC5FF64717D55401618A4":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2800},"EVID-3169F24E668515676CDAEC06":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-338FBC5F582A0343A81D5D35":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":228},"EVID-34D2BE323D88FEFBD52BC157":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-3B28A16644A2A57DA7060FEB":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-48F5313AC3181ACA7638598F":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-496E780302F53950272CD89F":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-4DBA88B2BC78EFFDE0289BF2":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-4E3B3CFBE454C52D06E172D9":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":72},"EVID-573AE828EB0C16FFBDF39D89":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-5BAB9AE2F58AF32F2026C26F":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-5C6906863C57EB98A8D88F66":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-5F2D4AB39AABF5BAADEEEC14":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-683B1AE13834CF7A72976437":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":14500.0},"EVID-6A828E733BFBF0C431954454":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":12760.0},"EVID-6CDFF811B60AA588BA20E158":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-71FFD313D781A7EB30D0E021":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":3},"EVID-754094313E68ACA0FA861C99":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":11000},"EVID-79E52EE17204D63C325353E3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":6659.65},"EVID-7A0828DFF3D741851110137B":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-7C48F59A969F6B4129C6A6F7":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-7D9F1BB280D23FF7B2FCA3C7":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-84E8ACC912EFD5A45DC90F5F":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-8AF8AB5698F5F3CBA88B0794":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-9BFCB9789587DE8B131F843F":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-9C0887EA9BBD5DE729F8D5C2":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-A0D653C7E7295C8A6FCCA24B":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-A15E47B73E05ED02C3C19CD2":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-A3B4AC4B648CA9BA139F8C4F":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-A41BC0C2030EB101CE85B820":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-A8EFF5F2B461614CF5DBAA12":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-AC454960F83731A41C18B2E6":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-B5C6E9BC8D6DB4E66C7DEC14":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-C0E81BB6EA014B400613A97D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-C3766CBA9521FE51088A3D5D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-C57BD8997AEF9DA09175FE80":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-D279C5B2E8AE57BAA1C94081":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-D563A904AF61289F7E0D5BFE":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-D828BA2B7CE2902D2014DD21":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-D9C2F551D19A9FB621D5851F":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-E22A43BF0CCBA0DC7437C8CC":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-E42C4D645EC2B254E217C4BD":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-F8B206CAB99AC6B2BBEEEB53":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-FBBD7CA62DAF0F3CE7D41AA7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-FCE8F183005B58ACEF7C85B4":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":675}}</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="AA11" s="19" t="n">
-        <v>-176826.67</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="19" t="n">
         <v>0</v>
@@ -4330,14 +4330,14 @@
         <v>163840</v>
       </c>
       <c r="AF11" s="19" t="n">
-        <v>340666.67</v>
+        <v>163840</v>
       </c>
       <c r="AG11" s="20" t="n">
         <v>0</v>
       </c>
       <c r="AH11" s="14" t="inlineStr">
         <is>
-          <t>SCN-41BF7EE984C5C0ED6D4476A1</t>
+          <t>SCN-30936F51711A163A3B65FB99</t>
         </is>
       </c>
       <c r="AI11" s="15" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="AO11" s="16" t="inlineStr">
         <is>
-          <t>OPTIMIZATION_AVAILABLE</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="AP11" s="16" t="inlineStr">
@@ -4388,7 +4388,7 @@
         <v>0</v>
       </c>
       <c r="AT11" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU11" s="17" t="n">
         <v>0</v>
@@ -4403,11 +4403,11 @@
         <v>0</v>
       </c>
       <c r="AY11" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AZ11" s="16" t="inlineStr">
         <is>
-          <t>Size SMALL [NO_CHANGE] | Max 2 [NO_CHANGE] | Min 1 [NO_CHANGE] | Auto-stop 120→30 [BLOCKED] | Type PRO→SERVERLESS [TEST_REQUIRED] | Channel CURRENT [NO_CHANGE]</t>
+          <t>Size SMALL [NO_CHANGE] | Max 2 [NO_CHANGE] | Min 1 [NO_CHANGE] | Auto-stop 120→30 [BLOCKED] | Type PRO [INSUFFICIENT_EVIDENCE] | Channel CURRENT [NO_CHANGE]</t>
         </is>
       </c>
       <c r="BA11" s="16" t="inlineStr">
@@ -4422,12 +4422,12 @@
       </c>
       <c r="BC11" s="22" t="inlineStr">
         <is>
-          <t>["SCN-41BF7EE984C5C0ED6D4476A1","SCN-FDB5EC0875B1F59325F0FADD"]</t>
+          <t>["SCN-30936F51711A163A3B65FB99","SCN-128613E6F87821956FC1EC4B"]</t>
         </is>
       </c>
       <c r="BD11" s="22" t="inlineStr">
         <is>
-          <t>["CAND-BE64253C1F5541854D9D5F73","CAND-D5D6479CF95BC13FC20D6F5F","CAND-754355444A1A789B2EC1DC71","CAND-B2C77C0E282E77BA3CA93FFD","CAND-05ECA8EB06C456A0556818F8","CAND-D1C8429D0D427860A3152AFC"]</t>
+          <t>["CAND-8FC877BAEE26947E63D85BAC","CAND-C2FAFFBA66195CD03818B824","CAND-846E33011FE609606A10FA5B","CAND-20D4E14BE93B700A40985E38","CAND-802B5C5EAE5E3991FDB65CA7","CAND-6B089B819AB4B39987DDEE98"]</t>
         </is>
       </c>
       <c r="BE11" s="22" t="inlineStr">
@@ -4437,14 +4437,14 @@
       </c>
       <c r="BF11" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-07150EBD7C85821371FC5C6D":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-08183391992A779E604BF66F":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-0C9E319B71D62381F589D216":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-11DE4B9E2CE51DBAE4B4614C":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":3},"EVID-164D4D97F7515BF86F925145":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-18637E3CA6358E9E46DF826D":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-1A988C9435A4C646C054795C":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-1C88354197DE4989BF278EC4":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-1DA1B37749AB7CAF629DC62B":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-21CA29942CA50C940F7D85F5":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-222B0A26CEBB4F6CFFCEE77A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-2452143F8B9B2CED497389CF":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-2466A868745928C7FD331536":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-28CD210DF4ED6451A92DA63F":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-2ADB478E1643572CD5941C8A":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-33DCA8B89A2B49AF5DF37795":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-38718E7800609FF827476BF7":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-38E12A59BDB085C9ED17E3D5":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-3BAC65585521CF919E44102B":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-3FC965DD5530031ABE3CF979":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-437994D2A9758FE4A0245CBF":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-43CC9F6E44DCD88D951C6080":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-53C42F047891ECE385CAFC98":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-6F2210B4A714E07FF2B336E5":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-72FB3CFBF04B362625A5DCD4":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":192},"EVID-747CC412E5A28693E648C692":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":1800},"EVID-755CFD7941CE94A93847E0B3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":151840.0},"EVID-7665354F4642CB67866F4828":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-81A9089491437728148A8B5A":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-8938B516CD96332F08779D49":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-935962377953AEF38189FA9F":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2400},"EVID-9F356459A3FA55B3F1CB5D7E":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":96},"EVID-AE59227B08C58DEA635C4681":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":80.0},"EVID-B90BF660B79B024B199EFC4B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":600},"EVID-B990A2C0CB6B6E40A93AD8B6":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-BA5DFBF6A766BB887B518D2D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-BB0A39E40BDCA511D223ED23":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":3},"EVID-C1F4909D7B9F54E1D4FE0B08":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-C39DD2C1AB5242026F7CC137":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-CF2C3BD20C77D10B63ED3718":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8000},"EVID-D6B273BC561A1E053AB22E8C":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":10560.0},"EVID-D933EFAFAF243FC9D57DF4B1":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-D966A16760B03C5442A116EF":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-DAD524D94B365093E6990606":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-DE3386120F2F186DF02F2001":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-E85A4C9B3B5A439FE6F3D488":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-EBCE9854B773D00DADF903B9":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-ECEA4B5972B35E88B483B834":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":12000.0},"EVID-F06B58DBEE8A6313BDCAAB01":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-F50B89D1981BBC41BE24B65F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-FD5E9C86633A3F34080BECF7":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1}}</t>
+          <t>{"EVID-07150EBD7C85821371FC5C6D":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-08183391992A779E604BF66F":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-0C9E319B71D62381F589D216":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-11DE4B9E2CE51DBAE4B4614C":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":3},"EVID-164D4D97F7515BF86F925145":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-18637E3CA6358E9E46DF826D":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-19A0CD94320ACC8CE6577AB0":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-1C88354197DE4989BF278EC4":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-1DA1B37749AB7CAF629DC62B":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-21CA29942CA50C940F7D85F5":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-222B0A26CEBB4F6CFFCEE77A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-242E046D548E372E51BAB181":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-2452143F8B9B2CED497389CF":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-2466A868745928C7FD331536":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-28CD210DF4ED6451A92DA63F":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-2ADB478E1643572CD5941C8A":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-33DCA8B89A2B49AF5DF37795":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-38718E7800609FF827476BF7":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-38E12A59BDB085C9ED17E3D5":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-3FC965DD5530031ABE3CF979":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-437994D2A9758FE4A0245CBF":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-43CC9F6E44DCD88D951C6080":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-53C42F047891ECE385CAFC98":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-6F2210B4A714E07FF2B336E5":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-72FB3CFBF04B362625A5DCD4":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":192},"EVID-747CC412E5A28693E648C692":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":1800},"EVID-755CFD7941CE94A93847E0B3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":151840.0},"EVID-81A9089491437728148A8B5A":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-8938B516CD96332F08779D49":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-8D52106E13681C2F50F82B9E":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-935962377953AEF38189FA9F":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2400},"EVID-9F356459A3FA55B3F1CB5D7E":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":96},"EVID-AE59227B08C58DEA635C4681":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":80.0},"EVID-B90BF660B79B024B199EFC4B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":600},"EVID-B990A2C0CB6B6E40A93AD8B6":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-BA5DFBF6A766BB887B518D2D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-BB0A39E40BDCA511D223ED23":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":3},"EVID-C1F4909D7B9F54E1D4FE0B08":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-C39DD2C1AB5242026F7CC137":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-CF2C3BD20C77D10B63ED3718":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8000},"EVID-D6B273BC561A1E053AB22E8C":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":10560.0},"EVID-D933EFAFAF243FC9D57DF4B1":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-D966A16760B03C5442A116EF":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-DE3386120F2F186DF02F2001":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-DFDC582DDAF10240DA9F7DAE":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-EBCE9854B773D00DADF903B9":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-ECEA4B5972B35E88B483B834":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":12000.0},"EVID-F06B58DBEE8A6313BDCAAB01":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-FD5E9C86633A3F34080BECF7":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1}}</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="AH12" s="14" t="inlineStr">
         <is>
-          <t>SCN-EFE76D0072038BA31048924A</t>
+          <t>SCN-A7F14CD75A7AA486F6E590A9</t>
         </is>
       </c>
       <c r="AI12" s="15" t="inlineStr">
@@ -4656,12 +4656,12 @@
       </c>
       <c r="BC12" s="22" t="inlineStr">
         <is>
-          <t>["SCN-EFE76D0072038BA31048924A","SCN-0DE5AFA24E42CA4905AA2E90"]</t>
+          <t>["SCN-A7F14CD75A7AA486F6E590A9","SCN-010708604C897CBD8CB6999B"]</t>
         </is>
       </c>
       <c r="BD12" s="22" t="inlineStr">
         <is>
-          <t>["CAND-8AE2220BFA703CEB2977138F","CAND-8CF2F68ED84D562D3D9E5560","CAND-D7E581D7637D85BCED1CACDC","CAND-B9252C817CCDE26D5CB43B2C","CAND-EB4C0826388DAF0095655F04","CAND-FF7A26AD3267B8B24B7DDE29"]</t>
+          <t>["CAND-BC0EEDE6473CF891F03E312D","CAND-B1DE4DC4AEBC6BA9039D5664","CAND-AAE2D61246CC19F3D31359B2","CAND-6BE294F5E618F24E926B049B","CAND-627B2620330D84D5C80F1643","CAND-71D893FD78F2362AC4404318"]</t>
         </is>
       </c>
       <c r="BE12" s="22" t="inlineStr">
@@ -4671,14 +4671,14 @@
       </c>
       <c r="BF12" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-010ABDFA627B23B226A3DE39":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":5500},"EVID-01337F937AD5E33DC77EC575":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":0},"EVID-0183D69D139344A5B63A4692":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-0A5EDD910EDA6604A2135A12":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-0B2D8687B4C5CC349527EF25":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-0EFC69DD796CDB2BB3A26C05":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":4},"EVID-1116318FCAEEE6C427983F44":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-13EB4B4FF84410D28683254C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-1556195FEAB1A5CF132FC710":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":5500},"EVID-163D38CEFC5E02464C492820":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":56000.0},"EVID-16D2A9F49BA8DA0CCB7F9646":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":0},"EVID-16F87622F0D96D469B6496DA":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-21334DD8CB15A285F6C275C3":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-2990A0D93C8B36C0E61B4460":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-2EA82A5DF902436D5F2AC6F5":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2F0017120F12F15E975E9770":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-33E061A2CE91CD7F047CEC55":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-3643FB63351B00006C91E749":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1800},"EVID-399A9B3F6C7C397202C68C56":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-4253557C05392B6E40ABDFE2":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-525CBF587D31215B90EBF9D6":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-5608F7EDDD7A89A523D78D43":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":10},"EVID-5DEEAD19532E64C0BBBA64A9":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":100.0},"EVID-6767B2DC53AFEA546EA87194":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-6B64C5D537A164CF2D9E9E83":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-7509E42EBDD3C2025EEECD35":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":269},"EVID-798F548D6E877B362DF24116":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":0.0},"EVID-7C38C1C5C0A50E5541957C70":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-82C9597A7E863C89ACD47773":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":733.33},"EVID-8D49DCB561BC25C03FAD67EC":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-9497EEFAC96FC0FF43049E5A":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-998294748DD31CF5089C376A":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-9A80D9741075BE7C0A437259":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":880},"EVID-A2CEA2EBAACB0B0BC33FA08F":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-A8308230B1476EEE1C7C1CD8":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"SERVERLESS"},"EVID-A8BF0B9309250A74132C5EBD":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-AA18BAE8BDFA353021FAA175":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":10},"EVID-AC8BB4FF1601DC693A4FC67D":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":45760.0},"EVID-AEC33BC02A330A7D397D1BA5":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":0.0},"EVID-B6F105CC07A5E815778807D4":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1760},"EVID-B8F98E64B70FB348AB5F2BB4":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":16500},"EVID-C1EF897F2209F5020FC5E87C":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-D29755684368C6080721CFC3":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-D60301ABD8C8BE18489743FD":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-D9753C2D5E31F0E204F772E6":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":52000.0},"EVID-DA3CD5BE88644D557E028E6B":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-DB06FB4F1E8030A7C256EE4C":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1920.0},"EVID-F4D8D4F24B968E2BDE359E7B":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.0}}</t>
+          <t>{"EVID-010ABDFA627B23B226A3DE39":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":5500},"EVID-01337F937AD5E33DC77EC575":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":0},"EVID-0183D69D139344A5B63A4692":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-0A5EDD910EDA6604A2135A12":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-0B2D8687B4C5CC349527EF25":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-0EFC69DD796CDB2BB3A26C05":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":4},"EVID-1116318FCAEEE6C427983F44":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-13EB4B4FF84410D28683254C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-1556195FEAB1A5CF132FC710":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":5500},"EVID-163D38CEFC5E02464C492820":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":56000.0},"EVID-16D2A9F49BA8DA0CCB7F9646":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":0},"EVID-16F87622F0D96D469B6496DA":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-21334DD8CB15A285F6C275C3":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-2990A0D93C8B36C0E61B4460":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-2EA82A5DF902436D5F2AC6F5":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2F0017120F12F15E975E9770":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-33E061A2CE91CD7F047CEC55":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-3643FB63351B00006C91E749":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1800},"EVID-399A9B3F6C7C397202C68C56":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-4253557C05392B6E40ABDFE2":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-525CBF587D31215B90EBF9D6":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-5608F7EDDD7A89A523D78D43":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":10},"EVID-5DEEAD19532E64C0BBBA64A9":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":100.0},"EVID-6767B2DC53AFEA546EA87194":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-6B64C5D537A164CF2D9E9E83":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-7509E42EBDD3C2025EEECD35":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":269},"EVID-798F548D6E877B362DF24116":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":0.0},"EVID-7C38C1C5C0A50E5541957C70":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-82C9597A7E863C89ACD47773":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":733.33},"EVID-8D49DCB561BC25C03FAD67EC":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-9497EEFAC96FC0FF43049E5A":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-998294748DD31CF5089C376A":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-9A80D9741075BE7C0A437259":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":880},"EVID-A14A6B1ED36B01E84398DF00":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-A2CEA2EBAACB0B0BC33FA08F":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-A8308230B1476EEE1C7C1CD8":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"SERVERLESS"},"EVID-A8BF0B9309250A74132C5EBD":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-AA18BAE8BDFA353021FAA175":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":10},"EVID-AC8BB4FF1601DC693A4FC67D":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":45760.0},"EVID-AEC33BC02A330A7D397D1BA5":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":0.0},"EVID-B6F105CC07A5E815778807D4":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1760},"EVID-B8F98E64B70FB348AB5F2BB4":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":16500},"EVID-C1EF897F2209F5020FC5E87C":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-D29755684368C6080721CFC3":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-D60301ABD8C8BE18489743FD":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-D9753C2D5E31F0E204F772E6":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":52000.0},"EVID-DA3CD5BE88644D557E028E6B":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-DB06FB4F1E8030A7C256EE4C":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1920.0},"EVID-F4D8D4F24B968E2BDE359E7B":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.0}}</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="AH13" s="14" t="inlineStr">
         <is>
-          <t>SCN-2AD1B1369F3CA903C33A7F0A</t>
+          <t>SCN-9082F31BD0DF2BCD069F29F7</t>
         </is>
       </c>
       <c r="AI13" s="15" t="inlineStr">
@@ -4894,12 +4894,12 @@
       </c>
       <c r="BC13" s="22" t="inlineStr">
         <is>
-          <t>["SCN-2AD1B1369F3CA903C33A7F0A","SCN-DB87EC8AF05431F8208079A0"]</t>
+          <t>["SCN-9082F31BD0DF2BCD069F29F7","SCN-0BEADBEFBF7332316DE55F3F"]</t>
         </is>
       </c>
       <c r="BD13" s="22" t="inlineStr">
         <is>
-          <t>["CAND-8C1381C8202F9B850CD6E472","CAND-B91739B640B2882103617ADC","CAND-1416408891B7644B4B970F3D","CAND-EB204DD074336232DC0C1B6A","CAND-FBB76A767C22C2098918D09A","CAND-E299C12314806ACD8AA15BB6"]</t>
+          <t>["CAND-453E404B55579ADA5E3CE252","CAND-03498DA37C2B00C97906A378","CAND-AA7121CBC49CC8D096B1A310","CAND-EF76206E257CE5ED39BC6191","CAND-13F09CD6F23B59AC9235B936","CAND-E16149DF1079E234A70FABFA"]</t>
         </is>
       </c>
       <c r="BE13" s="22" t="inlineStr">
@@ -4909,14 +4909,14 @@
       </c>
       <c r="BF13" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-079EAA62D4D2463F280DD636":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-0C21797178BF0546053B9CCA":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-0C4E337F432378BC4ABF82BB":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":192},"EVID-262B6F32A3311EAB0AEA956E":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":160.0},"EVID-28C27F2BFF375CFAC3A26164":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-2C06AAF783B5BE4F07CD8F11":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-32637602B73B998E62D2015F":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-35D18D87479D58503717BE9C":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3B0B5CEA1E220C0A96409685":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":384},"EVID-407FA82F270C2032644D2CE0":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-4358A7777647777705B43015":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.8},"EVID-44CB7956DAC1F37994F238B8":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-45CE0E82B14BDBD37414D241":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-4C5F394CE1E66392DB372C0E":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-4DF6E5161EC835521DB08092":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-50AC4F920960AAFFE49D6C13":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-544F97BCD83FF9A97476FE07":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":17000.0},"EVID-5755982F8C3E87CBDBBD762F":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":24},"EVID-576AD0041E307AD0E98A8B99":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-5C0183A03D3EB756B2D7C05E":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-605B6814A4D4E829CB5A5B66":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3000},"EVID-7BBFE58EB390ED9CE470DDBA":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":3600},"EVID-7F5D9CC3A93CF86EA6D35DFB":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-82F2F544BF285E0D48F629A2":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-8E55818AEA4051473E4E572D":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-94494E609884DD1061A1BAE8":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-95D1B823E29837B625350057":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-95F3AEE2D4248F3B8729BE25":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-B07C2C16B6BD9A10981E2118":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-B9FCE9EF48F56612B7574032":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-C2BC28961D71AEE7B4624583":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-C2CD370AACFD9F2B4229945B":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-C58346E61AE97D4F760ABDBD":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-CCA0AB4C53A92C8B3916ABDA":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":249},"EVID-CEE3C740E46B3ED08A890FD4":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-D5CE70495019334C5543184A":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":9000},"EVID-D69EE6A78CC33EAA81289A91":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E21F9261CD31D2A21EF533E4":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5488.19},"EVID-E548109D2824FF6673337CE2":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-E6F82DE3524205296B0288DB":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-E7AE32B925F94500C2F12FF9":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-EDC048377DB26691E0C059FB":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":85000},"EVID-EDD11801F242C17DD64F2799":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-F061026BE78747696C1238CE":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-F48024947EFAAED048529938":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F62D3E7730D5A803CE342120":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-F6A16121002CAEDD32814FF8":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":14960.0},"EVID-FA09B298BBED0188E79849C7":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-FA632D73262B55CF827D5211":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-FD670F422E4B757BEE0194C6":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":1200},"EVID-FE12840F9CF6363CB2E50AE5":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0}}</t>
+          <t>{"EVID-079EAA62D4D2463F280DD636":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-0C21797178BF0546053B9CCA":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-0C4E337F432378BC4ABF82BB":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":192},"EVID-262B6F32A3311EAB0AEA956E":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":160.0},"EVID-28C27F2BFF375CFAC3A26164":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-2C06AAF783B5BE4F07CD8F11":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-32637602B73B998E62D2015F":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-35D18D87479D58503717BE9C":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3B0B5CEA1E220C0A96409685":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":384},"EVID-3CBD002DD8F60BA15CC1ACF8":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-407FA82F270C2032644D2CE0":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-4358A7777647777705B43015":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.8},"EVID-44CB7956DAC1F37994F238B8":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-45CE0E82B14BDBD37414D241":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-4C5F394CE1E66392DB372C0E":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-4DF6E5161EC835521DB08092":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-50AC4F920960AAFFE49D6C13":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-544F97BCD83FF9A97476FE07":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":17000.0},"EVID-5755982F8C3E87CBDBBD762F":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":24},"EVID-576AD0041E307AD0E98A8B99":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-5C0183A03D3EB756B2D7C05E":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-605B6814A4D4E829CB5A5B66":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3000},"EVID-7BBFE58EB390ED9CE470DDBA":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":3600},"EVID-7F5D9CC3A93CF86EA6D35DFB":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-82F2F544BF285E0D48F629A2":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-8E55818AEA4051473E4E572D":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-94494E609884DD1061A1BAE8":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-95D1B823E29837B625350057":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-95F3AEE2D4248F3B8729BE25":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-B07C2C16B6BD9A10981E2118":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-B9FCE9EF48F56612B7574032":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-C2BC28961D71AEE7B4624583":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-C2CD370AACFD9F2B4229945B":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-C58346E61AE97D4F760ABDBD":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-CCA0AB4C53A92C8B3916ABDA":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":249},"EVID-CEE3C740E46B3ED08A890FD4":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-D5CE70495019334C5543184A":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":9000},"EVID-D69EE6A78CC33EAA81289A91":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E21F9261CD31D2A21EF533E4":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5488.19},"EVID-E548109D2824FF6673337CE2":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-E6F82DE3524205296B0288DB":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-E7AE32B925F94500C2F12FF9":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-EDC048377DB26691E0C059FB":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":85000},"EVID-EDD11801F242C17DD64F2799":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-F061026BE78747696C1238CE":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-F48024947EFAAED048529938":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F62D3E7730D5A803CE342120":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-F6A16121002CAEDD32814FF8":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":14960.0},"EVID-FA09B298BBED0188E79849C7":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-FA632D73262B55CF827D5211":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-FD670F422E4B757BEE0194C6":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":1200},"EVID-FE12840F9CF6363CB2E50AE5":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0}}</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="AH14" s="14" t="inlineStr">
         <is>
-          <t>SCN-3ADBD372252C701E8605FDBF</t>
+          <t>SCN-0AF33099B977B44DE891DB2F</t>
         </is>
       </c>
       <c r="AI14" s="15" t="inlineStr">
@@ -5132,12 +5132,12 @@
       </c>
       <c r="BC14" s="22" t="inlineStr">
         <is>
-          <t>["SCN-3ADBD372252C701E8605FDBF","SCN-3B15D95786681E2F1586255E"]</t>
+          <t>["SCN-0AF33099B977B44DE891DB2F","SCN-85DD6FDC4F7D607B91486DB3"]</t>
         </is>
       </c>
       <c r="BD14" s="22" t="inlineStr">
         <is>
-          <t>["CAND-6DAADF5C7A000999BB0EF2C1","CAND-44783D6FD480C2752BDBEC25","CAND-F66CC7C521D489A9BFE5369C","CAND-062229819F3FCAD00A4C42F2","CAND-184A3C392690D298B3EFD5E3","CAND-D3DD9FFE6744CCBBA9B4F934"]</t>
+          <t>["CAND-94B14CEE087AE61D01782199","CAND-6A591F792934B6D67437E104","CAND-75EEB2BB4814F605DFACC0A5","CAND-E538FA9D2E0002740D3A8291","CAND-1BF6312BDBD011BCBF5B17DD","CAND-208C05A9E348D11DAEE662DF"]</t>
         </is>
       </c>
       <c r="BE14" s="22" t="inlineStr">
@@ -5147,14 +5147,14 @@
       </c>
       <c r="BF14" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-026EA0A0C1CDA6D5BF6861E0":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-05E65620367F546ED7403371":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-100EE4E12A042B6CA6801300":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":1.0},"EVID-147B3F71E2FD2C372C751AA6":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":37670.23},"EVID-14D5F3273317129C41786ABC":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-1BB42907159AF707FE39C5B1":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":35.0},"EVID-1BFCD956061A5FF8AD162D6A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-1C01A17AAD8C207EF44692C1":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-1D9D72AFBDB7C1DC2B552C1B":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2805E2CB0E21815B548E32C4":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-36E316B362E683D130437B68":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":784},"EVID-38E4F9656837EFDE5FDBF34F":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-45040C819E97E97C0C3512DD":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-4A7E1844228F5FD433A998C6":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":392},"EVID-4FC2DA089D8E1230B40C62EC":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-51A58BE39546BE7B080FEF30":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-55EEA56CA02C609E862A91A9":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-5701A1693763AB907ED13F14":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-5DC3FDBE1BD0729F52CEC22D":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":7350},"EVID-5DCBE726277C51C2DE2EA638":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-61487496034534522AE52030":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":412},"EVID-63B44F71C0B9A791C79ACFAE":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-692C1AED9F82E4D968155B44":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":15.0},"EVID-774DFFF76A9BF347776727F1":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":36000},"EVID-7A4AC35DF8C26AD31C26B498":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":15.0},"EVID-84BB9FB2CC3C791B8780F9FD":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-8A2CA1F2CB0AE069280E449E":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-8F7E3338B58CABACD8A8F19C":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-9061C8B86A3E064D3068DD57":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":1.0},"EVID-961B35C0E85521646A2B48D9":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":2147483648},"EVID-9B8E1FCFDF764EB620F8627C":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-A0E6420717F746163C350A0E":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-A6B0629AF776267EC1BEFD1C":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-B14E29B030DF322078D9574C":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-B243D5AFB2596AB542DE4D0B":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-BE99070B2138778FAD6323C4":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-BF652AC51560329CFD9C0449":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":45},"EVID-BFABA7FE5F4CD649CD8BB5CF":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-C0985AE59F5D8278110173AD":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":11000},"EVID-C65E409498DAAC26BC9A7E6C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-CE5AAF49B736110C9BABD5DF":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":326.67},"EVID-D3B52F66FCD31062B1B0A0B3":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":1.0},"EVID-DE93964EDC1B9E5DCF7EDE95":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-E537D70782B304C239A5C196":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":58000.0},"EVID-E9763030D2ED61047B419AFA":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-EB4062CC3E2A9EE53D82DCE2":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":51040.0},"EVID-EC1BD88B388D79E675C955D2":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":98},"EVID-ECDDE17AA397C1C6C3A2165D":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-F434EE37F0A085340B6B5BEE":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":262},"EVID-F6050662637ABA0BDC2DBA35":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-FA3E117294ACCCC7A8F86BE4":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":4.2}}</t>
+          <t>{"EVID-026EA0A0C1CDA6D5BF6861E0":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-05E65620367F546ED7403371":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-100EE4E12A042B6CA6801300":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":1.0},"EVID-147B3F71E2FD2C372C751AA6":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":37670.23},"EVID-14D5F3273317129C41786ABC":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-1BB42907159AF707FE39C5B1":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":35.0},"EVID-1BFCD956061A5FF8AD162D6A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-1C01A17AAD8C207EF44692C1":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-1D9D72AFBDB7C1DC2B552C1B":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2805E2CB0E21815B548E32C4":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-36E316B362E683D130437B68":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":784},"EVID-38E4F9656837EFDE5FDBF34F":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-45040C819E97E97C0C3512DD":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-4A7E1844228F5FD433A998C6":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":392},"EVID-4FC2DA089D8E1230B40C62EC":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-51A58BE39546BE7B080FEF30":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-55EEA56CA02C609E862A91A9":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-5701A1693763AB907ED13F14":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-5DC3FDBE1BD0729F52CEC22D":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":7350},"EVID-5DCBE726277C51C2DE2EA638":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-61487496034534522AE52030":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":412},"EVID-63B44F71C0B9A791C79ACFAE":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-692C1AED9F82E4D968155B44":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":15.0},"EVID-774DFFF76A9BF347776727F1":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":36000},"EVID-7A4AC35DF8C26AD31C26B498":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":15.0},"EVID-84BB9FB2CC3C791B8780F9FD":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-8A2CA1F2CB0AE069280E449E":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-8F7E3338B58CABACD8A8F19C":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-9061C8B86A3E064D3068DD57":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":1.0},"EVID-961B35C0E85521646A2B48D9":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":2147483648},"EVID-9B8E1FCFDF764EB620F8627C":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-A0E6420717F746163C350A0E":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-A6B0629AF776267EC1BEFD1C":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-B14E29B030DF322078D9574C":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-B243D5AFB2596AB542DE4D0B":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-BE99070B2138778FAD6323C4":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-BF652AC51560329CFD9C0449":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":45},"EVID-BFABA7FE5F4CD649CD8BB5CF":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-C0985AE59F5D8278110173AD":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":11000},"EVID-C65E409498DAAC26BC9A7E6C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-C66F1B2AC854BD459A280659":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-CE5AAF49B736110C9BABD5DF":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":326.67},"EVID-D3B52F66FCD31062B1B0A0B3":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":1.0},"EVID-DE93964EDC1B9E5DCF7EDE95":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-E537D70782B304C239A5C196":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":58000.0},"EVID-E9763030D2ED61047B419AFA":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-EB4062CC3E2A9EE53D82DCE2":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":51040.0},"EVID-EC1BD88B388D79E675C955D2":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":98},"EVID-ECDDE17AA397C1C6C3A2165D":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-F434EE37F0A085340B6B5BEE":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":262},"EVID-F6050662637ABA0BDC2DBA35":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-FA3E117294ACCCC7A8F86BE4":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":4.2}}</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="AH15" s="14" t="inlineStr">
         <is>
-          <t>SCN-BBAAF3154665B37B8FCEA1E0</t>
+          <t>SCN-2933621CB20E77E39795A10D</t>
         </is>
       </c>
       <c r="AI15" s="15" t="inlineStr">
@@ -5370,12 +5370,12 @@
       </c>
       <c r="BC15" s="22" t="inlineStr">
         <is>
-          <t>["SCN-BBAAF3154665B37B8FCEA1E0","SCN-4C7F7B95C214EEBF380310D5"]</t>
+          <t>["SCN-2933621CB20E77E39795A10D","SCN-8CEE26C6FC4807B9693BC3A5"]</t>
         </is>
       </c>
       <c r="BD15" s="22" t="inlineStr">
         <is>
-          <t>["CAND-1531D4BD13B32E9441CF326C","CAND-B6913E34C50A503A1D6DBEA0","CAND-573D056D65CE4249801B3E1C","CAND-C1A802D5E5BEE703D8ED0085","CAND-0F14BBC11AE756EB5AFB1C96","CAND-53AF57B05EB45846CF76155B"]</t>
+          <t>["CAND-B18907413D2DF98545B33865","CAND-BBB38F2B1B9EA80282892372","CAND-75C376C9ADCC22E111CF436A","CAND-97D73C8B9AB1304A39EE9B0D","CAND-2B92AC15169DEA8C2A7CFA89","CAND-1B05132C1EC3D2449969E905"]</t>
         </is>
       </c>
       <c r="BE15" s="22" t="inlineStr">
@@ -5385,14 +5385,14 @@
       </c>
       <c r="BF15" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-01B0931797AD8E53145A691A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0D810E83CECE50954A7A685C":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-0ED6F46984B7429965251DFA":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-13D5BCA568FCB7051CE9D79D":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-16B432383FD0DDFEE4D012AE":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-1B042AC3F3DC722F7CBD7EFC":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-1DD7A19B3B0DF4143675E5FB":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-2C1A5879F6C5D019F73F53CF":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-2ECCAF2DEB31C4E6DA63B160":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-3A343CC6FF17D49FC9AD677E":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-407B8B7358879E2BF927FBC7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-4D0620980296070C0F13B308":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-4DE0BBBC3685DD0789E6ABE6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-507A4213371D1C316C1CC988":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":15500.0},"EVID-5461C38656FC772B05732F94":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-5F732C6BD12B85E05433189C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-634399DEE70438016F07F4AE":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-6BD43BFD6ABCD42659E7A67E":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-71AA2350F44ED33F293E9415":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-790EAB5EC858806D654BE4C3":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-7C5B36553FD4D6F24464AAE3":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-83C49754DBFBB0A3F73A8DF0":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-898523B3F6F9EF7659721E39":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-8DCFC6A0FCF3F29EDAC2E7F6":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":13640.0},"EVID-9EAB95FAF297AB482EC4BEDA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3615.24},"EVID-A0DF30623A058D588E6D05E6":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-A247506597147334B7EBC5FA":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-A385D4A375B81956644C007B":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":256},"EVID-A77090CFFE32A7F60C21BF7A":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-AAC19684A130CEDB6899D5A4":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-AAF37F5753DFBD8265CBC705":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":106.67},"EVID-B0F8165F4ECE68C2CAF2F705":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-B25BA1B63DF47E9357C97990":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-B45065D6E10A3C07E0278909":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":128},"EVID-B9988C289DDAA9B7B6A22290":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":800},"EVID-BA44DE5A4FFD511819D160D3":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":252},"EVID-BB24712E336B1DE6544A9089":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":90.0},"EVID-BFECCAA5C954B839B41B3F78":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-C051B133A3F60F2431CCB46B":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-C1A290503A730A2597E04F4F":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-D204E6427AA6DB80225C18CF":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-D68F79CF3972CCE5B1DFCEAD":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-DB0003F618B6A5F1F058A80A":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2000},"EVID-DF9F879685D647BC4173CCB3":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":2400},"EVID-EB0482919E76BABE5679717F":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-F130A53A660169C51BDDECBF":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-F3295EDE47B1C510743F895B":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-F68E95D9A0280257191BA4C5":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-F83AD8E314550D8512193F6A":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6000},"EVID-F9465E0B062F91CEDE4AB7CB":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F9A9C7240302A09DAA7D6DD6":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0}}</t>
+          <t>{"EVID-01B0931797AD8E53145A691A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0D810E83CECE50954A7A685C":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-0ED6F46984B7429965251DFA":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-13D5BCA568FCB7051CE9D79D":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-16B432383FD0DDFEE4D012AE":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-1B042AC3F3DC722F7CBD7EFC":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-1DD7A19B3B0DF4143675E5FB":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-2C1A5879F6C5D019F73F53CF":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-2ECCAF2DEB31C4E6DA63B160":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-3A343CC6FF17D49FC9AD677E":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-407B8B7358879E2BF927FBC7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-4D0620980296070C0F13B308":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-4DE0BBBC3685DD0789E6ABE6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-507A4213371D1C316C1CC988":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":15500.0},"EVID-5461C38656FC772B05732F94":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-5F732C6BD12B85E05433189C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-634399DEE70438016F07F4AE":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-6BD43BFD6ABCD42659E7A67E":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-71AA2350F44ED33F293E9415":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-790EAB5EC858806D654BE4C3":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-7C5B36553FD4D6F24464AAE3":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-83C49754DBFBB0A3F73A8DF0":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-898523B3F6F9EF7659721E39":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-8DCFC6A0FCF3F29EDAC2E7F6":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":13640.0},"EVID-9EAB95FAF297AB482EC4BEDA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3615.24},"EVID-A0DF30623A058D588E6D05E6":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-A247506597147334B7EBC5FA":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-A385D4A375B81956644C007B":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":256},"EVID-A77090CFFE32A7F60C21BF7A":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-AAC19684A130CEDB6899D5A4":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-AAF37F5753DFBD8265CBC705":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":106.67},"EVID-B0F8165F4ECE68C2CAF2F705":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-B25BA1B63DF47E9357C97990":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-B45065D6E10A3C07E0278909":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":128},"EVID-B9988C289DDAA9B7B6A22290":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":800},"EVID-BA44DE5A4FFD511819D160D3":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":252},"EVID-BB24712E336B1DE6544A9089":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":90.0},"EVID-BFECCAA5C954B839B41B3F78":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-C051B133A3F60F2431CCB46B":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-C1A290503A730A2597E04F4F":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-D204E6427AA6DB80225C18CF":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-D68F79CF3972CCE5B1DFCEAD":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-DB0003F618B6A5F1F058A80A":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2000},"EVID-DF9F879685D647BC4173CCB3":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":2400},"EVID-EB0482919E76BABE5679717F":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-F130A53A660169C51BDDECBF":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-F3295EDE47B1C510743F895B":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-F68E95D9A0280257191BA4C5":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-F83AD8E314550D8512193F6A":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6000},"EVID-F9465E0B062F91CEDE4AB7CB":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F9A9C7240302A09DAA7D6DD6":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-FABB267EC471BEB44A231F3C":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3}}</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="AH16" s="14" t="inlineStr">
         <is>
-          <t>SCN-B1AE3151CA3DFABC9D6F87A2</t>
+          <t>SCN-DC5D9238399C6A5D0C16D1D5</t>
         </is>
       </c>
       <c r="AI16" s="15" t="inlineStr">
@@ -5608,12 +5608,12 @@
       </c>
       <c r="BC16" s="22" t="inlineStr">
         <is>
-          <t>["SCN-B1AE3151CA3DFABC9D6F87A2","SCN-7AA042130907C622B3D829D7"]</t>
+          <t>["SCN-DC5D9238399C6A5D0C16D1D5","SCN-D6AA6A4FA46862F6334FBC5C"]</t>
         </is>
       </c>
       <c r="BD16" s="22" t="inlineStr">
         <is>
-          <t>["CAND-68B1A41A04A2F7483EAD9565","CAND-3B94CC5756DFC0077D2E12FE","CAND-F89285A886F733FCF48A39F5","CAND-924103D11A79912AF1188F2F","CAND-30A07501B51A2AE278F7EA92","CAND-AD58D34434A2170D1BF1A9B1"]</t>
+          <t>["CAND-7841A56D1EF08AEECA9362E6","CAND-D830ED375B9F86AA1F381EA4","CAND-DB36510075A8FBE14B50458C","CAND-0630B601A39B1E7F3ABDB138","CAND-5784A0970E1A5BFDF92DD2BB","CAND-D2AA37F564A2D82B828401D3"]</t>
         </is>
       </c>
       <c r="BE16" s="22" t="inlineStr">
@@ -5623,14 +5623,14 @@
       </c>
       <c r="BF16" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-05A39DE059C813C193661F07":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-075DC68712355A8DD4FE2603":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":22880.0},"EVID-0B236E96CFAADEA401D485D8":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-15C90A7069D97FFBF27141F6":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-1ACA7C8B9A9A293BE5CFEE4E":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":433.33},"EVID-1DD41E094BAD58A2025478A3":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-20B74C71235026CB1006D75D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-22BEC328AA4A66999655C284":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-23B98DC198C1A8170F8F9A99":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-25BA1C551957EAD856D93BB1":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7200},"EVID-27BF4F675CF47BE7ED7D92A7":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2981DA47184B33DAA0E0AEF3":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-2EB24474879263CAA7D55388":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-34338326D5389EC2477F90A1":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-4B8B2B525621ED89EA20CBB7":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-4D7719F0DCD578A9F64A53CF":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-4E5FAEE78D56DFC97676075D":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-51ABDD6192C632754DC043A4":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-51ED3C0701E326D181DDCBAD":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2100},"EVID-52F379B326B48A163DAD8F0B":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-5410112DFBC342DF891DBF46":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-54CEC3840D90DC23AE1DDB39":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-560228B799DA72762556AD39":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":520},"EVID-58873DCCF86A22B7C49B25C7":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-5A0984690AB60FAD1E646F57":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-5CE253A6ED0C92F5F4B58920":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-6E3CC48635A168300AFD9101":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-7470F3D044066BB776AA7526":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-7CBF6F506E34E48BF4007E49":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-7D9BF92BB726FFBAED23FE74":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5338.12},"EVID-818918115DFD85F2025E4AB5":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-8446876BD86846BC5B4A09B1":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-900367C6FD27EF69401875BB":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-987E8FBCED5AD351FFAAAA33":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":58.0},"EVID-9A48289F39C4CBF84AFA056D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-9C01DEB2842095BB47EE5CDE":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9750},"EVID-A0EDCF34958103470FFB3138":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1040},"EVID-AEAB494D17C5B4B7C451733A":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3250},"EVID-B272FC69B2AFFDD9F8CAA0ED":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-B497C3FF5ED3D8789DC6D823":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-BDE0805A170B0A4C92D6B573":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-C1B2C572B41553D2862081B7":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-C531CFB4DE60DA5DFFD90F03":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":256},"EVID-D09849AFFFB193163A0F1547":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-D3629BE0A19E65713B480452":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":26000.0},"EVID-D686C6BEE50D1122355032D0":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-DAD23F3F252736320B90B610":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DBA319585E47DD744C7C91FE":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-EAC15F6872ADFF0F3C60D54F":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-EC30765FCC5CC089BFE85916":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-F48AEEBA5FE65654FE81C0FC":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}}}</t>
+          <t>{"EVID-05A39DE059C813C193661F07":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-075DC68712355A8DD4FE2603":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":22880.0},"EVID-0B236E96CFAADEA401D485D8":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-15C90A7069D97FFBF27141F6":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-1ACA7C8B9A9A293BE5CFEE4E":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":433.33},"EVID-1DD41E094BAD58A2025478A3":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-20B74C71235026CB1006D75D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-22BEC328AA4A66999655C284":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-23B98DC198C1A8170F8F9A99":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-25BA1C551957EAD856D93BB1":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7200},"EVID-27BF4F675CF47BE7ED7D92A7":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2981DA47184B33DAA0E0AEF3":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-2EB24474879263CAA7D55388":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-34338326D5389EC2477F90A1":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-4B8B2B525621ED89EA20CBB7":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-4D7719F0DCD578A9F64A53CF":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-4E5FAEE78D56DFC97676075D":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-51ABDD6192C632754DC043A4":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-51ED3C0701E326D181DDCBAD":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2100},"EVID-52F379B326B48A163DAD8F0B":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-5410112DFBC342DF891DBF46":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-54CEC3840D90DC23AE1DDB39":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-560228B799DA72762556AD39":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":520},"EVID-58873DCCF86A22B7C49B25C7":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-5A0984690AB60FAD1E646F57":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-5CE253A6ED0C92F5F4B58920":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-6E3CC48635A168300AFD9101":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-7470F3D044066BB776AA7526":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-7CBF6F506E34E48BF4007E49":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-7D9BF92BB726FFBAED23FE74":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5338.12},"EVID-818918115DFD85F2025E4AB5":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-8446876BD86846BC5B4A09B1":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-900367C6FD27EF69401875BB":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-987E8FBCED5AD351FFAAAA33":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":58.0},"EVID-9A48289F39C4CBF84AFA056D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-9C01DEB2842095BB47EE5CDE":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9750},"EVID-A0EDCF34958103470FFB3138":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1040},"EVID-AEAB494D17C5B4B7C451733A":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3250},"EVID-B272FC69B2AFFDD9F8CAA0ED":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-B497C3FF5ED3D8789DC6D823":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-BDE0805A170B0A4C92D6B573":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-C1B2C572B41553D2862081B7":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-C531CFB4DE60DA5DFFD90F03":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":256},"EVID-D09849AFFFB193163A0F1547":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-D3629BE0A19E65713B480452":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":26000.0},"EVID-D686C6BEE50D1122355032D0":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-DAD23F3F252736320B90B610":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DBA319585E47DD744C7C91FE":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-EAC15F6872ADFF0F3C60D54F":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-EC30765FCC5CC089BFE85916":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-EF8F9819481D98F6C8919AB9":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-F48AEEBA5FE65654FE81C0FC":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}}}</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="AH17" s="14" t="inlineStr">
         <is>
-          <t>SCN-C7D4A73498A01E43CF2F1F99</t>
+          <t>SCN-999C878D6C51D4B139B49A57</t>
         </is>
       </c>
       <c r="AI17" s="15" t="inlineStr">
@@ -5846,12 +5846,12 @@
       </c>
       <c r="BC17" s="22" t="inlineStr">
         <is>
-          <t>["SCN-C7D4A73498A01E43CF2F1F99","SCN-C2B8462C39C6CBF67EA76272"]</t>
+          <t>["SCN-999C878D6C51D4B139B49A57","SCN-F5B38DFE81B5D7BBAF6911B1"]</t>
         </is>
       </c>
       <c r="BD17" s="22" t="inlineStr">
         <is>
-          <t>["CAND-36E93BF7B8CE7895B3350359","CAND-4D7163BFB57F1D099F93FBB4","CAND-E4FE1A1917EE61ADF0A90DD5","CAND-580A5D1DBAA9FF66F3497081","CAND-A69115976DE8B2D6CED3E2F9","CAND-0E7487FBA4179110E052404A"]</t>
+          <t>["CAND-FC7B2860CAAD03861AED5C53","CAND-61D8612587ADCC0F68698112","CAND-07075A2AF6885F9116290675","CAND-2FEA25EDC5E48395071F4EF6","CAND-0B255F5C4039607F30C4EE4A","CAND-C8B97E03CD532E0571F1A2F5"]</t>
         </is>
       </c>
       <c r="BE17" s="22" t="inlineStr">
@@ -5861,14 +5861,14 @@
       </c>
       <c r="BF17" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-058D81357EB5272C1DE9ED9B":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-07174CC5836579556EAE3FBA":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":18480.0},"EVID-15BC98689FE74269E3463311":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-19826A02AE03B4A846113469":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-1D08ADE1876B67CB8F50C528":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-223C7D3604E9DF00A1BEF7CC":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-25C1DA18EEB5F16EA1C37494":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-2CD27BF63AFEE3E528EEE1A4":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-2E961C8C26A8DD4D880DC0C3":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-36D86A2F5E0936332A1B2820":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-39C9D8D68FDB2B48EC1F8E06":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":4200},"EVID-3A43D2B90A2ADDC63154F1DC":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3BFFD13E796C679EC14F7CA3":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":2.0},"EVID-3FBBE1F8B66451E76AC07E04":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-43A9D4AA27211AD241140DA8":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":21000.0},"EVID-44A8E6640DAD4631893F4EB9":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-469489F4837B65DD18F63C9D":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-473DAE924D0494843A151322":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-4B7D594AEF10EB1994631521":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-4FF74009A0DFB40815A0A413":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-57A759616BDD3E869A9BD1B6":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":5400},"EVID-5821F563D2CDBB6D2A1B7AF1":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":2.0},"EVID-5F049D088166930E912ED0CA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":2932.53},"EVID-61E092FB1CF8E0D4F83E7C75":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-65D1AD0CE53C4B489DEF9257":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-814B842EA1F2BD7336C2E67C":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":233},"EVID-8A92D5F7019BF02D403BCB98":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-8C834AFA4684E60064532F4A":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-8F2AFB31A724A7DCC1A017B4":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-978B04F1AA38AA4C2EF6D66F":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-9B5F3B007AF6B0C87B636B00":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-A360A570EBEE8B5F549A53E0":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-A8479D37C2BD6296B01193CA":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":7},"EVID-A8A9397A693D4D562A86DAC3":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-B05D9F6F28424A0150AE0161":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-C45D5F5AEEEFC5D7036ABEFB":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-CA2FD32DD6DA1B4179B6677F":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":288},"EVID-D74AEF3FA0511AE5AC0CDAD8":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-D7B86E8FA15817630DB367C9":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-D84F7646519258747323D10D":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-DCDF95C6A1F733063FB0FF40":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-DFCDBC00C82164F40BF36FB7":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-E02CC741A5434D31B5A71083":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":576},"EVID-E09655B4C8E5A7904441CDAF":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-E0A9E6F5CF1C6CC89EF49539":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":16000},"EVID-E11EAFF1B6EDF5B5DA7152A2":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-E6197B84E314F1E28F08BB9E":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-ECA8EC5793FCAC7E93A8CB70":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-F06D6C88947D665948ED9A70":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":240.0},"EVID-F508A01058EA0B6B9B6F94A6":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-FEA1A86964875B556D58A600":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"}}</t>
+          <t>{"EVID-058D81357EB5272C1DE9ED9B":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-07174CC5836579556EAE3FBA":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":18480.0},"EVID-15BC98689FE74269E3463311":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-19826A02AE03B4A846113469":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-1D08ADE1876B67CB8F50C528":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-223C7D3604E9DF00A1BEF7CC":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-25C1DA18EEB5F16EA1C37494":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-2CD27BF63AFEE3E528EEE1A4":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-2E961C8C26A8DD4D880DC0C3":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-36D86A2F5E0936332A1B2820":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-39C9D8D68FDB2B48EC1F8E06":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":4200},"EVID-3A43D2B90A2ADDC63154F1DC":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3BFFD13E796C679EC14F7CA3":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":2.0},"EVID-3FBBE1F8B66451E76AC07E04":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-43A9D4AA27211AD241140DA8":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":21000.0},"EVID-44A8E6640DAD4631893F4EB9":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-469489F4837B65DD18F63C9D":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-473DAE924D0494843A151322":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-4B7D594AEF10EB1994631521":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-4FF74009A0DFB40815A0A413":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-57A759616BDD3E869A9BD1B6":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":5400},"EVID-5821F563D2CDBB6D2A1B7AF1":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":2.0},"EVID-5F049D088166930E912ED0CA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":2932.53},"EVID-61E092FB1CF8E0D4F83E7C75":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-65D1AD0CE53C4B489DEF9257":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-814B842EA1F2BD7336C2E67C":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":233},"EVID-8A92D5F7019BF02D403BCB98":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-8C834AFA4684E60064532F4A":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-8F2AFB31A724A7DCC1A017B4":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-978B04F1AA38AA4C2EF6D66F":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-9B5F3B007AF6B0C87B636B00":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-A360A570EBEE8B5F549A53E0":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-A8479D37C2BD6296B01193CA":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":7},"EVID-A8A9397A693D4D562A86DAC3":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-AE5017E437240372E2E797B8":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-B05D9F6F28424A0150AE0161":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-C45D5F5AEEEFC5D7036ABEFB":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-CA2FD32DD6DA1B4179B6677F":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":288},"EVID-D74AEF3FA0511AE5AC0CDAD8":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-D7B86E8FA15817630DB367C9":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-D84F7646519258747323D10D":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-DCDF95C6A1F733063FB0FF40":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-DFCDBC00C82164F40BF36FB7":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-E02CC741A5434D31B5A71083":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":576},"EVID-E09655B4C8E5A7904441CDAF":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-E0A9E6F5CF1C6CC89EF49539":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":16000},"EVID-E11EAFF1B6EDF5B5DA7152A2":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-E6197B84E314F1E28F08BB9E":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-ECA8EC5793FCAC7E93A8CB70":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-F06D6C88947D665948ED9A70":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":240.0},"EVID-F508A01058EA0B6B9B6F94A6":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-FEA1A86964875B556D58A600":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"}}</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -5999,7 +5999,7 @@
       </c>
       <c r="AH18" s="14" t="inlineStr">
         <is>
-          <t>SCN-90F84EEF462106B503D5FCD5</t>
+          <t>SCN-21882722E00BEBBB1248C9B9</t>
         </is>
       </c>
       <c r="AI18" s="15" t="inlineStr">
@@ -6084,12 +6084,12 @@
       </c>
       <c r="BC18" s="22" t="inlineStr">
         <is>
-          <t>["SCN-90F84EEF462106B503D5FCD5","SCN-C76B1BF0BE04F2268A48C457"]</t>
+          <t>["SCN-21882722E00BEBBB1248C9B9","SCN-C2EBBB483BA454145E5C3C56"]</t>
         </is>
       </c>
       <c r="BD18" s="22" t="inlineStr">
         <is>
-          <t>["CAND-48E992E09B6FDDDA184620BB","CAND-7AD7357E0749467C6A7B878C","CAND-4AD0C5CF56FFE443109E075C","CAND-49A88561475837189D75A95B","CAND-CBCF6ED4CDF8B9664828018A","CAND-0CF01F172DB34D3AE5983193"]</t>
+          <t>["CAND-C4A7C16CD04A96235E2A96F0","CAND-C5123BB77CACC1CED8BB907A","CAND-BF43E30DCCBF2197D86C4A47","CAND-C51D33CA45FD919D45D2C3AC","CAND-5C6283E0FB5D37B9AF951A35","CAND-C83A18C81BA3F8F01454DD46"]</t>
         </is>
       </c>
       <c r="BE18" s="22" t="inlineStr">
@@ -6099,14 +6099,14 @@
       </c>
       <c r="BF18" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0645324E21523AC72540EBFB":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":122},"EVID-0BA05DFEDB55A3C639CBDE3C":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":11.25},"EVID-11E47EFC2708CBFEDD50ADF5":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-195F46F60FABA88715E01BF8":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-2005A26A4E686F61F138D184":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-2717985C1ABCB4F82F0C3207":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-277695726D78445956FE494F":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-2D1C834F33B47D7C597813BC":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3757B07B85F990B0A9264097":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-376B961B29D12F53A747A949":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":33},"EVID-3BE897690A2172D19236EC85":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":5},"EVID-3DCBC6489AC48EDCE794F393":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-3E185CE21A5B0320DDCB65EB":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-406AF2C15F491C90EC38F696":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-473C88A56036CF4722376661":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-48AD911004D78BC5B629A2CD":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-48B5752A7517C832C6F13F16":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-4B624F4A3B3E05F869CEBB81":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-4E79642ADEB6BD83CF237522":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-5B91767FD693F50EFD0576F7":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-60929AEB71973AE52157CA34":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-6D0F865829FDA770BA2D1F50":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-7A436410CF1C8EE2567C00A8":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-7C1343FE613D1C19015BD7B1":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-803FE025612A1F6D4A58355B":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-81BB2260DF67AC5CE9D9AEF5":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.5},"EVID-82F8B6438164A878220C92CF":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-86F8174A6943E8D4F2C7FAFE":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":3},"EVID-877CBDBF73660A76F7D7B906":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-8945206B7EFE7B399B2C2E7E":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":2816.0},"EVID-8BFB6DBCD41163D4975AC2D0":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-9094DED8046D5939494E72F6":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":4000},"EVID-90E0282E95C7A75CCA70207C":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-93044B07330628C211B83BB0":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-9C5BA1A542982FAA1650BA7C":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":45.0},"EVID-9D5FF441E9A83BA2016A7779":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":3200.0},"EVID-A39D869989EE20E8F0FA4661":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-AA062B5DFCC4DBB6962C7CA9":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1600},"EVID-AA1588DBCF52F271FDBDC1CB":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-AF2A27B54B6E2E92040B22C3":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-BB70599C732C9AF2C89E8F69":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3733.77},"EVID-BFA6C64A9A6B80359A92DDCF":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-C0FDA37896D08BB3EC313B88":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-C93E53FFBF15C2C059DD7551":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-CF1D42DA66B6EDAFCB6EBB2A":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-D3C92F624741AE9991AFF968":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":2},"EVID-DF7FBF457C19FB28EF5FD820":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-ED017CC07FEB8357DD377236":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F0FEE41C0A094A7E4BC8355D":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-F289972C47C0295FAC5F5901":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F306F90358EC1E71F324BC0D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0}}</t>
+          <t>{"EVID-0645324E21523AC72540EBFB":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":122},"EVID-0BA05DFEDB55A3C639CBDE3C":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":11.25},"EVID-11E47EFC2708CBFEDD50ADF5":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-195F46F60FABA88715E01BF8":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-2005A26A4E686F61F138D184":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-2717985C1ABCB4F82F0C3207":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-277695726D78445956FE494F":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-2BE3AE8039A7B379DAA21484":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-2D1C834F33B47D7C597813BC":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-3757B07B85F990B0A9264097":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-376B961B29D12F53A747A949":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":33},"EVID-3BE897690A2172D19236EC85":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":5},"EVID-3DCBC6489AC48EDCE794F393":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-3E185CE21A5B0320DDCB65EB":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-406AF2C15F491C90EC38F696":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-473C88A56036CF4722376661":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-48AD911004D78BC5B629A2CD":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-48B5752A7517C832C6F13F16":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-4B624F4A3B3E05F869CEBB81":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-4E79642ADEB6BD83CF237522":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-5B91767FD693F50EFD0576F7":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-60929AEB71973AE52157CA34":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-6D0F865829FDA770BA2D1F50":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-7A436410CF1C8EE2567C00A8":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-7C1343FE613D1C19015BD7B1":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-803FE025612A1F6D4A58355B":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-81BB2260DF67AC5CE9D9AEF5":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.5},"EVID-82F8B6438164A878220C92CF":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-86F8174A6943E8D4F2C7FAFE":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":3},"EVID-877CBDBF73660A76F7D7B906":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-8945206B7EFE7B399B2C2E7E":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":2816.0},"EVID-8BFB6DBCD41163D4975AC2D0":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-9094DED8046D5939494E72F6":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":4000},"EVID-90E0282E95C7A75CCA70207C":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-93044B07330628C211B83BB0":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-9C5BA1A542982FAA1650BA7C":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":45.0},"EVID-9D5FF441E9A83BA2016A7779":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":3200.0},"EVID-A39D869989EE20E8F0FA4661":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-AA062B5DFCC4DBB6962C7CA9":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1600},"EVID-AA1588DBCF52F271FDBDC1CB":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-AF2A27B54B6E2E92040B22C3":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-BB70599C732C9AF2C89E8F69":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3733.77},"EVID-BFA6C64A9A6B80359A92DDCF":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-C0FDA37896D08BB3EC313B88":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-C93E53FFBF15C2C059DD7551":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-CF1D42DA66B6EDAFCB6EBB2A":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-D3C92F624741AE9991AFF968":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":2},"EVID-DF7FBF457C19FB28EF5FD820":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-ED017CC07FEB8357DD377236":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F0FEE41C0A094A7E4BC8355D":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-F289972C47C0295FAC5F5901":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-F306F90358EC1E71F324BC0D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0}}</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="AH19" s="14" t="inlineStr">
         <is>
-          <t>SCN-CD13BC97911EDD734CF17B6B</t>
+          <t>SCN-5F795672B44D350C3E296BF1</t>
         </is>
       </c>
       <c r="AI19" s="15" t="inlineStr">
@@ -6322,12 +6322,12 @@
       </c>
       <c r="BC19" s="22" t="inlineStr">
         <is>
-          <t>["SCN-CD13BC97911EDD734CF17B6B","SCN-D90F0090AC8A9492249F19B8"]</t>
+          <t>["SCN-5F795672B44D350C3E296BF1","SCN-871471461B50CF97B71AE728"]</t>
         </is>
       </c>
       <c r="BD19" s="22" t="inlineStr">
         <is>
-          <t>["CAND-73A72B66CCC5DF6F66CAC2FE","CAND-20A04702FCD63664C07653A5","CAND-9ADFC70F5FC112A2499B5375","CAND-F52F904EE62AFA4706B94D7E","CAND-C08CF1BBC9ECD83993F5BCE2","CAND-A33DFC4B60027DE5B92ED694"]</t>
+          <t>["CAND-ACCF6F438E9B7DD1C243642F","CAND-2ABC4239192B22E3E0541016","CAND-ACA9A2EEB098AFFFB5C5CDD7","CAND-F7FAB3EBC34F7F42BB4CB9AB","CAND-5BD0417FF74CCA4CE750987C","CAND-254186ED0FFA404D809AF606"]</t>
         </is>
       </c>
       <c r="BE19" s="22" t="inlineStr">
@@ -6337,7 +6337,7 @@
       </c>
       <c r="BF19" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-04AFCA0AAC20E78DB30EAB77":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-05DD86E0F6613765BFBA1E18":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":8793.82},"EVID-07A2D8FB5FCCD61519B96CC3":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-0D49EBE0456D3AC0425D6040":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-15E61DCCCDC9640AEECEDE52":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-168734B9927A9EB76E8DD271":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-21BAEB92A93F4EA1EFA4BE25":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-25018FD718DF5EACF142F830":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":5},"EVID-2A52B7303B96A6106B59F7DD":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":11},"EVID-2B410DD070DE49F4BA280AC0":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-2D14233C22D92C6645004C4B":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-2ED156DA3F1E6A8E1ECD0756":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-30684DDD3BC0545735D7BE84":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":880},"EVID-35105E35476552EC4996467A":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-44114512A244D39710D4F01E":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-4D2EA7CDCF00512B9AD8016B":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-53CBA2DB88E1E98F95E78F57":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-5744D477056B6D4DDA2B3C9A":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":33000.0},"EVID-6697A43FF1953B6DD17B7E3A":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-76A6F57147432ADF9195AB8A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-76CC7EFCB0C616F7636449A1":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2300},"EVID-8061388EF01AF88966780FE8":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-813B76ABCC2E92AFB79A8CEC":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-86522A92DD2115BE645B0597":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-8749654928EDA932BF981D0D":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-93FF7D4EC33F9B836AB6A5B1":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":440},"EVID-94A443A0D3C916891029D716":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-97BB222802772AFEA5FAD120":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-992E8BC51B6B9DAF16486239":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-A8BE846EED36B67068AA40E0":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":29040.0},"EVID-ABE50E8BB95F0A3555F82500":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-AE8923033C2E33B284017783":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":65.0},"EVID-AF279CE943239F24018B7A6B":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-AFCCD0D5FA6B5D57006462F7":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-B4DC16A94706160A1FD2D15E":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-BA8A411AD317A6E434A8FB8B":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":366.67},"EVID-BD5A2CE5E7D1A27A48EA67AD":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":8250},"EVID-C5ED523E62D944AA6BE91E28":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-C6A2F9009A7F7A4E149AD155":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-CB895D6D4CF4E45D8C39BD25":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-CDF4EEEA440FFA47B7C7CA28":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-CE464D57463AF05E9E2B1B2E":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-D83B486744833AA5B4728EAA":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8500},"EVID-D9FA7D75F1F9F500B957BAF9":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-DA02736184DF2A70345CF47D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-EBE7FEB8EDF8384AFCA4023F":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-EDFF0EB8D8E64AA2F579F299":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-F45B3F25E72C93572E60D363":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-F7616687094FA66C2BA94FEF":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-F7625C8D7909DB61C7DD76C3":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-FB2B4A65C10DA970E465C7C5":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}}}</t>
+          <t>{"EVID-04AFCA0AAC20E78DB30EAB77":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-05DD86E0F6613765BFBA1E18":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":8793.82},"EVID-07A2D8FB5FCCD61519B96CC3":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-0D49EBE0456D3AC0425D6040":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-15E61DCCCDC9640AEECEDE52":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-168734B9927A9EB76E8DD271":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-21BAEB92A93F4EA1EFA4BE25":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-25018FD718DF5EACF142F830":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":5},"EVID-2A52B7303B96A6106B59F7DD":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":11},"EVID-2B410DD070DE49F4BA280AC0":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-2D14233C22D92C6645004C4B":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-2ED156DA3F1E6A8E1ECD0756":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-30684DDD3BC0545735D7BE84":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":880},"EVID-35105E35476552EC4996467A":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-44114512A244D39710D4F01E":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-4BF5518163DAD5705703F01C":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-4D2EA7CDCF00512B9AD8016B":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-53CBA2DB88E1E98F95E78F57":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-5744D477056B6D4DDA2B3C9A":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":33000.0},"EVID-6697A43FF1953B6DD17B7E3A":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-76A6F57147432ADF9195AB8A":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-76CC7EFCB0C616F7636449A1":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2300},"EVID-8061388EF01AF88966780FE8":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-813B76ABCC2E92AFB79A8CEC":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-86522A92DD2115BE645B0597":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-8749654928EDA932BF981D0D":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-93FF7D4EC33F9B836AB6A5B1":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":440},"EVID-94A443A0D3C916891029D716":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-97BB222802772AFEA5FAD120":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-992E8BC51B6B9DAF16486239":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-A8BE846EED36B67068AA40E0":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":29040.0},"EVID-ABE50E8BB95F0A3555F82500":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-AE8923033C2E33B284017783":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":65.0},"EVID-AF279CE943239F24018B7A6B":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-AFCCD0D5FA6B5D57006462F7":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-B4DC16A94706160A1FD2D15E":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-BA8A411AD317A6E434A8FB8B":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":366.67},"EVID-BD5A2CE5E7D1A27A48EA67AD":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":8250},"EVID-C5ED523E62D944AA6BE91E28":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-C6A2F9009A7F7A4E149AD155":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-CB895D6D4CF4E45D8C39BD25":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-CDF4EEEA440FFA47B7C7CA28":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-CE464D57463AF05E9E2B1B2E":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-D83B486744833AA5B4728EAA":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8500},"EVID-D9FA7D75F1F9F500B957BAF9":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-DA02736184DF2A70345CF47D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-EBE7FEB8EDF8384AFCA4023F":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-EDFF0EB8D8E64AA2F579F299":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-F45B3F25E72C93572E60D363":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-F7616687094FA66C2BA94FEF":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-F7625C8D7909DB61C7DD76C3":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-FB2B4A65C10DA970E465C7C5":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}}}</t>
         </is>
       </c>
     </row>
@@ -7129,12 +7129,12 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SCN-F6C96142718566E6610757F4</t>
+          <t>SCN-E1D619112BE62AFA050EA71A</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -7290,12 +7290,12 @@
       </c>
       <c r="AP5" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-CDC9DD7E27E8CA6ED23E9CEB","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-4CD23256DB0CA20822638058","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-F7CD1FD114943EA1AAB92DF2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":8207.57,"high":11021.59,"low":4690.04},"dbu":{"base":10241.38,"high":23648.28,"low":-6517.24},"total":{"base":18448.95,"high":34669.87,"low":-1827.2}}},"recommended_value":1,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-1EB011ABA71F8CF380C298A8","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":9252.28,"high":11725.1,"low":5386.51},"dbu":{"base":15218.69,"high":27000.0,"low":-3199.03},"total":{"base":24470.97,"high":38725.1,"low":2187.48}}},"recommended_value":30,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-DAC9E910F2A94A05B67B302A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-567E1FFD79E2F9A61A59510F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-585D0C22F7A86D37CE5BCDE5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":8207.57,"high":11021.59,"low":4690.04},"dbu":{"base":10241.38,"high":23648.28,"low":-6517.24},"total":{"base":18448.95,"high":34669.87,"low":-1827.2}}},"recommended_value":1,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-B72E480BD8ADA0BAAADDB594","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":9252.28,"high":11725.1,"low":5386.51},"dbu":{"base":15218.69,"high":27000.0,"low":-3199.03},"total":{"base":24470.97,"high":38725.1,"low":2187.48}}},"recommended_value":30,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ5" s="22" t="inlineStr">
         <is>
-          <t>["CAND-CDC9DD7E27E8CA6ED23E9CEB","CAND-4CD23256DB0CA20822638058","CAND-F7CD1FD114943EA1AAB92DF2","CAND-1EB011ABA71F8CF380C298A8"]</t>
+          <t>["CAND-DAC9E910F2A94A05B67B302A","CAND-567E1FFD79E2F9A61A59510F","CAND-585D0C22F7A86D37CE5BCDE5","CAND-B72E480BD8ADA0BAAADDB594"]</t>
         </is>
       </c>
       <c r="AR5" s="22" t="inlineStr">
@@ -7312,12 +7312,12 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SCN-4CE208EB461A228615816740</t>
+          <t>SCN-B49B73B0344B4AF52B454990</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -7479,12 +7479,12 @@
       </c>
       <c r="AP6" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-78762B303EA11AF80300E2C3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":11725.1,"high":11725.1,"low":11725.1},"dbu":{"base":693.69,"high":13846.85,"low":693.69},"total":{"base":12418.79,"high":25571.95,"low":12418.79}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-D7C2183B68BBD711C74005C7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":11725.1,"high":11725.1,"low":11725.1},"dbu":{"base":693.69,"high":13846.85,"low":693.69},"total":{"base":12418.79,"high":25571.95,"low":12418.79}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ6" s="22" t="inlineStr">
         <is>
-          <t>["CAND-78762B303EA11AF80300E2C3"]</t>
+          <t>["CAND-D7C2183B68BBD711C74005C7"]</t>
         </is>
       </c>
       <c r="AR6" s="22" t="inlineStr">
@@ -7501,12 +7501,12 @@
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SCN-CB5E8798D5A13F523639541D</t>
+          <t>SCN-2EEA487274E8B4C2D2A00C65</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -7662,12 +7662,12 @@
       </c>
       <c r="AP7" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-F6DA76343C4F0EEC6747DD79","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"X_LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-19440.12,"high":7476.97,"low":-59815.76},"dbu":{"base":-25600.0,"high":0.0,"low":-64000.0},"total":{"base":-45040.12,"high":7476.97,"low":-123815.76}}},"recommended_value":"2X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-A122082B3BB2FB0568C91BF4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13849.65,"high":14930.93,"low":-56088.78},"dbu":{"base":-20283.08,"high":7089.23,"low":-60455.38},"total":{"base":-34132.73,"high":22020.16,"low":-116544.16}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-3107EA199EA58282439B64F2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"X_LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-19440.12,"high":7476.97,"low":-59815.76},"dbu":{"base":-25600.0,"high":0.0,"low":-64000.0},"total":{"base":-45040.12,"high":7476.97,"low":-123815.76}}},"recommended_value":"2X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-CDA61DCEC36313DD1885DFD7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13849.65,"high":14930.93,"low":-56088.78},"dbu":{"base":-20283.08,"high":7089.23,"low":-60455.38},"total":{"base":-34132.73,"high":22020.16,"low":-116544.16}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ7" s="22" t="inlineStr">
         <is>
-          <t>["CAND-F6DA76343C4F0EEC6747DD79","CAND-A122082B3BB2FB0568C91BF4"]</t>
+          <t>["CAND-3107EA199EA58282439B64F2","CAND-CDA61DCEC36313DD1885DFD7"]</t>
         </is>
       </c>
       <c r="AR7" s="22" t="inlineStr">
@@ -7684,12 +7684,12 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SCN-AF126D31FABFB5905E6640A4</t>
+          <t>SCN-69AD699F056B046156191604</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -7851,12 +7851,12 @@
       </c>
       <c r="AP8" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-335D8BD4AAC3CB041A5DB0CB","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":74769.7,"high":74769.7,"low":74769.7},"dbu":{"base":-103752.53,"high":38191.92,"low":-116656.57},"total":{"base":-28982.83,"high":112961.62,"low":-41886.87}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-5FD3D0884B03CB55AFDD5092","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":74769.7,"high":74769.7,"low":74769.7},"dbu":{"base":-103752.53,"high":38191.92,"low":-116656.57},"total":{"base":-28982.83,"high":112961.62,"low":-41886.87}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ8" s="22" t="inlineStr">
         <is>
-          <t>["CAND-335D8BD4AAC3CB041A5DB0CB"]</t>
+          <t>["CAND-5FD3D0884B03CB55AFDD5092"]</t>
         </is>
       </c>
       <c r="AR8" s="22" t="inlineStr">
@@ -7873,12 +7873,12 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SCN-CE4B0C3CDE2534722A4AAADE</t>
+          <t>SCN-F7FD9602740588A931526FB1</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -8034,12 +8034,12 @@
       </c>
       <c r="AP9" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-C86EF28A42FC56DB5AD00959","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-0B0E829222AD5BA2CA4E7612","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":6,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":4,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-E2B81BBFEB2D221645C6CC57","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":14219.04,"high":18646.52,"low":8514.39},"dbu":{"base":15028.97,"high":35685.52,"low":-11586.21},"total":{"base":29248.01,"high":54332.04,"low":-3071.82}}},"recommended_value":2,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-028FA513EA788FFB1FAADF4E","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":15975.13,"high":20987.98,"low":9685.12},"dbu":{"base":23222.07,"high":46609.66,"low":-6124.14},"total":{"base":39197.2,"high":67597.64,"low":3560.98}}},"recommended_value":45,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-FF852A8F55F23A58470A0F50","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-6A370586BC9EDB6A5FE47F5D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":6,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":4,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-6F350B226F959664414114EB","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":14219.04,"high":18646.52,"low":8514.39},"dbu":{"base":15028.97,"high":35685.52,"low":-11586.21},"total":{"base":29248.01,"high":54332.04,"low":-3071.82}}},"recommended_value":2,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-99A7041317161930A14478B9","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":15975.13,"high":20987.98,"low":9685.12},"dbu":{"base":23222.07,"high":46609.66,"low":-6124.14},"total":{"base":39197.2,"high":67597.64,"low":3560.98}}},"recommended_value":45,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ9" s="22" t="inlineStr">
         <is>
-          <t>["CAND-C86EF28A42FC56DB5AD00959","CAND-0B0E829222AD5BA2CA4E7612","CAND-E2B81BBFEB2D221645C6CC57","CAND-028FA513EA788FFB1FAADF4E"]</t>
+          <t>["CAND-FF852A8F55F23A58470A0F50","CAND-6A370586BC9EDB6A5FE47F5D","CAND-6F350B226F959664414114EB","CAND-99A7041317161930A14478B9"]</t>
         </is>
       </c>
       <c r="AR9" s="22" t="inlineStr">
@@ -8056,12 +8056,12 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SCN-68F9545F52E814CE6E2CDC73</t>
+          <t>SCN-260783C9E116C39D21DA207C</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -8223,12 +8223,12 @@
       </c>
       <c r="AP10" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-B994ABE33118C0EA458EFC1D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":21285.98,"high":21285.98,"low":21285.98},"dbu":{"base":242.99,"high":32081.0,"low":242.99},"total":{"base":21528.97,"high":53366.98,"low":21528.97}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-99EF846309D3820B9095938B","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":21285.98,"high":21285.98,"low":21285.98},"dbu":{"base":242.99,"high":32081.0,"low":242.99},"total":{"base":21528.97,"high":53366.98,"low":21528.97}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ10" s="22" t="inlineStr">
         <is>
-          <t>["CAND-B994ABE33118C0EA458EFC1D"]</t>
+          <t>["CAND-99EF846309D3820B9095938B"]</t>
         </is>
       </c>
       <c r="AR10" s="22" t="inlineStr">
@@ -8245,12 +8245,12 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SCN-CC786000B1366D95D0796012</t>
+          <t>SCN-11A38429F99045CFB20CD972</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -8412,12 +8412,12 @@
       </c>
       <c r="AP11" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-80AFEAAC17B90B6740091CD3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"READY","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-807.02,"high":0.0,"low":-1614.05},"dbu":{"base":-5400.0,"high":0.0,"low":-10800.0},"total":{"base":-6207.02,"high":0.0,"low":-12414.05}}},"recommended_value":3,"step":1,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-INCREASE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":2,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-0076DB22E0A75900B6DEDFC0","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"READY","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-807.02,"high":0.0,"low":-1614.05},"dbu":{"base":-5400.0,"high":0.0,"low":-10800.0},"total":{"base":-6207.02,"high":0.0,"low":-12414.05}}},"recommended_value":3,"step":1,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-INCREASE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":2,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ11" s="22" t="inlineStr">
         <is>
-          <t>["CAND-80AFEAAC17B90B6740091CD3"]</t>
+          <t>["CAND-0076DB22E0A75900B6DEDFC0"]</t>
         </is>
       </c>
       <c r="AR11" s="22" t="inlineStr">
@@ -8434,12 +8434,12 @@
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SCN-AE1383D5FC2C30D7B1E8A625</t>
+          <t>SCN-38846EB94CC8C77FF71512AF</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -8601,12 +8601,12 @@
       </c>
       <c r="AP12" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-02A4A2C622C961DA8C1E29A5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5380.16,"high":5380.16,"low":5380.16},"dbu":{"base":23929.13,"high":27952.76,"low":19905.51},"total":{"base":29309.29,"high":33332.92,"low":25285.67}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-778A29A01C5B19EC469FD4F6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5380.16,"high":5380.16,"low":5380.16},"dbu":{"base":23929.13,"high":27952.76,"low":19905.51},"total":{"base":29309.29,"high":33332.92,"low":25285.67}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ12" s="22" t="inlineStr">
         <is>
-          <t>["CAND-02A4A2C622C961DA8C1E29A5"]</t>
+          <t>["CAND-778A29A01C5B19EC469FD4F6"]</t>
         </is>
       </c>
       <c r="AR12" s="22" t="inlineStr">
@@ -8623,12 +8623,12 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SCN-1B656E36C1F436B2D31FEE71</t>
+          <t>SCN-7B8535F47F089440D4CC3A6C</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -8784,12 +8784,12 @@
       </c>
       <c r="AP13" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-54F63D00E2EFC9427B7F8293","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-E0276ED21AF1CA6ABDA3685B","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-5BDB30FEB9889EFB8854DA36","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-7EAB4FCCBC7AFDB42AB9A6AD","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ13" s="22" t="inlineStr">
         <is>
-          <t>["CAND-54F63D00E2EFC9427B7F8293","CAND-E0276ED21AF1CA6ABDA3685B"]</t>
+          <t>["CAND-5BDB30FEB9889EFB8854DA36","CAND-7EAB4FCCBC7AFDB42AB9A6AD"]</t>
         </is>
       </c>
       <c r="AR13" s="22" t="inlineStr">
@@ -8806,12 +8806,12 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SCN-562458A34AA20834D8E26D00</t>
+          <t>SCN-ACAFEDE99BA9CDD0084D6217</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -8973,12 +8973,12 @@
       </c>
       <c r="AP14" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-6E8B69CCEE3CE8F4973519A4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5646.94,"high":5646.94,"low":5646.94},"dbu":{"base":5330.58,"high":9553.72,"low":1107.44},"total":{"base":10977.52,"high":15200.66,"low":6754.38}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-F9500B9F40B865363F195297","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5646.94,"high":5646.94,"low":5646.94},"dbu":{"base":5330.58,"high":9553.72,"low":1107.44},"total":{"base":10977.52,"high":15200.66,"low":6754.38}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ14" s="22" t="inlineStr">
         <is>
-          <t>["CAND-6E8B69CCEE3CE8F4973519A4"]</t>
+          <t>["CAND-F9500B9F40B865363F195297"]</t>
         </is>
       </c>
       <c r="AR14" s="22" t="inlineStr">
@@ -8995,12 +8995,12 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SCN-D7CBE49F5C50DE0E816A9CD2</t>
+          <t>SCN-3F6C04F0A9ED249FBC064295</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -9156,12 +9156,12 @@
       </c>
       <c r="AP15" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-F878D946224283BA589FD98A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-8931F3BE78641A385D65130D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":2,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-2B65CE34434D627E7C4E7D0B","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":5379.0,"high":6659.65,"low":3674.79},"dbu":{"base":8731.0,"high":14500.0,"low":1054.0},"total":{"base":14110.0,"high":21159.65,"low":4728.79}}},"recommended_value":15,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-1DF24738E803FAC91A3628A9","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-79B0BE87400A9CFA38C8B82A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":2,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-F05F1CA9672C73FA7DBC8109","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":5379.0,"high":6659.65,"low":3674.79},"dbu":{"base":8731.0,"high":14500.0,"low":1054.0},"total":{"base":14110.0,"high":21159.65,"low":4728.79}}},"recommended_value":15,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ15" s="22" t="inlineStr">
         <is>
-          <t>["CAND-F878D946224283BA589FD98A","CAND-8931F3BE78641A385D65130D","CAND-2B65CE34434D627E7C4E7D0B"]</t>
+          <t>["CAND-1DF24738E803FAC91A3628A9","CAND-79B0BE87400A9CFA38C8B82A","CAND-F05F1CA9672C73FA7DBC8109"]</t>
         </is>
       </c>
       <c r="AR15" s="22" t="inlineStr">
@@ -9178,12 +9178,12 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SCN-509F0B84125F5B7EFD41B34F</t>
+          <t>SCN-B39CD91F38AECF06C4899822</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -9345,12 +9345,12 @@
       </c>
       <c r="AP16" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-5D8E6A15050D0BC21F82DB67","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6659.65,"high":6659.65,"low":6659.65},"dbu":{"base":-441.52,"high":-441.52,"low":-441.52},"total":{"base":6218.13,"high":6218.13,"low":6218.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-BC13A971B047ACEFA8054A4E","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6659.65,"high":6659.65,"low":6659.65},"dbu":{"base":-441.52,"high":-441.52,"low":-441.52},"total":{"base":6218.13,"high":6218.13,"low":6218.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ16" s="22" t="inlineStr">
         <is>
-          <t>["CAND-5D8E6A15050D0BC21F82DB67"]</t>
+          <t>["CAND-BC13A971B047ACEFA8054A4E"]</t>
         </is>
       </c>
       <c r="AR16" s="22" t="inlineStr">
@@ -9367,12 +9367,12 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>SCN-41BF7EE984C5C0ED6D4476A1</t>
+          <t>SCN-30936F51711A163A3B65FB99</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -9558,12 +9558,12 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>SCN-FDB5EC0875B1F59325F0FADD</t>
+          <t>SCN-128613E6F87821956FC1EC4B</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -9588,12 +9588,12 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>Plan B — Serverless migration experiment</t>
+          <t>Plan B — Pro migration experiment</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>WAREHOUSE_TYPE_MIGRATION</t>
+          <t>IN_PLACE_OPTIMIZATION</t>
         </is>
       </c>
       <c r="I18" s="18" t="inlineStr">
@@ -9605,11 +9605,11 @@
         <v>0</v>
       </c>
       <c r="K18" s="21" t="n">
-        <v>0.61</v>
+        <v>1</v>
       </c>
       <c r="L18" s="18" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="M18" s="16" t="inlineStr">
@@ -9634,7 +9634,7 @@
       </c>
       <c r="Q18" s="18" t="inlineStr">
         <is>
-          <t>COST_INCREASE</t>
+          <t>NO_CHANGE</t>
         </is>
       </c>
       <c r="R18" s="19" t="n">
@@ -9647,44 +9647,44 @@
         <v>163840</v>
       </c>
       <c r="U18" s="19" t="n">
-        <v>-328666.67</v>
+        <v>0</v>
       </c>
       <c r="V18" s="19" t="n">
-        <v>-328666.67</v>
+        <v>0</v>
       </c>
       <c r="W18" s="19" t="n">
-        <v>-328666.67</v>
+        <v>0</v>
       </c>
       <c r="X18" s="19" t="n">
-        <v>151840</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="19" t="n">
-        <v>151840</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="19" t="n">
-        <v>151840</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="19" t="n">
-        <v>-176826.67</v>
+        <v>0</v>
       </c>
       <c r="AB18" s="19" t="n">
-        <v>-176826.67</v>
+        <v>0</v>
       </c>
       <c r="AC18" s="19" t="n">
-        <v>-176826.67</v>
+        <v>0</v>
       </c>
       <c r="AD18" s="19" t="n">
-        <v>340666.67</v>
+        <v>163840</v>
       </c>
       <c r="AE18" s="19" t="n">
-        <v>340666.67</v>
+        <v>163840</v>
       </c>
       <c r="AF18" s="19" t="n">
-        <v>340666.67</v>
+        <v>163840</v>
       </c>
       <c r="AG18" s="16" t="inlineStr">
         <is>
-          <t>PRE_CANARY_MODELED_RANGE</t>
+          <t>NO_DELTA_MODELED</t>
         </is>
       </c>
       <c r="AH18" s="19" t="inlineStr">
@@ -9704,33 +9704,35 @@
       </c>
       <c r="AK18" s="16" t="inlineStr">
         <is>
-          <t>Plan B — Serverless migration experiment | 1. VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY [REQUIRED] | 2. warehouse_type PRO→SERVERLESS [READY_FOR_CANARY]; priced AUTHORITATIVE | 3. REMEASURE_AND_REGENERATE [REQUIRED]; remeasure 7d</t>
+          <t>Plan B — Pro migration experiment</t>
         </is>
       </c>
       <c r="AL18" s="18" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM18" s="17" t="n">
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="AM18" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="AN18" s="22" t="inlineStr">
         <is>
-          <t>[{"check":"aws_region_serverless_availability","details":"{\"policy\":\"Databricks documents Serverless SQL warehouse support across AWS regions.\",\"region\":\"us-east-1\"}","evidence_refs":["EVID-F50B89D1981BBC41BE24B65F"],"requires_hitl":false,"status":"PASS"},{"check":"workspace_serverless_observed","details":"true","evidence_refs":["EVID-DAD524D94B365093E6990606"],"requires_hitl":false,"status":"PASS"},{"check":"workspace_serverless_enablement","details":"true","evidence_refs":["EVID-1A988C9435A4C646C054795C"],"requires_hitl":false,"status":"PASS"},{"check":"external_legacy_hive_metastore_workspace_setting","details":"{\"config_keys\":[],\"detected\":false}","evidence_refs":["EVID-7665354F4642CB67866F4828"],"requires_hitl":false,"status":"PASS"},{"check":"s3_access_policy_compatibility","details":"\"UNKNOWN\"","evidence_refs":["EVID-E85A4C9B3B5A439FE6F3D488"],"requires_hitl":true,"status":"UNKNOWN"},{"check":"legacy_hive_metastore_sql_reference","details":"{\"reference_queries\":0,\"visible_pct\":100.0}","evidence_refs":["EVID-3BAC65585521CF919E44102B"],"requires_hitl":true,"status":"UNKNOWN"}]</t>
+          <t>[{"check":"workspace_pro_classic_observed","details":"true","evidence_refs":["EVID-242E046D548E372E51BAB181"],"requires_hitl":false,"status":"PASS"},{"check":"pro_warehouse_type_enabled","details":"true","evidence_refs":["EVID-8D52106E13681C2F50F82B9E"],"requires_hitl":false,"status":"PASS"},{"check":"aws_price_registry_region","details":"\"us-east-1\"","evidence_refs":["EVID-DFDC582DDAF10240DA9F7DAE"],"requires_hitl":false,"status":"PASS"}]</t>
         </is>
       </c>
       <c r="AO18" s="22" t="inlineStr">
         <is>
-          <t>[{"check":"s3_access_policy_compatibility","details":"\"UNKNOWN\"","evidence_refs":["EVID-E85A4C9B3B5A439FE6F3D488"],"requires_hitl":true,"status":"UNKNOWN"},{"check":"legacy_hive_metastore_sql_reference","details":"{\"reference_queries\":0,\"visible_pct\":100.0}","evidence_refs":["EVID-3BAC65585521CF919E44102B"],"requires_hitl":true,"status":"UNKNOWN"}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AP18" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.61},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-D1C8429D0D427860A3152AFC","confidence":{"components":{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.61},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":151840.0,"high":151840.0,"low":151840.0},"dbu":{"base":-328666.67,"high":-328666.67,"low":-328666.67},"total":{"base":-176826.67,"high":-176826.67,"low":-176826.67}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AQ18" s="22" t="inlineStr">
         <is>
-          <t>["CAND-D1C8429D0D427860A3152AFC"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AR18" s="22" t="inlineStr">
@@ -9740,19 +9742,19 @@
       </c>
       <c r="AS18" s="22" t="inlineStr">
         <is>
-          <t>["auto_stop_minutes","max_clusters","min_clusters","warehouse_size"]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>SCN-EFE76D0072038BA31048924A</t>
+          <t>SCN-A7F14CD75A7AA486F6E590A9</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -9908,12 +9910,12 @@
       </c>
       <c r="AP19" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-8CF2F68ED84D562D3D9E5560","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-D7E581D7637D85BCED1CACDC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":10,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":5,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-B1DE4DC4AEBC6BA9039D5664","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-AAE2D61246CC19F3D31359B2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":10,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":5,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ19" s="22" t="inlineStr">
         <is>
-          <t>["CAND-8CF2F68ED84D562D3D9E5560","CAND-D7E581D7637D85BCED1CACDC"]</t>
+          <t>["CAND-B1DE4DC4AEBC6BA9039D5664","CAND-AAE2D61246CC19F3D31359B2"]</t>
         </is>
       </c>
       <c r="AR19" s="22" t="inlineStr">
@@ -9930,12 +9932,12 @@
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>SCN-0DE5AFA24E42CA4905AA2E90</t>
+          <t>SCN-010708604C897CBD8CB6999B</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
@@ -10097,12 +10099,12 @@
       </c>
       <c r="AP20" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-FF7A26AD3267B8B24B7DDE29","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SERVERLESS","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-9482.94,"high":-2709.41,"low":-10837.65},"dbu":{"base":-16386.62,"high":32460.97,"low":-26156.13},"total":{"base":-25869.56,"high":29751.56,"low":-36993.78}}},"recommended_value":"PRO","step":2,"step_type":"CANDIDATE","technique_id":"WH-PRO-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-71D893FD78F2362AC4404318","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SERVERLESS","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-9482.94,"high":-2709.41,"low":-10837.65},"dbu":{"base":-16386.62,"high":32460.97,"low":-26156.13},"total":{"base":-25869.56,"high":29751.56,"low":-36993.78}}},"recommended_value":"PRO","step":2,"step_type":"CANDIDATE","technique_id":"WH-PRO-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ20" s="22" t="inlineStr">
         <is>
-          <t>["CAND-FF7A26AD3267B8B24B7DDE29"]</t>
+          <t>["CAND-71D893FD78F2362AC4404318"]</t>
         </is>
       </c>
       <c r="AR20" s="22" t="inlineStr">
@@ -10119,12 +10121,12 @@
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>SCN-2AD1B1369F3CA903C33A7F0A</t>
+          <t>SCN-9082F31BD0DF2BCD069F29F7</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -10280,12 +10282,12 @@
       </c>
       <c r="AP21" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-B91739B640B2882103617ADC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-1416408891B7644B4B970F3D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-03498DA37C2B00C97906A378","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-AA7121CBC49CC8D096B1A310","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ21" s="22" t="inlineStr">
         <is>
-          <t>["CAND-B91739B640B2882103617ADC","CAND-1416408891B7644B4B970F3D"]</t>
+          <t>["CAND-03498DA37C2B00C97906A378","CAND-AA7121CBC49CC8D096B1A310"]</t>
         </is>
       </c>
       <c r="AR21" s="22" t="inlineStr">
@@ -10302,12 +10304,12 @@
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>SCN-DB87EC8AF05431F8208079A0</t>
+          <t>SCN-0BEADBEFBF7332316DE55F3F</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -10469,12 +10471,12 @@
       </c>
       <c r="AP22" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-E299C12314806ACD8AA15BB6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5488.19,"high":5488.19,"low":5488.19},"dbu":{"base":4686.75,"high":8791.16,"low":582.33},"total":{"base":10174.94,"high":14279.35,"low":6070.52}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-E16149DF1079E234A70FABFA","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5488.19,"high":5488.19,"low":5488.19},"dbu":{"base":4686.75,"high":8791.16,"low":582.33},"total":{"base":10174.94,"high":14279.35,"low":6070.52}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ22" s="22" t="inlineStr">
         <is>
-          <t>["CAND-E299C12314806ACD8AA15BB6"]</t>
+          <t>["CAND-E16149DF1079E234A70FABFA"]</t>
         </is>
       </c>
       <c r="AR22" s="22" t="inlineStr">
@@ -10491,12 +10493,12 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>SCN-3ADBD372252C701E8605FDBF</t>
+          <t>SCN-0AF33099B977B44DE891DB2F</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -10652,12 +10654,12 @@
       </c>
       <c r="AP23" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-44783D6FD480C2752BDBEC25","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-15068.09,"high":0.0,"low":-37670.23},"dbu":{"base":-23200.0,"high":0.0,"low":-58000.0},"total":{"base":-38268.09,"high":0.0,"low":-95670.23}}},"recommended_value":"X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-184A3C392690D298B3EFD5E3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":45,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13565.92,"high":2002.9,"low":-36668.78},"dbu":{"base":-20887.14,"high":3083.82,"low":-56458.09},"total":{"base":-34453.06,"high":5086.72,"low":-93126.87}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-6A591F792934B6D67437E104","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-15068.09,"high":0.0,"low":-37670.23},"dbu":{"base":-23200.0,"high":0.0,"low":-58000.0},"total":{"base":-38268.09,"high":0.0,"low":-95670.23}}},"recommended_value":"X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-1BF6312BDBD011BCBF5B17DD","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":45,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13565.92,"high":2002.9,"low":-36668.78},"dbu":{"base":-20887.14,"high":3083.82,"low":-56458.09},"total":{"base":-34453.06,"high":5086.72,"low":-93126.87}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ23" s="22" t="inlineStr">
         <is>
-          <t>["CAND-44783D6FD480C2752BDBEC25","CAND-184A3C392690D298B3EFD5E3"]</t>
+          <t>["CAND-6A591F792934B6D67437E104","CAND-1BF6312BDBD011BCBF5B17DD"]</t>
         </is>
       </c>
       <c r="AR23" s="22" t="inlineStr">
@@ -10674,12 +10676,12 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>SCN-3B15D95786681E2F1586255E</t>
+          <t>SCN-85DD6FDC4F7D607B91486DB3</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -10841,12 +10843,12 @@
       </c>
       <c r="AP24" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-D3DD9FFE6744CCBBA9B4F934","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":37670.23,"high":37670.23,"low":37670.23},"dbu":{"base":-26516.54,"high":44997.46,"low":-33017.81},"total":{"base":11153.69,"high":82667.69,"low":4652.42}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-208C05A9E348D11DAEE662DF","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":37670.23,"high":37670.23,"low":37670.23},"dbu":{"base":-26516.54,"high":44997.46,"low":-33017.81},"total":{"base":11153.69,"high":82667.69,"low":4652.42}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ24" s="22" t="inlineStr">
         <is>
-          <t>["CAND-D3DD9FFE6744CCBBA9B4F934"]</t>
+          <t>["CAND-208C05A9E348D11DAEE662DF"]</t>
         </is>
       </c>
       <c r="AR24" s="22" t="inlineStr">
@@ -10863,12 +10865,12 @@
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>SCN-BBAAF3154665B37B8FCEA1E0</t>
+          <t>SCN-2933621CB20E77E39795A10D</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -11024,12 +11026,12 @@
       </c>
       <c r="AP25" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-B6913E34C50A503A1D6DBEA0","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1265.33,"high":1626.86,"low":813.43},"dbu":{"base":5425.0,"high":6975.0,"low":3487.5},"total":{"base":6690.33,"high":8601.86,"low":4300.93}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-C1A802D5E5BEE703D8ED0085","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1672.05,"high":2440.29,"low":813.43},"dbu":{"base":7168.75,"high":10462.5,"low":3487.5},"total":{"base":8840.8,"high":12902.79,"low":4300.93}}},"recommended_value":1,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-0F14BBC11AE756EB5AFB1C96","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1940.48,"high":2798.2,"low":992.38},"dbu":{"base":8319.62,"high":11997.0,"low":4254.75},"total":{"base":10260.1,"high":14795.2,"low":5247.13}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-BBB38F2B1B9EA80282892372","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1265.33,"high":1626.86,"low":813.43},"dbu":{"base":5425.0,"high":6975.0,"low":3487.5},"total":{"base":6690.33,"high":8601.86,"low":4300.93}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-97D73C8B9AB1304A39EE9B0D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1672.05,"high":2440.29,"low":813.43},"dbu":{"base":7168.75,"high":10462.5,"low":3487.5},"total":{"base":8840.8,"high":12902.79,"low":4300.93}}},"recommended_value":1,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-2B92AC15169DEA8C2A7CFA89","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1940.48,"high":2798.2,"low":992.38},"dbu":{"base":8319.62,"high":11997.0,"low":4254.75},"total":{"base":10260.1,"high":14795.2,"low":5247.13}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ25" s="22" t="inlineStr">
         <is>
-          <t>["CAND-B6913E34C50A503A1D6DBEA0","CAND-C1A802D5E5BEE703D8ED0085","CAND-0F14BBC11AE756EB5AFB1C96"]</t>
+          <t>["CAND-BBB38F2B1B9EA80282892372","CAND-97D73C8B9AB1304A39EE9B0D","CAND-2B92AC15169DEA8C2A7CFA89"]</t>
         </is>
       </c>
       <c r="AR25" s="22" t="inlineStr">
@@ -11046,12 +11048,12 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>SCN-4C7F7B95C214EEBF380310D5</t>
+          <t>SCN-8CEE26C6FC4807B9693BC3A5</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -11213,12 +11215,12 @@
       </c>
       <c r="AP26" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-53AF57B05EB45846CF76155B","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3615.24,"high":3615.24,"low":3615.24},"dbu":{"base":7388.89,"high":11444.44,"low":7388.89},"total":{"base":11004.13,"high":15059.68,"low":11004.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-1B05132C1EC3D2449969E905","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3615.24,"high":3615.24,"low":3615.24},"dbu":{"base":7388.89,"high":11444.44,"low":7388.89},"total":{"base":11004.13,"high":15059.68,"low":11004.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ26" s="22" t="inlineStr">
         <is>
-          <t>["CAND-53AF57B05EB45846CF76155B"]</t>
+          <t>["CAND-1B05132C1EC3D2449969E905"]</t>
         </is>
       </c>
       <c r="AR26" s="22" t="inlineStr">
@@ -11235,12 +11237,12 @@
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>SCN-B1AE3151CA3DFABC9D6F87A2</t>
+          <t>SCN-DC5D9238399C6A5D0C16D1D5</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -11396,12 +11398,12 @@
       </c>
       <c r="AP27" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-3B94CC5756DFC0077D2E12FE","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-F89285A886F733FCF48A39F5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":8,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-D830ED375B9F86AA1F381EA4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-DB36510075A8FBE14B50458C","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":8,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ27" s="22" t="inlineStr">
         <is>
-          <t>["CAND-3B94CC5756DFC0077D2E12FE","CAND-F89285A886F733FCF48A39F5"]</t>
+          <t>["CAND-D830ED375B9F86AA1F381EA4","CAND-DB36510075A8FBE14B50458C"]</t>
         </is>
       </c>
       <c r="AR27" s="22" t="inlineStr">
@@ -11418,12 +11420,12 @@
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>SCN-7AA042130907C622B3D829D7</t>
+          <t>SCN-D6AA6A4FA46862F6334FBC5C</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
@@ -11585,12 +11587,12 @@
       </c>
       <c r="AP28" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-AD58D34434A2170D1BF1A9B1","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5338.12,"high":5338.12,"low":5338.12},"dbu":{"base":14023.44,"high":18015.63,"low":10031.25},"total":{"base":19361.56,"high":23353.75,"low":15369.37}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-D2AA37F564A2D82B828401D3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5338.12,"high":5338.12,"low":5338.12},"dbu":{"base":14023.44,"high":18015.63,"low":10031.25},"total":{"base":19361.56,"high":23353.75,"low":15369.37}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ28" s="22" t="inlineStr">
         <is>
-          <t>["CAND-AD58D34434A2170D1BF1A9B1"]</t>
+          <t>["CAND-D2AA37F564A2D82B828401D3"]</t>
         </is>
       </c>
       <c r="AR28" s="22" t="inlineStr">
@@ -11607,12 +11609,12 @@
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>SCN-C7D4A73498A01E43CF2F1F99</t>
+          <t>SCN-999C878D6C51D4B139B49A57</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -11768,12 +11770,12 @@
       </c>
       <c r="AP29" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-4D7163BFB57F1D099F93FBB4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1026.39,"high":1319.64,"low":659.82},"dbu":{"base":7350.0,"high":9450.0,"low":4725.0},"total":{"base":8376.39,"high":10769.64,"low":5384.82}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-A69115976DE8B2D6CED3E2F9","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1158.35,"high":1495.59,"low":747.8},"dbu":{"base":8295.0,"high":10710.0,"low":5355.0},"total":{"base":9453.35,"high":12205.59,"low":6102.8}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-61D8612587ADCC0F68698112","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1026.39,"high":1319.64,"low":659.82},"dbu":{"base":7350.0,"high":9450.0,"low":4725.0},"total":{"base":8376.39,"high":10769.64,"low":5384.82}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-0B255F5C4039607F30C4EE4A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1158.35,"high":1495.59,"low":747.8},"dbu":{"base":8295.0,"high":10710.0,"low":5355.0},"total":{"base":9453.35,"high":12205.59,"low":6102.8}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ29" s="22" t="inlineStr">
         <is>
-          <t>["CAND-4D7163BFB57F1D099F93FBB4","CAND-A69115976DE8B2D6CED3E2F9"]</t>
+          <t>["CAND-61D8612587ADCC0F68698112","CAND-0B255F5C4039607F30C4EE4A"]</t>
         </is>
       </c>
       <c r="AR29" s="22" t="inlineStr">
@@ -11790,12 +11792,12 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>SCN-C2B8462C39C6CBF67EA76272</t>
+          <t>SCN-F5B38DFE81B5D7BBAF6911B1</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -11957,12 +11959,12 @@
       </c>
       <c r="AP30" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-0E7487FBA4179110E052404A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":2932.53,"high":2932.53,"low":2932.53},"dbu":{"base":14420.6,"high":16613.73,"low":12227.47},"total":{"base":17353.13,"high":19546.26,"low":15160.0}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-C8B97E03CD532E0571F1A2F5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":2932.53,"high":2932.53,"low":2932.53},"dbu":{"base":14420.6,"high":16613.73,"low":12227.47},"total":{"base":17353.13,"high":19546.26,"low":15160.0}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ30" s="22" t="inlineStr">
         <is>
-          <t>["CAND-0E7487FBA4179110E052404A"]</t>
+          <t>["CAND-C8B97E03CD532E0571F1A2F5"]</t>
         </is>
       </c>
       <c r="AR30" s="22" t="inlineStr">
@@ -11979,12 +11981,12 @@
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>SCN-90F84EEF462106B503D5FCD5</t>
+          <t>SCN-21882722E00BEBBB1248C9B9</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -12170,12 +12172,12 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>SCN-C76B1BF0BE04F2268A48C457</t>
+          <t>SCN-C2EBBB483BA454145E5C3C56</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -12337,12 +12339,12 @@
       </c>
       <c r="AP32" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.731},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-0CF01F172DB34D3AE5983193","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":0.09,"signal":1.0,"stability":0.725},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.731},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3733.77,"high":3733.77,"low":3733.77},"dbu":{"base":-5177.05,"high":-5177.05,"low":-5177.05},"total":{"base":-1443.28,"high":-1443.28,"low":-1443.28}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.731},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-C83A18C81BA3F8F01454DD46","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":0.09,"signal":1.0,"stability":0.725},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.731},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3733.77,"high":3733.77,"low":3733.77},"dbu":{"base":-5177.05,"high":-5177.05,"low":-5177.05},"total":{"base":-1443.28,"high":-1443.28,"low":-1443.28}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ32" s="22" t="inlineStr">
         <is>
-          <t>["CAND-0CF01F172DB34D3AE5983193"]</t>
+          <t>["CAND-C83A18C81BA3F8F01454DD46"]</t>
         </is>
       </c>
       <c r="AR32" s="22" t="inlineStr">
@@ -12359,12 +12361,12 @@
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>SCN-CD13BC97911EDD734CF17B6B</t>
+          <t>SCN-5F795672B44D350C3E296BF1</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -12520,12 +12522,12 @@
       </c>
       <c r="AP33" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-20A04702FCD63664C07653A5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-9ADFC70F5FC112A2499B5375","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":5,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-C08CF1BBC9ECD83993F5BCE2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":2409.51,"high":3623.05,"low":932.15},"dbu":{"base":-4016.37,"high":3019.8,"low":-12582.14},"total":{"base":-1606.86,"high":6642.85,"low":-11649.99}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-2ABC4239192B22E3E0541016","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-ACA9A2EEB098AFFFB5C5CDD7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":5,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-5BD0417FF74CCA4CE750987C","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":2409.51,"high":3623.05,"low":932.15},"dbu":{"base":-4016.37,"high":3019.8,"low":-12582.14},"total":{"base":-1606.86,"high":6642.85,"low":-11649.99}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ33" s="22" t="inlineStr">
         <is>
-          <t>["CAND-20A04702FCD63664C07653A5","CAND-9ADFC70F5FC112A2499B5375","CAND-C08CF1BBC9ECD83993F5BCE2"]</t>
+          <t>["CAND-2ABC4239192B22E3E0541016","CAND-ACA9A2EEB098AFFFB5C5CDD7","CAND-5BD0417FF74CCA4CE750987C"]</t>
         </is>
       </c>
       <c r="AR33" s="22" t="inlineStr">
@@ -12542,12 +12544,12 @@
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>SCN-D90F0090AC8A9492249F19B8</t>
+          <t>SCN-871471461B50CF97B71AE728</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -12709,12 +12711,12 @@
       </c>
       <c r="AP34" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-A33DFC4B60027DE5B92ED694","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":8793.82,"high":8793.82,"low":8793.82},"dbu":{"base":13270.27,"high":19846.85,"low":6693.69},"total":{"base":22064.09,"high":28640.67,"low":15487.51}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-254186ED0FFA404D809AF606","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":8793.82,"high":8793.82,"low":8793.82},"dbu":{"base":13270.27,"high":19846.85,"low":6693.69},"total":{"base":22064.09,"high":28640.67,"low":15487.51}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ34" s="22" t="inlineStr">
         <is>
-          <t>["CAND-A33DFC4B60027DE5B92ED694"]</t>
+          <t>["CAND-254186ED0FFA404D809AF606"]</t>
         </is>
       </c>
       <c r="AR34" s="22" t="inlineStr">
@@ -13462,12 +13464,12 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>CAND-7228133F8C9DCD58D5450164</t>
+          <t>CAND-2FF10B6D104A88133435FFC9</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -13693,12 +13695,12 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>CAND-CDC9DD7E27E8CA6ED23E9CEB</t>
+          <t>CAND-DAC9E910F2A94A05B67B302A</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -13872,7 +13874,7 @@
       </c>
       <c r="AR6" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS6" s="22" t="inlineStr">
@@ -13882,17 +13884,17 @@
       </c>
       <c r="AT6" s="22" t="inlineStr">
         <is>
-          <t>["EVID-832712B10A432503BA1E0ADE","EVID-A8636AD7291DF641B4479F73","EVID-B2362D5F32380977A933F401","EVID-FDBFFBC774D23EA471B31E96","EVID-4D3C96F560A56E7EC4E79822","EVID-6EA74D3474DEBD48A2D18AA3","EVID-A86EAA13EE5082AEC4DF0A44","EVID-844D3CCD8E1426B8521EC841","EVID-816032E26FD5D0505D12B7B5","EVID-671AEFC2D527CBB61D748323","EVID-37B58153FD21C4097D6839AF","EVID-8FDC7E9818FEE739EB1C3E96"]</t>
+          <t>["EVID-832712B10A432503BA1E0ADE","EVID-A8636AD7291DF641B4479F73","EVID-B2362D5F32380977A933F401","EVID-FDBFFBC774D23EA471B31E96","EVID-4D3C96F560A56E7EC4E79822","EVID-756332815C5D1223CA4A8740","EVID-6EA74D3474DEBD48A2D18AA3","EVID-A86EAA13EE5082AEC4DF0A44","EVID-844D3CCD8E1426B8521EC841","EVID-816032E26FD5D0505D12B7B5","EVID-671AEFC2D527CBB61D748323","EVID-37B58153FD21C4097D6839AF","EVID-8FDC7E9818FEE739EB1C3E96"]</t>
         </is>
       </c>
       <c r="AU6" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-37B58153FD21C4097D6839AF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-37B58153FD21C4097D6839AF","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-4D3C96F560A56E7EC4E79822":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4D3C96F560A56E7EC4E79822","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-671AEFC2D527CBB61D748323":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-671AEFC2D527CBB61D748323","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-6EA74D3474DEBD48A2D18AA3":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6EA74D3474DEBD48A2D18AA3","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2500},"EVID-816032E26FD5D0505D12B7B5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-816032E26FD5D0505D12B7B5","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-832712B10A432503BA1E0ADE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-832712B10A432503BA1E0ADE","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-844D3CCD8E1426B8521EC841":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-844D3CCD8E1426B8521EC841","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-8FDC7E9818FEE739EB1C3E96":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8FDC7E9818FEE739EB1C3E96","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A8636AD7291DF641B4479F73":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-A8636AD7291DF641B4479F73","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-A86EAA13EE5082AEC4DF0A44":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-A86EAA13EE5082AEC4DF0A44","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":10000},"EVID-B2362D5F32380977A933F401":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-B2362D5F32380977A933F401","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-FDBFFBC774D23EA471B31E96":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-FDBFFBC774D23EA471B31E96","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0}}</t>
+          <t>{"EVID-37B58153FD21C4097D6839AF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-37B58153FD21C4097D6839AF","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-4D3C96F560A56E7EC4E79822":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4D3C96F560A56E7EC4E79822","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-671AEFC2D527CBB61D748323":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-671AEFC2D527CBB61D748323","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-6EA74D3474DEBD48A2D18AA3":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6EA74D3474DEBD48A2D18AA3","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2500},"EVID-756332815C5D1223CA4A8740":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-756332815C5D1223CA4A8740","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-816032E26FD5D0505D12B7B5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-816032E26FD5D0505D12B7B5","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-832712B10A432503BA1E0ADE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-832712B10A432503BA1E0ADE","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-844D3CCD8E1426B8521EC841":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-844D3CCD8E1426B8521EC841","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-8FDC7E9818FEE739EB1C3E96":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8FDC7E9818FEE739EB1C3E96","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A8636AD7291DF641B4479F73":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-A8636AD7291DF641B4479F73","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-A86EAA13EE5082AEC4DF0A44":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-A86EAA13EE5082AEC4DF0A44","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":10000},"EVID-B2362D5F32380977A933F401":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-B2362D5F32380977A933F401","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-FDBFFBC774D23EA471B31E96":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-FDBFFBC774D23EA471B31E96","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0}}</t>
         </is>
       </c>
       <c r="AV6" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-A8636AD7291DF641B4479F73","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-B2362D5F32380977A933F401","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-FDBFFBC774D23EA471B31E96","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-4D3C96F560A56E7EC4E79822","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-6EA74D3474DEBD48A2D18AA3","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-A86EAA13EE5082AEC4DF0A44","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-A8636AD7291DF641B4479F73","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-B2362D5F32380977A933F401","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-FDBFFBC774D23EA471B31E96","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-4D3C96F560A56E7EC4E79822","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-756332815C5D1223CA4A8740","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-6EA74D3474DEBD48A2D18AA3","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-A86EAA13EE5082AEC4DF0A44","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW6" s="22" t="inlineStr">
@@ -13912,7 +13914,7 @@
       </c>
       <c r="AZ6" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-F6C96142718566E6610757F4","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-E1D619112BE62AFA050EA71A","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA6" s="22" t="inlineStr">
@@ -13924,12 +13926,12 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>CAND-4CD23256DB0CA20822638058</t>
+          <t>CAND-567E1FFD79E2F9A61A59510F</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -14139,7 +14141,7 @@
       </c>
       <c r="AZ7" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F6C96142718566E6610757F4","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-E1D619112BE62AFA050EA71A","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA7" s="22" t="inlineStr">
@@ -14151,12 +14153,12 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>CAND-F7CD1FD114943EA1AAB92DF2</t>
+          <t>CAND-585D0C22F7A86D37CE5BCDE5</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -14366,7 +14368,7 @@
       </c>
       <c r="AZ8" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F6C96142718566E6610757F4","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-E1D619112BE62AFA050EA71A","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA8" s="22" t="inlineStr">
@@ -14378,12 +14380,12 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>CAND-1EB011ABA71F8CF380C298A8</t>
+          <t>CAND-B72E480BD8ADA0BAAADDB594</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -14593,7 +14595,7 @@
       </c>
       <c r="AZ9" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F6C96142718566E6610757F4","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-E1D619112BE62AFA050EA71A","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
         </is>
       </c>
       <c r="BA9" s="22" t="inlineStr">
@@ -14605,12 +14607,12 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PKG-CAA063CBB4924A9B7B8E4514</t>
+          <t>PKG-3BA4F39CA2D09D98401702A2</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>CAND-78762B303EA11AF80300E2C3</t>
+          <t>CAND-D7C2183B68BBD711C74005C7</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -14824,7 +14826,7 @@
       </c>
       <c r="AZ10" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-4CE208EB461A228615816740","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-B49B73B0344B4AF52B454990","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA10" s="22" t="inlineStr">
@@ -14836,12 +14838,12 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>CAND-BB5D8BD2733924BAA2A2BB82</t>
+          <t>CAND-BBCE77B209F653D5A121588C</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -15067,12 +15069,12 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>CAND-F6DA76343C4F0EEC6747DD79</t>
+          <t>CAND-3107EA199EA58282439B64F2</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -15246,7 +15248,7 @@
       </c>
       <c r="AR12" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS12" s="22" t="inlineStr">
@@ -15256,17 +15258,17 @@
       </c>
       <c r="AT12" s="22" t="inlineStr">
         <is>
-          <t>["EVID-8686A768FBB341A60EA85745","EVID-88AEFDEA380CDAD006F80001","EVID-0A7D5DF3B5E2F45BE27DFD19","EVID-BB7DFD2862AB2ADD1FA0CF31","EVID-EA733691C9BFE7B18FA8EE7E","EVID-F96600E8808D60DFD7238304","EVID-9FFE6B7A17D42D283F900800","EVID-61A44CDFF8B383C5ABB509D9","EVID-823A180D36962C7150FEB320","EVID-31544533FEDFC669EB9E511D","EVID-60346EE4CD6A756F88C9A889","EVID-10635B972051ED8C2A7BEF9D"]</t>
+          <t>["EVID-8686A768FBB341A60EA85745","EVID-88AEFDEA380CDAD006F80001","EVID-0A7D5DF3B5E2F45BE27DFD19","EVID-BB7DFD2862AB2ADD1FA0CF31","EVID-EA733691C9BFE7B18FA8EE7E","EVID-EC04540FF7292F7272B822B1","EVID-F96600E8808D60DFD7238304","EVID-9FFE6B7A17D42D283F900800","EVID-61A44CDFF8B383C5ABB509D9","EVID-823A180D36962C7150FEB320","EVID-31544533FEDFC669EB9E511D","EVID-60346EE4CD6A756F88C9A889","EVID-10635B972051ED8C2A7BEF9D"]</t>
         </is>
       </c>
       <c r="AU12" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0A7D5DF3B5E2F45BE27DFD19":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-0A7D5DF3B5E2F45BE27DFD19","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":422},"EVID-10635B972051ED8C2A7BEF9D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-10635B972051ED8C2A7BEF9D","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-31544533FEDFC669EB9E511D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-31544533FEDFC669EB9E511D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0},"EVID-60346EE4CD6A756F88C9A889":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-60346EE4CD6A756F88C9A889","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-61A44CDFF8B383C5ABB509D9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-61A44CDFF8B383C5ABB509D9","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-823A180D36962C7150FEB320":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-823A180D36962C7150FEB320","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-8686A768FBB341A60EA85745":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8686A768FBB341A60EA85745","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"X_LARGE"},"EVID-88AEFDEA380CDAD006F80001":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-88AEFDEA380CDAD006F80001","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":6.5},"EVID-9FFE6B7A17D42D283F900800":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9FFE6B7A17D42D283F900800","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":48000},"EVID-BB7DFD2862AB2ADD1FA0CF31":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BB7DFD2862AB2ADD1FA0CF31","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":3221225472},"EVID-EA733691C9BFE7B18FA8EE7E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EA733691C9BFE7B18FA8EE7E","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.8},"EVID-F96600E8808D60DFD7238304":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F96600E8808D60DFD7238304","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":14000}}</t>
+          <t>{"EVID-0A7D5DF3B5E2F45BE27DFD19":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-0A7D5DF3B5E2F45BE27DFD19","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":422},"EVID-10635B972051ED8C2A7BEF9D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-10635B972051ED8C2A7BEF9D","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-31544533FEDFC669EB9E511D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-31544533FEDFC669EB9E511D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0},"EVID-60346EE4CD6A756F88C9A889":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-60346EE4CD6A756F88C9A889","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-61A44CDFF8B383C5ABB509D9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-61A44CDFF8B383C5ABB509D9","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-823A180D36962C7150FEB320":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-823A180D36962C7150FEB320","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-8686A768FBB341A60EA85745":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8686A768FBB341A60EA85745","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"X_LARGE"},"EVID-88AEFDEA380CDAD006F80001":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-88AEFDEA380CDAD006F80001","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":6.5},"EVID-9FFE6B7A17D42D283F900800":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9FFE6B7A17D42D283F900800","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":48000},"EVID-BB7DFD2862AB2ADD1FA0CF31":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BB7DFD2862AB2ADD1FA0CF31","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":3221225472},"EVID-EA733691C9BFE7B18FA8EE7E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EA733691C9BFE7B18FA8EE7E","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.8},"EVID-EC04540FF7292F7272B822B1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EC04540FF7292F7272B822B1","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-F96600E8808D60DFD7238304":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F96600E8808D60DFD7238304","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":14000}}</t>
         </is>
       </c>
       <c r="AV12" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-88AEFDEA380CDAD006F80001","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-0A7D5DF3B5E2F45BE27DFD19","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-BB7DFD2862AB2ADD1FA0CF31","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-EA733691C9BFE7B18FA8EE7E","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F96600E8808D60DFD7238304","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-9FFE6B7A17D42D283F900800","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-88AEFDEA380CDAD006F80001","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-0A7D5DF3B5E2F45BE27DFD19","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-BB7DFD2862AB2ADD1FA0CF31","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-EA733691C9BFE7B18FA8EE7E","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-EC04540FF7292F7272B822B1","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F96600E8808D60DFD7238304","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-9FFE6B7A17D42D283F900800","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW12" s="22" t="inlineStr">
@@ -15286,7 +15288,7 @@
       </c>
       <c r="AZ12" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY","scenario_id":"SCN-CB5E8798D5A13F523639541D","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY","scenario_id":"SCN-2EEA487274E8B4C2D2A00C65","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA12" s="22" t="inlineStr">
@@ -15298,12 +15300,12 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CAND-19E6151216E0827A2A6FA085</t>
+          <t>CAND-59AA68AE5112DDA5910F67FF</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -15525,12 +15527,12 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CAND-CF1FEEFF3DB94CBE4A3A7DCC</t>
+          <t>CAND-EBBDB2090AA5F8307AFCB223</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -15752,12 +15754,12 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>CAND-A122082B3BB2FB0568C91BF4</t>
+          <t>CAND-CDA61DCEC36313DD1885DFD7</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -15967,7 +15969,7 @@
       </c>
       <c r="AZ15" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-CB5E8798D5A13F523639541D","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-2EEA487274E8B4C2D2A00C65","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA15" s="22" t="inlineStr">
@@ -15979,12 +15981,12 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PKG-3542FB38D0CE64996A1D7C9D</t>
+          <t>PKG-94708DA4314591AE1A094826</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>CAND-335D8BD4AAC3CB041A5DB0CB</t>
+          <t>CAND-5FD3D0884B03CB55AFDD5092</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -16198,7 +16200,7 @@
       </c>
       <c r="AZ16" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-AF126D31FABFB5905E6640A4","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-69AD699F056B046156191604","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA16" s="22" t="inlineStr">
@@ -16210,12 +16212,12 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>CAND-B2CDD1956666E75CF94834A6</t>
+          <t>CAND-5D7C7CA2D483F31C69008B3F</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -16441,12 +16443,12 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>CAND-C86EF28A42FC56DB5AD00959</t>
+          <t>CAND-FF852A8F55F23A58470A0F50</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -16620,7 +16622,7 @@
       </c>
       <c r="AR18" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS18" s="22" t="inlineStr">
@@ -16630,17 +16632,17 @@
       </c>
       <c r="AT18" s="22" t="inlineStr">
         <is>
-          <t>["EVID-7EE079F6E39AE969EB70AD13","EVID-7DE4C6A55F99666E0EA5E572","EVID-75681E00F1AFFAE2ED2A7EE6","EVID-1D3DC4ADB1D13DC74AC5E8BA","EVID-5377620EA4B90F62C3412859","EVID-895BAEEB75D06CB18730FA3E","EVID-1614F9F08839318F3E399E84","EVID-B10D381B0DF19402AF720873","EVID-990E7C65C9A55CFB360EA05A","EVID-3DE1D1B65EC8D6C5C825F4CD","EVID-A5222E97CA81F6CAE91BF10A","EVID-2774AF84EAE8D6AA54B380CA"]</t>
+          <t>["EVID-7EE079F6E39AE969EB70AD13","EVID-7DE4C6A55F99666E0EA5E572","EVID-75681E00F1AFFAE2ED2A7EE6","EVID-1D3DC4ADB1D13DC74AC5E8BA","EVID-5377620EA4B90F62C3412859","EVID-F597D49E500FDB24F9B8434F","EVID-895BAEEB75D06CB18730FA3E","EVID-1614F9F08839318F3E399E84","EVID-B10D381B0DF19402AF720873","EVID-990E7C65C9A55CFB360EA05A","EVID-3DE1D1B65EC8D6C5C825F4CD","EVID-A5222E97CA81F6CAE91BF10A","EVID-2774AF84EAE8D6AA54B380CA"]</t>
         </is>
       </c>
       <c r="AU18" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1614F9F08839318F3E399E84":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1614F9F08839318F3E399E84","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6500},"EVID-1D3DC4ADB1D13DC74AC5E8BA":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-1D3DC4ADB1D13DC74AC5E8BA","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-2774AF84EAE8D6AA54B380CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2774AF84EAE8D6AA54B380CA","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-3DE1D1B65EC8D6C5C825F4CD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3DE1D1B65EC8D6C5C825F4CD","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-5377620EA4B90F62C3412859":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5377620EA4B90F62C3412859","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-75681E00F1AFFAE2ED2A7EE6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-75681E00F1AFFAE2ED2A7EE6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-7DE4C6A55F99666E0EA5E572":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-7DE4C6A55F99666E0EA5E572","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-7EE079F6E39AE969EB70AD13":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7EE079F6E39AE969EB70AD13","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-895BAEEB75D06CB18730FA3E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-895BAEEB75D06CB18730FA3E","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1900},"EVID-990E7C65C9A55CFB360EA05A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-990E7C65C9A55CFB360EA05A","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-A5222E97CA81F6CAE91BF10A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A5222E97CA81F6CAE91BF10A","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-B10D381B0DF19402AF720873":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B10D381B0DF19402AF720873","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0}}</t>
+          <t>{"EVID-1614F9F08839318F3E399E84":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1614F9F08839318F3E399E84","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6500},"EVID-1D3DC4ADB1D13DC74AC5E8BA":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-1D3DC4ADB1D13DC74AC5E8BA","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-2774AF84EAE8D6AA54B380CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2774AF84EAE8D6AA54B380CA","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-3DE1D1B65EC8D6C5C825F4CD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3DE1D1B65EC8D6C5C825F4CD","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-5377620EA4B90F62C3412859":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5377620EA4B90F62C3412859","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-75681E00F1AFFAE2ED2A7EE6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-75681E00F1AFFAE2ED2A7EE6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-7DE4C6A55F99666E0EA5E572":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-7DE4C6A55F99666E0EA5E572","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-7EE079F6E39AE969EB70AD13":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7EE079F6E39AE969EB70AD13","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-895BAEEB75D06CB18730FA3E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-895BAEEB75D06CB18730FA3E","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1900},"EVID-990E7C65C9A55CFB360EA05A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-990E7C65C9A55CFB360EA05A","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-A5222E97CA81F6CAE91BF10A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A5222E97CA81F6CAE91BF10A","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-B10D381B0DF19402AF720873":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B10D381B0DF19402AF720873","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-F597D49E500FDB24F9B8434F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F597D49E500FDB24F9B8434F","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
         </is>
       </c>
       <c r="AV18" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-7DE4C6A55F99666E0EA5E572","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-75681E00F1AFFAE2ED2A7EE6","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-1D3DC4ADB1D13DC74AC5E8BA","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-5377620EA4B90F62C3412859","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-895BAEEB75D06CB18730FA3E","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-1614F9F08839318F3E399E84","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-7DE4C6A55F99666E0EA5E572","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-75681E00F1AFFAE2ED2A7EE6","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-1D3DC4ADB1D13DC74AC5E8BA","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-5377620EA4B90F62C3412859","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F597D49E500FDB24F9B8434F","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-895BAEEB75D06CB18730FA3E","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-1614F9F08839318F3E399E84","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW18" s="22" t="inlineStr">
@@ -16660,7 +16662,7 @@
       </c>
       <c r="AZ18" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-CE4B0C3CDE2534722A4AAADE","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-F7FD9602740588A931526FB1","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA18" s="22" t="inlineStr">
@@ -16672,12 +16674,12 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>CAND-0B0E829222AD5BA2CA4E7612</t>
+          <t>CAND-6A370586BC9EDB6A5FE47F5D</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -16887,7 +16889,7 @@
       </c>
       <c r="AZ19" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-CE4B0C3CDE2534722A4AAADE","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F7FD9602740588A931526FB1","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA19" s="22" t="inlineStr">
@@ -16899,12 +16901,12 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>CAND-E2B81BBFEB2D221645C6CC57</t>
+          <t>CAND-6F350B226F959664414114EB</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
@@ -17114,7 +17116,7 @@
       </c>
       <c r="AZ20" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-CE4B0C3CDE2534722A4AAADE","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F7FD9602740588A931526FB1","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA20" s="22" t="inlineStr">
@@ -17126,12 +17128,12 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>CAND-028FA513EA788FFB1FAADF4E</t>
+          <t>CAND-99A7041317161930A14478B9</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -17341,7 +17343,7 @@
       </c>
       <c r="AZ21" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-CE4B0C3CDE2534722A4AAADE","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F7FD9602740588A931526FB1","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
         </is>
       </c>
       <c r="BA21" s="22" t="inlineStr">
@@ -17353,12 +17355,12 @@
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>PKG-C269EAEEE79C014B6AC9A50D</t>
+          <t>PKG-A88C246FEB82985004538A4B</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>CAND-B994ABE33118C0EA458EFC1D</t>
+          <t>CAND-99EF846309D3820B9095938B</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -17572,7 +17574,7 @@
       </c>
       <c r="AZ22" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-68F9545F52E814CE6E2CDC73","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-260783C9E116C39D21DA207C","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA22" s="22" t="inlineStr">
@@ -17584,12 +17586,12 @@
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>CAND-377F9ED8A2D81DF0AEB07C32</t>
+          <t>CAND-E9365F5C153DFAA7DE67E118</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -17815,12 +17817,12 @@
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>CAND-F183F7D1929B7C7CD565A918</t>
+          <t>CAND-594FA1A7DB150BCEAACADDBB</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -18012,7 +18014,7 @@
       </c>
       <c r="AR24" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS24" s="22" t="inlineStr">
@@ -18022,17 +18024,17 @@
       </c>
       <c r="AT24" s="22" t="inlineStr">
         <is>
-          <t>["EVID-A49976C5217F3BD58CB83CF6","EVID-DE39AAE7BF440BBDEED43AE7","EVID-5B6C5E71AB278ACD11F995EE","EVID-ACF2755A20123E6FB62F422E","EVID-B568E4C752C9E441A2D4C225","EVID-F711CDE22C38E70F8CB18F5F","EVID-C39CBA43019A7E2E41D52699","EVID-1AAD84553C8E637E76730749","EVID-038E46D416CD216AAD824440","EVID-08768924F23A35F26342A6B5","EVID-0E02597D3213CE7CBA74C86C","EVID-EE9A980D23EE91DC1253C3A7"]</t>
+          <t>["EVID-A49976C5217F3BD58CB83CF6","EVID-DE39AAE7BF440BBDEED43AE7","EVID-5B6C5E71AB278ACD11F995EE","EVID-ACF2755A20123E6FB62F422E","EVID-B568E4C752C9E441A2D4C225","EVID-2EBC5B132CA40C28109BD66A","EVID-F711CDE22C38E70F8CB18F5F","EVID-C39CBA43019A7E2E41D52699","EVID-1AAD84553C8E637E76730749","EVID-038E46D416CD216AAD824440","EVID-08768924F23A35F26342A6B5","EVID-0E02597D3213CE7CBA74C86C","EVID-EE9A980D23EE91DC1253C3A7"]</t>
         </is>
       </c>
       <c r="AU24" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-038E46D416CD216AAD824440":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-038E46D416CD216AAD824440","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-08768924F23A35F26342A6B5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-08768924F23A35F26342A6B5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-0E02597D3213CE7CBA74C86C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0E02597D3213CE7CBA74C86C","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-1AAD84553C8E637E76730749":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1AAD84553C8E637E76730749","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-5B6C5E71AB278ACD11F995EE":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-5B6C5E71AB278ACD11F995EE","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-A49976C5217F3BD58CB83CF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A49976C5217F3BD58CB83CF6","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-ACF2755A20123E6FB62F422E":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-ACF2755A20123E6FB62F422E","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-B568E4C752C9E441A2D4C225":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-B568E4C752C9E441A2D4C225","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":12.0},"EVID-C39CBA43019A7E2E41D52699":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C39CBA43019A7E2E41D52699","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":15000},"EVID-DE39AAE7BF440BBDEED43AE7":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-DE39AAE7BF440BBDEED43AE7","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-EE9A980D23EE91DC1253C3A7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE9A980D23EE91DC1253C3A7","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-F711CDE22C38E70F8CB18F5F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F711CDE22C38E70F8CB18F5F","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3600}}</t>
+          <t>{"EVID-038E46D416CD216AAD824440":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-038E46D416CD216AAD824440","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-08768924F23A35F26342A6B5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-08768924F23A35F26342A6B5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-0E02597D3213CE7CBA74C86C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0E02597D3213CE7CBA74C86C","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-1AAD84553C8E637E76730749":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1AAD84553C8E637E76730749","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-2EBC5B132CA40C28109BD66A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-2EBC5B132CA40C28109BD66A","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-5B6C5E71AB278ACD11F995EE":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-5B6C5E71AB278ACD11F995EE","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-A49976C5217F3BD58CB83CF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A49976C5217F3BD58CB83CF6","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-ACF2755A20123E6FB62F422E":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-ACF2755A20123E6FB62F422E","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-B568E4C752C9E441A2D4C225":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-B568E4C752C9E441A2D4C225","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":12.0},"EVID-C39CBA43019A7E2E41D52699":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C39CBA43019A7E2E41D52699","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":15000},"EVID-DE39AAE7BF440BBDEED43AE7":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-DE39AAE7BF440BBDEED43AE7","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-EE9A980D23EE91DC1253C3A7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE9A980D23EE91DC1253C3A7","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-F711CDE22C38E70F8CB18F5F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F711CDE22C38E70F8CB18F5F","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3600}}</t>
         </is>
       </c>
       <c r="AV24" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-DE39AAE7BF440BBDEED43AE7","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-5B6C5E71AB278ACD11F995EE","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-ACF2755A20123E6FB62F422E","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-B568E4C752C9E441A2D4C225","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F711CDE22C38E70F8CB18F5F","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C39CBA43019A7E2E41D52699","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-DE39AAE7BF440BBDEED43AE7","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-5B6C5E71AB278ACD11F995EE","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-ACF2755A20123E6FB62F422E","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-B568E4C752C9E441A2D4C225","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-2EBC5B132CA40C28109BD66A","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F711CDE22C38E70F8CB18F5F","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C39CBA43019A7E2E41D52699","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW24" s="22" t="inlineStr">
@@ -18064,12 +18066,12 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>CAND-80AFEAAC17B90B6740091CD3</t>
+          <t>CAND-0076DB22E0A75900B6DEDFC0</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -18279,7 +18281,7 @@
       </c>
       <c r="AZ25" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY","scenario_id":"SCN-CC786000B1366D95D0796012","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY","scenario_id":"SCN-11A38429F99045CFB20CD972","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA25" s="22" t="inlineStr">
@@ -18291,12 +18293,12 @@
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>CAND-0EF3E4718784E98BA23D5C7D</t>
+          <t>CAND-3E445C7CDDA306563C04C796</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -18518,12 +18520,12 @@
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>CAND-CEA5FCCDA651DD76B15D02CA</t>
+          <t>CAND-05ACDA7D28A13AAFDF7F3D64</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -18745,12 +18747,12 @@
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>PKG-CC33BDB742BBCA3EB867C0A2</t>
+          <t>PKG-2F1E4946047B169734FD3E7C</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>CAND-02A4A2C622C961DA8C1E29A5</t>
+          <t>CAND-778A29A01C5B19EC469FD4F6</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
@@ -18964,7 +18966,7 @@
       </c>
       <c r="AZ28" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-AE1383D5FC2C30D7B1E8A625","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-38846EB94CC8C77FF71512AF","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA28" s="22" t="inlineStr">
@@ -18976,12 +18978,12 @@
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>CAND-8E9FD2A57101E24DC21989E6</t>
+          <t>CAND-1A583E97BA46A3119E6BC8BB</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -19207,12 +19209,12 @@
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>CAND-54F63D00E2EFC9427B7F8293</t>
+          <t>CAND-5BDB30FEB9889EFB8854DA36</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -19386,7 +19388,7 @@
       </c>
       <c r="AR30" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS30" s="22" t="inlineStr">
@@ -19396,17 +19398,17 @@
       </c>
       <c r="AT30" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4AD9BFC520F810E375C9F267","EVID-CE93052A4088BD04DDDFC0B4","EVID-565A318F59FE2D81C60059DB","EVID-8337939F0AFF21D2C6FE2977","EVID-91B0650858728DBD33B126CD","EVID-5E83882E9CB63D27C16F478D","EVID-FAA816B37A09EEEF7686D7A7","EVID-7A91A2021AA57C5F33FA42C6","EVID-736AEF23E7ED9DFBA2AA3EED","EVID-81523112C9E873756ADB144D","EVID-D75BC7CEF9C5E360F50654AF","EVID-A75501B0489D683DBC75D3A9"]</t>
+          <t>["EVID-4AD9BFC520F810E375C9F267","EVID-CE93052A4088BD04DDDFC0B4","EVID-565A318F59FE2D81C60059DB","EVID-8337939F0AFF21D2C6FE2977","EVID-91B0650858728DBD33B126CD","EVID-32A60495C6A356B84CEDB62C","EVID-5E83882E9CB63D27C16F478D","EVID-FAA816B37A09EEEF7686D7A7","EVID-7A91A2021AA57C5F33FA42C6","EVID-736AEF23E7ED9DFBA2AA3EED","EVID-81523112C9E873756ADB144D","EVID-D75BC7CEF9C5E360F50654AF","EVID-A75501B0489D683DBC75D3A9"]</t>
         </is>
       </c>
       <c r="AU30" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-4AD9BFC520F810E375C9F267":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AD9BFC520F810E375C9F267","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-565A318F59FE2D81C60059DB":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-565A318F59FE2D81C60059DB","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-5E83882E9CB63D27C16F478D":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5E83882E9CB63D27C16F478D","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2200},"EVID-736AEF23E7ED9DFBA2AA3EED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-736AEF23E7ED9DFBA2AA3EED","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-7A91A2021AA57C5F33FA42C6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A91A2021AA57C5F33FA42C6","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-81523112C9E873756ADB144D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-81523112C9E873756ADB144D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-8337939F0AFF21D2C6FE2977":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8337939F0AFF21D2C6FE2977","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-91B0650858728DBD33B126CD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-91B0650858728DBD33B126CD","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.2},"EVID-A75501B0489D683DBC75D3A9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A75501B0489D683DBC75D3A9","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242},"EVID-CE93052A4088BD04DDDFC0B4":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-CE93052A4088BD04DDDFC0B4","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D75BC7CEF9C5E360F50654AF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D75BC7CEF9C5E360F50654AF","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-FAA816B37A09EEEF7686D7A7":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FAA816B37A09EEEF7686D7A7","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7000}}</t>
+          <t>{"EVID-32A60495C6A356B84CEDB62C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-32A60495C6A356B84CEDB62C","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-4AD9BFC520F810E375C9F267":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AD9BFC520F810E375C9F267","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-565A318F59FE2D81C60059DB":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-565A318F59FE2D81C60059DB","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-5E83882E9CB63D27C16F478D":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5E83882E9CB63D27C16F478D","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2200},"EVID-736AEF23E7ED9DFBA2AA3EED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-736AEF23E7ED9DFBA2AA3EED","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-7A91A2021AA57C5F33FA42C6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A91A2021AA57C5F33FA42C6","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-81523112C9E873756ADB144D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-81523112C9E873756ADB144D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-8337939F0AFF21D2C6FE2977":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8337939F0AFF21D2C6FE2977","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-91B0650858728DBD33B126CD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-91B0650858728DBD33B126CD","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.2},"EVID-A75501B0489D683DBC75D3A9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A75501B0489D683DBC75D3A9","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242},"EVID-CE93052A4088BD04DDDFC0B4":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-CE93052A4088BD04DDDFC0B4","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D75BC7CEF9C5E360F50654AF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D75BC7CEF9C5E360F50654AF","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-FAA816B37A09EEEF7686D7A7":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FAA816B37A09EEEF7686D7A7","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7000}}</t>
         </is>
       </c>
       <c r="AV30" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-CE93052A4088BD04DDDFC0B4","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-565A318F59FE2D81C60059DB","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-8337939F0AFF21D2C6FE2977","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-91B0650858728DBD33B126CD","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-5E83882E9CB63D27C16F478D","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-FAA816B37A09EEEF7686D7A7","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-CE93052A4088BD04DDDFC0B4","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-565A318F59FE2D81C60059DB","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-8337939F0AFF21D2C6FE2977","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-91B0650858728DBD33B126CD","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-32A60495C6A356B84CEDB62C","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-5E83882E9CB63D27C16F478D","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-FAA816B37A09EEEF7686D7A7","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW30" s="22" t="inlineStr">
@@ -19426,7 +19428,7 @@
       </c>
       <c r="AZ30" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-1B656E36C1F436B2D31FEE71","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-7B8535F47F089440D4CC3A6C","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA30" s="22" t="inlineStr">
@@ -19438,12 +19440,12 @@
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>CAND-E0276ED21AF1CA6ABDA3685B</t>
+          <t>CAND-7EAB4FCCBC7AFDB42AB9A6AD</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -19653,7 +19655,7 @@
       </c>
       <c r="AZ31" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-1B656E36C1F436B2D31FEE71","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-7B8535F47F089440D4CC3A6C","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA31" s="22" t="inlineStr">
@@ -19665,12 +19667,12 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>CAND-C84C3FCC5EB73EA428D9DCED</t>
+          <t>CAND-95461AE6689D3B91CFE81AB8</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -19892,12 +19894,12 @@
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>CAND-E390311B2EF9D01C3C6F7D26</t>
+          <t>CAND-161D0B44D8BDFBCB35A95C44</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -20119,12 +20121,12 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>PKG-69BA220DC5EC020D84CA55CB</t>
+          <t>PKG-1A36A56E13C0F1C844A9B720</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>CAND-6E8B69CCEE3CE8F4973519A4</t>
+          <t>CAND-F9500B9F40B865363F195297</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -20338,7 +20340,7 @@
       </c>
       <c r="AZ34" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-562458A34AA20834D8E26D00","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-ACAFEDE99BA9CDD0084D6217","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA34" s="22" t="inlineStr">
@@ -20350,12 +20352,12 @@
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>CAND-6B9EEF223CD62A0B0720714A</t>
+          <t>CAND-D1C4FA26B6E3600A9A21AC88</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -20581,12 +20583,12 @@
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>CAND-F878D946224283BA589FD98A</t>
+          <t>CAND-1DF24738E803FAC91A3628A9</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -20760,7 +20762,7 @@
       </c>
       <c r="AR36" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS36" s="22" t="inlineStr">
@@ -20770,17 +20772,17 @@
       </c>
       <c r="AT36" s="22" t="inlineStr">
         <is>
-          <t>["EVID-FBBD7CA62DAF0F3CE7D41AA7","EVID-3B28A16644A2A57DA7060FEB","EVID-A15E47B73E05ED02C3C19CD2","EVID-D279C5B2E8AE57BAA1C94081","EVID-9BFCB9789587DE8B131F843F","EVID-29BAC5FF64717D55401618A4","EVID-754094313E68ACA0FA861C99","EVID-48F5313AC3181ACA7638598F","EVID-6A828E733BFBF0C431954454","EVID-683B1AE13834CF7A72976437","EVID-79E52EE17204D63C325353E3","EVID-338FBC5F582A0343A81D5D35"]</t>
+          <t>["EVID-FBBD7CA62DAF0F3CE7D41AA7","EVID-3B28A16644A2A57DA7060FEB","EVID-A15E47B73E05ED02C3C19CD2","EVID-D279C5B2E8AE57BAA1C94081","EVID-9BFCB9789587DE8B131F843F","EVID-7D9F1BB280D23FF7B2FCA3C7","EVID-29BAC5FF64717D55401618A4","EVID-754094313E68ACA0FA861C99","EVID-48F5313AC3181ACA7638598F","EVID-6A828E733BFBF0C431954454","EVID-683B1AE13834CF7A72976437","EVID-79E52EE17204D63C325353E3","EVID-338FBC5F582A0343A81D5D35"]</t>
         </is>
       </c>
       <c r="AU36" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-29BAC5FF64717D55401618A4":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-29BAC5FF64717D55401618A4","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2800},"EVID-338FBC5F582A0343A81D5D35":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-338FBC5F582A0343A81D5D35","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-3B28A16644A2A57DA7060FEB":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-3B28A16644A2A57DA7060FEB","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-48F5313AC3181ACA7638598F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48F5313AC3181ACA7638598F","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-683B1AE13834CF7A72976437":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-683B1AE13834CF7A72976437","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-6A828E733BFBF0C431954454":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6A828E733BFBF0C431954454","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-754094313E68ACA0FA861C99":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-754094313E68ACA0FA861C99","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":11000},"EVID-79E52EE17204D63C325353E3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-79E52EE17204D63C325353E3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-9BFCB9789587DE8B131F843F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9BFCB9789587DE8B131F843F","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-A15E47B73E05ED02C3C19CD2":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-A15E47B73E05ED02C3C19CD2","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-D279C5B2E8AE57BAA1C94081":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-D279C5B2E8AE57BAA1C94081","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-FBBD7CA62DAF0F3CE7D41AA7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FBBD7CA62DAF0F3CE7D41AA7","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"}}</t>
+          <t>{"EVID-29BAC5FF64717D55401618A4":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-29BAC5FF64717D55401618A4","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2800},"EVID-338FBC5F582A0343A81D5D35":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-338FBC5F582A0343A81D5D35","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-3B28A16644A2A57DA7060FEB":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-3B28A16644A2A57DA7060FEB","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-48F5313AC3181ACA7638598F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48F5313AC3181ACA7638598F","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-683B1AE13834CF7A72976437":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-683B1AE13834CF7A72976437","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-6A828E733BFBF0C431954454":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6A828E733BFBF0C431954454","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-754094313E68ACA0FA861C99":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-754094313E68ACA0FA861C99","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":11000},"EVID-79E52EE17204D63C325353E3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-79E52EE17204D63C325353E3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-7D9F1BB280D23FF7B2FCA3C7":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-7D9F1BB280D23FF7B2FCA3C7","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-9BFCB9789587DE8B131F843F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9BFCB9789587DE8B131F843F","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-A15E47B73E05ED02C3C19CD2":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-A15E47B73E05ED02C3C19CD2","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-D279C5B2E8AE57BAA1C94081":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-D279C5B2E8AE57BAA1C94081","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-FBBD7CA62DAF0F3CE7D41AA7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FBBD7CA62DAF0F3CE7D41AA7","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"}}</t>
         </is>
       </c>
       <c r="AV36" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-3B28A16644A2A57DA7060FEB","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-A15E47B73E05ED02C3C19CD2","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-D279C5B2E8AE57BAA1C94081","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-9BFCB9789587DE8B131F843F","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-29BAC5FF64717D55401618A4","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-754094313E68ACA0FA861C99","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-3B28A16644A2A57DA7060FEB","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-A15E47B73E05ED02C3C19CD2","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-D279C5B2E8AE57BAA1C94081","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-9BFCB9789587DE8B131F843F","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-7D9F1BB280D23FF7B2FCA3C7","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-29BAC5FF64717D55401618A4","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-754094313E68ACA0FA861C99","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW36" s="22" t="inlineStr">
@@ -20800,7 +20802,7 @@
       </c>
       <c r="AZ36" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-D7CBE49F5C50DE0E816A9CD2","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-3F6C04F0A9ED249FBC064295","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA36" s="22" t="inlineStr">
@@ -20812,12 +20814,12 @@
     <row r="37" ht="32" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>CAND-8931F3BE78641A385D65130D</t>
+          <t>CAND-79B0BE87400A9CFA38C8B82A</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -21027,7 +21029,7 @@
       </c>
       <c r="AZ37" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-D7CBE49F5C50DE0E816A9CD2","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-3F6C04F0A9ED249FBC064295","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA37" s="22" t="inlineStr">
@@ -21039,12 +21041,12 @@
     <row r="38" ht="32" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>CAND-1D1B4EC16ED60AB22768C5E8</t>
+          <t>CAND-61DB2D99CF2B5F9EA7BB61F6</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -21266,12 +21268,12 @@
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>CAND-2B65CE34434D627E7C4E7D0B</t>
+          <t>CAND-F05F1CA9672C73FA7DBC8109</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -21481,7 +21483,7 @@
       </c>
       <c r="AZ39" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-D7CBE49F5C50DE0E816A9CD2","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-3F6C04F0A9ED249FBC064295","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA39" s="22" t="inlineStr">
@@ -21493,12 +21495,12 @@
     <row r="40" ht="32" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>PKG-1B297C98438DC42F237017DA</t>
+          <t>PKG-2A3B6FE2F6DF3951AD5A991C</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>CAND-5D8E6A15050D0BC21F82DB67</t>
+          <t>CAND-BC13A971B047ACEFA8054A4E</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
@@ -21712,7 +21714,7 @@
       </c>
       <c r="AZ40" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-509F0B84125F5B7EFD41B34F","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-B39CD91F38AECF06C4899822","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA40" s="22" t="inlineStr">
@@ -21724,12 +21726,12 @@
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>CAND-BE64253C1F5541854D9D5F73</t>
+          <t>CAND-8FC877BAEE26947E63D85BAC</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -21955,12 +21957,12 @@
     <row r="42" ht="32" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>CAND-D5D6479CF95BC13FC20D6F5F</t>
+          <t>CAND-C2FAFFBA66195CD03818B824</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
@@ -22152,7 +22154,7 @@
       </c>
       <c r="AR42" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS42" s="22" t="inlineStr">
@@ -22162,17 +22164,17 @@
       </c>
       <c r="AT42" s="22" t="inlineStr">
         <is>
-          <t>["EVID-6F2210B4A714E07FF2B336E5","EVID-2ADB478E1643572CD5941C8A","EVID-07150EBD7C85821371FC5C6D","EVID-2452143F8B9B2CED497389CF","EVID-1C88354197DE4989BF278EC4","EVID-935962377953AEF38189FA9F","EVID-CF2C3BD20C77D10B63ED3718","EVID-38E12A59BDB085C9ED17E3D5","EVID-D6B273BC561A1E053AB22E8C","EVID-ECEA4B5972B35E88B483B834","EVID-755CFD7941CE94A93847E0B3","EVID-11DE4B9E2CE51DBAE4B4614C"]</t>
+          <t>["EVID-6F2210B4A714E07FF2B336E5","EVID-2ADB478E1643572CD5941C8A","EVID-07150EBD7C85821371FC5C6D","EVID-2452143F8B9B2CED497389CF","EVID-1C88354197DE4989BF278EC4","EVID-19A0CD94320ACC8CE6577AB0","EVID-935962377953AEF38189FA9F","EVID-CF2C3BD20C77D10B63ED3718","EVID-38E12A59BDB085C9ED17E3D5","EVID-D6B273BC561A1E053AB22E8C","EVID-ECEA4B5972B35E88B483B834","EVID-755CFD7941CE94A93847E0B3","EVID-11DE4B9E2CE51DBAE4B4614C"]</t>
         </is>
       </c>
       <c r="AU42" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-07150EBD7C85821371FC5C6D":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-07150EBD7C85821371FC5C6D","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-11DE4B9E2CE51DBAE4B4614C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-11DE4B9E2CE51DBAE4B4614C","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-1C88354197DE4989BF278EC4":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1C88354197DE4989BF278EC4","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-2452143F8B9B2CED497389CF":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2452143F8B9B2CED497389CF","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-2ADB478E1643572CD5941C8A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2ADB478E1643572CD5941C8A","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-38E12A59BDB085C9ED17E3D5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-38E12A59BDB085C9ED17E3D5","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-6F2210B4A714E07FF2B336E5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6F2210B4A714E07FF2B336E5","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-755CFD7941CE94A93847E0B3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-755CFD7941CE94A93847E0B3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-935962377953AEF38189FA9F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-935962377953AEF38189FA9F","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2400},"EVID-CF2C3BD20C77D10B63ED3718":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-CF2C3BD20C77D10B63ED3718","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":8000},"EVID-D6B273BC561A1E053AB22E8C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D6B273BC561A1E053AB22E8C","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-ECEA4B5972B35E88B483B834":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ECEA4B5972B35E88B483B834","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0}}</t>
+          <t>{"EVID-07150EBD7C85821371FC5C6D":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-07150EBD7C85821371FC5C6D","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-11DE4B9E2CE51DBAE4B4614C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-11DE4B9E2CE51DBAE4B4614C","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-19A0CD94320ACC8CE6577AB0":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-19A0CD94320ACC8CE6577AB0","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-1C88354197DE4989BF278EC4":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1C88354197DE4989BF278EC4","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-2452143F8B9B2CED497389CF":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2452143F8B9B2CED497389CF","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-2ADB478E1643572CD5941C8A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2ADB478E1643572CD5941C8A","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-38E12A59BDB085C9ED17E3D5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-38E12A59BDB085C9ED17E3D5","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-6F2210B4A714E07FF2B336E5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6F2210B4A714E07FF2B336E5","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-755CFD7941CE94A93847E0B3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-755CFD7941CE94A93847E0B3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-935962377953AEF38189FA9F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-935962377953AEF38189FA9F","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2400},"EVID-CF2C3BD20C77D10B63ED3718":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-CF2C3BD20C77D10B63ED3718","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":8000},"EVID-D6B273BC561A1E053AB22E8C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D6B273BC561A1E053AB22E8C","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-ECEA4B5972B35E88B483B834":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ECEA4B5972B35E88B483B834","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0}}</t>
         </is>
       </c>
       <c r="AV42" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-2ADB478E1643572CD5941C8A","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-07150EBD7C85821371FC5C6D","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-2452143F8B9B2CED497389CF","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-1C88354197DE4989BF278EC4","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-935962377953AEF38189FA9F","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-CF2C3BD20C77D10B63ED3718","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-2ADB478E1643572CD5941C8A","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-07150EBD7C85821371FC5C6D","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-2452143F8B9B2CED497389CF","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-1C88354197DE4989BF278EC4","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-19A0CD94320ACC8CE6577AB0","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-935962377953AEF38189FA9F","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-CF2C3BD20C77D10B63ED3718","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW42" s="22" t="inlineStr">
@@ -22204,12 +22206,12 @@
     <row r="43" ht="32" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>CAND-754355444A1A789B2EC1DC71</t>
+          <t>CAND-846E33011FE609606A10FA5B</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr">
@@ -22431,12 +22433,12 @@
     <row r="44" ht="32" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>CAND-B2C77C0E282E77BA3CA93FFD</t>
+          <t>CAND-20D4E14BE93B700A40985E38</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
@@ -22658,12 +22660,12 @@
     <row r="45" ht="32" customHeight="1">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>CAND-05ECA8EB06C456A0556818F8</t>
+          <t>CAND-802B5C5EAE5E3991FDB65CA7</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr">
@@ -22909,17 +22911,17 @@
     <row r="46" ht="32" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>PKG-174715E982DCBFB8A89E70C3</t>
+          <t>PKG-C2BA122DB9F5C7BA674FEB5A</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>CAND-D1C8429D0D427860A3152AFC</t>
+          <t>CAND-6B089B819AB4B39987DDEE98</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>WH-SERVERLESS-MIGRATE-001</t>
+          <t>WH-WAREHOUSE-TYPE-ASSESS-001</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
@@ -22954,7 +22956,7 @@
       </c>
       <c r="J46" s="18" t="inlineStr">
         <is>
-          <t>TEST_REQUIRED</t>
+          <t>INSUFFICIENT_EVIDENCE</t>
         </is>
       </c>
       <c r="K46" s="15" t="inlineStr">
@@ -22969,24 +22971,24 @@
       </c>
       <c r="M46" s="15" t="inlineStr">
         <is>
-          <t>SERVERLESS</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="N46" s="15" t="inlineStr">
         <is>
-          <t>Serverless is evaluated as a separate migration experiment with a pre-canary DBU/AWS counterfactual and deterministic compatibility gate.</t>
+          <t>Migration is judged on a pre-canary cost comparison, but the current epoch has fewer than 7 days of billing history to price it.</t>
         </is>
       </c>
       <c r="O46" s="21" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="P46" s="18" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="Q46" s="18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R46" s="16" t="inlineStr">
         <is>
@@ -22995,7 +22997,7 @@
       </c>
       <c r="S46" s="18" t="inlineStr">
         <is>
-          <t>COST_INCREASE</t>
+          <t>UNAVAILABLE</t>
         </is>
       </c>
       <c r="T46" s="19" t="n">
@@ -23007,41 +23009,65 @@
       <c r="V46" s="19" t="n">
         <v>163840</v>
       </c>
-      <c r="W46" s="19" t="n">
-        <v>-328666.67</v>
-      </c>
-      <c r="X46" s="19" t="n">
-        <v>-328666.67</v>
-      </c>
-      <c r="Y46" s="19" t="n">
-        <v>-328666.67</v>
-      </c>
-      <c r="Z46" s="19" t="n">
-        <v>151840</v>
-      </c>
-      <c r="AA46" s="19" t="n">
-        <v>151840</v>
-      </c>
-      <c r="AB46" s="19" t="n">
-        <v>151840</v>
-      </c>
-      <c r="AC46" s="19" t="n">
-        <v>-176826.67</v>
-      </c>
-      <c r="AD46" s="19" t="n">
-        <v>-176826.67</v>
-      </c>
-      <c r="AE46" s="19" t="n">
-        <v>-176826.67</v>
-      </c>
-      <c r="AF46" s="19" t="n">
-        <v>340666.67</v>
-      </c>
-      <c r="AG46" s="19" t="n">
-        <v>340666.67</v>
-      </c>
-      <c r="AH46" s="19" t="n">
-        <v>340666.67</v>
+      <c r="W46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="X46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="Y46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="Z46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AA46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AB46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AC46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AD46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AE46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AF46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AG46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AH46" s="19" t="inlineStr">
+        <is>
+          <t>UNAVAILABLE</t>
+        </is>
       </c>
       <c r="AI46" s="18" t="b">
         <v>0</v>
@@ -23093,7 +23119,7 @@
       </c>
       <c r="AS46" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":1.0,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
         </is>
       </c>
       <c r="AT46" s="22" t="inlineStr">
@@ -23118,17 +23144,17 @@
       </c>
       <c r="AX46" s="22" t="inlineStr">
         <is>
-          <t>["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AY46" s="22" t="inlineStr">
         <is>
-          <t>["A_B_COST_PERFORMANCE_VALIDATION_REQUIRED"]</t>
+          <t>["COST_HISTORY_INSUFFICIENT"]</t>
         </is>
       </c>
       <c r="AZ46" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-FDB5EC0875B1F59325F0FADD","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="BA46" s="22" t="inlineStr">
@@ -23140,12 +23166,12 @@
     <row r="47" ht="32" customHeight="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>CAND-8AE2220BFA703CEB2977138F</t>
+          <t>CAND-BC0EEDE6473CF891F03E312D</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">
@@ -23371,12 +23397,12 @@
     <row r="48" ht="32" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>CAND-8CF2F68ED84D562D3D9E5560</t>
+          <t>CAND-B1DE4DC4AEBC6BA9039D5664</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
@@ -23550,7 +23576,7 @@
       </c>
       <c r="AR48" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS48" s="22" t="inlineStr">
@@ -23560,17 +23586,17 @@
       </c>
       <c r="AT48" s="22" t="inlineStr">
         <is>
-          <t>["EVID-7C38C1C5C0A50E5541957C70","EVID-9497EEFAC96FC0FF43049E5A","EVID-6B64C5D537A164CF2D9E9E83","EVID-2990A0D93C8B36C0E61B4460","EVID-0183D69D139344A5B63A4692","EVID-3643FB63351B00006C91E749","EVID-1556195FEAB1A5CF132FC710","EVID-0B2D8687B4C5CC349527EF25","EVID-AC8BB4FF1601DC693A4FC67D","EVID-D9753C2D5E31F0E204F772E6","EVID-AEC33BC02A330A7D397D1BA5","EVID-7509E42EBDD3C2025EEECD35"]</t>
+          <t>["EVID-7C38C1C5C0A50E5541957C70","EVID-9497EEFAC96FC0FF43049E5A","EVID-6B64C5D537A164CF2D9E9E83","EVID-2990A0D93C8B36C0E61B4460","EVID-0183D69D139344A5B63A4692","EVID-A14A6B1ED36B01E84398DF00","EVID-3643FB63351B00006C91E749","EVID-1556195FEAB1A5CF132FC710","EVID-0B2D8687B4C5CC349527EF25","EVID-AC8BB4FF1601DC693A4FC67D","EVID-D9753C2D5E31F0E204F772E6","EVID-AEC33BC02A330A7D397D1BA5","EVID-7509E42EBDD3C2025EEECD35"]</t>
         </is>
       </c>
       <c r="AU48" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0183D69D139344A5B63A4692":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0183D69D139344A5B63A4692","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-0B2D8687B4C5CC349527EF25":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0B2D8687B4C5CC349527EF25","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-1556195FEAB1A5CF132FC710":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1556195FEAB1A5CF132FC710","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":5500},"EVID-2990A0D93C8B36C0E61B4460":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2990A0D93C8B36C0E61B4460","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-3643FB63351B00006C91E749":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-3643FB63351B00006C91E749","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1800},"EVID-6B64C5D537A164CF2D9E9E83":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-6B64C5D537A164CF2D9E9E83","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-7509E42EBDD3C2025EEECD35":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7509E42EBDD3C2025EEECD35","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-7C38C1C5C0A50E5541957C70":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7C38C1C5C0A50E5541957C70","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-9497EEFAC96FC0FF43049E5A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-9497EEFAC96FC0FF43049E5A","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-AC8BB4FF1601DC693A4FC67D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC8BB4FF1601DC693A4FC67D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-AEC33BC02A330A7D397D1BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AEC33BC02A330A7D397D1BA5","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-D9753C2D5E31F0E204F772E6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D9753C2D5E31F0E204F772E6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0}}</t>
+          <t>{"EVID-0183D69D139344A5B63A4692":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0183D69D139344A5B63A4692","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-0B2D8687B4C5CC349527EF25":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0B2D8687B4C5CC349527EF25","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-1556195FEAB1A5CF132FC710":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1556195FEAB1A5CF132FC710","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":5500},"EVID-2990A0D93C8B36C0E61B4460":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2990A0D93C8B36C0E61B4460","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-3643FB63351B00006C91E749":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-3643FB63351B00006C91E749","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1800},"EVID-6B64C5D537A164CF2D9E9E83":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-6B64C5D537A164CF2D9E9E83","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-7509E42EBDD3C2025EEECD35":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7509E42EBDD3C2025EEECD35","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-7C38C1C5C0A50E5541957C70":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7C38C1C5C0A50E5541957C70","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-9497EEFAC96FC0FF43049E5A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-9497EEFAC96FC0FF43049E5A","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-A14A6B1ED36B01E84398DF00":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-A14A6B1ED36B01E84398DF00","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-AC8BB4FF1601DC693A4FC67D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC8BB4FF1601DC693A4FC67D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-AEC33BC02A330A7D397D1BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AEC33BC02A330A7D397D1BA5","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-D9753C2D5E31F0E204F772E6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D9753C2D5E31F0E204F772E6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0}}</t>
         </is>
       </c>
       <c r="AV48" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-9497EEFAC96FC0FF43049E5A","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-6B64C5D537A164CF2D9E9E83","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-2990A0D93C8B36C0E61B4460","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-0183D69D139344A5B63A4692","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-3643FB63351B00006C91E749","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-1556195FEAB1A5CF132FC710","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-9497EEFAC96FC0FF43049E5A","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-6B64C5D537A164CF2D9E9E83","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-2990A0D93C8B36C0E61B4460","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-0183D69D139344A5B63A4692","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-A14A6B1ED36B01E84398DF00","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-3643FB63351B00006C91E749","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-1556195FEAB1A5CF132FC710","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW48" s="22" t="inlineStr">
@@ -23590,7 +23616,7 @@
       </c>
       <c r="AZ48" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-EFE76D0072038BA31048924A","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-A7F14CD75A7AA486F6E590A9","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA48" s="22" t="inlineStr">
@@ -23602,12 +23628,12 @@
     <row r="49" ht="32" customHeight="1">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>CAND-D7E581D7637D85BCED1CACDC</t>
+          <t>CAND-AAE2D61246CC19F3D31359B2</t>
         </is>
       </c>
       <c r="C49" s="14" t="inlineStr">
@@ -23817,7 +23843,7 @@
       </c>
       <c r="AZ49" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-EFE76D0072038BA31048924A","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-A7F14CD75A7AA486F6E590A9","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA49" s="22" t="inlineStr">
@@ -23829,12 +23855,12 @@
     <row r="50" ht="32" customHeight="1">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>CAND-B9252C817CCDE26D5CB43B2C</t>
+          <t>CAND-6BE294F5E618F24E926B049B</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
@@ -24056,12 +24082,12 @@
     <row r="51" ht="32" customHeight="1">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>CAND-EB4C0826388DAF0095655F04</t>
+          <t>CAND-627B2620330D84D5C80F1643</t>
         </is>
       </c>
       <c r="C51" s="14" t="inlineStr">
@@ -24283,12 +24309,12 @@
     <row r="52" ht="32" customHeight="1">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>PKG-127DD763EAF773382520242A</t>
+          <t>PKG-0BF64043B3246E34077278A4</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>CAND-FF7A26AD3267B8B24B7DDE29</t>
+          <t>CAND-71D893FD78F2362AC4404318</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
@@ -24502,7 +24528,7 @@
       </c>
       <c r="AZ52" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-0DE5AFA24E42CA4905AA2E90","scenario_name":"Plan B — Pro migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-010708604C897CBD8CB6999B","scenario_name":"Plan B — Pro migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA52" s="22" t="inlineStr">
@@ -24514,12 +24540,12 @@
     <row r="53" ht="32" customHeight="1">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>CAND-8C1381C8202F9B850CD6E472</t>
+          <t>CAND-453E404B55579ADA5E3CE252</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
@@ -24745,12 +24771,12 @@
     <row r="54" ht="32" customHeight="1">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>CAND-B91739B640B2882103617ADC</t>
+          <t>CAND-03498DA37C2B00C97906A378</t>
         </is>
       </c>
       <c r="C54" s="14" t="inlineStr">
@@ -24924,7 +24950,7 @@
       </c>
       <c r="AR54" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS54" s="22" t="inlineStr">
@@ -24934,17 +24960,17 @@
       </c>
       <c r="AT54" s="22" t="inlineStr">
         <is>
-          <t>["EVID-B07C2C16B6BD9A10981E2118","EVID-8E55818AEA4051473E4E572D","EVID-407FA82F270C2032644D2CE0","EVID-95F3AEE2D4248F3B8729BE25","EVID-C58346E61AE97D4F760ABDBD","EVID-605B6814A4D4E829CB5A5B66","EVID-D5CE70495019334C5543184A","EVID-E7AE32B925F94500C2F12FF9","EVID-F6A16121002CAEDD32814FF8","EVID-544F97BCD83FF9A97476FE07","EVID-E21F9261CD31D2A21EF533E4","EVID-CCA0AB4C53A92C8B3916ABDA"]</t>
+          <t>["EVID-B07C2C16B6BD9A10981E2118","EVID-8E55818AEA4051473E4E572D","EVID-407FA82F270C2032644D2CE0","EVID-95F3AEE2D4248F3B8729BE25","EVID-C58346E61AE97D4F760ABDBD","EVID-3CBD002DD8F60BA15CC1ACF8","EVID-605B6814A4D4E829CB5A5B66","EVID-D5CE70495019334C5543184A","EVID-E7AE32B925F94500C2F12FF9","EVID-F6A16121002CAEDD32814FF8","EVID-544F97BCD83FF9A97476FE07","EVID-E21F9261CD31D2A21EF533E4","EVID-CCA0AB4C53A92C8B3916ABDA"]</t>
         </is>
       </c>
       <c r="AU54" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-407FA82F270C2032644D2CE0":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-407FA82F270C2032644D2CE0","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-544F97BCD83FF9A97476FE07":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-544F97BCD83FF9A97476FE07","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-605B6814A4D4E829CB5A5B66":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-605B6814A4D4E829CB5A5B66","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3000},"EVID-8E55818AEA4051473E4E572D":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8E55818AEA4051473E4E572D","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-95F3AEE2D4248F3B8729BE25":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-95F3AEE2D4248F3B8729BE25","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-B07C2C16B6BD9A10981E2118":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B07C2C16B6BD9A10981E2118","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-C58346E61AE97D4F760ABDBD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C58346E61AE97D4F760ABDBD","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-CCA0AB4C53A92C8B3916ABDA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CCA0AB4C53A92C8B3916ABDA","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-D5CE70495019334C5543184A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D5CE70495019334C5543184A","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":9000},"EVID-E21F9261CD31D2A21EF533E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E21F9261CD31D2A21EF533E4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-E7AE32B925F94500C2F12FF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7AE32B925F94500C2F12FF9","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-F6A16121002CAEDD32814FF8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F6A16121002CAEDD32814FF8","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0}}</t>
+          <t>{"EVID-3CBD002DD8F60BA15CC1ACF8":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-3CBD002DD8F60BA15CC1ACF8","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-407FA82F270C2032644D2CE0":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-407FA82F270C2032644D2CE0","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-544F97BCD83FF9A97476FE07":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-544F97BCD83FF9A97476FE07","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-605B6814A4D4E829CB5A5B66":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-605B6814A4D4E829CB5A5B66","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3000},"EVID-8E55818AEA4051473E4E572D":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8E55818AEA4051473E4E572D","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-95F3AEE2D4248F3B8729BE25":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-95F3AEE2D4248F3B8729BE25","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-B07C2C16B6BD9A10981E2118":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B07C2C16B6BD9A10981E2118","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-C58346E61AE97D4F760ABDBD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C58346E61AE97D4F760ABDBD","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-CCA0AB4C53A92C8B3916ABDA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CCA0AB4C53A92C8B3916ABDA","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-D5CE70495019334C5543184A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D5CE70495019334C5543184A","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":9000},"EVID-E21F9261CD31D2A21EF533E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E21F9261CD31D2A21EF533E4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-E7AE32B925F94500C2F12FF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7AE32B925F94500C2F12FF9","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-F6A16121002CAEDD32814FF8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F6A16121002CAEDD32814FF8","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0}}</t>
         </is>
       </c>
       <c r="AV54" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-8E55818AEA4051473E4E572D","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-407FA82F270C2032644D2CE0","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-95F3AEE2D4248F3B8729BE25","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C58346E61AE97D4F760ABDBD","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-605B6814A4D4E829CB5A5B66","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-D5CE70495019334C5543184A","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-8E55818AEA4051473E4E572D","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-407FA82F270C2032644D2CE0","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-95F3AEE2D4248F3B8729BE25","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C58346E61AE97D4F760ABDBD","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-3CBD002DD8F60BA15CC1ACF8","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-605B6814A4D4E829CB5A5B66","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-D5CE70495019334C5543184A","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW54" s="22" t="inlineStr">
@@ -24964,7 +24990,7 @@
       </c>
       <c r="AZ54" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-2AD1B1369F3CA903C33A7F0A","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-9082F31BD0DF2BCD069F29F7","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA54" s="22" t="inlineStr">
@@ -24976,12 +25002,12 @@
     <row r="55" ht="32" customHeight="1">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>CAND-1416408891B7644B4B970F3D</t>
+          <t>CAND-AA7121CBC49CC8D096B1A310</t>
         </is>
       </c>
       <c r="C55" s="14" t="inlineStr">
@@ -25191,7 +25217,7 @@
       </c>
       <c r="AZ55" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-2AD1B1369F3CA903C33A7F0A","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-9082F31BD0DF2BCD069F29F7","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA55" s="22" t="inlineStr">
@@ -25203,12 +25229,12 @@
     <row r="56" ht="32" customHeight="1">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>CAND-EB204DD074336232DC0C1B6A</t>
+          <t>CAND-EF76206E257CE5ED39BC6191</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
@@ -25430,12 +25456,12 @@
     <row r="57" ht="32" customHeight="1">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>CAND-FBB76A767C22C2098918D09A</t>
+          <t>CAND-13F09CD6F23B59AC9235B936</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -25681,12 +25707,12 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>PKG-B2D290A3E27C723FA701C058</t>
+          <t>PKG-94221A88FCC26CDD4E97C3DB</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>CAND-E299C12314806ACD8AA15BB6</t>
+          <t>CAND-E16149DF1079E234A70FABFA</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
@@ -25900,7 +25926,7 @@
       </c>
       <c r="AZ58" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-DB87EC8AF05431F8208079A0","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-0BEADBEFBF7332316DE55F3F","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA58" s="22" t="inlineStr">
@@ -25912,12 +25938,12 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>CAND-6DAADF5C7A000999BB0EF2C1</t>
+          <t>CAND-94B14CEE087AE61D01782199</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -26143,12 +26169,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>CAND-44783D6FD480C2752BDBEC25</t>
+          <t>CAND-6A591F792934B6D67437E104</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
@@ -26322,7 +26348,7 @@
       </c>
       <c r="AR60" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS60" s="22" t="inlineStr">
@@ -26332,17 +26358,17 @@
       </c>
       <c r="AT60" s="22" t="inlineStr">
         <is>
-          <t>["EVID-45040C819E97E97C0C3512DD","EVID-FA3E117294ACCCC7A8F86BE4","EVID-61487496034534522AE52030","EVID-961B35C0E85521646A2B48D9","EVID-D3B52F66FCD31062B1B0A0B3","EVID-C0985AE59F5D8278110173AD","EVID-774DFFF76A9BF347776727F1","EVID-1C01A17AAD8C207EF44692C1","EVID-EB4062CC3E2A9EE53D82DCE2","EVID-E537D70782B304C239A5C196","EVID-147B3F71E2FD2C372C751AA6","EVID-F434EE37F0A085340B6B5BEE"]</t>
+          <t>["EVID-45040C819E97E97C0C3512DD","EVID-FA3E117294ACCCC7A8F86BE4","EVID-61487496034534522AE52030","EVID-961B35C0E85521646A2B48D9","EVID-D3B52F66FCD31062B1B0A0B3","EVID-C66F1B2AC854BD459A280659","EVID-C0985AE59F5D8278110173AD","EVID-774DFFF76A9BF347776727F1","EVID-1C01A17AAD8C207EF44692C1","EVID-EB4062CC3E2A9EE53D82DCE2","EVID-E537D70782B304C239A5C196","EVID-147B3F71E2FD2C372C751AA6","EVID-F434EE37F0A085340B6B5BEE"]</t>
         </is>
       </c>
       <c r="AU60" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-147B3F71E2FD2C372C751AA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-147B3F71E2FD2C372C751AA6","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-1C01A17AAD8C207EF44692C1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1C01A17AAD8C207EF44692C1","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-45040C819E97E97C0C3512DD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-45040C819E97E97C0C3512DD","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-61487496034534522AE52030":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-61487496034534522AE52030","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":412},"EVID-774DFFF76A9BF347776727F1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-774DFFF76A9BF347776727F1","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":36000},"EVID-961B35C0E85521646A2B48D9":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-961B35C0E85521646A2B48D9","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":2147483648},"EVID-C0985AE59F5D8278110173AD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C0985AE59F5D8278110173AD","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":11000},"EVID-D3B52F66FCD31062B1B0A0B3":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D3B52F66FCD31062B1B0A0B3","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":1.0},"EVID-E537D70782B304C239A5C196":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E537D70782B304C239A5C196","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-EB4062CC3E2A9EE53D82DCE2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EB4062CC3E2A9EE53D82DCE2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0},"EVID-F434EE37F0A085340B6B5BEE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F434EE37F0A085340B6B5BEE","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-FA3E117294ACCCC7A8F86BE4":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-FA3E117294ACCCC7A8F86BE4","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":4.2}}</t>
+          <t>{"EVID-147B3F71E2FD2C372C751AA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-147B3F71E2FD2C372C751AA6","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-1C01A17AAD8C207EF44692C1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1C01A17AAD8C207EF44692C1","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-45040C819E97E97C0C3512DD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-45040C819E97E97C0C3512DD","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-61487496034534522AE52030":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-61487496034534522AE52030","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":412},"EVID-774DFFF76A9BF347776727F1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-774DFFF76A9BF347776727F1","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":36000},"EVID-961B35C0E85521646A2B48D9":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-961B35C0E85521646A2B48D9","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":2147483648},"EVID-C0985AE59F5D8278110173AD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C0985AE59F5D8278110173AD","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":11000},"EVID-C66F1B2AC854BD459A280659":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-C66F1B2AC854BD459A280659","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-D3B52F66FCD31062B1B0A0B3":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D3B52F66FCD31062B1B0A0B3","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":1.0},"EVID-E537D70782B304C239A5C196":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E537D70782B304C239A5C196","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-EB4062CC3E2A9EE53D82DCE2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EB4062CC3E2A9EE53D82DCE2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0},"EVID-F434EE37F0A085340B6B5BEE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F434EE37F0A085340B6B5BEE","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-FA3E117294ACCCC7A8F86BE4":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-FA3E117294ACCCC7A8F86BE4","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":4.2}}</t>
         </is>
       </c>
       <c r="AV60" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-FA3E117294ACCCC7A8F86BE4","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-61487496034534522AE52030","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-961B35C0E85521646A2B48D9","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-D3B52F66FCD31062B1B0A0B3","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C0985AE59F5D8278110173AD","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-774DFFF76A9BF347776727F1","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-FA3E117294ACCCC7A8F86BE4","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-61487496034534522AE52030","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-961B35C0E85521646A2B48D9","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-D3B52F66FCD31062B1B0A0B3","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C66F1B2AC854BD459A280659","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-C0985AE59F5D8278110173AD","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-774DFFF76A9BF347776727F1","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW60" s="22" t="inlineStr">
@@ -26362,7 +26388,7 @@
       </c>
       <c r="AZ60" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY","scenario_id":"SCN-3ADBD372252C701E8605FDBF","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY","scenario_id":"SCN-0AF33099B977B44DE891DB2F","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA60" s="22" t="inlineStr">
@@ -26374,12 +26400,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>CAND-F66CC7C521D489A9BFE5369C</t>
+          <t>CAND-75EEB2BB4814F605DFACC0A5</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
@@ -26601,12 +26627,12 @@
     <row r="62" ht="32" customHeight="1">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>CAND-062229819F3FCAD00A4C42F2</t>
+          <t>CAND-E538FA9D2E0002740D3A8291</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
@@ -26828,12 +26854,12 @@
     <row r="63" ht="32" customHeight="1">
       <c r="A63" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>CAND-184A3C392690D298B3EFD5E3</t>
+          <t>CAND-1BF6312BDBD011BCBF5B17DD</t>
         </is>
       </c>
       <c r="C63" s="14" t="inlineStr">
@@ -27043,7 +27069,7 @@
       </c>
       <c r="AZ63" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-3ADBD372252C701E8605FDBF","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-0AF33099B977B44DE891DB2F","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA63" s="22" t="inlineStr">
@@ -27055,12 +27081,12 @@
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>PKG-07F463C0C249905A57984274</t>
+          <t>PKG-BA66C219708DB217FA5D16CD</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>CAND-D3DD9FFE6744CCBBA9B4F934</t>
+          <t>CAND-208C05A9E348D11DAEE662DF</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
@@ -27274,7 +27300,7 @@
       </c>
       <c r="AZ64" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-3B15D95786681E2F1586255E","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-85DD6FDC4F7D607B91486DB3","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA64" s="22" t="inlineStr">
@@ -27286,12 +27312,12 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>CAND-1531D4BD13B32E9441CF326C</t>
+          <t>CAND-B18907413D2DF98545B33865</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
@@ -27517,12 +27543,12 @@
     <row r="66" ht="32" customHeight="1">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>CAND-B6913E34C50A503A1D6DBEA0</t>
+          <t>CAND-BBB38F2B1B9EA80282892372</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
@@ -27696,7 +27722,7 @@
       </c>
       <c r="AR66" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS66" s="22" t="inlineStr">
@@ -27706,17 +27732,17 @@
       </c>
       <c r="AT66" s="22" t="inlineStr">
         <is>
-          <t>["EVID-407B8B7358879E2BF927FBC7","EVID-0D810E83CECE50954A7A685C","EVID-4DE0BBBC3685DD0789E6ABE6","EVID-1B042AC3F3DC722F7CBD7EFC","EVID-EB0482919E76BABE5679717F","EVID-DB0003F618B6A5F1F058A80A","EVID-F83AD8E314550D8512193F6A","EVID-13D5BCA568FCB7051CE9D79D","EVID-8DCFC6A0FCF3F29EDAC2E7F6","EVID-507A4213371D1C316C1CC988","EVID-9EAB95FAF297AB482EC4BEDA","EVID-BA44DE5A4FFD511819D160D3"]</t>
+          <t>["EVID-407B8B7358879E2BF927FBC7","EVID-0D810E83CECE50954A7A685C","EVID-4DE0BBBC3685DD0789E6ABE6","EVID-1B042AC3F3DC722F7CBD7EFC","EVID-EB0482919E76BABE5679717F","EVID-FABB267EC471BEB44A231F3C","EVID-DB0003F618B6A5F1F058A80A","EVID-F83AD8E314550D8512193F6A","EVID-13D5BCA568FCB7051CE9D79D","EVID-8DCFC6A0FCF3F29EDAC2E7F6","EVID-507A4213371D1C316C1CC988","EVID-9EAB95FAF297AB482EC4BEDA","EVID-BA44DE5A4FFD511819D160D3"]</t>
         </is>
       </c>
       <c r="AU66" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0D810E83CECE50954A7A685C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-0D810E83CECE50954A7A685C","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-13D5BCA568FCB7051CE9D79D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-13D5BCA568FCB7051CE9D79D","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-1B042AC3F3DC722F7CBD7EFC":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-1B042AC3F3DC722F7CBD7EFC","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-407B8B7358879E2BF927FBC7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-407B8B7358879E2BF927FBC7","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-4DE0BBBC3685DD0789E6ABE6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-4DE0BBBC3685DD0789E6ABE6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-507A4213371D1C316C1CC988":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-507A4213371D1C316C1CC988","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-8DCFC6A0FCF3F29EDAC2E7F6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8DCFC6A0FCF3F29EDAC2E7F6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-9EAB95FAF297AB482EC4BEDA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9EAB95FAF297AB482EC4BEDA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-BA44DE5A4FFD511819D160D3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BA44DE5A4FFD511819D160D3","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-DB0003F618B6A5F1F058A80A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DB0003F618B6A5F1F058A80A","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2000},"EVID-EB0482919E76BABE5679717F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EB0482919E76BABE5679717F","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-F83AD8E314550D8512193F6A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F83AD8E314550D8512193F6A","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6000}}</t>
+          <t>{"EVID-0D810E83CECE50954A7A685C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-0D810E83CECE50954A7A685C","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-13D5BCA568FCB7051CE9D79D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-13D5BCA568FCB7051CE9D79D","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-1B042AC3F3DC722F7CBD7EFC":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-1B042AC3F3DC722F7CBD7EFC","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-407B8B7358879E2BF927FBC7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-407B8B7358879E2BF927FBC7","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-4DE0BBBC3685DD0789E6ABE6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-4DE0BBBC3685DD0789E6ABE6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-507A4213371D1C316C1CC988":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-507A4213371D1C316C1CC988","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-8DCFC6A0FCF3F29EDAC2E7F6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8DCFC6A0FCF3F29EDAC2E7F6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-9EAB95FAF297AB482EC4BEDA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9EAB95FAF297AB482EC4BEDA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-BA44DE5A4FFD511819D160D3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BA44DE5A4FFD511819D160D3","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-DB0003F618B6A5F1F058A80A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DB0003F618B6A5F1F058A80A","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2000},"EVID-EB0482919E76BABE5679717F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EB0482919E76BABE5679717F","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-F83AD8E314550D8512193F6A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F83AD8E314550D8512193F6A","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6000},"EVID-FABB267EC471BEB44A231F3C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FABB267EC471BEB44A231F3C","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
         </is>
       </c>
       <c r="AV66" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-0D810E83CECE50954A7A685C","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-4DE0BBBC3685DD0789E6ABE6","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-1B042AC3F3DC722F7CBD7EFC","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-EB0482919E76BABE5679717F","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-DB0003F618B6A5F1F058A80A","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F83AD8E314550D8512193F6A","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-0D810E83CECE50954A7A685C","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-4DE0BBBC3685DD0789E6ABE6","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-1B042AC3F3DC722F7CBD7EFC","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-EB0482919E76BABE5679717F","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-FABB267EC471BEB44A231F3C","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-DB0003F618B6A5F1F058A80A","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-F83AD8E314550D8512193F6A","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW66" s="22" t="inlineStr">
@@ -27736,7 +27762,7 @@
       </c>
       <c r="AZ66" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-BBAAF3154665B37B8FCEA1E0","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-2933621CB20E77E39795A10D","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA66" s="22" t="inlineStr">
@@ -27748,12 +27774,12 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>CAND-573D056D65CE4249801B3E1C</t>
+          <t>CAND-75C376C9ADCC22E111CF436A</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
@@ -27975,12 +28001,12 @@
     <row r="68" ht="32" customHeight="1">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>CAND-C1A802D5E5BEE703D8ED0085</t>
+          <t>CAND-97D73C8B9AB1304A39EE9B0D</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
@@ -28190,7 +28216,7 @@
       </c>
       <c r="AZ68" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-BBAAF3154665B37B8FCEA1E0","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-2933621CB20E77E39795A10D","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA68" s="22" t="inlineStr">
@@ -28202,12 +28228,12 @@
     <row r="69" ht="32" customHeight="1">
       <c r="A69" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>CAND-0F14BBC11AE756EB5AFB1C96</t>
+          <t>CAND-2B92AC15169DEA8C2A7CFA89</t>
         </is>
       </c>
       <c r="C69" s="14" t="inlineStr">
@@ -28417,7 +28443,7 @@
       </c>
       <c r="AZ69" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-BBAAF3154665B37B8FCEA1E0","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-2933621CB20E77E39795A10D","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA69" s="22" t="inlineStr">
@@ -28429,12 +28455,12 @@
     <row r="70" ht="32" customHeight="1">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>PKG-860F9BF3834486EBE41DF046</t>
+          <t>PKG-B359CEE309463C67727F4737</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>CAND-53AF57B05EB45846CF76155B</t>
+          <t>CAND-1B05132C1EC3D2449969E905</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
@@ -28648,7 +28674,7 @@
       </c>
       <c r="AZ70" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-4C7F7B95C214EEBF380310D5","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-8CEE26C6FC4807B9693BC3A5","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA70" s="22" t="inlineStr">
@@ -28660,12 +28686,12 @@
     <row r="71" ht="32" customHeight="1">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>CAND-68B1A41A04A2F7483EAD9565</t>
+          <t>CAND-7841A56D1EF08AEECA9362E6</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
@@ -28891,12 +28917,12 @@
     <row r="72" ht="32" customHeight="1">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>CAND-3B94CC5756DFC0077D2E12FE</t>
+          <t>CAND-D830ED375B9F86AA1F381EA4</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
@@ -29070,7 +29096,7 @@
       </c>
       <c r="AR72" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS72" s="22" t="inlineStr">
@@ -29080,17 +29106,17 @@
       </c>
       <c r="AT72" s="22" t="inlineStr">
         <is>
-          <t>["EVID-5A0984690AB60FAD1E646F57","EVID-0B236E96CFAADEA401D485D8","EVID-2EB24474879263CAA7D55388","EVID-7CBF6F506E34E48BF4007E49","EVID-4E5FAEE78D56DFC97676075D","EVID-51ED3C0701E326D181DDCBAD","EVID-25BA1C551957EAD856D93BB1","EVID-DBA319585E47DD744C7C91FE","EVID-075DC68712355A8DD4FE2603","EVID-D3629BE0A19E65713B480452","EVID-7D9BF92BB726FFBAED23FE74","EVID-C531CFB4DE60DA5DFFD90F03"]</t>
+          <t>["EVID-5A0984690AB60FAD1E646F57","EVID-0B236E96CFAADEA401D485D8","EVID-2EB24474879263CAA7D55388","EVID-7CBF6F506E34E48BF4007E49","EVID-4E5FAEE78D56DFC97676075D","EVID-EF8F9819481D98F6C8919AB9","EVID-51ED3C0701E326D181DDCBAD","EVID-25BA1C551957EAD856D93BB1","EVID-DBA319585E47DD744C7C91FE","EVID-075DC68712355A8DD4FE2603","EVID-D3629BE0A19E65713B480452","EVID-7D9BF92BB726FFBAED23FE74","EVID-C531CFB4DE60DA5DFFD90F03"]</t>
         </is>
       </c>
       <c r="AU72" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-075DC68712355A8DD4FE2603":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-075DC68712355A8DD4FE2603","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-0B236E96CFAADEA401D485D8":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-0B236E96CFAADEA401D485D8","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-25BA1C551957EAD856D93BB1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-25BA1C551957EAD856D93BB1","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7200},"EVID-2EB24474879263CAA7D55388":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2EB24474879263CAA7D55388","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-4E5FAEE78D56DFC97676075D":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4E5FAEE78D56DFC97676075D","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-51ED3C0701E326D181DDCBAD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-51ED3C0701E326D181DDCBAD","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2100},"EVID-5A0984690AB60FAD1E646F57":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5A0984690AB60FAD1E646F57","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-7CBF6F506E34E48BF4007E49":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-7CBF6F506E34E48BF4007E49","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-7D9BF92BB726FFBAED23FE74":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7D9BF92BB726FFBAED23FE74","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-C531CFB4DE60DA5DFFD90F03":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C531CFB4DE60DA5DFFD90F03","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-D3629BE0A19E65713B480452":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3629BE0A19E65713B480452","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0},"EVID-DBA319585E47DD744C7C91FE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DBA319585E47DD744C7C91FE","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0}}</t>
+          <t>{"EVID-075DC68712355A8DD4FE2603":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-075DC68712355A8DD4FE2603","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-0B236E96CFAADEA401D485D8":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-0B236E96CFAADEA401D485D8","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-25BA1C551957EAD856D93BB1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-25BA1C551957EAD856D93BB1","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7200},"EVID-2EB24474879263CAA7D55388":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2EB24474879263CAA7D55388","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-4E5FAEE78D56DFC97676075D":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4E5FAEE78D56DFC97676075D","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-51ED3C0701E326D181DDCBAD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-51ED3C0701E326D181DDCBAD","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2100},"EVID-5A0984690AB60FAD1E646F57":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5A0984690AB60FAD1E646F57","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-7CBF6F506E34E48BF4007E49":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-7CBF6F506E34E48BF4007E49","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-7D9BF92BB726FFBAED23FE74":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7D9BF92BB726FFBAED23FE74","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-C531CFB4DE60DA5DFFD90F03":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C531CFB4DE60DA5DFFD90F03","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-D3629BE0A19E65713B480452":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3629BE0A19E65713B480452","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0},"EVID-DBA319585E47DD744C7C91FE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DBA319585E47DD744C7C91FE","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-EF8F9819481D98F6C8919AB9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF8F9819481D98F6C8919AB9","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
         </is>
       </c>
       <c r="AV72" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-0B236E96CFAADEA401D485D8","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-2EB24474879263CAA7D55388","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-7CBF6F506E34E48BF4007E49","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-4E5FAEE78D56DFC97676075D","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-51ED3C0701E326D181DDCBAD","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-25BA1C551957EAD856D93BB1","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-0B236E96CFAADEA401D485D8","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-2EB24474879263CAA7D55388","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-7CBF6F506E34E48BF4007E49","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-4E5FAEE78D56DFC97676075D","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-EF8F9819481D98F6C8919AB9","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-51ED3C0701E326D181DDCBAD","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-25BA1C551957EAD856D93BB1","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW72" s="22" t="inlineStr">
@@ -29110,7 +29136,7 @@
       </c>
       <c r="AZ72" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-B1AE3151CA3DFABC9D6F87A2","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-DC5D9238399C6A5D0C16D1D5","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA72" s="22" t="inlineStr">
@@ -29122,12 +29148,12 @@
     <row r="73" ht="32" customHeight="1">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>CAND-F89285A886F733FCF48A39F5</t>
+          <t>CAND-DB36510075A8FBE14B50458C</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
@@ -29337,7 +29363,7 @@
       </c>
       <c r="AZ73" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-B1AE3151CA3DFABC9D6F87A2","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-DC5D9238399C6A5D0C16D1D5","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA73" s="22" t="inlineStr">
@@ -29349,12 +29375,12 @@
     <row r="74" ht="32" customHeight="1">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>CAND-924103D11A79912AF1188F2F</t>
+          <t>CAND-0630B601A39B1E7F3ABDB138</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
@@ -29576,12 +29602,12 @@
     <row r="75" ht="32" customHeight="1">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>CAND-30A07501B51A2AE278F7EA92</t>
+          <t>CAND-5784A0970E1A5BFDF92DD2BB</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
@@ -29803,12 +29829,12 @@
     <row r="76" ht="32" customHeight="1">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>PKG-7BBB53D3EBA7FF15A78C71B4</t>
+          <t>PKG-E9241458D19D86459E878919</t>
         </is>
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>CAND-AD58D34434A2170D1BF1A9B1</t>
+          <t>CAND-D2AA37F564A2D82B828401D3</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
@@ -30022,7 +30048,7 @@
       </c>
       <c r="AZ76" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-7AA042130907C622B3D829D7","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-D6AA6A4FA46862F6334FBC5C","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA76" s="22" t="inlineStr">
@@ -30034,12 +30060,12 @@
     <row r="77" ht="32" customHeight="1">
       <c r="A77" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>CAND-36E93BF7B8CE7895B3350359</t>
+          <t>CAND-FC7B2860CAAD03861AED5C53</t>
         </is>
       </c>
       <c r="C77" s="14" t="inlineStr">
@@ -30265,12 +30291,12 @@
     <row r="78" ht="32" customHeight="1">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>CAND-4D7163BFB57F1D099F93FBB4</t>
+          <t>CAND-61D8612587ADCC0F68698112</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
@@ -30444,7 +30470,7 @@
       </c>
       <c r="AR78" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS78" s="22" t="inlineStr">
@@ -30454,17 +30480,17 @@
       </c>
       <c r="AT78" s="22" t="inlineStr">
         <is>
-          <t>["EVID-DCDF95C6A1F733063FB0FF40","EVID-473DAE924D0494843A151322","EVID-2E961C8C26A8DD4D880DC0C3","EVID-9B5F3B007AF6B0C87B636B00","EVID-25C1DA18EEB5F16EA1C37494","EVID-39C9D8D68FDB2B48EC1F8E06","EVID-E0A9E6F5CF1C6CC89EF49539","EVID-4FF74009A0DFB40815A0A413","EVID-07174CC5836579556EAE3FBA","EVID-43A9D4AA27211AD241140DA8","EVID-5F049D088166930E912ED0CA","EVID-814B842EA1F2BD7336C2E67C"]</t>
+          <t>["EVID-DCDF95C6A1F733063FB0FF40","EVID-473DAE924D0494843A151322","EVID-2E961C8C26A8DD4D880DC0C3","EVID-9B5F3B007AF6B0C87B636B00","EVID-25C1DA18EEB5F16EA1C37494","EVID-AE5017E437240372E2E797B8","EVID-39C9D8D68FDB2B48EC1F8E06","EVID-E0A9E6F5CF1C6CC89EF49539","EVID-4FF74009A0DFB40815A0A413","EVID-07174CC5836579556EAE3FBA","EVID-43A9D4AA27211AD241140DA8","EVID-5F049D088166930E912ED0CA","EVID-814B842EA1F2BD7336C2E67C"]</t>
         </is>
       </c>
       <c r="AU78" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-07174CC5836579556EAE3FBA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-07174CC5836579556EAE3FBA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-25C1DA18EEB5F16EA1C37494":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-25C1DA18EEB5F16EA1C37494","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-2E961C8C26A8DD4D880DC0C3":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2E961C8C26A8DD4D880DC0C3","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-39C9D8D68FDB2B48EC1F8E06":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-39C9D8D68FDB2B48EC1F8E06","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":4200},"EVID-43A9D4AA27211AD241140DA8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-43A9D4AA27211AD241140DA8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0},"EVID-473DAE924D0494843A151322":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-473DAE924D0494843A151322","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-4FF74009A0DFB40815A0A413":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4FF74009A0DFB40815A0A413","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-5F049D088166930E912ED0CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5F049D088166930E912ED0CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-814B842EA1F2BD7336C2E67C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-814B842EA1F2BD7336C2E67C","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-9B5F3B007AF6B0C87B636B00":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-9B5F3B007AF6B0C87B636B00","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-DCDF95C6A1F733063FB0FF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DCDF95C6A1F733063FB0FF40","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-E0A9E6F5CF1C6CC89EF49539":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E0A9E6F5CF1C6CC89EF49539","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":16000}}</t>
+          <t>{"EVID-07174CC5836579556EAE3FBA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-07174CC5836579556EAE3FBA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-25C1DA18EEB5F16EA1C37494":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-25C1DA18EEB5F16EA1C37494","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-2E961C8C26A8DD4D880DC0C3":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2E961C8C26A8DD4D880DC0C3","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-39C9D8D68FDB2B48EC1F8E06":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-39C9D8D68FDB2B48EC1F8E06","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":4200},"EVID-43A9D4AA27211AD241140DA8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-43A9D4AA27211AD241140DA8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0},"EVID-473DAE924D0494843A151322":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-473DAE924D0494843A151322","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-4FF74009A0DFB40815A0A413":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4FF74009A0DFB40815A0A413","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-5F049D088166930E912ED0CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5F049D088166930E912ED0CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-814B842EA1F2BD7336C2E67C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-814B842EA1F2BD7336C2E67C","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-9B5F3B007AF6B0C87B636B00":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-9B5F3B007AF6B0C87B636B00","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-AE5017E437240372E2E797B8":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-AE5017E437240372E2E797B8","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-DCDF95C6A1F733063FB0FF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DCDF95C6A1F733063FB0FF40","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-E0A9E6F5CF1C6CC89EF49539":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E0A9E6F5CF1C6CC89EF49539","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":16000}}</t>
         </is>
       </c>
       <c r="AV78" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-473DAE924D0494843A151322","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-2E961C8C26A8DD4D880DC0C3","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-9B5F3B007AF6B0C87B636B00","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-25C1DA18EEB5F16EA1C37494","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-39C9D8D68FDB2B48EC1F8E06","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-E0A9E6F5CF1C6CC89EF49539","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-473DAE924D0494843A151322","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-2E961C8C26A8DD4D880DC0C3","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-9B5F3B007AF6B0C87B636B00","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-25C1DA18EEB5F16EA1C37494","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-AE5017E437240372E2E797B8","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-39C9D8D68FDB2B48EC1F8E06","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-E0A9E6F5CF1C6CC89EF49539","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW78" s="22" t="inlineStr">
@@ -30484,7 +30510,7 @@
       </c>
       <c r="AZ78" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-C7D4A73498A01E43CF2F1F99","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-999C878D6C51D4B139B49A57","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA78" s="22" t="inlineStr">
@@ -30496,12 +30522,12 @@
     <row r="79" ht="32" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>CAND-E4FE1A1917EE61ADF0A90DD5</t>
+          <t>CAND-07075A2AF6885F9116290675</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
@@ -30723,12 +30749,12 @@
     <row r="80" ht="32" customHeight="1">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>CAND-580A5D1DBAA9FF66F3497081</t>
+          <t>CAND-2FEA25EDC5E48395071F4EF6</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
@@ -30950,12 +30976,12 @@
     <row r="81" ht="32" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>CAND-A69115976DE8B2D6CED3E2F9</t>
+          <t>CAND-0B255F5C4039607F30C4EE4A</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
@@ -31165,7 +31191,7 @@
       </c>
       <c r="AZ81" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-C7D4A73498A01E43CF2F1F99","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-999C878D6C51D4B139B49A57","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA81" s="22" t="inlineStr">
@@ -31177,12 +31203,12 @@
     <row r="82" ht="32" customHeight="1">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>PKG-64D236F637ADCD1FA2350E7B</t>
+          <t>PKG-B63013D458FDCDAA74198601</t>
         </is>
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>CAND-0E7487FBA4179110E052404A</t>
+          <t>CAND-C8B97E03CD532E0571F1A2F5</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
@@ -31396,7 +31422,7 @@
       </c>
       <c r="AZ82" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-C2B8462C39C6CBF67EA76272","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-F5B38DFE81B5D7BBAF6911B1","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA82" s="22" t="inlineStr">
@@ -31408,12 +31434,12 @@
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>CAND-48E992E09B6FDDDA184620BB</t>
+          <t>CAND-C4A7C16CD04A96235E2A96F0</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
@@ -31639,12 +31665,12 @@
     <row r="84" ht="32" customHeight="1">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>CAND-7AD7357E0749467C6A7B878C</t>
+          <t>CAND-C5123BB77CACC1CED8BB907A</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
@@ -31836,7 +31862,7 @@
       </c>
       <c r="AR84" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS84" s="22" t="inlineStr">
@@ -31846,17 +31872,17 @@
       </c>
       <c r="AT84" s="22" t="inlineStr">
         <is>
-          <t>["EVID-7A436410CF1C8EE2567C00A8","EVID-DF7FBF457C19FB28EF5FD820","EVID-AF2A27B54B6E2E92040B22C3","EVID-277695726D78445956FE494F","EVID-A39D869989EE20E8F0FA4661","EVID-AA062B5DFCC4DBB6962C7CA9","EVID-9094DED8046D5939494E72F6","EVID-877CBDBF73660A76F7D7B906","EVID-8945206B7EFE7B399B2C2E7E","EVID-9D5FF441E9A83BA2016A7779","EVID-BB70599C732C9AF2C89E8F69","EVID-0645324E21523AC72540EBFB"]</t>
+          <t>["EVID-7A436410CF1C8EE2567C00A8","EVID-DF7FBF457C19FB28EF5FD820","EVID-AF2A27B54B6E2E92040B22C3","EVID-277695726D78445956FE494F","EVID-A39D869989EE20E8F0FA4661","EVID-2BE3AE8039A7B379DAA21484","EVID-AA062B5DFCC4DBB6962C7CA9","EVID-9094DED8046D5939494E72F6","EVID-877CBDBF73660A76F7D7B906","EVID-8945206B7EFE7B399B2C2E7E","EVID-9D5FF441E9A83BA2016A7779","EVID-BB70599C732C9AF2C89E8F69","EVID-0645324E21523AC72540EBFB"]</t>
         </is>
       </c>
       <c r="AU84" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0645324E21523AC72540EBFB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0645324E21523AC72540EBFB","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":122},"EVID-277695726D78445956FE494F":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-277695726D78445956FE494F","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-7A436410CF1C8EE2567C00A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A436410CF1C8EE2567C00A8","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-877CBDBF73660A76F7D7B906":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-877CBDBF73660A76F7D7B906","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-8945206B7EFE7B399B2C2E7E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8945206B7EFE7B399B2C2E7E","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":2816.0},"EVID-9094DED8046D5939494E72F6":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9094DED8046D5939494E72F6","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":4000},"EVID-9D5FF441E9A83BA2016A7779":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9D5FF441E9A83BA2016A7779","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":3200.0},"EVID-A39D869989EE20E8F0FA4661":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-A39D869989EE20E8F0FA4661","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-AA062B5DFCC4DBB6962C7CA9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-AA062B5DFCC4DBB6962C7CA9","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1600},"EVID-AF2A27B54B6E2E92040B22C3":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-AF2A27B54B6E2E92040B22C3","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-BB70599C732C9AF2C89E8F69":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BB70599C732C9AF2C89E8F69","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3733.77},"EVID-DF7FBF457C19FB28EF5FD820":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-DF7FBF457C19FB28EF5FD820","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0}}</t>
+          <t>{"EVID-0645324E21523AC72540EBFB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0645324E21523AC72540EBFB","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":122},"EVID-277695726D78445956FE494F":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-277695726D78445956FE494F","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-2BE3AE8039A7B379DAA21484":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-2BE3AE8039A7B379DAA21484","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-7A436410CF1C8EE2567C00A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A436410CF1C8EE2567C00A8","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-877CBDBF73660A76F7D7B906":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-877CBDBF73660A76F7D7B906","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-8945206B7EFE7B399B2C2E7E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8945206B7EFE7B399B2C2E7E","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":2816.0},"EVID-9094DED8046D5939494E72F6":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9094DED8046D5939494E72F6","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":4000},"EVID-9D5FF441E9A83BA2016A7779":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9D5FF441E9A83BA2016A7779","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":3200.0},"EVID-A39D869989EE20E8F0FA4661":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-A39D869989EE20E8F0FA4661","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-AA062B5DFCC4DBB6962C7CA9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-AA062B5DFCC4DBB6962C7CA9","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1600},"EVID-AF2A27B54B6E2E92040B22C3":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-AF2A27B54B6E2E92040B22C3","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-BB70599C732C9AF2C89E8F69":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BB70599C732C9AF2C89E8F69","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3733.77},"EVID-DF7FBF457C19FB28EF5FD820":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-DF7FBF457C19FB28EF5FD820","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0}}</t>
         </is>
       </c>
       <c r="AV84" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-DF7FBF457C19FB28EF5FD820","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-AF2A27B54B6E2E92040B22C3","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-277695726D78445956FE494F","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-A39D869989EE20E8F0FA4661","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-AA062B5DFCC4DBB6962C7CA9","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-9094DED8046D5939494E72F6","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-DF7FBF457C19FB28EF5FD820","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-AF2A27B54B6E2E92040B22C3","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-277695726D78445956FE494F","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-A39D869989EE20E8F0FA4661","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-2BE3AE8039A7B379DAA21484","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-AA062B5DFCC4DBB6962C7CA9","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-9094DED8046D5939494E72F6","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW84" s="22" t="inlineStr">
@@ -31888,12 +31914,12 @@
     <row r="85" ht="32" customHeight="1">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>CAND-4AD0C5CF56FFE443109E075C</t>
+          <t>CAND-BF43E30DCCBF2197D86C4A47</t>
         </is>
       </c>
       <c r="C85" s="14" t="inlineStr">
@@ -32115,12 +32141,12 @@
     <row r="86" ht="32" customHeight="1">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>CAND-49A88561475837189D75A95B</t>
+          <t>CAND-C51D33CA45FD919D45D2C3AC</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
@@ -32342,12 +32368,12 @@
     <row r="87" ht="32" customHeight="1">
       <c r="A87" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B87" s="14" t="inlineStr">
         <is>
-          <t>CAND-CBCF6ED4CDF8B9664828018A</t>
+          <t>CAND-5C6283E0FB5D37B9AF951A35</t>
         </is>
       </c>
       <c r="C87" s="14" t="inlineStr">
@@ -32593,12 +32619,12 @@
     <row r="88" ht="32" customHeight="1">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>PKG-B1B32F263A12954F8161595B</t>
+          <t>PKG-C8E9F9F3FE6FECF8B1F2C852</t>
         </is>
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>CAND-0CF01F172DB34D3AE5983193</t>
+          <t>CAND-C83A18C81BA3F8F01454DD46</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
@@ -32812,7 +32838,7 @@
       </c>
       <c r="AZ88" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-C76B1BF0BE04F2268A48C457","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-C2EBBB483BA454145E5C3C56","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA88" s="22" t="inlineStr">
@@ -32824,12 +32850,12 @@
     <row r="89" ht="32" customHeight="1">
       <c r="A89" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B89" s="14" t="inlineStr">
         <is>
-          <t>CAND-73A72B66CCC5DF6F66CAC2FE</t>
+          <t>CAND-ACCF6F438E9B7DD1C243642F</t>
         </is>
       </c>
       <c r="C89" s="14" t="inlineStr">
@@ -33055,12 +33081,12 @@
     <row r="90" ht="32" customHeight="1">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B90" s="14" t="inlineStr">
         <is>
-          <t>CAND-20A04702FCD63664C07653A5</t>
+          <t>CAND-2ABC4239192B22E3E0541016</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
@@ -33234,7 +33260,7 @@
       </c>
       <c r="AR90" s="15" t="inlineStr">
         <is>
-          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
+          <t>spill_query_pct_30 &gt;= upsize signal 2.0; spill_queries_30 &gt;= evidence minimum for upsize 20; p95_spill_bytes_when_spilled_30 &gt;= upsize signal 1073741824; queued_query_pct_30 &lt;= downsize-safe 0.5; failure_cancel_pct_30 &lt;= downsize-safe 5.0; p95_execution_ms_30 &lt;= downsize-safe 5000; p99_execution_ms_30 &lt;= downsize-safe 30000</t>
         </is>
       </c>
       <c r="AS90" s="22" t="inlineStr">
@@ -33244,17 +33270,17 @@
       </c>
       <c r="AT90" s="22" t="inlineStr">
         <is>
-          <t>["EVID-F45B3F25E72C93572E60D363","EVID-ABE50E8BB95F0A3555F82500","EVID-EBE7FEB8EDF8384AFCA4023F","EVID-6697A43FF1953B6DD17B7E3A","EVID-168734B9927A9EB76E8DD271","EVID-76CC7EFCB0C616F7636449A1","EVID-D83B486744833AA5B4728EAA","EVID-CE464D57463AF05E9E2B1B2E","EVID-A8BE846EED36B67068AA40E0","EVID-5744D477056B6D4DDA2B3C9A","EVID-05DD86E0F6613765BFBA1E18","EVID-4D2EA7CDCF00512B9AD8016B"]</t>
+          <t>["EVID-F45B3F25E72C93572E60D363","EVID-ABE50E8BB95F0A3555F82500","EVID-EBE7FEB8EDF8384AFCA4023F","EVID-6697A43FF1953B6DD17B7E3A","EVID-168734B9927A9EB76E8DD271","EVID-4BF5518163DAD5705703F01C","EVID-76CC7EFCB0C616F7636449A1","EVID-D83B486744833AA5B4728EAA","EVID-CE464D57463AF05E9E2B1B2E","EVID-A8BE846EED36B67068AA40E0","EVID-5744D477056B6D4DDA2B3C9A","EVID-05DD86E0F6613765BFBA1E18","EVID-4D2EA7CDCF00512B9AD8016B"]</t>
         </is>
       </c>
       <c r="AU90" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-05DD86E0F6613765BFBA1E18":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-05DD86E0F6613765BFBA1E18","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":8793.82},"EVID-168734B9927A9EB76E8DD271":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-168734B9927A9EB76E8DD271","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-4D2EA7CDCF00512B9AD8016B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4D2EA7CDCF00512B9AD8016B","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-5744D477056B6D4DDA2B3C9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5744D477056B6D4DDA2B3C9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":33000.0},"EVID-6697A43FF1953B6DD17B7E3A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-6697A43FF1953B6DD17B7E3A","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-76CC7EFCB0C616F7636449A1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-76CC7EFCB0C616F7636449A1","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2300},"EVID-A8BE846EED36B67068AA40E0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A8BE846EED36B67068AA40E0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":29040.0},"EVID-ABE50E8BB95F0A3555F82500":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-ABE50E8BB95F0A3555F82500","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-CE464D57463AF05E9E2B1B2E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CE464D57463AF05E9E2B1B2E","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-D83B486744833AA5B4728EAA":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D83B486744833AA5B4728EAA","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":8500},"EVID-EBE7FEB8EDF8384AFCA4023F":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-EBE7FEB8EDF8384AFCA4023F","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-F45B3F25E72C93572E60D363":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F45B3F25E72C93572E60D363","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"}}</t>
+          <t>{"EVID-05DD86E0F6613765BFBA1E18":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-05DD86E0F6613765BFBA1E18","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":8793.82},"EVID-168734B9927A9EB76E8DD271":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-168734B9927A9EB76E8DD271","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-4BF5518163DAD5705703F01C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4BF5518163DAD5705703F01C","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-4D2EA7CDCF00512B9AD8016B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4D2EA7CDCF00512B9AD8016B","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-5744D477056B6D4DDA2B3C9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5744D477056B6D4DDA2B3C9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":33000.0},"EVID-6697A43FF1953B6DD17B7E3A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-6697A43FF1953B6DD17B7E3A","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-76CC7EFCB0C616F7636449A1":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-76CC7EFCB0C616F7636449A1","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2300},"EVID-A8BE846EED36B67068AA40E0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A8BE846EED36B67068AA40E0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":29040.0},"EVID-ABE50E8BB95F0A3555F82500":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-ABE50E8BB95F0A3555F82500","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-CE464D57463AF05E9E2B1B2E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CE464D57463AF05E9E2B1B2E","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-D83B486744833AA5B4728EAA":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D83B486744833AA5B4728EAA","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":8500},"EVID-EBE7FEB8EDF8384AFCA4023F":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-EBE7FEB8EDF8384AFCA4023F","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-F45B3F25E72C93572E60D363":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F45B3F25E72C93572E60D363","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"}}</t>
         </is>
       </c>
       <c r="AV90" s="22" t="inlineStr">
         <is>
-          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-ABE50E8BB95F0A3555F82500","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-EBE7FEB8EDF8384AFCA4023F","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-6697A43FF1953B6DD17B7E3A","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-168734B9927A9EB76E8DD271","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-76CC7EFCB0C616F7636449A1","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-D83B486744833AA5B4728EAA","metric":"p99_execution_ms_30","threshold":30000}]</t>
+          <t>[{"comparator":"&gt;= upsize signal","evidence_id":"EVID-ABE50E8BB95F0A3555F82500","metric":"spill_query_pct_30","threshold":2.0},{"comparator":"&gt;= evidence minimum for upsize","evidence_id":"EVID-EBE7FEB8EDF8384AFCA4023F","metric":"spill_queries_30","threshold":20},{"comparator":"&gt;= upsize signal","evidence_id":"EVID-6697A43FF1953B6DD17B7E3A","metric":"p95_spill_bytes_when_spilled_30","threshold":1073741824},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-168734B9927A9EB76E8DD271","metric":"queued_query_pct_30","threshold":0.5},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-4BF5518163DAD5705703F01C","metric":"failure_cancel_pct_30","threshold":5.0},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-76CC7EFCB0C616F7636449A1","metric":"p95_execution_ms_30","threshold":5000},{"comparator":"&lt;= downsize-safe","evidence_id":"EVID-D83B486744833AA5B4728EAA","metric":"p99_execution_ms_30","threshold":30000}]</t>
         </is>
       </c>
       <c r="AW90" s="22" t="inlineStr">
@@ -33274,7 +33300,7 @@
       </c>
       <c r="AZ90" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-CD13BC97911EDD734CF17B6B","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-5F795672B44D350C3E296BF1","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA90" s="22" t="inlineStr">
@@ -33286,12 +33312,12 @@
     <row r="91" ht="32" customHeight="1">
       <c r="A91" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B91" s="14" t="inlineStr">
         <is>
-          <t>CAND-9ADFC70F5FC112A2499B5375</t>
+          <t>CAND-ACA9A2EEB098AFFFB5C5CDD7</t>
         </is>
       </c>
       <c r="C91" s="14" t="inlineStr">
@@ -33501,7 +33527,7 @@
       </c>
       <c r="AZ91" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-CD13BC97911EDD734CF17B6B","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-5F795672B44D350C3E296BF1","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA91" s="22" t="inlineStr">
@@ -33513,12 +33539,12 @@
     <row r="92" ht="32" customHeight="1">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B92" s="14" t="inlineStr">
         <is>
-          <t>CAND-F52F904EE62AFA4706B94D7E</t>
+          <t>CAND-F7FAB3EBC34F7F42BB4CB9AB</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
@@ -33740,12 +33766,12 @@
     <row r="93" ht="32" customHeight="1">
       <c r="A93" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B93" s="14" t="inlineStr">
         <is>
-          <t>CAND-C08CF1BBC9ECD83993F5BCE2</t>
+          <t>CAND-5BD0417FF74CCA4CE750987C</t>
         </is>
       </c>
       <c r="C93" s="14" t="inlineStr">
@@ -33955,7 +33981,7 @@
       </c>
       <c r="AZ93" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-CD13BC97911EDD734CF17B6B","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-5F795672B44D350C3E296BF1","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA93" s="22" t="inlineStr">
@@ -33967,12 +33993,12 @@
     <row r="94" ht="32" customHeight="1">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>PKG-8A3D702F2E106E66AE0DA92A</t>
+          <t>PKG-78B04335C6149C99A956F907</t>
         </is>
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>CAND-A33DFC4B60027DE5B92ED694</t>
+          <t>CAND-254186ED0FFA404D809AF606</t>
         </is>
       </c>
       <c r="C94" s="14" t="inlineStr">
@@ -34186,7 +34212,7 @@
       </c>
       <c r="AZ94" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-D90F0090AC8A9492249F19B8","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-871471461B50CF97B71AE728","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA94" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Review fixes: SQL-scoped 30-day watermark, replayed short-history CV, demo CV; add group B proposals
- Watermark query looks back 30 days and is limited to the SQL product so a
  stalled feed is not mistaken for no watermark.
- Evidence replay treats CV <= short history as unknown (pre-fix evidence stored 0.0).
- Demo generator no longer reports a CV for a 3-day warehouse.
- Cost-history floor comment corrected; midnight/timezone caveat documented.
- docs/proposals/audit-m-group-b.md: unexecuted designs for M1, M2, M3b, M4, M9.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo_output/workbook.xlsx
+++ b/examples/demo_output/workbook.xlsx
@@ -21795,7 +21795,7 @@
         </is>
       </c>
       <c r="O41" s="21" t="n">
-        <v>0.58</v>
+        <v>0.443</v>
       </c>
       <c r="P41" s="18" t="inlineStr">
         <is>
@@ -21910,7 +21910,7 @@
       </c>
       <c r="AS41" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":null}</t>
         </is>
       </c>
       <c r="AT41" s="22" t="inlineStr">
@@ -22026,7 +22026,7 @@
         </is>
       </c>
       <c r="O42" s="21" t="n">
-        <v>0.58</v>
+        <v>0.443</v>
       </c>
       <c r="P42" s="18" t="inlineStr">
         <is>
@@ -22159,7 +22159,7 @@
       </c>
       <c r="AS42" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":null}</t>
         </is>
       </c>
       <c r="AT42" s="22" t="inlineStr">
@@ -22271,7 +22271,7 @@
         </is>
       </c>
       <c r="O43" s="21" t="n">
-        <v>0.58</v>
+        <v>0.443</v>
       </c>
       <c r="P43" s="18" t="inlineStr">
         <is>
@@ -22386,7 +22386,7 @@
       </c>
       <c r="AS43" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":null}</t>
         </is>
       </c>
       <c r="AT43" s="22" t="inlineStr">
@@ -22498,7 +22498,7 @@
         </is>
       </c>
       <c r="O44" s="21" t="n">
-        <v>0.58</v>
+        <v>0.443</v>
       </c>
       <c r="P44" s="18" t="inlineStr">
         <is>
@@ -22613,7 +22613,7 @@
       </c>
       <c r="AS44" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":null}</t>
         </is>
       </c>
       <c r="AT44" s="22" t="inlineStr">
@@ -22725,7 +22725,7 @@
         </is>
       </c>
       <c r="O45" s="21" t="n">
-        <v>0.58</v>
+        <v>0.443</v>
       </c>
       <c r="P45" s="18" t="inlineStr">
         <is>
@@ -22864,7 +22864,7 @@
       </c>
       <c r="AS45" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":null}</t>
         </is>
       </c>
       <c r="AT45" s="22" t="inlineStr">
@@ -22980,7 +22980,7 @@
         </is>
       </c>
       <c r="O46" s="21" t="n">
-        <v>0.58</v>
+        <v>0.443</v>
       </c>
       <c r="P46" s="18" t="inlineStr">
         <is>
@@ -23119,7 +23119,7 @@
       </c>
       <c r="AS46" s="22" t="inlineStr">
         <is>
-          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":0.91}</t>
+          <t>{"coverage":0.033,"epoch_maturity":0.1,"sample":1.0,"signal":0.7,"stability":null}</t>
         </is>
       </c>
       <c r="AT46" s="22" t="inlineStr">

</xml_diff>

<commit_message>
G2: keep usage with no list price as unpriced DBU; unknown cost stays null
EPOCH_DAILY_COST_SQL left-joins list_prices (one price per usage record,
latest price_start_time) and reports unpriced_dbu_quantity. Unpriced DBU in
the trailing window makes the actual DBU cost null; inside the current-epoch
forecast basis it makes the forward DBU cost null. Estimates are withheld
(DBU_COST_UNAVAILABLE), migration is INSUFFICIENT_EVIDENCE, epoch cost for
calibration is null, and nulls survive evidence replay. Adds the golden
scenario harness and fixture C32. Publisher 2.10.0; modeler, optimizer,
estimator and bundle versions bumped; demo regenerated (values unchanged).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo_output/workbook.xlsx
+++ b/examples/demo_output/workbook.xlsx
@@ -2799,7 +2799,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="AH5" s="14" t="inlineStr">
         <is>
-          <t>SCN-863D86733C17ECB8516EF093</t>
+          <t>SCN-0F323C820C480A6DB359983B</t>
         </is>
       </c>
       <c r="AI5" s="15" t="inlineStr">
@@ -3030,12 +3030,12 @@
       </c>
       <c r="BF5" s="22" t="inlineStr">
         <is>
-          <t>["SCN-863D86733C17ECB8516EF093","SCN-145D50BED02E3BA2BE197B7F"]</t>
+          <t>["SCN-0F323C820C480A6DB359983B","SCN-05AEB24D88A789A8A5B3097C"]</t>
         </is>
       </c>
       <c r="BG5" s="22" t="inlineStr">
         <is>
-          <t>["CAND-7766A2738B430E52A7885D34","CAND-EE57C678D7321484C82E7EC4","CAND-7C972C46E6BADA6422EF650F","CAND-759D0E09D0D3D1DF01FBBA2B","CAND-AF9E15C01CEAC8C1A0D722AB","CAND-E9A7141D8480ED7AC73076CC"]</t>
+          <t>["CAND-30CABA362591DD08BBD7EEFF","CAND-19BB082E74D6C1E39FFF482D","CAND-FACB02F992DE84FD0C6488B6","CAND-F52C33A9DDA0277D8F79D9E6","CAND-8FB89535DFCD63C9A63BF39E","CAND-B5D201CF9262CAC1AA7E3182"]</t>
         </is>
       </c>
       <c r="BH5" s="22" t="inlineStr">
@@ -3045,14 +3045,14 @@
       </c>
       <c r="BI5" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-02C377DDCAB735229EEC24A6":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-0465D6B752AD0AB46330483B":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2667},"EVID-05ABEF123F82DD14B9089E15":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-0769A5E646320DA500332309":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-1738AF6A4068640602ECD84E":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-1ACF5B01162FE1C9B407F0AA":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-23834E1D614A63BF7B745F8B":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":10000},"EVID-249028FA99BFDEE68A2645DB":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-25CAE9179FEBB6FA2D425213":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-267BE325DB935326F0ECD0CA":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":480},"EVID-2B38163DC5B241CCC5D6E4DE":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2C2557D4DA122C44D293B116":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-35D70FC33D4A591A8B2F1AB3":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-36D1387C3DAB197C2F09456E":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-3F20250831BDAE21F08D1FA3":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-3FA53CA4EC8C609E6C60F9CF":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-43A874D251CBC13D278C1E5F":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2500},"EVID-492656489A02189691212637":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-581184092AAF568D86DE312B":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-592F211E9EDB3223E49035DF":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9000},"EVID-5CE57275336FF7A99147DCC0":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-619414E4B31300D140BA8FB0":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":80.0},"EVID-819197156A69EF5E136BCD0D":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-82E7AD7A0BFE9AC6A7E9E8E3":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-849F13DCD8F8A626942FED31":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-8B432207CE81E1B5453FBA36":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-8CFC377DC61A584AFF2B89D5":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-9165453291690C68D73C499A":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3000},"EVID-95D4200101460975CFB0113A":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-9A7BE346494C09B0348F5402":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-A10762D366E7024D1873F50A":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-A260A94FAD60AB2B5B984E15":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":400.0},"EVID-A30D883A534722C9BCA5AEE0":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-A94431E86D58DBE8F3A0F596":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-AD5C166A82B775E709ABF751":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-BC460C11441EEA3635B6CEF6":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":27000.0},"EVID-C0024AE90132BFF522B946EA":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-C3D2E64A89DE473CEF3F10A8":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-C8BD459AEE7D00E30C81E085":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":11725.1},"EVID-CE1E8D70F4C1F4F7211BEBB2":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-D0948F3BBDA2C1A885CCD2E8":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":8},"EVID-D1D3CCC01ECDAD227F11E100":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-D31130A3622EA96577F699ED":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-E172A6102448FF828423C618":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-E2BFCCA76EB8534DA44771CC":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":23760.0},"EVID-E6FDF0DED766BE36DBCF9B85":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-EE439C26D0E760A7878BFAEA":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-F0838A46641CA4DF579874C2":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-F2975CBD0F7435B6DE4E6A1E":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-FBADEF6B92F4CD5C57558A64":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":960},"EVID-FCFFAB99D6FF292E4BC8DC8F":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-FE30CB96733BF18D9469D45B":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0}}</t>
+          <t>{"EVID-02C377DDCAB735229EEC24A6":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-0465D6B752AD0AB46330483B":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2667},"EVID-05ABEF123F82DD14B9089E15":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-0769A5E646320DA500332309":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-1738AF6A4068640602ECD84E":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-1ACF5B01162FE1C9B407F0AA":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-23834E1D614A63BF7B745F8B":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":10000},"EVID-249028FA99BFDEE68A2645DB":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-25CAE9179FEBB6FA2D425213":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-267BE325DB935326F0ECD0CA":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":480},"EVID-2B38163DC5B241CCC5D6E4DE":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2C2557D4DA122C44D293B116":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-35D70FC33D4A591A8B2F1AB3":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-36D1387C3DAB197C2F09456E":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-3F20250831BDAE21F08D1FA3":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-3FA53CA4EC8C609E6C60F9CF":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-43A874D251CBC13D278C1E5F":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2500},"EVID-492656489A02189691212637":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-581184092AAF568D86DE312B":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-592F211E9EDB3223E49035DF":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9000},"EVID-5CE57275336FF7A99147DCC0":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-609ECEA12D01A7D7EE1FB3B0":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":27000.0},"EVID-619414E4B31300D140BA8FB0":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":80.0},"EVID-819197156A69EF5E136BCD0D":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-82E7AD7A0BFE9AC6A7E9E8E3":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-849F13DCD8F8A626942FED31":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-8B432207CE81E1B5453FBA36":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-8CFC377DC61A584AFF2B89D5":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-9165453291690C68D73C499A":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3000},"EVID-95D4200101460975CFB0113A":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-9A7BE346494C09B0348F5402":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-A10762D366E7024D1873F50A":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-A260A94FAD60AB2B5B984E15":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":400.0},"EVID-A30D883A534722C9BCA5AEE0":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-A94431E86D58DBE8F3A0F596":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-AD5C166A82B775E709ABF751":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-C0024AE90132BFF522B946EA":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-C3D2E64A89DE473CEF3F10A8":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-C8BD459AEE7D00E30C81E085":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":11725.1},"EVID-CE1E8D70F4C1F4F7211BEBB2":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-D0948F3BBDA2C1A885CCD2E8":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":8},"EVID-D1D3CCC01ECDAD227F11E100":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-D31130A3622EA96577F699ED":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-E172A6102448FF828423C618":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-E2BFCCA76EB8534DA44771CC":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":23760.0},"EVID-E6FDF0DED766BE36DBCF9B85":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-EE439C26D0E760A7878BFAEA":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-F0838A46641CA4DF579874C2":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-F2975CBD0F7435B6DE4E6A1E":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-FBADEF6B92F4CD5C57558A64":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":960},"EVID-FCFFAB99D6FF292E4BC8DC8F":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-FE30CB96733BF18D9469D45B":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0}}</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="AH6" s="14" t="inlineStr">
         <is>
-          <t>SCN-B31B08FCFCF16CF8C3ED3133</t>
+          <t>SCN-EB2C0C39F179860453FE1B76</t>
         </is>
       </c>
       <c r="AI6" s="15" t="inlineStr">
@@ -3283,12 +3283,12 @@
       </c>
       <c r="BF6" s="22" t="inlineStr">
         <is>
-          <t>["SCN-B31B08FCFCF16CF8C3ED3133","SCN-49F9E59C5DC51E8EA18565EB"]</t>
+          <t>["SCN-EB2C0C39F179860453FE1B76","SCN-BA79A1BAC0F873D6CDE9EC20"]</t>
         </is>
       </c>
       <c r="BG6" s="22" t="inlineStr">
         <is>
-          <t>["CAND-828F9A162C1D262C1F78972E","CAND-725D8CE810F7854F0B4F0599","CAND-0A41949888B511BF5079790D","CAND-E76392F60728B051B8FFF1A6","CAND-CC561F3665974267980305C7","CAND-FBE101BD35EAD540544961F6"]</t>
+          <t>["CAND-16E28D4A7F0B58A50DBE0DFE","CAND-429785936CDB1BB844384CE3","CAND-0EB9378528832881336CC3CB","CAND-147B23ADCB8854F570950756","CAND-9036A0CCF32202C187B847C1","CAND-50DDBBB8A017E60563909CE4"]</t>
         </is>
       </c>
       <c r="BH6" s="22" t="inlineStr">
@@ -3298,14 +3298,14 @@
       </c>
       <c r="BI6" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-108CC2BBEE3480D859C1460C":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-191D2612CC2320CF4E6B71A8":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-1C1403E5FDC40ADF27F58E2E":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-1E3C87A385079E3183BA0AA9":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":14000},"EVID-1F9B7F008085483A33F93C00":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-238FF507E88B1AC45C97415F":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":260},"EVID-317694A250D14B0CB5738BDB":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"X_LARGE"},"EVID-3466FCD5ACCCF0CB40F076F6":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-37BBA0C0F054D3E379D30D26":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-397653A8F7424B807EC69A77":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-3F6A911A1B67177259CD0328":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-44A316ECBA6BF84EB02F0D48":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":48000},"EVID-4AC0A6B6BF0BFFF9604E16E8":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-4B0A26E4BCE89FB67759E226":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-4B6CAD51D6E6CC690F238328":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-4C9BD346490AA494BABDC248":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-563CF3DD0B11F9EE318B64CA":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":216.67},"EVID-5679CAD31A1AC2F9C5E2AC0B":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-5A8EA64D13B38C8F14D75DFA":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":12.0},"EVID-5CA339D2D13816847797EB99":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":4875},"EVID-5FAA6569BBF4163B44E3BB5F":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":264},"EVID-64C33490C6C8E7457B3DECE3":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-6BA862424AEB0E713F6C4C3E":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-6D57B4495F16EF2F1F11A058":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":520},"EVID-6F5C81C659714CBD71F96903":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-7362CB175D2D3EE7F7FD836B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-7700F4C8B0DDF3241F3EF7E2":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.8},"EVID-798CAF1B6E59A5A6800BFDA6":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":56320.0},"EVID-7F3FBCF285A330187414CCE9":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-8089B2A88341C92E810E6D25":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":25.0},"EVID-856AE353D873B76613562142":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":74769.7},"EVID-88260E5CAA85A2862B0AF592":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":3221225472},"EVID-93786EC662829319601327D0":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":422},"EVID-9B47E8DD6C50F547AD614266":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-AD892CA77594BB00A48A1B37":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-B2195A64E32504F7CA0F938B":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-BAA92FC68151FBCB7BAC6577":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-BB853687EABCE34F9D34DE1A":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.8},"EVID-BCF105F24D33111D31C3E82A":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":6.5},"EVID-CCA7709442092923BEC9EDFD":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.8},"EVID-D0A63A8CF2088FDE42703300":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-D353A0904BB6A241CD4A8FCF":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-D36E9B4C473DB25466DABDB8":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-DD4AB7148F9EA2F96522D001":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":64000.0},"EVID-E4B7509030D6AA1C7EE0DC48":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E991D606CA5CF64A0BF34205":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-EF19965DFBC5EC58CB587207":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":12.0},"EVID-F038199F302C038B0F28F6E0":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-F099780A8C11FAFA04AFEAA2":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-F16D4AB2E6B3FE48E318CC61":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-F2F3E51797850FB6D31B3CE9":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-FADEC648D4D98214CD4E0817":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":52}}</t>
+          <t>{"EVID-108CC2BBEE3480D859C1460C":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-191D2612CC2320CF4E6B71A8":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-1C1403E5FDC40ADF27F58E2E":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-1E3C87A385079E3183BA0AA9":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":14000},"EVID-1F9B7F008085483A33F93C00":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-238FF507E88B1AC45C97415F":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":260},"EVID-317694A250D14B0CB5738BDB":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"X_LARGE"},"EVID-3466FCD5ACCCF0CB40F076F6":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-37BBA0C0F054D3E379D30D26":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-397653A8F7424B807EC69A77":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-3F6A911A1B67177259CD0328":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-44A316ECBA6BF84EB02F0D48":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":48000},"EVID-48AB665BCC0F78BDF2A9678D":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":64000.0},"EVID-4AC0A6B6BF0BFFF9604E16E8":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-4B0A26E4BCE89FB67759E226":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-4B6CAD51D6E6CC690F238328":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-4C9BD346490AA494BABDC248":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-563CF3DD0B11F9EE318B64CA":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":216.67},"EVID-5679CAD31A1AC2F9C5E2AC0B":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-5A8EA64D13B38C8F14D75DFA":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":12.0},"EVID-5CA339D2D13816847797EB99":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":4875},"EVID-5FAA6569BBF4163B44E3BB5F":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":264},"EVID-64C33490C6C8E7457B3DECE3":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":5000},"EVID-6BA862424AEB0E713F6C4C3E":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-6D57B4495F16EF2F1F11A058":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":520},"EVID-6F5C81C659714CBD71F96903":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-7362CB175D2D3EE7F7FD836B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-7700F4C8B0DDF3241F3EF7E2":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.8},"EVID-798CAF1B6E59A5A6800BFDA6":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":56320.0},"EVID-7F3FBCF285A330187414CCE9":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-8089B2A88341C92E810E6D25":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":25.0},"EVID-856AE353D873B76613562142":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":74769.7},"EVID-88260E5CAA85A2862B0AF592":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":3221225472},"EVID-93786EC662829319601327D0":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":422},"EVID-9B47E8DD6C50F547AD614266":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-AD892CA77594BB00A48A1B37":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-B2195A64E32504F7CA0F938B":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-BAA92FC68151FBCB7BAC6577":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-BB853687EABCE34F9D34DE1A":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.8},"EVID-BCF105F24D33111D31C3E82A":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":6.5},"EVID-CCA7709442092923BEC9EDFD":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.8},"EVID-D0A63A8CF2088FDE42703300":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-D353A0904BB6A241CD4A8FCF":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-D36E9B4C473DB25466DABDB8":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-E4B7509030D6AA1C7EE0DC48":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E991D606CA5CF64A0BF34205":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-EF19965DFBC5EC58CB587207":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":12.0},"EVID-F038199F302C038B0F28F6E0":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-F099780A8C11FAFA04AFEAA2":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-F16D4AB2E6B3FE48E318CC61":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-F2F3E51797850FB6D31B3CE9":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-FADEC648D4D98214CD4E0817":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":52}}</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="AH7" s="14" t="inlineStr">
         <is>
-          <t>SCN-9D2CE3A1C8DF6267C795DB02</t>
+          <t>SCN-26E77B55DE75D30BC7D94E62</t>
         </is>
       </c>
       <c r="AI7" s="15" t="inlineStr">
@@ -3536,12 +3536,12 @@
       </c>
       <c r="BF7" s="22" t="inlineStr">
         <is>
-          <t>["SCN-9D2CE3A1C8DF6267C795DB02","SCN-3E24BF4E2EB1FFD6BD97C5EF"]</t>
+          <t>["SCN-26E77B55DE75D30BC7D94E62","SCN-DF356B65FC7D9469319D516C"]</t>
         </is>
       </c>
       <c r="BG7" s="22" t="inlineStr">
         <is>
-          <t>["CAND-19114E8F568FBD08CD0E7342","CAND-EB8642E918D1FD97EE3FA4E2","CAND-40DECBD0C64F73A246651419","CAND-47C39CB54A496B16C7C5535D","CAND-7B32E8C35D19CC2C522779EC","CAND-1E5BC9641C5288D175C688E2"]</t>
+          <t>["CAND-470FD4CCBBE164E952753E39","CAND-983E960CC6715CCFDAFC3353","CAND-925E95E6BA6DA0ED59A9A733","CAND-C01B3B61787F253552AB5722","CAND-014DD489DCA84594FA96ACC7","CAND-C8B00F2B86A8B7AF7549A783"]</t>
         </is>
       </c>
       <c r="BH7" s="22" t="inlineStr">
@@ -3551,14 +3551,14 @@
       </c>
       <c r="BI7" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0469DF8349DF92AE11B1D733":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":6},"EVID-06FC310FC9843E52C293EC95":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-0D4AD27CEF1BC4E014A366E0":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-0E04A6B3AFE0680824E42A87":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":60000.0},"EVID-138DC2A3D2FA80EC64571C3B":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":42240.0},"EVID-18DEA81AF9B9B09E66190314":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-1A7EE4BB1C6CB7A9A2364274":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1200},"EVID-1E15FCB045036DE3E4936272":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":600},"EVID-1F30B9F5C01C5C2958401FB4":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3750},"EVID-26B4226E972D76B87D6EFDC7":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-28F961BADB1773C5BBE0E0FC":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":88.0},"EVID-2B6F729499188E4516712DEF":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-2BE6464F016F9F52AD9CB0A6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-2F5A12215CC813683545D25C":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-3DF032BEFA85DB8FC552AEB3":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-3E1EFFF63FE150372B9DD4CB":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-4B2FA824AF34D1756613D802":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-511D1D18D1235C9B3444A79E":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6500},"EVID-528AF7AEAFDF42798FFAF40D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-5C11623129047EDA95ACBCAE":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-5F47555F958537E30D6B43EB":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-634883B72B148A9943D89C0E":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-64A7680E004B2C425704B7E9":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1900},"EVID-66A17A5BB4510C9DBCA2C477":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-70DB2AE41192F0BE08EDA0E4":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":48000.0},"EVID-7A3A3F9E60677F3A4138A318":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-7D237D1142C76BF20FE66F78":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-83E6ACE6F898190CF078E276":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-843F72CCFB337DC9D837A0C8":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":21285.98},"EVID-90FD7EC9CBD2C8836D6B0FFF":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":3},"EVID-962883EA791AE7B18476787C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-9B76D9DF13646CF492DF7A42":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-9C062F46FF3DD1C51BE0F5CF":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":3},"EVID-9F97153165BA0D87B5E65DAB":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":11250},"EVID-AB8C9AA0F1F72AAFD024A28C":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-ADBD9F5EF2B25F6F2301AC5D":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-AECADC84F1D8CBD06E73BED8":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":500.0},"EVID-AFA35C81985D592CA48145FD":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-BF740AE5AD36DB91FC871C3E":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-C14B4CFFD829954127F98C95":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-C54D688D7F24665423F4E1C8":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-C6C9F93AA2CBE86496C750A8":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-CA4D7EC185EB84B896178975":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-CB02952CE3269D257AC973ED":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-D42D7396E4078F59ED71E357":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":5500.0},"EVID-D98ED418DDC55A2585D8D062":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":214},"EVID-DCED59AF916F6BE35E271AE4":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-DF6A451DEEB6FF200327D202":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-DFFE4AC535CD891824D51F47":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-E5644C6E4E95CA9DFC6EA17E":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-F1CA50ECF9487421AC834976":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-FCA7D73825895E13A667605E":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0}}</t>
+          <t>{"EVID-0469DF8349DF92AE11B1D733":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":6},"EVID-06FC310FC9843E52C293EC95":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-0D4AD27CEF1BC4E014A366E0":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-0E04A6B3AFE0680824E42A87":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":60000.0},"EVID-138DC2A3D2FA80EC64571C3B":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":42240.0},"EVID-18DEA81AF9B9B09E66190314":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-1A7EE4BB1C6CB7A9A2364274":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1200},"EVID-1E15FCB045036DE3E4936272":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":600},"EVID-1F30B9F5C01C5C2958401FB4":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3750},"EVID-26B4226E972D76B87D6EFDC7":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-28F961BADB1773C5BBE0E0FC":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":88.0},"EVID-2B6F729499188E4516712DEF":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-2BE6464F016F9F52AD9CB0A6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-2F5A12215CC813683545D25C":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-3DF032BEFA85DB8FC552AEB3":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-3E1EFFF63FE150372B9DD4CB":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-4AE16179F3F066BEB4F4D971":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":48000.0},"EVID-4B2FA824AF34D1756613D802":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-511D1D18D1235C9B3444A79E":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6500},"EVID-528AF7AEAFDF42798FFAF40D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-5C11623129047EDA95ACBCAE":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-5F47555F958537E30D6B43EB":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-634883B72B148A9943D89C0E":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-64A7680E004B2C425704B7E9":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1900},"EVID-66A17A5BB4510C9DBCA2C477":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-7A3A3F9E60677F3A4138A318":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-7D237D1142C76BF20FE66F78":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-83E6ACE6F898190CF078E276":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-843F72CCFB337DC9D837A0C8":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":21285.98},"EVID-90FD7EC9CBD2C8836D6B0FFF":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":3},"EVID-962883EA791AE7B18476787C":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-9B76D9DF13646CF492DF7A42":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-9C062F46FF3DD1C51BE0F5CF":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":3},"EVID-9F97153165BA0D87B5E65DAB":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":11250},"EVID-AB8C9AA0F1F72AAFD024A28C":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-ADBD9F5EF2B25F6F2301AC5D":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-AECADC84F1D8CBD06E73BED8":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":500.0},"EVID-AFA35C81985D592CA48145FD":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-BF740AE5AD36DB91FC871C3E":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-C14B4CFFD829954127F98C95":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-C54D688D7F24665423F4E1C8":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-C6C9F93AA2CBE86496C750A8":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-CA4D7EC185EB84B896178975":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-CB02952CE3269D257AC973ED":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-D42D7396E4078F59ED71E357":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":5500.0},"EVID-D98ED418DDC55A2585D8D062":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":214},"EVID-DCED59AF916F6BE35E271AE4":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-DF6A451DEEB6FF200327D202":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-DFFE4AC535CD891824D51F47":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-E5644C6E4E95CA9DFC6EA17E":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-F1CA50ECF9487421AC834976":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-FCA7D73825895E13A667605E":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0}}</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="AH8" s="14" t="inlineStr">
         <is>
-          <t>SCN-68E82895D5D2754159603420</t>
+          <t>SCN-268144CE4DBE7F2E116E140E</t>
         </is>
       </c>
       <c r="AI8" s="15" t="inlineStr">
@@ -3789,12 +3789,12 @@
       </c>
       <c r="BF8" s="22" t="inlineStr">
         <is>
-          <t>["SCN-68E82895D5D2754159603420","SCN-EC35EE7A8A459E1030386BDF"]</t>
+          <t>["SCN-268144CE4DBE7F2E116E140E","SCN-7541A4581D52616B7887204B"]</t>
         </is>
       </c>
       <c r="BG8" s="22" t="inlineStr">
         <is>
-          <t>["CAND-77B660B87F881D16821F65A4","CAND-B2761F18473F72B19D49C194","CAND-2132EFA0CCC25A00B16EA2CF","CAND-8677BE4DC1B511B57B6B894C","CAND-E193BAA623F56B14C771BC33","CAND-A64CA3E68A669D150AAA07D6"]</t>
+          <t>["CAND-A8E0C6C2514B7B2907081D31","CAND-6746672461AA4563E3A5F445","CAND-6B2DDE23EC751D22DE4F7914","CAND-73961AD4AD35D7CCF0FE42DD","CAND-FE18BD942E427F6BFF3FD25D","CAND-05E76611FED4F59744C22AB8"]</t>
         </is>
       </c>
       <c r="BH8" s="22" t="inlineStr">
@@ -3804,14 +3804,14 @@
       </c>
       <c r="BI8" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-081574EC86CCBD9D2F1F4CA7":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0AD97717D45EF6A9B235338F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-0CDFBA17157E22093D86EADE":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-11B2E705A613CE480286F6F3":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-1A9FB4971218B885A774B43B":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-28D2862523167B2FE81853B6":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1440},"EVID-33BB28CF6EC356A46BE6650D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-358F61DFBB7111D4CFD58A1A":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-35B29B2F02D863EAADFD08F3":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-387B8FBC6D85BF1D0A585F82":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-3E3D4D117F217EA7DB1596CE":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-46D6FDAC99EA6600704976B5":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-4B254C8301F2AC01CC84CE76":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":30.0},"EVID-4CD8C8C1F0430C6A0156057C":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3600},"EVID-4D3A60329DCF7E143BD06023":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-5427DFBFB88B9EBFC0C27786":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-5559E287993BB07DE138FDF6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-57741F660C40486486D51EFB":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-57F17FFFCFEDA0A9A60A1FD8":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":13500},"EVID-679B0BB84F874895FE357CF9":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":36000.0},"EVID-6C649CEB38C11AD9F545A814":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-753982E08475C2D3F33CAC84":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-7C07E0575343482778154975":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":45.0},"EVID-8CF90399EB348CA2E57A41FC":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-8F4C40C92A48DE9D5B743C29":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-91E83CACE07F654C8375E91B":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":31680.0},"EVID-943CC5DA406961E6EB3068F0":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-947C133A7AF95BA119BCA9FF":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-A3FFF81B3A1797CA534E3F69":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-A4F5DF730DDC736B98D2A1D2":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-A64BE1A219A5E17C9CF9589A":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-A6BDE580C0266C39CA6313B6":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-B5A32995ECFF3B005A70D952":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-B829726708E678EF6D0D4FFD":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-BC390FACE6BB107FDA76E438":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5380.16},"EVID-C5B21CB96D957B10D42BA42D":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1200.0},"EVID-C78D83012F1308C65615F356":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-C9561CB7C3F62405C4518E23":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":254},"EVID-CEB50ADB444DABFFABD2448A":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":12.0},"EVID-CEF597117FDE03FC75D46082":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":2160},"EVID-D5234CFF6B2C514C67CA7887":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-D8ED1DBE0C9CA9FD5031A804":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-DC3612A9EEBCACBD7708CC0E":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":15000},"EVID-DCD165B1F77962F8297C7F4D":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":12.0},"EVID-E09FD1F994ABB868559DF515":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":600.0},"EVID-E1011CEF886F3D479CF5E863":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":45.0},"EVID-E14BE0884B6E34FCB998C395":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-E56F010E6353E5FD20061D06":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":720},"EVID-E9801B0191E0C020D4E6D167":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":4500},"EVID-EA77D49C07D5FE5F9FA22988":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-ED798F026DC7D4813C8D1BD7":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":12.0},"EVID-F76F8313D068DA94D8D128E3":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0}}</t>
+          <t>{"EVID-081574EC86CCBD9D2F1F4CA7":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0AD97717D45EF6A9B235338F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-0CDFBA17157E22093D86EADE":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-11B2E705A613CE480286F6F3":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-120A7F0AFA3DF21C0BF51872":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":36000.0},"EVID-1A9FB4971218B885A774B43B":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-28D2862523167B2FE81853B6":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1440},"EVID-33BB28CF6EC356A46BE6650D":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-358F61DFBB7111D4CFD58A1A":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-35B29B2F02D863EAADFD08F3":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-387B8FBC6D85BF1D0A585F82":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-3E3D4D117F217EA7DB1596CE":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-46D6FDAC99EA6600704976B5":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-4B254C8301F2AC01CC84CE76":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":30.0},"EVID-4CD8C8C1F0430C6A0156057C":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3600},"EVID-4D3A60329DCF7E143BD06023":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-5427DFBFB88B9EBFC0C27786":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-5559E287993BB07DE138FDF6":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-57741F660C40486486D51EFB":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-57F17FFFCFEDA0A9A60A1FD8":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":13500},"EVID-6C649CEB38C11AD9F545A814":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-753982E08475C2D3F33CAC84":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-7C07E0575343482778154975":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":45.0},"EVID-8CF90399EB348CA2E57A41FC":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-8F4C40C92A48DE9D5B743C29":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-91E83CACE07F654C8375E91B":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":31680.0},"EVID-943CC5DA406961E6EB3068F0":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-947C133A7AF95BA119BCA9FF":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-A3FFF81B3A1797CA534E3F69":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-A4F5DF730DDC736B98D2A1D2":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-A64BE1A219A5E17C9CF9589A":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-A6BDE580C0266C39CA6313B6":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-B5A32995ECFF3B005A70D952":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-B829726708E678EF6D0D4FFD":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-BC390FACE6BB107FDA76E438":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5380.16},"EVID-C5B21CB96D957B10D42BA42D":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1200.0},"EVID-C78D83012F1308C65615F356":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":65000},"EVID-C9561CB7C3F62405C4518E23":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":254},"EVID-CEB50ADB444DABFFABD2448A":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":12.0},"EVID-CEF597117FDE03FC75D46082":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":2160},"EVID-D5234CFF6B2C514C67CA7887":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-D8ED1DBE0C9CA9FD5031A804":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-DC3612A9EEBCACBD7708CC0E":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":15000},"EVID-DCD165B1F77962F8297C7F4D":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":12.0},"EVID-E09FD1F994ABB868559DF515":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":600.0},"EVID-E1011CEF886F3D479CF5E863":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":45.0},"EVID-E14BE0884B6E34FCB998C395":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-E56F010E6353E5FD20061D06":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":720},"EVID-E9801B0191E0C020D4E6D167":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":4500},"EVID-EA77D49C07D5FE5F9FA22988":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-ED798F026DC7D4813C8D1BD7":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":12.0},"EVID-F76F8313D068DA94D8D128E3":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0}}</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="AH9" s="14" t="inlineStr">
         <is>
-          <t>SCN-819DAEDF07A8F0192D7A247C</t>
+          <t>SCN-434C077126B079E5142CDF8C</t>
         </is>
       </c>
       <c r="AI9" s="15" t="inlineStr">
@@ -4042,12 +4042,12 @@
       </c>
       <c r="BF9" s="22" t="inlineStr">
         <is>
-          <t>["SCN-819DAEDF07A8F0192D7A247C","SCN-0C81CFCDAF78B26D6BFDAC1D"]</t>
+          <t>["SCN-434C077126B079E5142CDF8C","SCN-46131C6A05E4B40940D8714B"]</t>
         </is>
       </c>
       <c r="BG9" s="22" t="inlineStr">
         <is>
-          <t>["CAND-2A21A45EFF69356D0EDB4F30","CAND-AB3963A519CBBB85D39C5C32","CAND-04FD915BC6811A9ABF866B65","CAND-441EF1F7D10C5596117E1DEB","CAND-94C56D19D728CCD8E36E75F2","CAND-DBDB7630ED062E15E33B2B7A"]</t>
+          <t>["CAND-2DC77701D9463A039A4A3430","CAND-BA05FACF1A2AF701F6188BBC","CAND-4701F5AB0B552D8BE3E4E34C","CAND-27600366920A82E7674E3D7A","CAND-8B9D97017D3CAA5DA66961BB","CAND-2F116D492B169CDC7BFE4A4F"]</t>
         </is>
       </c>
       <c r="BH9" s="22" t="inlineStr">
@@ -4057,14 +4057,14 @@
       </c>
       <c r="BI9" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00476B7B0F3D8275B2936132":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-00BF09BDCBF894CCAF9C092F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-01F71FB33E6FD6577DC5BBB0":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7000},"EVID-08358BCEEA08EE19FE1FBAA3":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-0BA5CC7CA3B1F6049EB4670D":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0F38E2F7D06930B4B0B76120":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2200},"EVID-138128BA4272677A4B0AB7F4":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2333},"EVID-143518477975AC9C25611AB6":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-197A8C457D558504B0E953FA":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-25F2E397DF6F0BAE15813FE3":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-29E798CD3E14E9ED7476BC9B":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":360},"EVID-2C2B923FC13043FC6E4F00E9":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2DF8660439C625CDBD529815":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-30E518A1606B6C1EDEC6D0A3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5646.94},"EVID-36F22BE2CCDB16F3AD7E178F":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":62.0},"EVID-38DC7D3FF78924866B901CD2":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-44397AB78F278179197384EA":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":15840.0},"EVID-4985D186823206E5659AD9FF":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-49AC15C11B05FE0E025B4079":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-4CA277CD5E12D2564A4386D8":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.2},"EVID-58AAD17D87FDB89D4BE902B2":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":1.0},"EVID-5B682EEE7197C853378411F5":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":18},"EVID-604AC4779AD4C783C7EFA4CC":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-623DCE1B20F50ED2CC8F4149":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-62DB75214B161FAE24013595":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":7},"EVID-673C5350CF07282A55EA50CF":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":18000.0},"EVID-740D9017E7AC3B9814EF6F2B":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-74D377B844B0F634529FA379":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-7A6837724378711D474A758F":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":300.0},"EVID-7D4E39BC0F2BDAAF60D528F0":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-7F91993E1D9D087F839A562B":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-850D0D650424A506C00A22F9":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":6750},"EVID-8867C09103F24942A1655AA8":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.2},"EVID-8A99CBFA2631BA084AEDDF22":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":1.0},"EVID-8D939FBAAD70DE609CEEA32C":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-8F84F05872E6435005166D8D":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.2},"EVID-95141085DD5DC4861990625B":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-A8BFB204051100D76FD32275":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AC243B02F6E32FEE516B7F1A":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":2250},"EVID-AFD7FB4C9DCB9C5F2EC567AE":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-B566F403908A6960BED17E0C":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-BBD71C8135AF7545976EE916":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-BFD933D03EDDB6B88F5B4CAF":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-C7CC6C62FD487AC658763422":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-D1C799F1FF7272E4DA285A38":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-D4AA5B75F719775A0DE24274":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-E84E8CD881597CF3498F5149":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-EEB8E13A0DB907A0E6067CAA":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-F06620CFA61363C1EB9B89DC":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-F5E9C24305F9D197F7BE1862":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-F7405E951F0792C6F09AD862":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":242},"EVID-FE0CC0129747B52484AF90AA":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":720}}</t>
+          <t>{"EVID-00476B7B0F3D8275B2936132":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-00BF09BDCBF894CCAF9C092F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-01F71FB33E6FD6577DC5BBB0":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7000},"EVID-08358BCEEA08EE19FE1FBAA3":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-0BA5CC7CA3B1F6049EB4670D":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0F38E2F7D06930B4B0B76120":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2200},"EVID-138128BA4272677A4B0AB7F4":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2333},"EVID-143518477975AC9C25611AB6":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-197A8C457D558504B0E953FA":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-25F2E397DF6F0BAE15813FE3":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-29E798CD3E14E9ED7476BC9B":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":360},"EVID-2C2B923FC13043FC6E4F00E9":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2DF8660439C625CDBD529815":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-30E518A1606B6C1EDEC6D0A3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5646.94},"EVID-36F22BE2CCDB16F3AD7E178F":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":62.0},"EVID-38DC7D3FF78924866B901CD2":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-44397AB78F278179197384EA":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":15840.0},"EVID-4985D186823206E5659AD9FF":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-49AC15C11B05FE0E025B4079":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-4CA277CD5E12D2564A4386D8":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.2},"EVID-58AAD17D87FDB89D4BE902B2":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":1.0},"EVID-5B682EEE7197C853378411F5":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":18},"EVID-604AC4779AD4C783C7EFA4CC":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-623DCE1B20F50ED2CC8F4149":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-62DB75214B161FAE24013595":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":7},"EVID-740D9017E7AC3B9814EF6F2B":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-74D377B844B0F634529FA379":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-7A6837724378711D474A758F":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":300.0},"EVID-7D4E39BC0F2BDAAF60D528F0":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-7F91993E1D9D087F839A562B":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-850D0D650424A506C00A22F9":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":6750},"EVID-8867C09103F24942A1655AA8":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.2},"EVID-8A99CBFA2631BA084AEDDF22":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":1.0},"EVID-8D939FBAAD70DE609CEEA32C":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-8F84F05872E6435005166D8D":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.2},"EVID-95141085DD5DC4861990625B":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-97CE51EBFF3652C229CC3237":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":18000.0},"EVID-A8BFB204051100D76FD32275":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AC243B02F6E32FEE516B7F1A":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":2250},"EVID-AFD7FB4C9DCB9C5F2EC567AE":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-B566F403908A6960BED17E0C":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-BBD71C8135AF7545976EE916":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-BFD933D03EDDB6B88F5B4CAF":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-C7CC6C62FD487AC658763422":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-D1C799F1FF7272E4DA285A38":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-D4AA5B75F719775A0DE24274":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-E84E8CD881597CF3498F5149":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-EEB8E13A0DB907A0E6067CAA":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-F06620CFA61363C1EB9B89DC":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-F5E9C24305F9D197F7BE1862":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-F7405E951F0792C6F09AD862":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":242},"EVID-FE0CC0129747B52484AF90AA":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":720}}</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="AH10" s="14" t="inlineStr">
         <is>
-          <t>SCN-FFA03F647640FAFA848CFDF5</t>
+          <t>SCN-C3C9758E12BA36251A7A8421</t>
         </is>
       </c>
       <c r="AI10" s="15" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="BF10" s="22" t="inlineStr">
         <is>
-          <t>["SCN-FFA03F647640FAFA848CFDF5","SCN-B9518765A9CBB3B850E61ABC"]</t>
+          <t>["SCN-C3C9758E12BA36251A7A8421","SCN-582CD070FCA0E22EFE63E1A6"]</t>
         </is>
       </c>
       <c r="BG10" s="22" t="inlineStr">
         <is>
-          <t>["CAND-539A61990AAE80EB5F7FEA28","CAND-91BB40F77CB18835E431CCE6","CAND-9B652249BD980BF64F75C35A","CAND-941E7EE62D080D90E6C38505","CAND-912302CE7FA8ECEADF68A266","CAND-2CBB771D8661A0443D52D973"]</t>
+          <t>["CAND-4A1F51AB39038A7D21FFE467","CAND-5021E6E6585A4FEE342CB4BB","CAND-3CDD1DCF71D56AF9C3F59C6F","CAND-70CACBDA2D7EC45AA36032AE","CAND-1CDA6A7761D3E39DAA39959D","CAND-1FAD9418FB980278274923BD"]</t>
         </is>
       </c>
       <c r="BH10" s="22" t="inlineStr">
@@ -4310,14 +4310,14 @@
       </c>
       <c r="BI10" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-004F3A89FEF01598F8C11996":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-086E9F10584C5D0E6D857229":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-088D18F498BE6F6075DD5EE7":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0D702A232EC127629AA49DFE":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-10DD8E20CFD0843967535C3D":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-2569CCF4C70D2EC05D37B00E":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":72},"EVID-279BE51B7ECBECFDA834F95C":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2F27CB2083773BD3028BCFA7":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-3119B00455317B76FC9BAA56":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-32C2CD35574FD6E3A50F0D21":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-3423168674B585D72291AF40":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":14500.0},"EVID-3A74C56DDC296093EECF0652":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-3AC8106EC1B53C26EA9AFFF3":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-3AEA4349F78415A6D5F2A5AF":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-3F89F4000A47FE9CCF922B1E":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-45C4272AA3511B69A47B5B6A":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-466B497A774CAF498A6BA9B6":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-5A333AAE306257AB660C6EF1":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":36},"EVID-68D1E890FA429A7A1DFE9334":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":228},"EVID-69E5E89F43AFCABAB7C89422":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":30.0},"EVID-7A0DB47C7FA59832F2B414AD":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-7C54411923FB6D23463A13EC":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-88E6B93132F288B55F9EB1C7":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-8C03476C65C1A1FCE93F5FB5":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":11000},"EVID-902FC6EB18A50B9E4F86E87E":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-9223F725D7B62642F79C74BE":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-932F65A95D13BD774AC110D4":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-95E864FEF55573BF9580AC47":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":6659.65},"EVID-97A3FB96A83D9D61FF54C1D5":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-9836F65D6D3460015BC6F93E":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-AC85EC83EF0D7DA5FBE17B45":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AE75973FFC8EE1632018BC85":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-AF646F8CF6ACFB35721CE7A5":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-B21546F751C7C8A3A49A2CE3":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-B5D676918ED2DA9FF88A6D1D":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":12760.0},"EVID-B91AB0D86D5DD19043793E83":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-BC2F2A3126DBAE90BE88DB4C":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-C28DA97AA52F62A75E31930A":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-C721CB58A713E142353C518C":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":675},"EVID-C94B20B41C675AC388CC8348":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-C987973F5DA3C85B77BC6628":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-D89261AA21BB363F17428F63":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-E32751AAF6F198EC3ABDE795":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-E436F2B99029CFFC1A356400":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E64F9D530A85A59E200D0361":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-EBE1AA8740CF77C3D09FD892":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-EF86C7A16AAF04754D43BD71":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2800},"EVID-F309A4ABDF88FBD0EDAFF02F":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-F60B902C091A7275F66D6800":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-F92148DD59D012DE5D45E077":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-F97697F36DAAB95BEA42DFBC":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":3},"EVID-FBE987F7046EE4D3FB3A43E3":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0}}</t>
+          <t>{"EVID-004F3A89FEF01598F8C11996":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-086E9F10584C5D0E6D857229":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-088D18F498BE6F6075DD5EE7":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0D702A232EC127629AA49DFE":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-10DD8E20CFD0843967535C3D":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-2569CCF4C70D2EC05D37B00E":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":72},"EVID-279BE51B7ECBECFDA834F95C":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2F27CB2083773BD3028BCFA7":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-3119B00455317B76FC9BAA56":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-32C2CD35574FD6E3A50F0D21":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-3A74C56DDC296093EECF0652":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-3AC8106EC1B53C26EA9AFFF3":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-3AEA4349F78415A6D5F2A5AF":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-3F89F4000A47FE9CCF922B1E":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-45C4272AA3511B69A47B5B6A":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-466B497A774CAF498A6BA9B6":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-5A333AAE306257AB660C6EF1":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":36},"EVID-68D1E890FA429A7A1DFE9334":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":228},"EVID-69E5E89F43AFCABAB7C89422":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":30.0},"EVID-7A0DB47C7FA59832F2B414AD":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-7C54411923FB6D23463A13EC":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-88E6B93132F288B55F9EB1C7":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-8C03476C65C1A1FCE93F5FB5":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":11000},"EVID-902FC6EB18A50B9E4F86E87E":{"interpretation":"Compatibility check s3_access_policy_compatibility returned PASS_BY_EXISTING_SERVERLESS.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"PASS_BY_EXISTING_SERVERLESS"}},"EVID-9223F725D7B62642F79C74BE":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-932F65A95D13BD774AC110D4":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-95E864FEF55573BF9580AC47":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":6659.65},"EVID-97A3FB96A83D9D61FF54C1D5":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-9836F65D6D3460015BC6F93E":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-AC85EC83EF0D7DA5FBE17B45":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AE75973FFC8EE1632018BC85":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-AF646F8CF6ACFB35721CE7A5":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-B21546F751C7C8A3A49A2CE3":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-B5D676918ED2DA9FF88A6D1D":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":12760.0},"EVID-B91AB0D86D5DD19043793E83":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-BC2F2A3126DBAE90BE88DB4C":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-C28DA97AA52F62A75E31930A":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-C721CB58A713E142353C518C":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":675},"EVID-C94B20B41C675AC388CC8348":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-C987973F5DA3C85B77BC6628":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-D89261AA21BB363F17428F63":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-E32751AAF6F198EC3ABDE795":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-E436F2B99029CFFC1A356400":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-E64F9D530A85A59E200D0361":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-EBE1AA8740CF77C3D09FD892":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-EF86C7A16AAF04754D43BD71":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2800},"EVID-F309A4ABDF88FBD0EDAFF02F":{"interpretation":"Compatibility check workspace_serverless_observed returned PASS.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":true,"status":"PASS"}},"EVID-F60B902C091A7275F66D6800":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-F92148DD59D012DE5D45E077":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-F97697F36DAAB95BEA42DFBC":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":3},"EVID-FBE987F7046EE4D3FB3A43E3":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-FDAAC0BC5E85652E7A547DED":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":14500.0}}</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="AH11" s="14" t="inlineStr">
         <is>
-          <t>SCN-DFF0F7B21E7E59997E295C89</t>
+          <t>SCN-0AC9FD46A1C9A180B84B6313</t>
         </is>
       </c>
       <c r="AI11" s="15" t="inlineStr">
@@ -4548,12 +4548,12 @@
       </c>
       <c r="BF11" s="22" t="inlineStr">
         <is>
-          <t>["SCN-DFF0F7B21E7E59997E295C89","SCN-271D4A0780CD3BBEC0341F84"]</t>
+          <t>["SCN-0AC9FD46A1C9A180B84B6313","SCN-81FA38FBB36266F1B735E002"]</t>
         </is>
       </c>
       <c r="BG11" s="22" t="inlineStr">
         <is>
-          <t>["CAND-D02211BBD5905FD5780AB565","CAND-7D5805D2FF2492BB3634AF1C","CAND-4345B5FAFDB5E955A5FD97F9","CAND-411A0364EF7BDE3A2D8A1FC4","CAND-687CCF977D322BBD979CD3F1","CAND-66E8F8CE41F453720A81BDE7"]</t>
+          <t>["CAND-2AB73E156C1AAF3CDDA0CA86","CAND-332EED83B1AA249101A44265","CAND-75CB5E15D22B4E0E72A3CCBC","CAND-2A0FC9335E57A3C9B7F9C7B8","CAND-9E9049ADCEEB150F7DAC6289","CAND-7E49B030E1FF3BD2B17E40BF"]</t>
         </is>
       </c>
       <c r="BH11" s="22" t="inlineStr">
@@ -4563,14 +4563,14 @@
       </c>
       <c r="BI11" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03B043795BC8E94DD967C7AF":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":96},"EVID-03B05DA96489C34CE2110208":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8000},"EVID-089CD33D495CC6061EFF7764":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-166A67EED614A58D24276B2F":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-17967E4F367F91174E4DD90A":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-1E8EDA23B2F72B36B1D93744":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-1F147A54A4B903EA9FF757E1":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-22737B2A74C73AA4C040BE38":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":3},"EVID-260136938BF8F30C964EF511":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2FCC248C10E9F48BD4D77F54":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-3138604EBCD528E08EA037B3":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1},"EVID-330787B0D67DADCBF273B64B":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-46F28580C58548862BD2A95B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":600},"EVID-56715B4903BFF401AF13B22C":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-58EC282F7FC8A787ECCBF4CA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":151840.0},"EVID-5E4A3CABCB119CF19F211D5E":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-64D30D4AB8C6E6421AD90719":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-686AD89E86CEBC94CB6BED6C":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-6F897904B230528E289C4123":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2400},"EVID-73AF487F3DD1F81B6D0219B3":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-75644FA33C29D8ED513B803F":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":10560.0},"EVID-81CFE973454DD11FB7E57FAD":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":1800},"EVID-87899198CD3D28F8AF6A0665":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-91B8D540E9B7FD033C34AA62":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-9EBEB2F65E2632EC2AE72129":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-B13D8C673679E8D15718908E":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-B6AB0F518D240C586B6A9BAA":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-B733CE4EA148EA8A95C45B40":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":3},"EVID-B8B275A31ABAE4DF12904B0D":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-BB0C712245F54E1792FB4DFF":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-BD604BDEFD4EA94581027C35":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-CC158A559E6C492D009CC048":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":80.0},"EVID-CD5D8CB70FA3A41B08E180E2":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-D3EEA70AC8B32F968D671AC3":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":12000.0},"EVID-D856366644C3446CA8C9738B":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-DB69FA385B9B0EC01CC13C6E":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-DC8EDE09C90729113AE9AB54":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-DD24119637B30D9234FEEA1B":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-DED90243F1C5B80CE20CDB44":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":192},"EVID-DFFC77E0EA06DD119782A5C8":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-E3969B0FEA1EC3E2953E6635":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-E3F075A72C222D8EBDE27B38":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-E7592E31B8FF567DFD8C4BAC":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-E868B02D7C51E1D2B2C65B3E":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-ED313069E9F61EFA0C5EFD56":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-EF6BEBBCCBDCFF649C090BB2":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-F6216CA683B090EFED8D549C":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-FD23561554D253F349F128BD":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-FEA1593579C33BD7E3F5E803":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0}}</t>
+          <t>{"EVID-03B043795BC8E94DD967C7AF":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":96},"EVID-03B05DA96489C34CE2110208":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8000},"EVID-089CD33D495CC6061EFF7764":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-166A67EED614A58D24276B2F":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-17967E4F367F91174E4DD90A":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-1E8EDA23B2F72B36B1D93744":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-1F147A54A4B903EA9FF757E1":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-22737B2A74C73AA4C040BE38":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":3},"EVID-260136938BF8F30C964EF511":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2FCC248C10E9F48BD4D77F54":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-3138604EBCD528E08EA037B3":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1},"EVID-330787B0D67DADCBF273B64B":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-46F28580C58548862BD2A95B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":600},"EVID-56715B4903BFF401AF13B22C":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-58EC282F7FC8A787ECCBF4CA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":151840.0},"EVID-5E4A3CABCB119CF19F211D5E":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-64D30D4AB8C6E6421AD90719":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-686AD89E86CEBC94CB6BED6C":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-6F897904B230528E289C4123":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2400},"EVID-73AF487F3DD1F81B6D0219B3":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-75644FA33C29D8ED513B803F":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":10560.0},"EVID-81CFE973454DD11FB7E57FAD":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":1800},"EVID-87899198CD3D28F8AF6A0665":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-91B8D540E9B7FD033C34AA62":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-9EBEB2F65E2632EC2AE72129":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-B13D8C673679E8D15718908E":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-B6AB0F518D240C586B6A9BAA":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-B733CE4EA148EA8A95C45B40":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":3},"EVID-B8B275A31ABAE4DF12904B0D":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-BB0C712245F54E1792FB4DFF":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-BD604BDEFD4EA94581027C35":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-CC158A559E6C492D009CC048":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":80.0},"EVID-CD5D8CB70FA3A41B08E180E2":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-D856366644C3446CA8C9738B":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-DB69FA385B9B0EC01CC13C6E":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-DC8EDE09C90729113AE9AB54":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-DD24119637B30D9234FEEA1B":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-DED90243F1C5B80CE20CDB44":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":192},"EVID-DFFC77E0EA06DD119782A5C8":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-E051999032917A838DDCD461":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":12000.0},"EVID-E3969B0FEA1EC3E2953E6635":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-E3F075A72C222D8EBDE27B38":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-E7592E31B8FF567DFD8C4BAC":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-E868B02D7C51E1D2B2C65B3E":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-ED313069E9F61EFA0C5EFD56":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-EF6BEBBCCBDCFF649C090BB2":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-F6216CA683B090EFED8D549C":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-FD23561554D253F349F128BD":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-FEA1593579C33BD7E3F5E803":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0}}</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="AH12" s="14" t="inlineStr">
         <is>
-          <t>SCN-25C50A8B284AD6025A2723EA</t>
+          <t>SCN-69D437D3D8FDDFE6F953315B</t>
         </is>
       </c>
       <c r="AI12" s="15" t="inlineStr">
@@ -4797,12 +4797,12 @@
       </c>
       <c r="BF12" s="22" t="inlineStr">
         <is>
-          <t>["SCN-25C50A8B284AD6025A2723EA","SCN-BF14FB572683C696D02CD7EA"]</t>
+          <t>["SCN-69D437D3D8FDDFE6F953315B","SCN-27D656892CFF54E7DE80A40B"]</t>
         </is>
       </c>
       <c r="BG12" s="22" t="inlineStr">
         <is>
-          <t>["CAND-00CB68D319FAA492A409545D","CAND-EDB08C1E32CD5DFD2B45A9F1","CAND-064DD3A175BE92BD9C658F7C","CAND-66F4CCF16FDA6E5ED2780272","CAND-F4D441B77DA39A68A9B6983C","CAND-1F3EBDB3DFBB20D0B1CD4658"]</t>
+          <t>["CAND-D701CCAADA13C792A1F2ABC4","CAND-0B53B1CF89A1FF45576E8ACD","CAND-F867AC6F987F34C1567B71E4","CAND-91319B61F24C51743453ED64","CAND-D955E2B2473C8669E75F5A3E","CAND-09EB817A3591B59B95A5BDA5"]</t>
         </is>
       </c>
       <c r="BH12" s="22" t="inlineStr">
@@ -4812,14 +4812,14 @@
       </c>
       <c r="BI12" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00F687C1E6EEFA91E74B77BC":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-01C10C33A653913CBECF537E":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":10},"EVID-08C70D3F461AA8C9C1E94646":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-0D2577F99A78F966A66B9B75":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":45760.0},"EVID-0DFBE3E1D8CA16638D34ABF6":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"SERVERLESS"},"EVID-126B0066E8ED9BC396AF90F5":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":733.33},"EVID-2276D86FAB7C2B5BC1B741C8":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-22BC61EE8E8120AFBAD301A8":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":269},"EVID-30BE7B268EBCA2C565E734CE":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-4266ECEA017A21660614C087":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":16500},"EVID-43CAB2D4F8BAA15A8A9A3F70":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-44095FB79A7F7BEF72DA46ED":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":0},"EVID-48E87CEE6D354F7DE92B8533":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":100.0},"EVID-51E1C6FB4D6767553EA80848":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":5500},"EVID-59FD4115ACB0EBCC2B63BCA7":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-6B7CC2A9F0FE053CF03DFB5E":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":5500},"EVID-6CF2C562A97DB25CEDFBA2E1":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-6FCA127FE42DCA1BFEA9DCDD":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-7DD72E73E5027A86095C5BAF":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":0.0},"EVID-85BF82D6ECB297978551A196":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-8AFB6F95D7C42F5401483897":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-95322770660C5432BDE5C66B":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-9747F4CBC71901286891D2E9":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-980190F3B2D822FEC1043D48":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-9AAC252ACF6900D791D2AD26":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":52000.0},"EVID-9ABB987739ABEE5C6E537210":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.0},"EVID-A151021739E107AC0765F6ED":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":56000.0},"EVID-A75FAB3134E0BBD8EC73EEB4":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-A86918C3CB8E0352D71F4318":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-A97EBA544AC3955018A16D3B":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-AC4441B3F007D44D4E87FF73":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1920.0},"EVID-ADA7AC1BCB3C988A132932FF":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-ADC407565C55B500C48F5ED2":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-B277B645978A6DDE26F31849":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":880},"EVID-BEB268DC8C1FCAFB79C58653":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-BFA0FD588E32AB1988FF8D52":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-C0F8D4DE805D4DB3E336717F":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-CF8BA68C57BA71F1BDD694FC":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":4},"EVID-D194EDED7F6F327969D292B4":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-D6A49DE19AB0D51EE2C9E21C":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-D6CDBCF2AF4AE9D6F8CE9653":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":10},"EVID-DB2D727300A84DFD591BEA88":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-E8A374E6704F50307F8F7829":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1800},"EVID-EAC3FD6CB132DD4EC094D307":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":0.0},"EVID-EF9DF359F0ABC4B35E372381":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-F41A422F78611D9A8DBC6C9F":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":0},"EVID-F5753F549769D56D0A75DE45":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1760},"EVID-F832B6C7EEAD59A8276C0A30":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-FA9EDB53BA7E51763A168D86":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0}}</t>
+          <t>{"EVID-00F687C1E6EEFA91E74B77BC":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-01C10C33A653913CBECF537E":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":10},"EVID-08C70D3F461AA8C9C1E94646":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-0D2577F99A78F966A66B9B75":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":45760.0},"EVID-0DFBE3E1D8CA16638D34ABF6":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"SERVERLESS"},"EVID-126B0066E8ED9BC396AF90F5":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":733.33},"EVID-2276D86FAB7C2B5BC1B741C8":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-22BC61EE8E8120AFBAD301A8":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":269},"EVID-30BE7B268EBCA2C565E734CE":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-4266ECEA017A21660614C087":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":16500},"EVID-43CAB2D4F8BAA15A8A9A3F70":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-44095FB79A7F7BEF72DA46ED":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":0},"EVID-48E87CEE6D354F7DE92B8533":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":100.0},"EVID-51E1C6FB4D6767553EA80848":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":5500},"EVID-59FD4115ACB0EBCC2B63BCA7":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-6B7CC2A9F0FE053CF03DFB5E":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":5500},"EVID-6CF2C562A97DB25CEDFBA2E1":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-6FCA127FE42DCA1BFEA9DCDD":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-7DD72E73E5027A86095C5BAF":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":0.0},"EVID-85BF82D6ECB297978551A196":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-8AFB6F95D7C42F5401483897":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-95322770660C5432BDE5C66B":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-9747F4CBC71901286891D2E9":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-980190F3B2D822FEC1043D48":{"interpretation":"Compatibility check pro_warehouse_type_enabled returned PASS.","metric":"compatibility.pro_warehouse_type_enabled","value":{"evidence":true,"status":"PASS"}},"EVID-9ABB987739ABEE5C6E537210":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.0},"EVID-A151021739E107AC0765F6ED":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":56000.0},"EVID-A75FAB3134E0BBD8EC73EEB4":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-A86918C3CB8E0352D71F4318":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-A97EBA544AC3955018A16D3B":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-AC4441B3F007D44D4E87FF73":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1920.0},"EVID-ADA7AC1BCB3C988A132932FF":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-ADC407565C55B500C48F5ED2":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-B277B645978A6DDE26F31849":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":880},"EVID-BEB268DC8C1FCAFB79C58653":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-BFA0FD588E32AB1988FF8D52":{"interpretation":"Compatibility check aws_price_registry_region returned PASS.","metric":"compatibility.aws_price_registry_region","value":{"evidence":"us-east-1","status":"PASS"}},"EVID-C0F8D4DE805D4DB3E336717F":{"interpretation":"Compatibility check workspace_pro_classic_observed returned PASS.","metric":"compatibility.workspace_pro_classic_observed","value":{"evidence":true,"status":"PASS"}},"EVID-CF8BA68C57BA71F1BDD694FC":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":4},"EVID-D194EDED7F6F327969D292B4":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-D6A49DE19AB0D51EE2C9E21C":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-D6CDBCF2AF4AE9D6F8CE9653":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":10},"EVID-DA09F55E9B9D4B9E274D1724":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":52000.0},"EVID-DB2D727300A84DFD591BEA88":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-E8A374E6704F50307F8F7829":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1800},"EVID-EAC3FD6CB132DD4EC094D307":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":0.0},"EVID-EF9DF359F0ABC4B35E372381":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-F41A422F78611D9A8DBC6C9F":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":0},"EVID-F5753F549769D56D0A75DE45":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1760},"EVID-F832B6C7EEAD59A8276C0A30":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-FA9EDB53BA7E51763A168D86":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0}}</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="AH13" s="14" t="inlineStr">
         <is>
-          <t>SCN-7999EC8BC5B2A2F2A072C81B</t>
+          <t>SCN-2CC0626945850CA914D1FE52</t>
         </is>
       </c>
       <c r="AI13" s="15" t="inlineStr">
@@ -5050,12 +5050,12 @@
       </c>
       <c r="BF13" s="22" t="inlineStr">
         <is>
-          <t>["SCN-7999EC8BC5B2A2F2A072C81B","SCN-2CF9865BFB2C9E9FFFB1F087"]</t>
+          <t>["SCN-2CC0626945850CA914D1FE52","SCN-1A607722905F5626F2592F39"]</t>
         </is>
       </c>
       <c r="BG13" s="22" t="inlineStr">
         <is>
-          <t>["CAND-F68319AE1BD26F3AE3D7C206","CAND-51124DC4FB8ADD3865AA63DB","CAND-A61DE0B24632CFBA54001A80","CAND-B374D8D47EA49C8263B110B4","CAND-2FBBF83290400F68817DBC65","CAND-FF15B75DF3EB05354881F56F"]</t>
+          <t>["CAND-328B32A3406D831E36A10996","CAND-9D796F49F0E013A31CC9883D","CAND-577A4357DFAC3AC2FC120CCC","CAND-0158D968DBF1312B9426F514","CAND-D698FAAC1DCEDE4698BD76F8","CAND-113EE95F32D6329E0F3A4C61"]</t>
         </is>
       </c>
       <c r="BH13" s="22" t="inlineStr">
@@ -5065,14 +5065,14 @@
       </c>
       <c r="BI13" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-059FE4330A15AD87E55A2739":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-157609D059EE617240F34DBA":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-15CF0A5DC41DD4B62D3D9890":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-1FE0A1D231A62E4C4F11DCD0":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.8},"EVID-30873B9A166C94B785F6DD9E":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-34F5EEC65A083C997173A336":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-35D1AC26AEE944960C554D47":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-3B99677A5BA12CD929F685C8":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5488.19},"EVID-3DCE404051777C9BAEF8B72E":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-3FA7FA11988FE0E694F141BC":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-40AB8EEB573EBBC490AC80C3":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-42094F6FB6165ECA71933317":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-503B61DBFF6F18290B1D0B98":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-57FF2359E7551FE22742D506":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-61F35E8FA5A8996603C62417":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":384},"EVID-65D3B2971A671665ED696DAB":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":24},"EVID-6665943F60B0947FC1DB72B0":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":14960.0},"EVID-6836034413538E0247BCD39C":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-709D8A90FB2DAC2E837F6CC4":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":1200},"EVID-81A596AD7DC138D8FF017479":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-84308FE592F273E313559071":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":9000},"EVID-86DC860E1A90F45258B79072":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-8B9D2E503AD6756D35F0BAB9":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-8CF968FBF50B177B3FEDC10A":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-8E56FA6625CBED82319654CD":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-91F2C85163E9C268917948AE":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-92DAC2328781D259CBBFBB85":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-98004CC96788E8AD51027C2D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-98CAA6224EA61D09431C73D8":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":17000.0},"EVID-9907A30A1D61046BB3CED706":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":3600},"EVID-9FD6DEBD0F2C18B06B0371E9":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-A32C46C7F9B097BBBB433A29":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-A8402360CEDF0C2D631CA71B":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-AEBD7278AEA481239BF5900E":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-B0ADC3F9BBD9ECB4740C747D":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-B4303033D02B81F9FB9A34FB":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-B475BD587CAF88BFD454BCEE":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-BA3C0617B4D759D9A07511BA":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-BBF9DD673AEF81FA3C8AA061":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":192},"EVID-C1375153ED8F081F94960AD2":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-D14FED294CE7E7E8308BB67E":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-D517C647FD60879252972C6F":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":249},"EVID-D7DBB679528E173F5E5E7B67":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-DAE8F937EC8E2BC926FB7373":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DC5EA1E87EB0CD581FE95A54":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-E264F0D7C3BF2400A7542F09":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":160.0},"EVID-E6D0D4FA10E482B278F54FFD":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-E7E44A13571351BB72C59DF7":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-ED7225D949D2C454A0AF5F1D":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-F589EAB431C557C66AD277CE":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3000},"EVID-FA63F69E827870908D19759E":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":85000}}</t>
+          <t>{"EVID-059FE4330A15AD87E55A2739":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-157609D059EE617240F34DBA":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-15CF0A5DC41DD4B62D3D9890":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-1FE0A1D231A62E4C4F11DCD0":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.8},"EVID-30873B9A166C94B785F6DD9E":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-34F5EEC65A083C997173A336":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-35D1AC26AEE944960C554D47":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-3B99677A5BA12CD929F685C8":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5488.19},"EVID-3DCE404051777C9BAEF8B72E":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-3FA7FA11988FE0E694F141BC":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-40AB8EEB573EBBC490AC80C3":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-42094F6FB6165ECA71933317":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-503B61DBFF6F18290B1D0B98":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-57FF2359E7551FE22742D506":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-61F35E8FA5A8996603C62417":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":384},"EVID-65D3B2971A671665ED696DAB":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":24},"EVID-6665943F60B0947FC1DB72B0":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":14960.0},"EVID-6836034413538E0247BCD39C":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":17000.0},"EVID-709D8A90FB2DAC2E837F6CC4":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":1200},"EVID-81A596AD7DC138D8FF017479":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-84308FE592F273E313559071":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":9000},"EVID-86DC860E1A90F45258B79072":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-8B9D2E503AD6756D35F0BAB9":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-8CF968FBF50B177B3FEDC10A":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-8E56FA6625CBED82319654CD":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-91F2C85163E9C268917948AE":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-92DAC2328781D259CBBFBB85":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-98004CC96788E8AD51027C2D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-9907A30A1D61046BB3CED706":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":3600},"EVID-9FD6DEBD0F2C18B06B0371E9":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-A32C46C7F9B097BBBB433A29":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-A8402360CEDF0C2D631CA71B":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-AEBD7278AEA481239BF5900E":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-B0ADC3F9BBD9ECB4740C747D":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-B4303033D02B81F9FB9A34FB":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-B475BD587CAF88BFD454BCEE":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-BA3C0617B4D759D9A07511BA":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-BBF9DD673AEF81FA3C8AA061":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":192},"EVID-C1375153ED8F081F94960AD2":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-D14FED294CE7E7E8308BB67E":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-D517C647FD60879252972C6F":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":249},"EVID-D7DBB679528E173F5E5E7B67":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-DAE8F937EC8E2BC926FB7373":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DC5EA1E87EB0CD581FE95A54":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":60.0},"EVID-E264F0D7C3BF2400A7542F09":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":160.0},"EVID-E6D0D4FA10E482B278F54FFD":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-E7E44A13571351BB72C59DF7":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-ED7225D949D2C454A0AF5F1D":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-F589EAB431C557C66AD277CE":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":3000},"EVID-FA63F69E827870908D19759E":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":85000}}</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="AH14" s="14" t="inlineStr">
         <is>
-          <t>SCN-6034F47F88FE870BCBD38A83</t>
+          <t>SCN-AC27CF4B8FF664CD14E343AA</t>
         </is>
       </c>
       <c r="AI14" s="15" t="inlineStr">
@@ -5303,12 +5303,12 @@
       </c>
       <c r="BF14" s="22" t="inlineStr">
         <is>
-          <t>["SCN-6034F47F88FE870BCBD38A83","SCN-60E6E4CF8B3C2E2611EA9BFA"]</t>
+          <t>["SCN-AC27CF4B8FF664CD14E343AA","SCN-7DA4C286CAFA46529A941D00"]</t>
         </is>
       </c>
       <c r="BG14" s="22" t="inlineStr">
         <is>
-          <t>["CAND-1E085EA645EBFB2349B07E26","CAND-0E877A6745803DC5EB83DB93","CAND-3E3533A2458836277B998E86","CAND-A3DE947D6AF269F223F3E0EF","CAND-497F0500B2853FDB8B49F0E2","CAND-3588FD08E2C2D20AB63356BE"]</t>
+          <t>["CAND-72B9F4A05D77B11C4A04BA02","CAND-B6EB43F303C4E8EE0A6DFB03","CAND-AEF82F4F82A158C8B6DEE7FC","CAND-E7EBDE9C9950918CFE5D7D41","CAND-347FA9E6410390B0FEC735D0","CAND-EDC5DB36F0D1AC83E7D2D87F"]</t>
         </is>
       </c>
       <c r="BH14" s="22" t="inlineStr">
@@ -5318,14 +5318,14 @@
       </c>
       <c r="BI14" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03A258EE64A16BEDB5966773":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":36000},"EVID-0E17892A53D58AB0E3D81DA9":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":15.0},"EVID-13DE1277A3F214D8F8E7400C":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":2147483648},"EVID-1484D2B86288BD9635B50252":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":58000.0},"EVID-17090E3CB43BF9A4A57ABFE7":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-173D30F30D973D96C190D660":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":412},"EVID-1DAF48D1163BBA61CD0056E0":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-2A056D89F1674EA69954505E":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":4.2},"EVID-425B9A2FF4A64BAA904964D0":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-44B03B2E73C720355A16DDE9":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":392},"EVID-4B874828C8EF72E08DEA0F30":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-5AC03ABF4E9741764C71D936":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-5C92297D19DABFC0D44936CE":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":15.0},"EVID-5F409B008B651F25022FB9F1":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-6463CC8FB6187D01932BF793":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-6AAE5CF1ECE6878C2CF26D21":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":45},"EVID-6E448D71588E95147EFF2F88":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-6F22403CC3615114ACF5B618":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-6F6A8539FD4499A3F56C3D3E":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-713796EA239C1695235EF207":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-7162B5A4A2E75540071E6568":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-77561C963E48CE1FD39A2EF6":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-78C22D80D0216E511EF28D8C":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":11000},"EVID-86A54913D98871BFD62DA3D6":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-86AA6C5EC99B8A9212BEB2BC":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-8A76454008C18D0CEFE51903":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-8AACAEEF28E431476CC1B4D7":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":1.0},"EVID-8D442199D3A610D39837FACC":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-8FDDF71E8ED766014CAF3614":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-90948AD02E9D2F3CDA3FCC77":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-9F221DC63C2B232A5A2F6CEA":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-A344FF415E43ADC4B5D305F8":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-AB2B7562E0C8B11CCC0C5784":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":262},"EVID-AFA585D0E5C1CA1B67E2DDE8":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":1.0},"EVID-B3729CEB99342E73AC28D761":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-B60E411C1121A2E587066DF4":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":37670.23},"EVID-BCF06BC5C9ABBA23587D9AAD":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":1.0},"EVID-BD171C03C212F63F5B6A670A":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-BF41760B14372497E2F416C7":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":35.0},"EVID-C54ADBED5D740B08A9ABDE1A":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-C59B9CC24DF2F6B383FBBDD7":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-C81F08A5E6EFA115692E37D1":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":7350},"EVID-D0E1731F851342CC365381CF":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-D120D5D150026DD0020186ED":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-D187DFEAE1763FDDD86483AA":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-DBEF4BFB75A13990DC561CF8":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-E7D093253C03B8E31471B2A1":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":326.67},"EVID-E96DF29A15DA7414D3724B94":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-EB97E31584CD7C2D55ED8084":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-EE90BBAB0C3D69CFB2392B54":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":51040.0},"EVID-F772EC513A5C2299BF08C8D9":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":98},"EVID-F92EDAAB3D1B901B5682377E":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":784}}</t>
+          <t>{"EVID-03A258EE64A16BEDB5966773":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":36000},"EVID-0E17892A53D58AB0E3D81DA9":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":15.0},"EVID-13DE1277A3F214D8F8E7400C":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":2147483648},"EVID-17090E3CB43BF9A4A57ABFE7":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-173D30F30D973D96C190D660":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":412},"EVID-1DAF48D1163BBA61CD0056E0":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-2A056D89F1674EA69954505E":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":4.2},"EVID-425B9A2FF4A64BAA904964D0":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-44B03B2E73C720355A16DDE9":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":392},"EVID-4B874828C8EF72E08DEA0F30":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-5AC03ABF4E9741764C71D936":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-5C92297D19DABFC0D44936CE":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":15.0},"EVID-5F409B008B651F25022FB9F1":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":130000.0},"EVID-6463CC8FB6187D01932BF793":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-6AAE5CF1ECE6878C2CF26D21":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":45},"EVID-6E448D71588E95147EFF2F88":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-6F22403CC3615114ACF5B618":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-6F6A8539FD4499A3F56C3D3E":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-713796EA239C1695235EF207":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-7162B5A4A2E75540071E6568":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-77561C963E48CE1FD39A2EF6":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-78C22D80D0216E511EF28D8C":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":11000},"EVID-86A54913D98871BFD62DA3D6":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-86AA6C5EC99B8A9212BEB2BC":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-8A76454008C18D0CEFE51903":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-8AACAEEF28E431476CC1B4D7":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":1.0},"EVID-8D442199D3A610D39837FACC":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-8FDDF71E8ED766014CAF3614":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-90948AD02E9D2F3CDA3FCC77":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-9F221DC63C2B232A5A2F6CEA":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":7},"EVID-A344FF415E43ADC4B5D305F8":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-AB2B7562E0C8B11CCC0C5784":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":262},"EVID-AFA585D0E5C1CA1B67E2DDE8":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":1.0},"EVID-B3729CEB99342E73AC28D761":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-B60E411C1121A2E587066DF4":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":37670.23},"EVID-BCF06BC5C9ABBA23587D9AAD":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":1.0},"EVID-BD171C03C212F63F5B6A670A":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-BF41760B14372497E2F416C7":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":35.0},"EVID-C54ADBED5D740B08A9ABDE1A":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-C59B9CC24DF2F6B383FBBDD7":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":9000},"EVID-C81F08A5E6EFA115692E37D1":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":7350},"EVID-CD777A9CADB66005FD36878A":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":58000.0},"EVID-D0E1731F851342CC365381CF":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-D120D5D150026DD0020186ED":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-D187DFEAE1763FDDD86483AA":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-DBEF4BFB75A13990DC561CF8":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-E7D093253C03B8E31471B2A1":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":326.67},"EVID-E96DF29A15DA7414D3724B94":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-EB97E31584CD7C2D55ED8084":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-EE90BBAB0C3D69CFB2392B54":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":51040.0},"EVID-F772EC513A5C2299BF08C8D9":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":98},"EVID-F92EDAAB3D1B901B5682377E":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":784}}</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="AH15" s="14" t="inlineStr">
         <is>
-          <t>SCN-F8D0AE11F3CFA07D7DFBD032</t>
+          <t>SCN-578A1D1819D737E19D5DEDBE</t>
         </is>
       </c>
       <c r="AI15" s="15" t="inlineStr">
@@ -5556,12 +5556,12 @@
       </c>
       <c r="BF15" s="22" t="inlineStr">
         <is>
-          <t>["SCN-F8D0AE11F3CFA07D7DFBD032","SCN-80FA6497D1269DF9BC6CDAC9"]</t>
+          <t>["SCN-578A1D1819D737E19D5DEDBE","SCN-D3A3FAD11AC31FEC9D1A2AB5"]</t>
         </is>
       </c>
       <c r="BG15" s="22" t="inlineStr">
         <is>
-          <t>["CAND-129F67319BADFA2CE089FF64","CAND-7ADCC0E72B9FC08857017FB5","CAND-55B90A7F8AD84F5FFABA5BD2","CAND-76FF89D1C033A3CA62741ACF","CAND-5763B8095F259B3EEED222B0","CAND-AC5879A21066084E08E49997"]</t>
+          <t>["CAND-8805373F493C9312FE14B270","CAND-4C2622B3D4EF1E9ED54322C7","CAND-6A4B2951E2A605857E3D99F2","CAND-016EDFB75AF0AF6A2C07E315","CAND-4C891B8A1136F219041C9F4E","CAND-C1507494ED1BA885FBF9071F"]</t>
         </is>
       </c>
       <c r="BH15" s="22" t="inlineStr">
@@ -5571,14 +5571,14 @@
       </c>
       <c r="BI15" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-01425C0BD47160649D9BDBF9":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-0226BD31F1B474314ECB9FDD":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-070F7AF4873DD67819657684":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-07DD446F0342AA9E5EE9CD19":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-0DAD979C2237FD3233FFDBB7":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-0DADE24E847363DC78BF885D":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":128},"EVID-18E049878DF524DEC1707E92":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-20B43961F3C6C1A2EE95A29D":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-24D506A8E7E2AEB695EA147B":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-2C3474A5C11EEF4B849349EF":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-39EADFD6CF9C66CE5165ED62":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-3E8E9407D28DA3636DD6D1DB":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-4093408BEE57005F6E49D35A":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":2400},"EVID-43592DE0B8462712436545A5":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-4A2C03CEA6A05D220F7D2277":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":800},"EVID-4E38AC87147767827FFDF2EC":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-5066EABB27208C07CAC1039A":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-50F616330E5AB32E27962258":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":13640.0},"EVID-5B407641EEE5BA93D851431E":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-5E2B2F90F6A7FB35A3F53418":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-5FEC7EBA259C7FFE299914B9":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-82066A1F9E22BA891367ABC2":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":90.0},"EVID-8B7E04D0182B235AA7CA4455":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-8C522E311D367BAF61F3E85A":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-8DEEE675FDE9D16D0002AF87":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-964D24D8B7D84854CFE55FA8":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":106.67},"EVID-979658122CEE3DF38426CB8E":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-99EACDD52661CD8933464BA5":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":15500.0},"EVID-9F434CDB24D2A3FE3556080D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-A9B9E90D64D9BB66A374C8AA":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-AD888A128A52C49972FDD70D":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-AF4D3B48D369F40E23E3E9BD":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AF75DEF9DB7D574EDF91EC64":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-B0FA3283F415F95E654D23E0":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-B8BA520171E53FD0595019DF":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6000},"EVID-BE35B69390609AEABE70E371":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-BECB952FE23A55CFA5BADC5E":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3615.24},"EVID-C182DDECD19F750F8D25FA15":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-CB205C7DCDC2DCF82E6A039B":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-D29573C2C46F89F85FAB8045":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":256},"EVID-D3FEC6D7C214B8D3BF551FE2":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-E027D765B3EFD2171CC0F0E5":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2000},"EVID-E06323EF562817A561795FDA":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-E1D312A511027E48D5E88AB0":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":252},"EVID-EBECC6E7D3E86EC9BF696CBC":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-EC39084808469B0496A22797":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-F00D55756F8FD6C9CF89C2AF":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-F13795802F91F9228B6FFB67":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-F33A6C8B22D19B62AED81051":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-FB48096C1335A2562EDE03B0":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-FB58541C718377C0AABCD1B9":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-FDF2A5D4010ABE92F736B48F":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}}}</t>
+          <t>{"EVID-01425C0BD47160649D9BDBF9":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-0226BD31F1B474314ECB9FDD":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-070F7AF4873DD67819657684":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-07DD446F0342AA9E5EE9CD19":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-0DAD979C2237FD3233FFDBB7":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-0DADE24E847363DC78BF885D":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":128},"EVID-18E049878DF524DEC1707E92":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-20B43961F3C6C1A2EE95A29D":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-24D506A8E7E2AEB695EA147B":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-2C3474A5C11EEF4B849349EF":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1333},"EVID-39EADFD6CF9C66CE5165ED62":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-3E8E9407D28DA3636DD6D1DB":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-4093408BEE57005F6E49D35A":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":2400},"EVID-43592DE0B8462712436545A5":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":4},"EVID-4A2C03CEA6A05D220F7D2277":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":800},"EVID-4E38AC87147767827FFDF2EC":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-5066EABB27208C07CAC1039A":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-50F616330E5AB32E27962258":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":13640.0},"EVID-5B407641EEE5BA93D851431E":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":7920.0},"EVID-5E2B2F90F6A7FB35A3F53418":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-5FEC7EBA259C7FFE299914B9":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-68034385A85814CE5E9D431D":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":15500.0},"EVID-82066A1F9E22BA891367ABC2":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":90.0},"EVID-8B7E04D0182B235AA7CA4455":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-8C522E311D367BAF61F3E85A":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-8DEEE675FDE9D16D0002AF87":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-964D24D8B7D84854CFE55FA8":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":106.67},"EVID-979658122CEE3DF38426CB8E":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-9F434CDB24D2A3FE3556080D":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":2},"EVID-A9B9E90D64D9BB66A374C8AA":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-AD888A128A52C49972FDD70D":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-AF4D3B48D369F40E23E3E9BD":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-AF75DEF9DB7D574EDF91EC64":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-B0FA3283F415F95E654D23E0":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-B8BA520171E53FD0595019DF":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":6000},"EVID-BE35B69390609AEABE70E371":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-BECB952FE23A55CFA5BADC5E":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3615.24},"EVID-C182DDECD19F750F8D25FA15":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-CB205C7DCDC2DCF82E6A039B":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-D29573C2C46F89F85FAB8045":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":256},"EVID-D3FEC6D7C214B8D3BF551FE2":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-E027D765B3EFD2171CC0F0E5":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2000},"EVID-E06323EF562817A561795FDA":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-E1D312A511027E48D5E88AB0":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":252},"EVID-EBECC6E7D3E86EC9BF696CBC":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-EC39084808469B0496A22797":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-F00D55756F8FD6C9CF89C2AF":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-F13795802F91F9228B6FFB67":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":40000.0},"EVID-F33A6C8B22D19B62AED81051":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-FB48096C1335A2562EDE03B0":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-FB58541C718377C0AABCD1B9":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-FDF2A5D4010ABE92F736B48F":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}}}</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="AH16" s="14" t="inlineStr">
         <is>
-          <t>SCN-6AF109497D3D72C350D1DB24</t>
+          <t>SCN-523803CD1056F839B5F4CF5A</t>
         </is>
       </c>
       <c r="AI16" s="15" t="inlineStr">
@@ -5809,12 +5809,12 @@
       </c>
       <c r="BF16" s="22" t="inlineStr">
         <is>
-          <t>["SCN-6AF109497D3D72C350D1DB24","SCN-1A718415E777F8AF64EDE335"]</t>
+          <t>["SCN-523803CD1056F839B5F4CF5A","SCN-79199C03A3C215D8409EAD4B"]</t>
         </is>
       </c>
       <c r="BG16" s="22" t="inlineStr">
         <is>
-          <t>["CAND-244B6A9BF1597473726DCECE","CAND-CD04AB68BD52CC1E1EB78D67","CAND-4D1C8BB67AC3293C91608AA1","CAND-911B8170B602DC4F576083D1","CAND-21808FD63999AEC86B578E0F","CAND-8DAE20517B39B4C87C5DB0F9"]</t>
+          <t>["CAND-69FB4749B4D73D743D4C0864","CAND-0E0C39CCFED2B26094B35BC6","CAND-16C467F705AC450DD5FB6F3F","CAND-17A18E302E55C3A7875CBEE5","CAND-26A61CADCADBE0C78C5ED6CC","CAND-3533B4E4348CE8BBC3CD27A3"]</t>
         </is>
       </c>
       <c r="BH16" s="22" t="inlineStr">
@@ -5824,14 +5824,14 @@
       </c>
       <c r="BI16" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00A3773856382E51F32E0890":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":520},"EVID-0273418DF08CF77E8FEA19EC":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-0B673BFB80ED7BCA73AD9E28":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-0B9354DFC8337B7FF4FBFEDD":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-10240CC6FE1740F33E7065A9":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-20AE8FF8C49B268F1050ADCD":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":433.33},"EVID-2184712B5D074BB210FB51B7":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-233AA44D11F809A7348519BE":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1040},"EVID-252BD3F3682258C790F28B6B":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-2D058786FA5DD49B24F1B760":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2E143851B2321E5658F0CAC4":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-2EEE40F816BC1314FC6D6794":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-34C490032C237ACC89D87EC2":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":22880.0},"EVID-3CD13C8C8685F803F84E6C0C":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-3DAFFB80935B845D569F18C4":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-45924CB6AA2E38CA92267128":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-49901827FD730943673C522F":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-5BA30663403D70E972E0FD56":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-5CB0B7A8854907E8F5396E26":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2100},"EVID-61FD8CB671DF85EFF00A4198":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-6231DA309B2890FEE5630D9F":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-64C8C669F3D65EB7D6DBE41D":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-67937AF881DA47B4E7F6F58F":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9750},"EVID-700C021192DC3C6830C6ACC5":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-71B1F5AA54FCF16B3FE8EDBA":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-73CA0CE74263D4F5F6B2418A":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-74FF3187C068E27FFD83A29D":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5338.12},"EVID-751B770717B686A49D65471D":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-75A390A72C67FC229F633E03":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-7E5A58CA120115D1E2ED5C61":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":256},"EVID-804BAA58EAAF38FFE577161F":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-88F5112E71B1CC7681FAE85F":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-8AE0144C4CD3EFAA8C1FEDD6":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":58.0},"EVID-94A46684F527C403627646A4":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-94C24C425D3C3E2BEBC29DD2":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-9919C3953E1E5DF2D700BD47":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-9A7629DAFB1FBA68EA7CC011":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-9E2A0ACE00349FC117E45E89":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-AB77AEF7838170C844F2636B":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-B2D7C2EE2968246DB663D751":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-B51C44C6D5D6295F37B69434":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-B53D17514F2583F70618DF69":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-B8F35C06BEA4E6B4653B2CA5":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-BA7BE08DA2BEE2DBBB5B7266":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-C132BD268C13FF70511A4C23":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-C2118EC102EA9703BF5A40AB":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-CA272E3BD0899A1D187BF510":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":26000.0},"EVID-D0676180FFB706041DF59124":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-D1B0E499E69AFDB6F3002005":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7200},"EVID-E62E849BC0654AAF5D85EAB7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-E90DF6D21AF730E06ED07EF2":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3250},"EVID-FE0A8787D4FE7A85E7328F2A":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0}}</t>
+          <t>{"EVID-00A3773856382E51F32E0890":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":520},"EVID-0273418DF08CF77E8FEA19EC":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-0B673BFB80ED7BCA73AD9E28":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-0B9354DFC8337B7FF4FBFEDD":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-10240CC6FE1740F33E7065A9":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-20AE8FF8C49B268F1050ADCD":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":433.33},"EVID-2184712B5D074BB210FB51B7":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":30},"EVID-233AA44D11F809A7348519BE":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":1040},"EVID-252BD3F3682258C790F28B6B":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-2D058786FA5DD49B24F1B760":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-2E143851B2321E5658F0CAC4":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-2EEE40F816BC1314FC6D6794":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-34C490032C237ACC89D87EC2":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":22880.0},"EVID-3CD13C8C8685F803F84E6C0C":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-3DAFFB80935B845D569F18C4":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-45924CB6AA2E38CA92267128":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-49901827FD730943673C522F":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-5BA30663403D70E972E0FD56":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-5CB0B7A8854907E8F5396E26":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2100},"EVID-61FD8CB671DF85EFF00A4198":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-6231DA309B2890FEE5630D9F":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-64C8C669F3D65EB7D6DBE41D":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-67937AF881DA47B4E7F6F58F":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":9750},"EVID-700C021192DC3C6830C6ACC5":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-71B1F5AA54FCF16B3FE8EDBA":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-73CA0CE74263D4F5F6B2418A":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-74FF3187C068E27FFD83A29D":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":5338.12},"EVID-751B770717B686A49D65471D":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":1728.0},"EVID-75A390A72C67FC229F633E03":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-7E5A58CA120115D1E2ED5C61":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":256},"EVID-804BAA58EAAF38FFE577161F":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-8866BAE17752BA680D35AD9A":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":26000.0},"EVID-88F5112E71B1CC7681FAE85F":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-8AE0144C4CD3EFAA8C1FEDD6":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":58.0},"EVID-94A46684F527C403627646A4":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-94C24C425D3C3E2BEBC29DD2":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-9919C3953E1E5DF2D700BD47":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-9A7629DAFB1FBA68EA7CC011":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-9E2A0ACE00349FC117E45E89":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-AB77AEF7838170C844F2636B":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-B2D7C2EE2968246DB663D751":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-B51C44C6D5D6295F37B69434":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-B53D17514F2583F70618DF69":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-B8F35C06BEA4E6B4653B2CA5":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-BA7BE08DA2BEE2DBBB5B7266":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":8},"EVID-C132BD268C13FF70511A4C23":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-C2118EC102EA9703BF5A40AB":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-D0676180FFB706041DF59124":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-D1B0E499E69AFDB6F3002005":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":7200},"EVID-E62E849BC0654AAF5D85EAB7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"MEDIUM"},"EVID-E90DF6D21AF730E06ED07EF2":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":3250},"EVID-FE0A8787D4FE7A85E7328F2A":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0}}</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="AH17" s="14" t="inlineStr">
         <is>
-          <t>SCN-3C4F23823E7323060F7D590E</t>
+          <t>SCN-66A9ACF16F67715AEDE3DD1E</t>
         </is>
       </c>
       <c r="AI17" s="15" t="inlineStr">
@@ -6062,12 +6062,12 @@
       </c>
       <c r="BF17" s="22" t="inlineStr">
         <is>
-          <t>["SCN-3C4F23823E7323060F7D590E","SCN-1B5457B19E85EA205F9057D6"]</t>
+          <t>["SCN-66A9ACF16F67715AEDE3DD1E","SCN-EEA1172BA764560AD0C5776C"]</t>
         </is>
       </c>
       <c r="BG17" s="22" t="inlineStr">
         <is>
-          <t>["CAND-AAB5D0F8604AAE069E7BB81F","CAND-CB50137D13AA86B1380E9225","CAND-55C42C4CB74E0DDB5E248AD5","CAND-065AC8BFFA6CD2F35B884972","CAND-ACD999430C8A059DFB38EBAC","CAND-32DF6FED0478FEF9963854FF"]</t>
+          <t>["CAND-209F8112923FB7D955D9E642","CAND-428D7886836325C1957B2FC7","CAND-5D881068EC81653BFBAE9057","CAND-E4E81DFEE63DC47048502757","CAND-6B0ACEABD2495B5A3B07846B","CAND-B9A432AC45556AC42F2CDE81"]</t>
         </is>
       </c>
       <c r="BH17" s="22" t="inlineStr">
@@ -6077,14 +6077,14 @@
       </c>
       <c r="BI17" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00BD6F78F73E54B4ED6BBBD0":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-0164D6D29E0EA5CF4E8AB303":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0AF4AC4CC2EFE0D7B0D04C7D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-0B74F9AC5B2FB5BA3961B896":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":2.0},"EVID-1741410CF2C554E6B884D7EE":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-180293A6D9DB38441576C299":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-19C6EC9C89DF11542B23C017":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":4200},"EVID-1C4C5F2DD86D5D02CEEC8DDF":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-1EC6339D5DE6445CE509F960":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":18480.0},"EVID-23708F72EC5B59C135E02F34":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-2C012211C1C911F47F72090F":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-2E939D43F5BB323DF22E4026":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-346B866635D3784872770C40":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":240.0},"EVID-34DC3E099426F015796451DA":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-363203EBE91A6BA8FE765D72":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":576},"EVID-36A7BD1B9906F3FAC507CA6E":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-37879E4CC18FB3E3DD0B4326":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-40AD09E7303B8B2EDD979703":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-4403DA2AD6FBF575B1913672":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-4651F04F55F5093F44CEAF83":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":233},"EVID-466AA6DFF5D422053A0304C3":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-49DDC09967250A39DC8AA8E3":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":2.0},"EVID-4B4458954444D6D1761F2B97":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-4C8D1DA4927D1E51EAFD5EF0":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-4D3BC0C4CD326B137F0E6E65":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-5C962F772A16D66A63DD8859":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-60FEA6406889613BF7D0D7B2":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-64535252D2DA01A6AA9B32FD":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-6877D38EED61AEE41EC2E4C9":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-6BD6044B2F8274556325FEA5":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-6DB47127905826426728EB23":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-6ECF76708502117135458415":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-7788ACC9A8B33D87E56CB271":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":16000},"EVID-7799CCE95E17579305B3C541":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":5400},"EVID-82B45567DA4A70CD40CCBF6C":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-8E35D24E8738FEA91F76B2F4":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-8E66F44EED7CB4EABFC52575":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-95AE888C192E87C9600B841A":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-95E2FB2242901BE5827CAF65":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-AB85741601676CEF4EC99624":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":2932.53},"EVID-ADA47AE99362347459714D8A":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-B4CF1A6ABE4A98216DB749FB":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-B779811345CC9113D2D9A1EB":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-BAA119A401A590AC412ABE46":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":21000.0},"EVID-C48F43336C1B2F7A7A8B6E1A":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-C6D7693171830636FB13018B":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":288},"EVID-D3229EED878B4951211AF5C1":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":7},"EVID-D53E2EF13F1E733634CCCD78":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-E1B10E4FB81AFD2B35E43242":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-F15353EC12D6ACAD2E076C5B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-F181CC0538E3C28FAA841E28":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-F929BDA3E021BD20ABF1A971":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}}}</t>
+          <t>{"EVID-00BD6F78F73E54B4ED6BBBD0":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-0164D6D29E0EA5CF4E8AB303":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-0A3918300145A810E01D7505":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":21000.0},"EVID-0AF4AC4CC2EFE0D7B0D04C7D":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-0B74F9AC5B2FB5BA3961B896":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":2.0},"EVID-1741410CF2C554E6B884D7EE":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-180293A6D9DB38441576C299":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-19C6EC9C89DF11542B23C017":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":4200},"EVID-1C4C5F2DD86D5D02CEEC8DDF":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-1EC6339D5DE6445CE509F960":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":18480.0},"EVID-23708F72EC5B59C135E02F34":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-2C012211C1C911F47F72090F":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-2E939D43F5BB323DF22E4026":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-346B866635D3784872770C40":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":240.0},"EVID-34DC3E099426F015796451DA":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-363203EBE91A6BA8FE765D72":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":576},"EVID-36A7BD1B9906F3FAC507CA6E":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-37879E4CC18FB3E3DD0B4326":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-40AD09E7303B8B2EDD979703":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-4403DA2AD6FBF575B1913672":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-4651F04F55F5093F44CEAF83":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":233},"EVID-466AA6DFF5D422053A0304C3":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":5},"EVID-49DDC09967250A39DC8AA8E3":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":2.0},"EVID-4B4458954444D6D1761F2B97":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":4},"EVID-4C8D1DA4927D1E51EAFD5EF0":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-4D3BC0C4CD326B137F0E6E65":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-5C962F772A16D66A63DD8859":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-60FEA6406889613BF7D0D7B2":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.1667},"EVID-64535252D2DA01A6AA9B32FD":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-6877D38EED61AEE41EC2E4C9":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-6BD6044B2F8274556325FEA5":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":55.0},"EVID-6DB47127905826426728EB23":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-6ECF76708502117135458415":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-7788ACC9A8B33D87E56CB271":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":16000},"EVID-7799CCE95E17579305B3C541":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":5400},"EVID-82B45567DA4A70CD40CCBF6C":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-8E35D24E8738FEA91F76B2F4":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-8E66F44EED7CB4EABFC52575":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-95AE888C192E87C9600B841A":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-95E2FB2242901BE5827CAF65":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-AB85741601676CEF4EC99624":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":2932.53},"EVID-ADA47AE99362347459714D8A":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":1000},"EVID-B4CF1A6ABE4A98216DB749FB":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-B779811345CC9113D2D9A1EB":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-C48F43336C1B2F7A7A8B6E1A":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-C6D7693171830636FB13018B":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":288},"EVID-D3229EED878B4951211AF5C1":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":7},"EVID-D53E2EF13F1E733634CCCD78":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-E1B10E4FB81AFD2B35E43242":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-F15353EC12D6ACAD2E076C5B":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-F181CC0538E3C28FAA841E28":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-F929BDA3E021BD20ABF1A971":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}}}</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PKG-02C2A3390BC1C4114197FDAD</t>
+          <t>PKG-664E535A61AEB69185D775A9</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="AH18" s="14" t="inlineStr">
         <is>
-          <t>SCN-8FDC6E54EE7012064F9C9683</t>
+          <t>SCN-43F5B63431477AC470A9522A</t>
         </is>
       </c>
       <c r="AI18" s="15" t="inlineStr">
@@ -6315,12 +6315,12 @@
       </c>
       <c r="BF18" s="22" t="inlineStr">
         <is>
-          <t>["SCN-8FDC6E54EE7012064F9C9683","SCN-39CB4EC90BE02170DAA80379"]</t>
+          <t>["SCN-43F5B63431477AC470A9522A","SCN-EB5A1A4A95D402FF8562792C"]</t>
         </is>
       </c>
       <c r="BG18" s="22" t="inlineStr">
         <is>
-          <t>["CAND-DF495D633D84F3AE8A813276","CAND-B1ED2C3FFE321E66E70DDEA3","CAND-725CF31F6E259EE88A0B613A","CAND-A167E0422FF656864EE0A59B","CAND-E2B65D1860279B86ED655385","CAND-FF6F464540547619819C2285"]</t>
+          <t>["CAND-186FCE93391AFC4EF35A6CBC","CAND-B53760F75B53442716A3FA4F","CAND-851FAED6DD515C85FA86FF07","CAND-52B3F4C627B29D5BAB8CFF88","CAND-F0373D6262BAB4AA88A836D9","CAND-E1F56BF222EF5FFED707D9C3"]</t>
         </is>
       </c>
       <c r="BH18" s="22" t="inlineStr">
@@ -6330,14 +6330,14 @@
       </c>
       <c r="BI18" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-05663CC3B2F16BDA6872F815":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-0780430512C23819DED79D5C":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0AD0589876F899B1952DAE24":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-0E39BB07A52CCA2264264F50":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":3200.0},"EVID-11BD92532930EC0A53F07D9D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-160E49D36662E0D31042F51A":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-1FACB7722CC3D6D36961D04E":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":11.25},"EVID-1FDA0700A45761E2E0DC6B81":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":2816.0},"EVID-21C81FA034E87B1F3F7F6DC2":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-24D5B79F9256B930AF1347AB":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-27955C45657420815891038E":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-2B9459F3394D8F98E3B82AA1":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-2E8779032372AE62F7A5B911":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-34F1847BE68B6EBBFA915B95":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1600},"EVID-34FCA371FD0F376A17EA29F8":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-4F1C02974E4C2865E7A50144":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-5045C3FC4FB05F520EFFF251":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":33},"EVID-5048EEF752FFDC02F573D115":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":5},"EVID-57ECB16438BC0501289666B3":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-616B75581FAF5783E6529E1D":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-63863E04521E55A5B64D6EA7":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-67F31581A04C53F6C09C2132":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-6C27B9E8BEE0D6837A9D7BB5":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-6DD782A2BB5F89EE62C99CA3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3733.77},"EVID-7204C8146CD0ECE7ABBDD178":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-738C19E56B6084DC96E07DFC":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-73C60CECF4EC6348178D77CA":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-76CE682449BA3088A5EBB4E1":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-7983B38362D1CC3EC0CE3291":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-828F5F1036D6622A2210D3EC":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-89B2E15FC06474BF301B094E":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-92ED300E01C85F9B5AF548B7":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":3},"EVID-9349C4F74710189DF28D26E5":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":122},"EVID-9520A9F3745C6B42827B881A":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-9C5A7D28B4BA43DE7C3220CD":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":4000},"EVID-9E575E9AFEFC84CDD908C6E2":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-A264A57620417E0913975A94":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":2},"EVID-A3B5D38B573515F1A3160299":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-B85976DAECB1E88018C6509B":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-C3A26BBE94815B44ABBAB98F":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-C6DEEB3C383C817D2C51F62F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-C6F3F79BC6004F797F66391D":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-C8DD5554A816A72AA6BFADCE":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-CD5D3B13B110CBF61F208478":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-CDC30A10A554D84D8C537CD3":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.5},"EVID-D13BA07AC4F2B2109C2C45B7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-DA2EDCB4ECB92BADC692A9C3":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-DA9A337A04DD6ADCBF6EA063":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-DB1D906A0D6DE794AFD7DB72":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-DEA2982F45002B6A998D521E":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-E4E6EBBFF99EE62F40D19F09":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-E74369C9127F37E94753C31E":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":45.0}}</t>
+          <t>{"EVID-05663CC3B2F16BDA6872F815":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-0780430512C23819DED79D5C":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0AD0589876F899B1952DAE24":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-11BD92532930EC0A53F07D9D":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-160E49D36662E0D31042F51A":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-1FACB7722CC3D6D36961D04E":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":11.25},"EVID-1FDA0700A45761E2E0DC6B81":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":2816.0},"EVID-21C81FA034E87B1F3F7F6DC2":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-24D5B79F9256B930AF1347AB":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.0},"EVID-27955C45657420815891038E":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-2B9459F3394D8F98E3B82AA1":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":10120.0},"EVID-2E8779032372AE62F7A5B911":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-34F1847BE68B6EBBFA915B95":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":1600},"EVID-34FCA371FD0F376A17EA29F8":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-4F1C02974E4C2865E7A50144":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-5045C3FC4FB05F520EFFF251":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":33},"EVID-5048EEF752FFDC02F573D115":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":5},"EVID-57ECB16438BC0501289666B3":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":120},"EVID-616B75581FAF5783E6529E1D":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-63863E04521E55A5B64D6EA7":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-67F31581A04C53F6C09C2132":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":1},"EVID-6C27B9E8BEE0D6837A9D7BB5":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.0},"EVID-6DD782A2BB5F89EE62C99CA3":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":3733.77},"EVID-7204C8146CD0ECE7ABBDD178":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":0},"EVID-738C19E56B6084DC96E07DFC":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-73C60CECF4EC6348178D77CA":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-76CE682449BA3088A5EBB4E1":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-7983B38362D1CC3EC0CE3291":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-828F5F1036D6622A2210D3EC":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-89B2E15FC06474BF301B094E":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.0},"EVID-92ED300E01C85F9B5AF548B7":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":3},"EVID-9349C4F74710189DF28D26E5":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":122},"EVID-9520A9F3745C6B42827B881A":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-9C5A7D28B4BA43DE7C3220CD":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":4000},"EVID-9E575E9AFEFC84CDD908C6E2":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-A264A57620417E0913975A94":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":2},"EVID-A3B5D38B573515F1A3160299":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-B85976DAECB1E88018C6509B":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-C3A26BBE94815B44ABBAB98F":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":0},"EVID-C6DEEB3C383C817D2C51F62F":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-C6F3F79BC6004F797F66391D":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-C8DD5554A816A72AA6BFADCE":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-CD5D3B13B110CBF61F208478":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-CDC30A10A554D84D8C537CD3":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.5},"EVID-D13BA07AC4F2B2109C2C45B7":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"SMALL"},"EVID-DA2EDCB4ECB92BADC692A9C3":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":2},"EVID-DA9A337A04DD6ADCBF6EA063":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":0},"EVID-DB1D906A0D6DE794AFD7DB72":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":20000.0},"EVID-DEA2982F45002B6A998D521E":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0},"EVID-E4E6EBBFF99EE62F40D19F09":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-E74369C9127F37E94753C31E":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":45.0},"EVID-F9AD519DB03E1D0381CB098E":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":3200.0}}</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PKG-AAD2A5F749FD290F3138AB5C</t>
+          <t>PKG-12310EDCE7FFCF9E8111114F</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="AH19" s="14" t="inlineStr">
         <is>
-          <t>SCN-8347382151702D72FD4C7016</t>
+          <t>SCN-F21183EC4EC78A0BBDAE0EBC</t>
         </is>
       </c>
       <c r="AI19" s="15" t="inlineStr">
@@ -6568,12 +6568,12 @@
       </c>
       <c r="BF19" s="22" t="inlineStr">
         <is>
-          <t>["SCN-8347382151702D72FD4C7016","SCN-2AA83F694744EABD32EBFDC8"]</t>
+          <t>["SCN-F21183EC4EC78A0BBDAE0EBC","SCN-0D507F5621CB3870A7FD7BE3"]</t>
         </is>
       </c>
       <c r="BG19" s="22" t="inlineStr">
         <is>
-          <t>["CAND-0BFA4AFAEB4B6BBBBFF81BD1","CAND-FD0EB76CB7D1BCCA6922F667","CAND-7B6686612C0DD9AC7B23D9D2","CAND-9702B2C7E3FDFBA0D271EF69","CAND-B655DB77EFCC30A1DD7E127C","CAND-AE90A6A42FD1F94FB256D883"]</t>
+          <t>["CAND-2EBFFE9A1BC3BC17D6166566","CAND-58C1DDD819272E9FEE9074A9","CAND-79A6AA57196043E2E050C701","CAND-8A8B962D786512042B09C749","CAND-B127AE44291FA0B54762C906","CAND-AD7E7D9A3D0FF3226E9F1282"]</t>
         </is>
       </c>
       <c r="BH19" s="22" t="inlineStr">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="BI19" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-013AF0D4100023303BDFD2A7":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-05DA23F1C23FE367A7DA3808":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-09E33179820C5EFC55542C66":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0D961CD8C3B4F20F72AEF2FF":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":880},"EVID-14C3C33548B7E08FE050F2CF":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-15C7C67119A67B5944AB2899":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-22BA61D33267AA7C1BC01567":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-2611DA9D50C11304C9973589":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-29DF47BE855B4DACDA7241A3":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2A164911C70A8C1108570671":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-33D06948BAFC6140DA56DD75":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-344F4D1BA3DF8BB13631E214":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-371DBDD605217D118F4E193F":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-383DCDB4EE07FF9C917545EB":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-510AFA9FBFF7BC81EFCBB501":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-54A4140751F39CF606C628AF":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-54C46A5FAD43CDFFAE089168":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":29040.0},"EVID-556FE78DCB047941101560A8":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-55DC30649E47B909EABCB8BC":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8500},"EVID-56D60AB28E872D0C2F0DD91A":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-5D64CF9B1C01826DDE0EE964":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-66456183B02AADC174EA2617":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":11},"EVID-688983026815DD8C0086D0F7":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":366.67},"EVID-6BBF4AAEBB864345F0F6DAF8":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-6C6F1C9D6A18448012C48FEA":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-6E637FA4341433EE45BF2B5A":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-72D57560B0F1C56E02B9F0CD":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-73EA2EB7AB5CB30D6B7D609D":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":8250},"EVID-7CE8DFF2A46AE4519DA451A6":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-7E9E7371827009D4D06C3F76":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":33000.0},"EVID-8402CBA053B29D588C9A9222":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-8612F5BB3349996472AEB3C8":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-8F5A1F6A957ADEB3B0906EC0":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-90055F47F4D5669251A316E7":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-943AD3BC9A40DF0CFFD309F5":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":8793.82},"EVID-9567B5B020FFAE348DA5D926":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-A3973250904BB40B76E1E527":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-A7F2920455F0333CC8955780":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-B1C6B7C6146EE7A3C63CDAAD":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-B37C5177BB01F6387791B8F1":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-B536166FAC942197556D371E":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-BA02237DA68F25CC23A0F0AB":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-BBE4F5C010E4B2F4059413E1":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":65.0},"EVID-BEFD899C14CEB4D6A16D2CBF":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-C02656417914FFA5B2403F89":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-C1C87C5A4518AC653A1E342B":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":5},"EVID-D11C52233B5E2BC24C8EC07E":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DEFCDDD672F31913742A7FA9":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-EB4F4DEAE95D3BF82604A74B":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-F175A7313421CDD6E1685A38":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2300},"EVID-F5E948F61EB0E0AD62C9AF94":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":440},"EVID-F6F97BF293DD5C6CC48C4DAD":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0}}</t>
+          <t>{"EVID-013AF0D4100023303BDFD2A7":{"interpretation":"Configured minimum scale.","metric":"min_clusters","value":1},"EVID-05DA23F1C23FE367A7DA3808":{"interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","value":0},"EVID-09E33179820C5EFC55542C66":{"interpretation":"Alert workload mix context.","metric":"alert_queries_30","value":0},"EVID-0D961CD8C3B4F20F72AEF2FF":{"interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","value":880},"EVID-14C3C33548B7E08FE050F2CF":{"interpretation":"Compatibility check workspace_serverless_enablement returned PASS.","metric":"compatibility.workspace_serverless_enablement","value":{"evidence":true,"status":"PASS"}},"EVID-15C7C67119A67B5944AB2899":{"interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","value":0},"EVID-22BA61D33267AA7C1BC01567":{"interpretation":"Compatibility check workspace_serverless_observed returned UNKNOWN.","metric":"compatibility.workspace_serverless_observed","value":{"evidence":false,"status":"UNKNOWN"}},"EVID-2611DA9D50C11304C9973589":{"interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","value":0},"EVID-29DF47BE855B4DACDA7241A3":{"interpretation":"Compatibility check external_legacy_hive_metastore_workspace_setting returned PASS.","metric":"compatibility.external_legacy_hive_metastore_workspace_setting","value":{"evidence":{"config_keys":[],"detected":false},"status":"PASS"}},"EVID-2A164911C70A8C1108570671":{"interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","value":0.1},"EVID-33D06948BAFC6140DA56DD75":{"interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-344F4D1BA3DF8BB13631E214":{"interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","value":"CURRENT"},"EVID-371DBDD605217D118F4E193F":{"interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","value":0},"EVID-383DCDB4EE07FF9C917545EB":{"interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","value":3500},"EVID-510AFA9FBFF7BC81EFCBB501":{"interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","value":0.3},"EVID-54A4140751F39CF606C628AF":{"interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","value":259},"EVID-54C46A5FAD43CDFFAE089168":{"interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","value":29040.0},"EVID-556FE78DCB047941101560A8":{"interpretation":"Current warehouse size.","metric":"warehouse_size","value":"LARGE"},"EVID-55DC30649E47B909EABCB8BC":{"interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","value":8500},"EVID-56D60AB28E872D0C2F0DD91A":{"interpretation":"Compatibility check s3_access_policy_compatibility returned UNKNOWN.","metric":"compatibility.s3_access_policy_compatibility","value":{"evidence":"UNKNOWN","status":"UNKNOWN"}},"EVID-5D64CF9B1C01826DDE0EE964":{"interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","value":3600.0},"EVID-66456183B02AADC174EA2617":{"interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","value":11},"EVID-688983026815DD8C0086D0F7":{"interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","value":366.67},"EVID-6BBF4AAEBB864345F0F6DAF8":{"interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","value":0.0},"EVID-6C6F1C9D6A18448012C48FEA":{"interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","value":30000.0},"EVID-6E637FA4341433EE45BF2B5A":{"interpretation":"Compatibility check legacy_hive_metastore_sql_reference returned PASS_WITH_LIMITATION.","metric":"compatibility.legacy_hive_metastore_sql_reference","value":{"evidence":{"reference_queries":0,"visible_pct":100.0},"status":"PASS_WITH_LIMITATION"}},"EVID-72D57560B0F1C56E02B9F0CD":{"interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","value":800},"EVID-73EA2EB7AB5CB30D6B7D609D":{"interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","value":8250},"EVID-7CE8DFF2A46AE4519DA451A6":{"interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","value":70.0},"EVID-8402CBA053B29D588C9A9222":{"interpretation":"Current warehouse type.","metric":"warehouse_type","value":"PRO"},"EVID-8612F5BB3349996472AEB3C8":{"interpretation":"Compatibility check aws_region_serverless_availability returned PASS.","metric":"compatibility.aws_region_serverless_availability","value":{"evidence":{"policy":"Databricks documents Serverless SQL warehouse support across AWS regions.","region":"us-east-1"},"status":"PASS"}},"EVID-8F5A1F6A957ADEB3B0906EC0":{"interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","value":0.1},"EVID-90055F47F4D5669251A316E7":{"interpretation":"Genie workload mix context.","metric":"genie_queries_30","value":0},"EVID-943AD3BC9A40DF0CFFD309F5":{"interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","value":8793.82},"EVID-9567B5B020FFAE348DA5D926":{"interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","value":0.0},"EVID-A3973250904BB40B76E1E527":{"interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","value":100.0},"EVID-A7F2920455F0333CC8955780":{"interpretation":"Job workload mix context.","metric":"job_queries_30","value":0},"EVID-B1C6B7C6146EE7A3C63CDAAD":{"interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","value":60},"EVID-B37C5177BB01F6387791B8F1":{"interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","value":0.0},"EVID-B536166FAC942197556D371E":{"interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","value":0.0},"EVID-BA02237DA68F25CC23A0F0AB":{"interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","value":6},"EVID-BBE4F5C010E4B2F4059413E1":{"interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","value":65.0},"EVID-BEFD899C14CEB4D6A16D2CBF":{"interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","value":35.0},"EVID-C02656417914FFA5B2403F89":{"interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","value":0.2},"EVID-C1C87C5A4518AC653A1E342B":{"interpretation":"Configured concurrency ceiling.","metric":"max_clusters","value":5},"EVID-CFC3799B9BB6502153FA55C0":{"interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","value":33000.0},"EVID-D11C52233B5E2BC24C8EC07E":{"interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","value":0},"EVID-DEFCDDD672F31913742A7FA9":{"interpretation":"Highest observed scale level.","metric":"max_observed_clusters","value":2},"EVID-EB4F4DEAE95D3BF82604A74B":{"interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","value":0.1},"EVID-F175A7313421CDD6E1685A38":{"interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","value":2300},"EVID-F5E948F61EB0E0AD62C9AF94":{"interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","value":440},"EVID-F6F97BF293DD5C6CC48C4DAD":{"interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","value":0}}</t>
         </is>
       </c>
     </row>
@@ -7375,12 +7375,12 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SCN-863D86733C17ECB8516EF093</t>
+          <t>SCN-0F323C820C480A6DB359983B</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -7536,12 +7536,12 @@
       </c>
       <c r="AP5" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-EE57C678D7321484C82E7EC4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-7C972C46E6BADA6422EF650F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-759D0E09D0D3D1DF01FBBA2B","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":8207.57,"high":11021.59,"low":4690.04},"dbu":{"base":10241.38,"high":23648.28,"low":-6517.24},"total":{"base":18448.95,"high":34669.87,"low":-1827.2}}},"recommended_value":1,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-AF9E15C01CEAC8C1A0D722AB","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":9252.28,"high":11725.1,"low":5386.51},"dbu":{"base":15218.69,"high":27000.0,"low":-3199.03},"total":{"base":24470.97,"high":38725.1,"low":2187.48}}},"recommended_value":30,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-19BB082E74D6C1E39FFF482D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-FACB02F992DE84FD0C6488B6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":6800.56,"high":8207.57,"low":4690.04},"dbu":{"base":3537.93,"high":10241.38,"low":-6517.24},"total":{"base":10338.49,"high":18448.95,"low":-1827.2}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-F52C33A9DDA0277D8F79D9E6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":8207.57,"high":11021.59,"low":4690.04},"dbu":{"base":10241.38,"high":23648.28,"low":-6517.24},"total":{"base":18448.95,"high":34669.87,"low":-1827.2}}},"recommended_value":1,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-8FB89535DFCD63C9A63BF39E","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":9252.28,"high":11725.1,"low":5386.51},"dbu":{"base":15218.69,"high":27000.0,"low":-3199.03},"total":{"base":24470.97,"high":38725.1,"low":2187.48}}},"recommended_value":30,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ5" s="22" t="inlineStr">
         <is>
-          <t>["CAND-EE57C678D7321484C82E7EC4","CAND-7C972C46E6BADA6422EF650F","CAND-759D0E09D0D3D1DF01FBBA2B","CAND-AF9E15C01CEAC8C1A0D722AB"]</t>
+          <t>["CAND-19BB082E74D6C1E39FFF482D","CAND-FACB02F992DE84FD0C6488B6","CAND-F52C33A9DDA0277D8F79D9E6","CAND-8FB89535DFCD63C9A63BF39E"]</t>
         </is>
       </c>
       <c r="AR5" s="22" t="inlineStr">
@@ -7558,12 +7558,12 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SCN-145D50BED02E3BA2BE197B7F</t>
+          <t>SCN-05AEB24D88A789A8A5B3097C</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -7725,12 +7725,12 @@
       </c>
       <c r="AP6" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-E9A7141D8480ED7AC73076CC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":11725.1,"high":11725.1,"low":11725.1},"dbu":{"base":693.69,"high":13846.85,"low":693.69},"total":{"base":12418.79,"high":25571.95,"low":12418.79}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-B5D201CF9262CAC1AA7E3182","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":11725.1,"high":11725.1,"low":11725.1},"dbu":{"base":693.69,"high":13846.85,"low":693.69},"total":{"base":12418.79,"high":25571.95,"low":12418.79}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ6" s="22" t="inlineStr">
         <is>
-          <t>["CAND-E9A7141D8480ED7AC73076CC"]</t>
+          <t>["CAND-B5D201CF9262CAC1AA7E3182"]</t>
         </is>
       </c>
       <c r="AR6" s="22" t="inlineStr">
@@ -7747,12 +7747,12 @@
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SCN-B31B08FCFCF16CF8C3ED3133</t>
+          <t>SCN-EB2C0C39F179860453FE1B76</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -7908,12 +7908,12 @@
       </c>
       <c r="AP7" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-725D8CE810F7854F0B4F0599","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"X_LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-19440.12,"high":7476.97,"low":-59815.76},"dbu":{"base":-25600.0,"high":0.0,"low":-64000.0},"total":{"base":-45040.12,"high":7476.97,"low":-123815.76}}},"recommended_value":"2X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-CC561F3665974267980305C7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13849.65,"high":14930.93,"low":-56088.78},"dbu":{"base":-20283.08,"high":7089.23,"low":-60455.38},"total":{"base":-34132.73,"high":22020.16,"low":-116544.16}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-429785936CDB1BB844384CE3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"X_LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-19440.12,"high":7476.97,"low":-59815.76},"dbu":{"base":-25600.0,"high":0.0,"low":-64000.0},"total":{"base":-45040.12,"high":7476.97,"low":-123815.76}}},"recommended_value":"2X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-9036A0CCF32202C187B847C1","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13849.65,"high":14930.93,"low":-56088.78},"dbu":{"base":-20283.08,"high":7089.23,"low":-60455.38},"total":{"base":-34132.73,"high":22020.16,"low":-116544.16}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ7" s="22" t="inlineStr">
         <is>
-          <t>["CAND-725D8CE810F7854F0B4F0599","CAND-CC561F3665974267980305C7"]</t>
+          <t>["CAND-429785936CDB1BB844384CE3","CAND-9036A0CCF32202C187B847C1"]</t>
         </is>
       </c>
       <c r="AR7" s="22" t="inlineStr">
@@ -7930,12 +7930,12 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SCN-49F9E59C5DC51E8EA18565EB</t>
+          <t>SCN-BA79A1BAC0F873D6CDE9EC20</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -8097,12 +8097,12 @@
       </c>
       <c r="AP8" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-FBE101BD35EAD540544961F6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":74769.7,"high":74769.7,"low":74769.7},"dbu":{"base":-103752.53,"high":38191.92,"low":-116656.57},"total":{"base":-28982.83,"high":112961.62,"low":-41886.87}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-50DDBBB8A017E60563909CE4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":74769.7,"high":74769.7,"low":74769.7},"dbu":{"base":-103752.53,"high":38191.92,"low":-116656.57},"total":{"base":-28982.83,"high":112961.62,"low":-41886.87}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ8" s="22" t="inlineStr">
         <is>
-          <t>["CAND-FBE101BD35EAD540544961F6"]</t>
+          <t>["CAND-50DDBBB8A017E60563909CE4"]</t>
         </is>
       </c>
       <c r="AR8" s="22" t="inlineStr">
@@ -8119,12 +8119,12 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SCN-9D2CE3A1C8DF6267C795DB02</t>
+          <t>SCN-26E77B55DE75D30BC7D94E62</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -8280,12 +8280,12 @@
       </c>
       <c r="AP9" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-EB8642E918D1FD97EE3FA4E2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-40DECBD0C64F73A246651419","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":6,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":4,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-47C39CB54A496B16C7C5535D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":14219.04,"high":18646.52,"low":8514.39},"dbu":{"base":15028.97,"high":35685.52,"low":-11586.21},"total":{"base":29248.01,"high":54332.04,"low":-3071.82}}},"recommended_value":2,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-7B32E8C35D19CC2C522779EC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":15975.13,"high":20987.98,"low":9685.12},"dbu":{"base":23222.07,"high":46609.66,"low":-6124.14},"total":{"base":39197.2,"high":67597.64,"low":3560.98}}},"recommended_value":45,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-983E960CC6715CCFDAFC3353","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-925E95E6BA6DA0ED59A9A733","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":6,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":12345.87,"high":14900.19,"low":8514.39},"dbu":{"base":6289.66,"high":18206.9,"low":-11586.21},"total":{"base":18635.53,"high":33107.09,"low":-3071.82}}},"recommended_value":4,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-C01B3B61787F253552AB5722","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":14219.04,"high":18646.52,"low":8514.39},"dbu":{"base":15028.97,"high":35685.52,"low":-11586.21},"total":{"base":29248.01,"high":54332.04,"low":-3071.82}}},"recommended_value":2,"step":3,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-014DD489DCA84594FA96ACC7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":15975.13,"high":20987.98,"low":9685.12},"dbu":{"base":23222.07,"high":46609.66,"low":-6124.14},"total":{"base":39197.2,"high":67597.64,"low":3560.98}}},"recommended_value":45,"step":4,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":5,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ9" s="22" t="inlineStr">
         <is>
-          <t>["CAND-EB8642E918D1FD97EE3FA4E2","CAND-40DECBD0C64F73A246651419","CAND-47C39CB54A496B16C7C5535D","CAND-7B32E8C35D19CC2C522779EC"]</t>
+          <t>["CAND-983E960CC6715CCFDAFC3353","CAND-925E95E6BA6DA0ED59A9A733","CAND-C01B3B61787F253552AB5722","CAND-014DD489DCA84594FA96ACC7"]</t>
         </is>
       </c>
       <c r="AR9" s="22" t="inlineStr">
@@ -8302,12 +8302,12 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SCN-3E24BF4E2EB1FFD6BD97C5EF</t>
+          <t>SCN-DF356B65FC7D9469319D516C</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AP10" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-1E5BC9641C5288D175C688E2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":21285.98,"high":21285.98,"low":21285.98},"dbu":{"base":242.99,"high":32081.0,"low":242.99},"total":{"base":21528.97,"high":53366.98,"low":21528.97}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-C8B00F2B86A8B7AF7549A783","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":21285.98,"high":21285.98,"low":21285.98},"dbu":{"base":242.99,"high":32081.0,"low":242.99},"total":{"base":21528.97,"high":53366.98,"low":21528.97}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ10" s="22" t="inlineStr">
         <is>
-          <t>["CAND-1E5BC9641C5288D175C688E2"]</t>
+          <t>["CAND-C8B00F2B86A8B7AF7549A783"]</t>
         </is>
       </c>
       <c r="AR10" s="22" t="inlineStr">
@@ -8491,12 +8491,12 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SCN-68E82895D5D2754159603420</t>
+          <t>SCN-268144CE4DBE7F2E116E140E</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -8658,12 +8658,12 @@
       </c>
       <c r="AP11" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-2132EFA0CCC25A00B16EA2CF","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"READY","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-807.02,"high":0.0,"low":-1614.05},"dbu":{"base":-5400.0,"high":0.0,"low":-10800.0},"total":{"base":-6207.02,"high":0.0,"low":-12414.05}}},"recommended_value":3,"step":1,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-INCREASE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":2,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-6B2DDE23EC751D22DE4F7914","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"READY","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-807.02,"high":0.0,"low":-1614.05},"dbu":{"base":-5400.0,"high":0.0,"low":-10800.0},"total":{"base":-6207.02,"high":0.0,"low":-12414.05}}},"recommended_value":3,"step":1,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-INCREASE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":2,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ11" s="22" t="inlineStr">
         <is>
-          <t>["CAND-2132EFA0CCC25A00B16EA2CF"]</t>
+          <t>["CAND-6B2DDE23EC751D22DE4F7914"]</t>
         </is>
       </c>
       <c r="AR11" s="22" t="inlineStr">
@@ -8680,12 +8680,12 @@
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SCN-EC35EE7A8A459E1030386BDF</t>
+          <t>SCN-7541A4581D52616B7887204B</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -8847,12 +8847,12 @@
       </c>
       <c r="AP12" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-A64CA3E68A669D150AAA07D6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5380.16,"high":5380.16,"low":5380.16},"dbu":{"base":23929.13,"high":27952.76,"low":19905.51},"total":{"base":29309.29,"high":33332.92,"low":25285.67}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-05E76611FED4F59744C22AB8","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5380.16,"high":5380.16,"low":5380.16},"dbu":{"base":23929.13,"high":27952.76,"low":19905.51},"total":{"base":29309.29,"high":33332.92,"low":25285.67}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ12" s="22" t="inlineStr">
         <is>
-          <t>["CAND-A64CA3E68A669D150AAA07D6"]</t>
+          <t>["CAND-05E76611FED4F59744C22AB8"]</t>
         </is>
       </c>
       <c r="AR12" s="22" t="inlineStr">
@@ -8869,12 +8869,12 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SCN-819DAEDF07A8F0192D7A247C</t>
+          <t>SCN-434C077126B079E5142CDF8C</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -9030,12 +9030,12 @@
       </c>
       <c r="AP13" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-AB3963A519CBBB85D39C5C32","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-04FD915BC6811A9ABF866B65","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-BA05FACF1A2AF701F6188BBC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-4701F5AB0B552D8BE3E4E34C","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1976.43,"high":2541.12,"low":1270.56},"dbu":{"base":2400.0,"high":4800.0,"low":-600.0},"total":{"base":4376.43,"high":7341.12,"low":670.56}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ13" s="22" t="inlineStr">
         <is>
-          <t>["CAND-AB3963A519CBBB85D39C5C32","CAND-04FD915BC6811A9ABF866B65"]</t>
+          <t>["CAND-BA05FACF1A2AF701F6188BBC","CAND-4701F5AB0B552D8BE3E4E34C"]</t>
         </is>
       </c>
       <c r="AR13" s="22" t="inlineStr">
@@ -9052,12 +9052,12 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SCN-0C81CFCDAF78B26D6BFDAC1D</t>
+          <t>SCN-46131C6A05E4B40940D8714B</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -9219,12 +9219,12 @@
       </c>
       <c r="AP14" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-DBDB7630ED062E15E33B2B7A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5646.94,"high":5646.94,"low":5646.94},"dbu":{"base":5330.58,"high":9553.72,"low":1107.44},"total":{"base":10977.52,"high":15200.66,"low":6754.38}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-2F116D492B169CDC7BFE4A4F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5646.94,"high":5646.94,"low":5646.94},"dbu":{"base":5330.58,"high":9553.72,"low":1107.44},"total":{"base":10977.52,"high":15200.66,"low":6754.38}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ14" s="22" t="inlineStr">
         <is>
-          <t>["CAND-DBDB7630ED062E15E33B2B7A"]</t>
+          <t>["CAND-2F116D492B169CDC7BFE4A4F"]</t>
         </is>
       </c>
       <c r="AR14" s="22" t="inlineStr">
@@ -9241,12 +9241,12 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SCN-FFA03F647640FAFA848CFDF5</t>
+          <t>SCN-C3C9758E12BA36251A7A8421</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -9402,12 +9402,12 @@
       </c>
       <c r="AP15" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-91BB40F77CB18835E431CCE6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-9B652249BD980BF64F75C35A","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":2,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-912302CE7FA8ECEADF68A266","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":5379.0,"high":6659.65,"low":3674.79},"dbu":{"base":8731.0,"high":14500.0,"low":1054.0},"total":{"base":14110.0,"high":21159.65,"low":4728.79}}},"recommended_value":15,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-5021E6E6585A4FEE342CB4BB","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-3CDD1DCF71D56AF9C3F59C6F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":3,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":3862.6,"high":4661.76,"low":2663.86},"dbu":{"base":1900.0,"high":5500.0,"low":-3500.0},"total":{"base":5762.6,"high":10161.76,"low":-836.14}}},"recommended_value":2,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-1CDA6A7761D3E39DAA39959D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":5379.0,"high":6659.65,"low":3674.79},"dbu":{"base":8731.0,"high":14500.0,"low":1054.0},"total":{"base":14110.0,"high":21159.65,"low":4728.79}}},"recommended_value":15,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ15" s="22" t="inlineStr">
         <is>
-          <t>["CAND-91BB40F77CB18835E431CCE6","CAND-9B652249BD980BF64F75C35A","CAND-912302CE7FA8ECEADF68A266"]</t>
+          <t>["CAND-5021E6E6585A4FEE342CB4BB","CAND-3CDD1DCF71D56AF9C3F59C6F","CAND-1CDA6A7761D3E39DAA39959D"]</t>
         </is>
       </c>
       <c r="AR15" s="22" t="inlineStr">
@@ -9424,12 +9424,12 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SCN-B9518765A9CBB3B850E61ABC</t>
+          <t>SCN-582CD070FCA0E22EFE63E1A6</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -9591,12 +9591,12 @@
       </c>
       <c r="AP16" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-2CBB771D8661A0443D52D973","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6659.65,"high":6659.65,"low":6659.65},"dbu":{"base":-441.52,"high":-441.52,"low":-441.52},"total":{"base":6218.13,"high":6218.13,"low":6218.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-1FAD9418FB980278274923BD","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":6659.65,"high":6659.65,"low":6659.65},"dbu":{"base":-441.52,"high":-441.52,"low":-441.52},"total":{"base":6218.13,"high":6218.13,"low":6218.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ16" s="22" t="inlineStr">
         <is>
-          <t>["CAND-2CBB771D8661A0443D52D973"]</t>
+          <t>["CAND-1FAD9418FB980278274923BD"]</t>
         </is>
       </c>
       <c r="AR16" s="22" t="inlineStr">
@@ -9613,12 +9613,12 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>SCN-DFF0F7B21E7E59997E295C89</t>
+          <t>SCN-0AC9FD46A1C9A180B84B6313</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -9804,12 +9804,12 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>SCN-271D4A0780CD3BBEC0341F84</t>
+          <t>SCN-81FA38FBB36266F1B735E002</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -9995,12 +9995,12 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>SCN-25C50A8B284AD6025A2723EA</t>
+          <t>SCN-69D437D3D8FDDFE6F953315B</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -10156,12 +10156,12 @@
       </c>
       <c r="AP19" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-EDB08C1E32CD5DFD2B45A9F1","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-064DD3A175BE92BD9C658F7C","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":10,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":5,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-0B53B1CF89A1FF45576E8ACD","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-F867AC6F987F34C1567B71E4","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":10,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":0.0,"high":0.0,"low":0.0},"dbu":{"base":18200.0,"high":23400.0,"low":11700.0},"total":{"base":18200.0,"high":23400.0,"low":11700.0}}},"recommended_value":5,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ19" s="22" t="inlineStr">
         <is>
-          <t>["CAND-EDB08C1E32CD5DFD2B45A9F1","CAND-064DD3A175BE92BD9C658F7C"]</t>
+          <t>["CAND-0B53B1CF89A1FF45576E8ACD","CAND-F867AC6F987F34C1567B71E4"]</t>
         </is>
       </c>
       <c r="AR19" s="22" t="inlineStr">
@@ -10178,12 +10178,12 @@
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>SCN-BF14FB572683C696D02CD7EA</t>
+          <t>SCN-27D656892CFF54E7DE80A40B</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
@@ -10345,12 +10345,12 @@
       </c>
       <c r="AP20" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-1F3EBDB3DFBB20D0B1CD4658","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SERVERLESS","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-9482.94,"high":-2709.41,"low":-10837.65},"dbu":{"base":-16386.62,"high":32460.97,"low":-26156.13},"total":{"base":-25869.56,"high":29751.56,"low":-36993.78}}},"recommended_value":"PRO","step":2,"step_type":"CANDIDATE","technique_id":"WH-PRO-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-09EB817A3591B59B95A5BDA5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SERVERLESS","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-9482.94,"high":-2709.41,"low":-10837.65},"dbu":{"base":-16386.62,"high":32460.97,"low":-26156.13},"total":{"base":-25869.56,"high":29751.56,"low":-36993.78}}},"recommended_value":"PRO","step":2,"step_type":"CANDIDATE","technique_id":"WH-PRO-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ20" s="22" t="inlineStr">
         <is>
-          <t>["CAND-1F3EBDB3DFBB20D0B1CD4658"]</t>
+          <t>["CAND-09EB817A3591B59B95A5BDA5"]</t>
         </is>
       </c>
       <c r="AR20" s="22" t="inlineStr">
@@ -10367,12 +10367,12 @@
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>SCN-7999EC8BC5B2A2F2A072C81B</t>
+          <t>SCN-2CC0626945850CA914D1FE52</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -10528,12 +10528,12 @@
       </c>
       <c r="AP21" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-51124DC4FB8ADD3865AA63DB","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-A61DE0B24632CFBA54001A80","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-9D796F49F0E013A31CC9883D","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-577A4357DFAC3AC2FC120CCC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":4,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1920.87,"high":2469.69,"low":1234.84},"dbu":{"base":5050.58,"high":6888.95,"low":2752.62},"total":{"base":6971.45,"high":9358.64,"low":3987.46}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ21" s="22" t="inlineStr">
         <is>
-          <t>["CAND-51124DC4FB8ADD3865AA63DB","CAND-A61DE0B24632CFBA54001A80"]</t>
+          <t>["CAND-9D796F49F0E013A31CC9883D","CAND-577A4357DFAC3AC2FC120CCC"]</t>
         </is>
       </c>
       <c r="AR21" s="22" t="inlineStr">
@@ -10550,12 +10550,12 @@
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>SCN-2CF9865BFB2C9E9FFFB1F087</t>
+          <t>SCN-1A607722905F5626F2592F39</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -10717,12 +10717,12 @@
       </c>
       <c r="AP22" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-FF15B75DF3EB05354881F56F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5488.19,"high":5488.19,"low":5488.19},"dbu":{"base":4686.75,"high":8791.16,"low":582.33},"total":{"base":10174.94,"high":14279.35,"low":6070.52}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-113EE95F32D6329E0F3A4C61","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5488.19,"high":5488.19,"low":5488.19},"dbu":{"base":4686.75,"high":8791.16,"low":582.33},"total":{"base":10174.94,"high":14279.35,"low":6070.52}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ22" s="22" t="inlineStr">
         <is>
-          <t>["CAND-FF15B75DF3EB05354881F56F"]</t>
+          <t>["CAND-113EE95F32D6329E0F3A4C61"]</t>
         </is>
       </c>
       <c r="AR22" s="22" t="inlineStr">
@@ -10739,12 +10739,12 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>SCN-6034F47F88FE870BCBD38A83</t>
+          <t>SCN-AC27CF4B8FF664CD14E343AA</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -10900,12 +10900,12 @@
       </c>
       <c r="AP23" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-0E877A6745803DC5EB83DB93","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-15068.09,"high":0.0,"low":-37670.23},"dbu":{"base":-23200.0,"high":0.0,"low":-58000.0},"total":{"base":-38268.09,"high":0.0,"low":-95670.23}}},"recommended_value":"X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-497F0500B2853FDB8B49F0E2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":45,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13565.92,"high":2002.9,"low":-36668.78},"dbu":{"base":-20887.14,"high":3083.82,"low":-56458.09},"total":{"base":-34453.06,"high":5086.72,"low":-93126.87}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-B6EB43F303C4E8EE0A6DFB03","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":-15068.09,"high":0.0,"low":-37670.23},"dbu":{"base":-23200.0,"high":0.0,"low":-58000.0},"total":{"base":-38268.09,"high":0.0,"low":-95670.23}}},"recommended_value":"X_LARGE","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-UPSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":[],"validation_type":"NONE"}},{"action":null,"candidate_id":"CAND-347FA9E6410390B0FEC735D0","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":45,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":-13565.92,"high":2002.9,"low":-36668.78},"dbu":{"base":-20887.14,"high":3083.82,"low":-56458.09},"total":{"base":-34453.06,"high":5086.72,"low":-93126.87}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ23" s="22" t="inlineStr">
         <is>
-          <t>["CAND-0E877A6745803DC5EB83DB93","CAND-497F0500B2853FDB8B49F0E2"]</t>
+          <t>["CAND-B6EB43F303C4E8EE0A6DFB03","CAND-347FA9E6410390B0FEC735D0"]</t>
         </is>
       </c>
       <c r="AR23" s="22" t="inlineStr">
@@ -10922,12 +10922,12 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>SCN-60E6E4CF8B3C2E2611EA9BFA</t>
+          <t>SCN-7DA4C286CAFA46529A941D00</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -11089,12 +11089,12 @@
       </c>
       <c r="AP24" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-3588FD08E2C2D20AB63356BE","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":37670.23,"high":37670.23,"low":37670.23},"dbu":{"base":-26516.54,"high":44997.46,"low":-33017.81},"total":{"base":11153.69,"high":82667.69,"low":4652.42}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-EDC5DB36F0D1AC83E7D2D87F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":37670.23,"high":37670.23,"low":37670.23},"dbu":{"base":-26516.54,"high":44997.46,"low":-33017.81},"total":{"base":11153.69,"high":82667.69,"low":4652.42}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ24" s="22" t="inlineStr">
         <is>
-          <t>["CAND-3588FD08E2C2D20AB63356BE"]</t>
+          <t>["CAND-EDC5DB36F0D1AC83E7D2D87F"]</t>
         </is>
       </c>
       <c r="AR24" s="22" t="inlineStr">
@@ -11111,12 +11111,12 @@
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>SCN-F8D0AE11F3CFA07D7DFBD032</t>
+          <t>SCN-578A1D1819D737E19D5DEDBE</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -11272,12 +11272,12 @@
       </c>
       <c r="AP25" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-7ADCC0E72B9FC08857017FB5","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1265.33,"high":1626.86,"low":813.43},"dbu":{"base":5425.0,"high":6975.0,"low":3487.5},"total":{"base":6690.33,"high":8601.86,"low":4300.93}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-76FF89D1C033A3CA62741ACF","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1672.05,"high":2440.29,"low":813.43},"dbu":{"base":7168.75,"high":10462.5,"low":3487.5},"total":{"base":8840.8,"high":12902.79,"low":4300.93}}},"recommended_value":1,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-5763B8095F259B3EEED222B0","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1940.48,"high":2798.2,"low":992.38},"dbu":{"base":8319.62,"high":11997.0,"low":4254.75},"total":{"base":10260.1,"high":14795.2,"low":5247.13}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-4C2622B3D4EF1E9ED54322C7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1265.33,"high":1626.86,"low":813.43},"dbu":{"base":5425.0,"high":6975.0,"low":3487.5},"total":{"base":6690.33,"high":8601.86,"low":4300.93}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-016EDFB75AF0AF6A2C07E315","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":2,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"},{"condition":null,"dependency_type":"KNOB","ref_id":"max_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":["auto_stop_minutes"],"knob":"min_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1672.05,"high":2440.29,"low":813.43},"dbu":{"base":7168.75,"high":10462.5,"low":3487.5},"total":{"base":8840.8,"high":12902.79,"low":4300.93}}},"recommended_value":1,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MIN-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-4C891B8A1136F219041C9F4E","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":120,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1940.48,"high":2798.2,"low":992.38},"dbu":{"base":8319.62,"high":11997.0,"low":4254.75},"total":{"base":10260.1,"high":14795.2,"low":5247.13}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ25" s="22" t="inlineStr">
         <is>
-          <t>["CAND-7ADCC0E72B9FC08857017FB5","CAND-76FF89D1C033A3CA62741ACF","CAND-5763B8095F259B3EEED222B0"]</t>
+          <t>["CAND-4C2622B3D4EF1E9ED54322C7","CAND-016EDFB75AF0AF6A2C07E315","CAND-4C891B8A1136F219041C9F4E"]</t>
         </is>
       </c>
       <c r="AR25" s="22" t="inlineStr">
@@ -11294,12 +11294,12 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>SCN-80FA6497D1269DF9BC6CDAC9</t>
+          <t>SCN-D3A3FAD11AC31FEC9D1A2AB5</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -11461,12 +11461,12 @@
       </c>
       <c r="AP26" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-AC5879A21066084E08E49997","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3615.24,"high":3615.24,"low":3615.24},"dbu":{"base":7388.89,"high":11444.44,"low":7388.89},"total":{"base":11004.13,"high":15059.68,"low":11004.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-C1507494ED1BA885FBF9071F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3615.24,"high":3615.24,"low":3615.24},"dbu":{"base":7388.89,"high":11444.44,"low":7388.89},"total":{"base":11004.13,"high":15059.68,"low":11004.13}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ26" s="22" t="inlineStr">
         <is>
-          <t>["CAND-AC5879A21066084E08E49997"]</t>
+          <t>["CAND-C1507494ED1BA885FBF9071F"]</t>
         </is>
       </c>
       <c r="AR26" s="22" t="inlineStr">
@@ -11483,12 +11483,12 @@
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>SCN-6AF109497D3D72C350D1DB24</t>
+          <t>SCN-523803CD1056F839B5F4CF5A</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -11644,12 +11644,12 @@
       </c>
       <c r="AP27" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-CD04AB68BD52CC1E1EB78D67","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-4D1C8BB67AC3293C91608AA1","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":8,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-0E0C39CCFED2B26094B35BC6","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"MEDIUM","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":"SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-16C467F705AC450DD5FB6F3F","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":8,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1868.34,"high":2402.15,"low":1201.08},"dbu":{"base":7724.42,"high":10536.05,"low":4209.88},"total":{"base":9592.76,"high":12938.2,"low":5410.96}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ27" s="22" t="inlineStr">
         <is>
-          <t>["CAND-CD04AB68BD52CC1E1EB78D67","CAND-4D1C8BB67AC3293C91608AA1"]</t>
+          <t>["CAND-0E0C39CCFED2B26094B35BC6","CAND-16C467F705AC450DD5FB6F3F"]</t>
         </is>
       </c>
       <c r="AR27" s="22" t="inlineStr">
@@ -11666,12 +11666,12 @@
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>SCN-1A718415E777F8AF64EDE335</t>
+          <t>SCN-79199C03A3C215D8409EAD4B</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
@@ -11833,12 +11833,12 @@
       </c>
       <c r="AP28" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-8DAE20517B39B4C87C5DB0F9","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5338.12,"high":5338.12,"low":5338.12},"dbu":{"base":14023.44,"high":18015.63,"low":10031.25},"total":{"base":19361.56,"high":23353.75,"low":15369.37}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-3533B4E4348CE8BBC3CD27A3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":5338.12,"high":5338.12,"low":5338.12},"dbu":{"base":14023.44,"high":18015.63,"low":10031.25},"total":{"base":19361.56,"high":23353.75,"low":15369.37}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ28" s="22" t="inlineStr">
         <is>
-          <t>["CAND-8DAE20517B39B4C87C5DB0F9"]</t>
+          <t>["CAND-3533B4E4348CE8BBC3CD27A3"]</t>
         </is>
       </c>
       <c r="AR28" s="22" t="inlineStr">
@@ -11855,12 +11855,12 @@
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>SCN-3C4F23823E7323060F7D590E</t>
+          <t>SCN-66A9ACF16F67715AEDE3DD1E</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -12016,12 +12016,12 @@
       </c>
       <c r="AP29" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-CB50137D13AA86B1380E9225","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1026.39,"high":1319.64,"low":659.82},"dbu":{"base":7350.0,"high":9450.0,"low":4725.0},"total":{"base":8376.39,"high":10769.64,"low":5384.82}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-ACD999430C8A059DFB38EBAC","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1158.35,"high":1495.59,"low":747.8},"dbu":{"base":8295.0,"high":10710.0,"low":5355.0},"total":{"base":9453.35,"high":12205.59,"low":6102.8}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-428D7886836325C1957B2FC7","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"SMALL","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1026.39,"high":1319.64,"low":659.82},"dbu":{"base":7350.0,"high":9450.0,"low":4725.0},"total":{"base":8376.39,"high":10769.64,"low":5384.82}}},"recommended_value":"X_SMALL","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-6B0ACEABD2495B5A3B07846B","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1158.35,"high":1495.59,"low":747.8},"dbu":{"base":8295.0,"high":10710.0,"low":5355.0},"total":{"base":9453.35,"high":12205.59,"low":6102.8}}},"recommended_value":30,"step":2,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ29" s="22" t="inlineStr">
         <is>
-          <t>["CAND-CB50137D13AA86B1380E9225","CAND-ACD999430C8A059DFB38EBAC"]</t>
+          <t>["CAND-428D7886836325C1957B2FC7","CAND-6B0ACEABD2495B5A3B07846B"]</t>
         </is>
       </c>
       <c r="AR29" s="22" t="inlineStr">
@@ -12038,12 +12038,12 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>SCN-1B5457B19E85EA205F9057D6</t>
+          <t>SCN-EEA1172BA764560AD0C5776C</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -12205,12 +12205,12 @@
       </c>
       <c r="AP30" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-32DF6FED0478FEF9963854FF","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":2932.53,"high":2932.53,"low":2932.53},"dbu":{"base":14420.6,"high":16613.73,"low":12227.47},"total":{"base":17353.13,"high":19546.26,"low":15160.0}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-B9A432AC45556AC42F2CDE81","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":2932.53,"high":2932.53,"low":2932.53},"dbu":{"base":14420.6,"high":16613.73,"low":12227.47},"total":{"base":17353.13,"high":19546.26,"low":15160.0}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ30" s="22" t="inlineStr">
         <is>
-          <t>["CAND-32DF6FED0478FEF9963854FF"]</t>
+          <t>["CAND-B9A432AC45556AC42F2CDE81"]</t>
         </is>
       </c>
       <c r="AR30" s="22" t="inlineStr">
@@ -12227,12 +12227,12 @@
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>PKG-02C2A3390BC1C4114197FDAD</t>
+          <t>PKG-664E535A61AEB69185D775A9</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>SCN-8FDC6E54EE7012064F9C9683</t>
+          <t>SCN-43F5B63431477AC470A9522A</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -12418,12 +12418,12 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>PKG-02C2A3390BC1C4114197FDAD</t>
+          <t>PKG-664E535A61AEB69185D775A9</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>SCN-39CB4EC90BE02170DAA80379</t>
+          <t>SCN-EB5A1A4A95D402FF8562792C</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -12585,12 +12585,12 @@
       </c>
       <c r="AP32" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.731},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-FF6F464540547619819C2285","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":0.09,"signal":1.0,"stability":0.725},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.731},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3733.77,"high":3733.77,"low":3733.77},"dbu":{"base":-5177.05,"high":-5177.05,"low":-5177.05},"total":{"base":-1443.28,"high":-1443.28,"low":-1443.28}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.731},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-E1F56BF222EF5FFED707D9C3","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":0.09,"signal":1.0,"stability":0.725},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.731},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":3733.77,"high":3733.77,"low":3733.77},"dbu":{"base":-5177.05,"high":-5177.05,"low":-5177.05},"total":{"base":-1443.28,"high":-1443.28,"low":-1443.28}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ32" s="22" t="inlineStr">
         <is>
-          <t>["CAND-FF6F464540547619819C2285"]</t>
+          <t>["CAND-E1F56BF222EF5FFED707D9C3"]</t>
         </is>
       </c>
       <c r="AR32" s="22" t="inlineStr">
@@ -12607,12 +12607,12 @@
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>PKG-AAD2A5F749FD290F3138AB5C</t>
+          <t>PKG-12310EDCE7FFCF9E8111114F</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>SCN-8347382151702D72FD4C7016</t>
+          <t>SCN-F21183EC4EC78A0BBDAE0EBC</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -12768,12 +12768,12 @@
       </c>
       <c r="AP33" s="22" t="inlineStr">
         <is>
-          <t>[{"action":null,"candidate_id":"CAND-FD0EB76CB7D1BCCA6922F667","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-7B6686612C0DD9AC7B23D9D2","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":5,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-B655DB77EFCC30A1DD7E127C","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":2409.51,"high":3623.05,"low":932.15},"dbu":{"base":-4016.37,"high":3019.8,"low":-12582.14},"total":{"base":-1606.86,"high":6642.85,"low":-11649.99}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":null,"candidate_id":"CAND-58C1DDD819272E9FEE9074A9","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"LARGE","dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_channel"}],"execution_state":"READY_FOR_CANARY","invalidates":["max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_size","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":"MEDIUM","step":1,"step_type":"CANDIDATE","technique_id":"WH-SIZE-DOWNSIZE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-79A6AA57196043E2E050C701","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":5,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"warehouse_size"}],"execution_state":"PENDING_REEVALUATION","invalidates":["min_clusters"],"knob":"max_clusters","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":1934.64,"high":2989.9,"low":615.57},"dbu":{"base":-6769.65,"high":-651.24,"low":-14417.66},"total":{"base":-4835.01,"high":2338.66,"low":-13802.09}}},"recommended_value":3,"step":2,"step_type":"CANDIDATE","technique_id":"WH-MAX-CLUSTER-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":null,"candidate_id":"CAND-B127AE44291FA0B54762C906","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"HIGH","method":"deterministic_evidence_score","score":0.93},"current_value":60,"dependencies":[{"condition":null,"dependency_type":"KNOB","ref_id":"min_clusters"}],"execution_state":"PENDING_REEVALUATION","invalidates":[],"knob":"auto_stop_minutes","projected_economics":{"pricing_basis":"CONTINGENT_PENDING_REEVALUATION","running_savings_365d":{"aws":{"base":2409.51,"high":3623.05,"low":932.15},"dbu":{"base":-4016.37,"high":3019.8,"low":-12582.14},"total":{"base":-1606.86,"high":6642.85,"low":-11649.99}}},"recommended_value":30,"step":3,"step_type":"CANDIDATE","technique_id":"WH-AUTOSTOP-REDUCE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":4,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ33" s="22" t="inlineStr">
         <is>
-          <t>["CAND-FD0EB76CB7D1BCCA6922F667","CAND-7B6686612C0DD9AC7B23D9D2","CAND-B655DB77EFCC30A1DD7E127C"]</t>
+          <t>["CAND-58C1DDD819272E9FEE9074A9","CAND-79A6AA57196043E2E050C701","CAND-B127AE44291FA0B54762C906"]</t>
         </is>
       </c>
       <c r="AR33" s="22" t="inlineStr">
@@ -12790,12 +12790,12 @@
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>PKG-AAD2A5F749FD290F3138AB5C</t>
+          <t>PKG-12310EDCE7FFCF9E8111114F</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>SCN-2AA83F694744EABD32EBFDC8</t>
+          <t>SCN-0D507F5621CB3870A7FD7BE3</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -12957,12 +12957,12 @@
       </c>
       <c r="AP34" s="22" t="inlineStr">
         <is>
-          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-AE90A6A42FD1F94FB256D883","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":8793.82,"high":8793.82,"low":8793.82},"dbu":{"base":13270.27,"high":19846.85,"low":6693.69},"total":{"base":22064.09,"high":28640.67,"low":15487.51}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
+          <t>[{"action":"VALIDATE_WAREHOUSE_TYPE_COMPATIBILITY","candidate_id":null,"confidence":{"components":{},"level":"MEDIUM","method":"compatibility_and_scenario_evidence","score":0.78},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":1,"step_type":"COMPATIBILITY_VALIDATION","technique_id":null,"validation":{"action_after":"CONTINUE_IF_PASS","remeasure_days":null,"success_metrics":[],"validation_type":"COMPATIBILITY"}},{"action":null,"candidate_id":"CAND-AD7E7D9A3D0FF3226E9F1282","confidence":{"components":{"coverage":1.0,"epoch_maturity":1.0,"sample":1.0,"signal":1.0,"stability":0.91},"level":"MEDIUM","method":"deterministic_evidence_score","score":0.78},"current_value":"PRO","dependencies":[],"execution_state":"READY_FOR_CANARY","invalidates":["warehouse_size","max_clusters","min_clusters","auto_stop_minutes"],"knob":"warehouse_type","projected_economics":{"pricing_basis":"AUTHORITATIVE","running_savings_365d":{"aws":{"base":8793.82,"high":8793.82,"low":8793.82},"dbu":{"base":13270.27,"high":19846.85,"low":6693.69},"total":{"base":22064.09,"high":28640.67,"low":15487.51}}},"recommended_value":"SERVERLESS","step":2,"step_type":"CANDIDATE","technique_id":"WH-SERVERLESS-MIGRATE-001","validation":{"action_after":null,"remeasure_days":null,"success_metrics":["p95_execution_ms","p99_execution_ms","failure_rate","queue_wait","dbu_cost","aws_cost"],"validation_type":"A_B_CANARY"}},{"action":"REMEASURE_AND_REGENERATE","candidate_id":null,"confidence":{"components":{"policy_gate":1.0},"level":"HIGH","method":"policy_gate","score":1.0},"current_value":null,"dependencies":[],"execution_state":"REQUIRED","invalidates":[],"knob":null,"projected_economics":null,"recommended_value":null,"step":3,"step_type":"REMEASURE","technique_id":null,"validation":{"action_after":"REGENERATE_RECOMMENDATIONS","remeasure_days":7,"success_metrics":[],"validation_type":"REMEASURE"}}]</t>
         </is>
       </c>
       <c r="AQ34" s="22" t="inlineStr">
         <is>
-          <t>["CAND-AE90A6A42FD1F94FB256D883"]</t>
+          <t>["CAND-AD7E7D9A3D0FF3226E9F1282"]</t>
         </is>
       </c>
       <c r="AR34" s="22" t="inlineStr">
@@ -13710,12 +13710,12 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>CAND-7766A2738B430E52A7885D34</t>
+          <t>CAND-30CABA362591DD08BBD7EEFF</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -13899,12 +13899,12 @@
       </c>
       <c r="AT5" s="22" t="inlineStr">
         <is>
-          <t>["EVID-D31130A3622EA96577F699ED","EVID-E2BFCCA76EB8534DA44771CC","EVID-BC460C11441EEA3635B6CEF6","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
+          <t>["EVID-D31130A3622EA96577F699ED","EVID-E2BFCCA76EB8534DA44771CC","EVID-609ECEA12D01A7D7EE1FB3B0","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
         </is>
       </c>
       <c r="AU5" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-BC460C11441EEA3635B6CEF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC460C11441EEA3635B6CEF6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-D31130A3622EA96577F699ED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D31130A3622EA96577F699ED","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0}}</t>
+          <t>{"EVID-609ECEA12D01A7D7EE1FB3B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-609ECEA12D01A7D7EE1FB3B0","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":27000.0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-D31130A3622EA96577F699ED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D31130A3622EA96577F699ED","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0}}</t>
         </is>
       </c>
       <c r="AV5" s="22" t="inlineStr">
@@ -13941,12 +13941,12 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>CAND-EE57C678D7321484C82E7EC4</t>
+          <t>CAND-19BB082E74D6C1E39FFF482D</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -14130,12 +14130,12 @@
       </c>
       <c r="AT6" s="22" t="inlineStr">
         <is>
-          <t>["EVID-CE1E8D70F4C1F4F7211BEBB2","EVID-AD5C166A82B775E709ABF751","EVID-581184092AAF568D86DE312B","EVID-C3D2E64A89DE473CEF3F10A8","EVID-FCFFAB99D6FF292E4BC8DC8F","EVID-249028FA99BFDEE68A2645DB","EVID-43A874D251CBC13D278C1E5F","EVID-23834E1D614A63BF7B745F8B","EVID-FE30CB96733BF18D9469D45B","EVID-E2BFCCA76EB8534DA44771CC","EVID-BC460C11441EEA3635B6CEF6","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
+          <t>["EVID-CE1E8D70F4C1F4F7211BEBB2","EVID-AD5C166A82B775E709ABF751","EVID-581184092AAF568D86DE312B","EVID-C3D2E64A89DE473CEF3F10A8","EVID-FCFFAB99D6FF292E4BC8DC8F","EVID-249028FA99BFDEE68A2645DB","EVID-43A874D251CBC13D278C1E5F","EVID-23834E1D614A63BF7B745F8B","EVID-FE30CB96733BF18D9469D45B","EVID-E2BFCCA76EB8534DA44771CC","EVID-609ECEA12D01A7D7EE1FB3B0","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
         </is>
       </c>
       <c r="AU6" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-23834E1D614A63BF7B745F8B":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-23834E1D614A63BF7B745F8B","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":10000},"EVID-249028FA99BFDEE68A2645DB":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-249028FA99BFDEE68A2645DB","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-43A874D251CBC13D278C1E5F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-43A874D251CBC13D278C1E5F","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2500},"EVID-581184092AAF568D86DE312B":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-581184092AAF568D86DE312B","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-AD5C166A82B775E709ABF751":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-AD5C166A82B775E709ABF751","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-BC460C11441EEA3635B6CEF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC460C11441EEA3635B6CEF6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-C3D2E64A89DE473CEF3F10A8":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-C3D2E64A89DE473CEF3F10A8","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-CE1E8D70F4C1F4F7211BEBB2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CE1E8D70F4C1F4F7211BEBB2","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-FCFFAB99D6FF292E4BC8DC8F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FCFFAB99D6FF292E4BC8DC8F","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-FE30CB96733BF18D9469D45B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FE30CB96733BF18D9469D45B","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0}}</t>
+          <t>{"EVID-23834E1D614A63BF7B745F8B":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-23834E1D614A63BF7B745F8B","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":10000},"EVID-249028FA99BFDEE68A2645DB":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-249028FA99BFDEE68A2645DB","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-43A874D251CBC13D278C1E5F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-43A874D251CBC13D278C1E5F","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2500},"EVID-581184092AAF568D86DE312B":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-581184092AAF568D86DE312B","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-609ECEA12D01A7D7EE1FB3B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-609ECEA12D01A7D7EE1FB3B0","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":27000.0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-AD5C166A82B775E709ABF751":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-AD5C166A82B775E709ABF751","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-C3D2E64A89DE473CEF3F10A8":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-C3D2E64A89DE473CEF3F10A8","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-CE1E8D70F4C1F4F7211BEBB2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CE1E8D70F4C1F4F7211BEBB2","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-FCFFAB99D6FF292E4BC8DC8F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FCFFAB99D6FF292E4BC8DC8F","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-FE30CB96733BF18D9469D45B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FE30CB96733BF18D9469D45B","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0}}</t>
         </is>
       </c>
       <c r="AV6" s="22" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="AZ6" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-863D86733C17ECB8516EF093","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-0F323C820C480A6DB359983B","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA6" s="22" t="inlineStr">
@@ -14172,12 +14172,12 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>CAND-7C972C46E6BADA6422EF650F</t>
+          <t>CAND-FACB02F992DE84FD0C6488B6</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -14357,12 +14357,12 @@
       </c>
       <c r="AT7" s="22" t="inlineStr">
         <is>
-          <t>["EVID-02C377DDCAB735229EEC24A6","EVID-25CAE9179FEBB6FA2D425213","EVID-2C2557D4DA122C44D293B116","EVID-3FA53CA4EC8C609E6C60F9CF","EVID-A10762D366E7024D1873F50A","EVID-05ABEF123F82DD14B9089E15","EVID-E2BFCCA76EB8534DA44771CC","EVID-BC460C11441EEA3635B6CEF6","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
+          <t>["EVID-02C377DDCAB735229EEC24A6","EVID-25CAE9179FEBB6FA2D425213","EVID-2C2557D4DA122C44D293B116","EVID-3FA53CA4EC8C609E6C60F9CF","EVID-A10762D366E7024D1873F50A","EVID-05ABEF123F82DD14B9089E15","EVID-E2BFCCA76EB8534DA44771CC","EVID-609ECEA12D01A7D7EE1FB3B0","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
         </is>
       </c>
       <c r="AU7" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-02C377DDCAB735229EEC24A6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-02C377DDCAB735229EEC24A6","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-05ABEF123F82DD14B9089E15":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-05ABEF123F82DD14B9089E15","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-25CAE9179FEBB6FA2D425213":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-25CAE9179FEBB6FA2D425213","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-2C2557D4DA122C44D293B116":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-2C2557D4DA122C44D293B116","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-3FA53CA4EC8C609E6C60F9CF":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-3FA53CA4EC8C609E6C60F9CF","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A10762D366E7024D1873F50A":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-A10762D366E7024D1873F50A","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-BC460C11441EEA3635B6CEF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC460C11441EEA3635B6CEF6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0}}</t>
+          <t>{"EVID-02C377DDCAB735229EEC24A6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-02C377DDCAB735229EEC24A6","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-05ABEF123F82DD14B9089E15":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-05ABEF123F82DD14B9089E15","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-25CAE9179FEBB6FA2D425213":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-25CAE9179FEBB6FA2D425213","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-2C2557D4DA122C44D293B116":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-2C2557D4DA122C44D293B116","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-3FA53CA4EC8C609E6C60F9CF":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-3FA53CA4EC8C609E6C60F9CF","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-609ECEA12D01A7D7EE1FB3B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-609ECEA12D01A7D7EE1FB3B0","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":27000.0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A10762D366E7024D1873F50A":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-A10762D366E7024D1873F50A","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0}}</t>
         </is>
       </c>
       <c r="AV7" s="22" t="inlineStr">
@@ -14387,7 +14387,7 @@
       </c>
       <c r="AZ7" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-863D86733C17ECB8516EF093","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-0F323C820C480A6DB359983B","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA7" s="22" t="inlineStr">
@@ -14399,12 +14399,12 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>CAND-759D0E09D0D3D1DF01FBBA2B</t>
+          <t>CAND-F52C33A9DDA0277D8F79D9E6</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -14584,12 +14584,12 @@
       </c>
       <c r="AT8" s="22" t="inlineStr">
         <is>
-          <t>["EVID-E6FDF0DED766BE36DBCF9B85","EVID-619414E4B31300D140BA8FB0","EVID-36D1387C3DAB197C2F09456E","EVID-849F13DCD8F8A626942FED31","EVID-E172A6102448FF828423C618","EVID-E2BFCCA76EB8534DA44771CC","EVID-BC460C11441EEA3635B6CEF6","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
+          <t>["EVID-E6FDF0DED766BE36DBCF9B85","EVID-619414E4B31300D140BA8FB0","EVID-36D1387C3DAB197C2F09456E","EVID-849F13DCD8F8A626942FED31","EVID-E172A6102448FF828423C618","EVID-E2BFCCA76EB8534DA44771CC","EVID-609ECEA12D01A7D7EE1FB3B0","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
         </is>
       </c>
       <c r="AU8" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-36D1387C3DAB197C2F09456E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-36D1387C3DAB197C2F09456E","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-619414E4B31300D140BA8FB0":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-619414E4B31300D140BA8FB0","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":80.0},"EVID-849F13DCD8F8A626942FED31":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-849F13DCD8F8A626942FED31","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-BC460C11441EEA3635B6CEF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC460C11441EEA3635B6CEF6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-E172A6102448FF828423C618":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-E172A6102448FF828423C618","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-E6FDF0DED766BE36DBCF9B85":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E6FDF0DED766BE36DBCF9B85","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2}}</t>
+          <t>{"EVID-36D1387C3DAB197C2F09456E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-36D1387C3DAB197C2F09456E","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-609ECEA12D01A7D7EE1FB3B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-609ECEA12D01A7D7EE1FB3B0","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":27000.0},"EVID-619414E4B31300D140BA8FB0":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-619414E4B31300D140BA8FB0","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":80.0},"EVID-849F13DCD8F8A626942FED31":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-849F13DCD8F8A626942FED31","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-E172A6102448FF828423C618":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-E172A6102448FF828423C618","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-E6FDF0DED766BE36DBCF9B85":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E6FDF0DED766BE36DBCF9B85","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2}}</t>
         </is>
       </c>
       <c r="AV8" s="22" t="inlineStr">
@@ -14614,7 +14614,7 @@
       </c>
       <c r="AZ8" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-863D86733C17ECB8516EF093","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-0F323C820C480A6DB359983B","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA8" s="22" t="inlineStr">
@@ -14626,12 +14626,12 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>CAND-AF9E15C01CEAC8C1A0D722AB</t>
+          <t>CAND-8FB89535DFCD63C9A63BF39E</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -14811,12 +14811,12 @@
       </c>
       <c r="AT9" s="22" t="inlineStr">
         <is>
-          <t>["EVID-492656489A02189691212637","EVID-A260A94FAD60AB2B5B984E15","EVID-267BE325DB935326F0ECD0CA","EVID-8B432207CE81E1B5453FBA36","EVID-D0948F3BBDA2C1A885CCD2E8","EVID-C0024AE90132BFF522B946EA","EVID-0465D6B752AD0AB46330483B","EVID-1ACF5B01162FE1C9B407F0AA","EVID-E2BFCCA76EB8534DA44771CC","EVID-BC460C11441EEA3635B6CEF6","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
+          <t>["EVID-492656489A02189691212637","EVID-A260A94FAD60AB2B5B984E15","EVID-267BE325DB935326F0ECD0CA","EVID-8B432207CE81E1B5453FBA36","EVID-D0948F3BBDA2C1A885CCD2E8","EVID-C0024AE90132BFF522B946EA","EVID-0465D6B752AD0AB46330483B","EVID-1ACF5B01162FE1C9B407F0AA","EVID-E2BFCCA76EB8534DA44771CC","EVID-609ECEA12D01A7D7EE1FB3B0","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
         </is>
       </c>
       <c r="AU9" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0465D6B752AD0AB46330483B":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-0465D6B752AD0AB46330483B","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2667},"EVID-1ACF5B01162FE1C9B407F0AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1ACF5B01162FE1C9B407F0AA","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-267BE325DB935326F0ECD0CA":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-267BE325DB935326F0ECD0CA","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":480},"EVID-492656489A02189691212637":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-492656489A02189691212637","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-8B432207CE81E1B5453FBA36":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-8B432207CE81E1B5453FBA36","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":40000.0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A260A94FAD60AB2B5B984E15":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A260A94FAD60AB2B5B984E15","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":400.0},"EVID-BC460C11441EEA3635B6CEF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC460C11441EEA3635B6CEF6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-C0024AE90132BFF522B946EA":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-C0024AE90132BFF522B946EA","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-D0948F3BBDA2C1A885CCD2E8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D0948F3BBDA2C1A885CCD2E8","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":8},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0}}</t>
+          <t>{"EVID-0465D6B752AD0AB46330483B":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-0465D6B752AD0AB46330483B","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2667},"EVID-1ACF5B01162FE1C9B407F0AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1ACF5B01162FE1C9B407F0AA","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-267BE325DB935326F0ECD0CA":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-267BE325DB935326F0ECD0CA","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":480},"EVID-492656489A02189691212637":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-492656489A02189691212637","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-609ECEA12D01A7D7EE1FB3B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-609ECEA12D01A7D7EE1FB3B0","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":27000.0},"EVID-8B432207CE81E1B5453FBA36":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-8B432207CE81E1B5453FBA36","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":40000.0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A260A94FAD60AB2B5B984E15":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A260A94FAD60AB2B5B984E15","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":400.0},"EVID-C0024AE90132BFF522B946EA":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-C0024AE90132BFF522B946EA","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-D0948F3BBDA2C1A885CCD2E8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D0948F3BBDA2C1A885CCD2E8","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":8},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0}}</t>
         </is>
       </c>
       <c r="AV9" s="22" t="inlineStr">
@@ -14841,7 +14841,7 @@
       </c>
       <c r="AZ9" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-863D86733C17ECB8516EF093","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-0F323C820C480A6DB359983B","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
         </is>
       </c>
       <c r="BA9" s="22" t="inlineStr">
@@ -14853,12 +14853,12 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PKG-6BBDFC6E7CA70D5342AE781F</t>
+          <t>PKG-4FA8754447022C3EC951FFF6</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>CAND-E9A7141D8480ED7AC73076CC</t>
+          <t>CAND-B5D201CF9262CAC1AA7E3182</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -15042,12 +15042,12 @@
       </c>
       <c r="AT10" s="22" t="inlineStr">
         <is>
-          <t>["EVID-5CE57275336FF7A99147DCC0","EVID-D1D3CCC01ECDAD227F11E100","EVID-0769A5E646320DA500332309","EVID-592F211E9EDB3223E49035DF","EVID-A30D883A534722C9BCA5AEE0","EVID-82E7AD7A0BFE9AC6A7E9E8E3","EVID-2B38163DC5B241CCC5D6E4DE","EVID-1738AF6A4068640602ECD84E","EVID-FBADEF6B92F4CD5C57558A64","EVID-9165453291690C68D73C499A","EVID-EE439C26D0E760A7878BFAEA","EVID-F0838A46641CA4DF579874C2","EVID-95D4200101460975CFB0113A","EVID-E2BFCCA76EB8534DA44771CC","EVID-BC460C11441EEA3635B6CEF6","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
+          <t>["EVID-5CE57275336FF7A99147DCC0","EVID-D1D3CCC01ECDAD227F11E100","EVID-0769A5E646320DA500332309","EVID-592F211E9EDB3223E49035DF","EVID-A30D883A534722C9BCA5AEE0","EVID-82E7AD7A0BFE9AC6A7E9E8E3","EVID-2B38163DC5B241CCC5D6E4DE","EVID-1738AF6A4068640602ECD84E","EVID-FBADEF6B92F4CD5C57558A64","EVID-9165453291690C68D73C499A","EVID-EE439C26D0E760A7878BFAEA","EVID-F0838A46641CA4DF579874C2","EVID-95D4200101460975CFB0113A","EVID-E2BFCCA76EB8534DA44771CC","EVID-609ECEA12D01A7D7EE1FB3B0","EVID-C8BD459AEE7D00E30C81E085","EVID-9A7BE346494C09B0348F5402"]</t>
         </is>
       </c>
       <c r="AU10" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0769A5E646320DA500332309":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0769A5E646320DA500332309","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-1738AF6A4068640602ECD84E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1738AF6A4068640602ECD84E","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-2B38163DC5B241CCC5D6E4DE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2B38163DC5B241CCC5D6E4DE","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-592F211E9EDB3223E49035DF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-592F211E9EDB3223E49035DF","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":9000},"EVID-5CE57275336FF7A99147DCC0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5CE57275336FF7A99147DCC0","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-82E7AD7A0BFE9AC6A7E9E8E3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-82E7AD7A0BFE9AC6A7E9E8E3","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-9165453291690C68D73C499A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9165453291690C68D73C499A","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":3000},"EVID-95D4200101460975CFB0113A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95D4200101460975CFB0113A","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A30D883A534722C9BCA5AEE0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A30D883A534722C9BCA5AEE0","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-BC460C11441EEA3635B6CEF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC460C11441EEA3635B6CEF6","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":27000.0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-D1D3CCC01ECDAD227F11E100":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D1D3CCC01ECDAD227F11E100","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-EE439C26D0E760A7878BFAEA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE439C26D0E760A7878BFAEA","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-F0838A46641CA4DF579874C2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F0838A46641CA4DF579874C2","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-FBADEF6B92F4CD5C57558A64":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FBADEF6B92F4CD5C57558A64","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":960}}</t>
+          <t>{"EVID-0769A5E646320DA500332309":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0769A5E646320DA500332309","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-1738AF6A4068640602ECD84E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1738AF6A4068640602ECD84E","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-2B38163DC5B241CCC5D6E4DE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2B38163DC5B241CCC5D6E4DE","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-592F211E9EDB3223E49035DF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-592F211E9EDB3223E49035DF","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":9000},"EVID-5CE57275336FF7A99147DCC0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5CE57275336FF7A99147DCC0","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-609ECEA12D01A7D7EE1FB3B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-609ECEA12D01A7D7EE1FB3B0","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":27000.0},"EVID-82E7AD7A0BFE9AC6A7E9E8E3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-82E7AD7A0BFE9AC6A7E9E8E3","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-9165453291690C68D73C499A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9165453291690C68D73C499A","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":3000},"EVID-95D4200101460975CFB0113A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95D4200101460975CFB0113A","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-9A7BE346494C09B0348F5402":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7BE346494C09B0348F5402","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":259},"EVID-A30D883A534722C9BCA5AEE0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A30D883A534722C9BCA5AEE0","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-C8BD459AEE7D00E30C81E085":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C8BD459AEE7D00E30C81E085","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":11725.1},"EVID-D1D3CCC01ECDAD227F11E100":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D1D3CCC01ECDAD227F11E100","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-E2BFCCA76EB8534DA44771CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E2BFCCA76EB8534DA44771CC","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":23760.0},"EVID-EE439C26D0E760A7878BFAEA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE439C26D0E760A7878BFAEA","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-F0838A46641CA4DF579874C2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F0838A46641CA4DF579874C2","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-FBADEF6B92F4CD5C57558A64":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FBADEF6B92F4CD5C57558A64","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":960}}</t>
         </is>
       </c>
       <c r="AV10" s="22" t="inlineStr">
@@ -15072,7 +15072,7 @@
       </c>
       <c r="AZ10" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-145D50BED02E3BA2BE197B7F","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-05AEB24D88A789A8A5B3097C","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA10" s="22" t="inlineStr">
@@ -15084,12 +15084,12 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>CAND-828F9A162C1D262C1F78972E</t>
+          <t>CAND-16E28D4A7F0B58A50DBE0DFE</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -15273,12 +15273,12 @@
       </c>
       <c r="AT11" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4B0A26E4BCE89FB67759E226","EVID-798CAF1B6E59A5A6800BFDA6","EVID-DD4AB7148F9EA2F96522D001","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
+          <t>["EVID-4B0A26E4BCE89FB67759E226","EVID-798CAF1B6E59A5A6800BFDA6","EVID-48AB665BCC0F78BDF2A9678D","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
         </is>
       </c>
       <c r="AU11" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-4B0A26E4BCE89FB67759E226":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B0A26E4BCE89FB67759E226","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-DD4AB7148F9EA2F96522D001":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DD4AB7148F9EA2F96522D001","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0}}</t>
+          <t>{"EVID-48AB665BCC0F78BDF2A9678D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48AB665BCC0F78BDF2A9678D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":64000.0},"EVID-4B0A26E4BCE89FB67759E226":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B0A26E4BCE89FB67759E226","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7}}</t>
         </is>
       </c>
       <c r="AV11" s="22" t="inlineStr">
@@ -15315,12 +15315,12 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>CAND-725D8CE810F7854F0B4F0599</t>
+          <t>CAND-429785936CDB1BB844384CE3</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -15504,12 +15504,12 @@
       </c>
       <c r="AT12" s="22" t="inlineStr">
         <is>
-          <t>["EVID-317694A250D14B0CB5738BDB","EVID-BCF105F24D33111D31C3E82A","EVID-93786EC662829319601327D0","EVID-88260E5CAA85A2862B0AF592","EVID-BB853687EABCE34F9D34DE1A","EVID-F099780A8C11FAFA04AFEAA2","EVID-1E3C87A385079E3183BA0AA9","EVID-44A316ECBA6BF84EB02F0D48","EVID-3F6A911A1B67177259CD0328","EVID-798CAF1B6E59A5A6800BFDA6","EVID-DD4AB7148F9EA2F96522D001","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
+          <t>["EVID-317694A250D14B0CB5738BDB","EVID-BCF105F24D33111D31C3E82A","EVID-93786EC662829319601327D0","EVID-88260E5CAA85A2862B0AF592","EVID-BB853687EABCE34F9D34DE1A","EVID-F099780A8C11FAFA04AFEAA2","EVID-1E3C87A385079E3183BA0AA9","EVID-44A316ECBA6BF84EB02F0D48","EVID-3F6A911A1B67177259CD0328","EVID-798CAF1B6E59A5A6800BFDA6","EVID-48AB665BCC0F78BDF2A9678D","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
         </is>
       </c>
       <c r="AU12" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1E3C87A385079E3183BA0AA9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1E3C87A385079E3183BA0AA9","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":14000},"EVID-317694A250D14B0CB5738BDB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-317694A250D14B0CB5738BDB","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"X_LARGE"},"EVID-3F6A911A1B67177259CD0328":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3F6A911A1B67177259CD0328","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-44A316ECBA6BF84EB02F0D48":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-44A316ECBA6BF84EB02F0D48","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":48000},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-88260E5CAA85A2862B0AF592":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-88260E5CAA85A2862B0AF592","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":3221225472},"EVID-93786EC662829319601327D0":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-93786EC662829319601327D0","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":422},"EVID-BB853687EABCE34F9D34DE1A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-BB853687EABCE34F9D34DE1A","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.8},"EVID-BCF105F24D33111D31C3E82A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BCF105F24D33111D31C3E82A","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":6.5},"EVID-DD4AB7148F9EA2F96522D001":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DD4AB7148F9EA2F96522D001","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0},"EVID-F099780A8C11FAFA04AFEAA2":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F099780A8C11FAFA04AFEAA2","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
+          <t>{"EVID-1E3C87A385079E3183BA0AA9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1E3C87A385079E3183BA0AA9","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":14000},"EVID-317694A250D14B0CB5738BDB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-317694A250D14B0CB5738BDB","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"X_LARGE"},"EVID-3F6A911A1B67177259CD0328":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3F6A911A1B67177259CD0328","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-44A316ECBA6BF84EB02F0D48":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-44A316ECBA6BF84EB02F0D48","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":48000},"EVID-48AB665BCC0F78BDF2A9678D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48AB665BCC0F78BDF2A9678D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":64000.0},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-88260E5CAA85A2862B0AF592":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-88260E5CAA85A2862B0AF592","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":3221225472},"EVID-93786EC662829319601327D0":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-93786EC662829319601327D0","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":422},"EVID-BB853687EABCE34F9D34DE1A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-BB853687EABCE34F9D34DE1A","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.8},"EVID-BCF105F24D33111D31C3E82A":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BCF105F24D33111D31C3E82A","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":6.5},"EVID-F099780A8C11FAFA04AFEAA2":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F099780A8C11FAFA04AFEAA2","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
         </is>
       </c>
       <c r="AV12" s="22" t="inlineStr">
@@ -15534,7 +15534,7 @@
       </c>
       <c r="AZ12" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY","scenario_id":"SCN-B31B08FCFCF16CF8C3ED3133","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY","scenario_id":"SCN-EB2C0C39F179860453FE1B76","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA12" s="22" t="inlineStr">
@@ -15546,12 +15546,12 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CAND-0A41949888B511BF5079790D</t>
+          <t>CAND-0EB9378528832881336CC3CB</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -15731,12 +15731,12 @@
       </c>
       <c r="AT13" s="22" t="inlineStr">
         <is>
-          <t>["EVID-397653A8F7424B807EC69A77","EVID-F16D4AB2E6B3FE48E318CC61","EVID-EF19965DFBC5EC58CB587207","EVID-CCA7709442092923BEC9EDFD","EVID-FADEC648D4D98214CD4E0817","EVID-4C9BD346490AA494BABDC248","EVID-798CAF1B6E59A5A6800BFDA6","EVID-DD4AB7148F9EA2F96522D001","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
+          <t>["EVID-397653A8F7424B807EC69A77","EVID-F16D4AB2E6B3FE48E318CC61","EVID-EF19965DFBC5EC58CB587207","EVID-CCA7709442092923BEC9EDFD","EVID-FADEC648D4D98214CD4E0817","EVID-4C9BD346490AA494BABDC248","EVID-798CAF1B6E59A5A6800BFDA6","EVID-48AB665BCC0F78BDF2A9678D","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
         </is>
       </c>
       <c r="AU13" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-397653A8F7424B807EC69A77":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-397653A8F7424B807EC69A77","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":8},"EVID-4C9BD346490AA494BABDC248":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-4C9BD346490AA494BABDC248","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":5000},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-CCA7709442092923BEC9EDFD":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-CCA7709442092923BEC9EDFD","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.8},"EVID-DD4AB7148F9EA2F96522D001":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DD4AB7148F9EA2F96522D001","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0},"EVID-EF19965DFBC5EC58CB587207":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF19965DFBC5EC58CB587207","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":12.0},"EVID-F16D4AB2E6B3FE48E318CC61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F16D4AB2E6B3FE48E318CC61","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":7},"EVID-FADEC648D4D98214CD4E0817":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-FADEC648D4D98214CD4E0817","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":52}}</t>
+          <t>{"EVID-397653A8F7424B807EC69A77":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-397653A8F7424B807EC69A77","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":8},"EVID-48AB665BCC0F78BDF2A9678D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48AB665BCC0F78BDF2A9678D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":64000.0},"EVID-4C9BD346490AA494BABDC248":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-4C9BD346490AA494BABDC248","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":5000},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-CCA7709442092923BEC9EDFD":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-CCA7709442092923BEC9EDFD","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.8},"EVID-EF19965DFBC5EC58CB587207":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF19965DFBC5EC58CB587207","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":12.0},"EVID-F16D4AB2E6B3FE48E318CC61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F16D4AB2E6B3FE48E318CC61","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":7},"EVID-FADEC648D4D98214CD4E0817":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-FADEC648D4D98214CD4E0817","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":52}}</t>
         </is>
       </c>
       <c r="AV13" s="22" t="inlineStr">
@@ -15773,12 +15773,12 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CAND-E76392F60728B051B8FFF1A6</t>
+          <t>CAND-147B23ADCB8854F570950756</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -15958,12 +15958,12 @@
       </c>
       <c r="AT14" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4B6CAD51D6E6CC690F238328","EVID-8089B2A88341C92E810E6D25","EVID-7700F4C8B0DDF3241F3EF7E2","EVID-64C33490C6C8E7457B3DECE3","EVID-5A8EA64D13B38C8F14D75DFA","EVID-798CAF1B6E59A5A6800BFDA6","EVID-DD4AB7148F9EA2F96522D001","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
+          <t>["EVID-4B6CAD51D6E6CC690F238328","EVID-8089B2A88341C92E810E6D25","EVID-7700F4C8B0DDF3241F3EF7E2","EVID-64C33490C6C8E7457B3DECE3","EVID-5A8EA64D13B38C8F14D75DFA","EVID-798CAF1B6E59A5A6800BFDA6","EVID-48AB665BCC0F78BDF2A9678D","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
         </is>
       </c>
       <c r="AU14" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-4B6CAD51D6E6CC690F238328":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B6CAD51D6E6CC690F238328","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2},"EVID-5A8EA64D13B38C8F14D75DFA":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-5A8EA64D13B38C8F14D75DFA","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":12.0},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-64C33490C6C8E7457B3DECE3":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-64C33490C6C8E7457B3DECE3","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":5000},"EVID-7700F4C8B0DDF3241F3EF7E2":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-7700F4C8B0DDF3241F3EF7E2","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.8},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-8089B2A88341C92E810E6D25":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-8089B2A88341C92E810E6D25","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":25.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-DD4AB7148F9EA2F96522D001":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DD4AB7148F9EA2F96522D001","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0}}</t>
+          <t>{"EVID-48AB665BCC0F78BDF2A9678D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48AB665BCC0F78BDF2A9678D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":64000.0},"EVID-4B6CAD51D6E6CC690F238328":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B6CAD51D6E6CC690F238328","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2},"EVID-5A8EA64D13B38C8F14D75DFA":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-5A8EA64D13B38C8F14D75DFA","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":12.0},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-64C33490C6C8E7457B3DECE3":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-64C33490C6C8E7457B3DECE3","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":5000},"EVID-7700F4C8B0DDF3241F3EF7E2":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-7700F4C8B0DDF3241F3EF7E2","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.8},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-8089B2A88341C92E810E6D25":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-8089B2A88341C92E810E6D25","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":25.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7}}</t>
         </is>
       </c>
       <c r="AV14" s="22" t="inlineStr">
@@ -16000,12 +16000,12 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>CAND-CC561F3665974267980305C7</t>
+          <t>CAND-9036A0CCF32202C187B847C1</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -16185,12 +16185,12 @@
       </c>
       <c r="AT15" s="22" t="inlineStr">
         <is>
-          <t>["EVID-D353A0904BB6A241CD4A8FCF","EVID-563CF3DD0B11F9EE318B64CA","EVID-238FF507E88B1AC45C97415F","EVID-1C1403E5FDC40ADF27F58E2E","EVID-9B47E8DD6C50F547AD614266","EVID-E991D606CA5CF64A0BF34205","EVID-F2F3E51797850FB6D31B3CE9","EVID-1F9B7F008085483A33F93C00","EVID-798CAF1B6E59A5A6800BFDA6","EVID-DD4AB7148F9EA2F96522D001","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
+          <t>["EVID-D353A0904BB6A241CD4A8FCF","EVID-563CF3DD0B11F9EE318B64CA","EVID-238FF507E88B1AC45C97415F","EVID-1C1403E5FDC40ADF27F58E2E","EVID-9B47E8DD6C50F547AD614266","EVID-E991D606CA5CF64A0BF34205","EVID-F2F3E51797850FB6D31B3CE9","EVID-1F9B7F008085483A33F93C00","EVID-798CAF1B6E59A5A6800BFDA6","EVID-48AB665BCC0F78BDF2A9678D","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
         </is>
       </c>
       <c r="AU15" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1C1403E5FDC40ADF27F58E2E":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-1C1403E5FDC40ADF27F58E2E","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":130000.0},"EVID-1F9B7F008085483A33F93C00":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1F9B7F008085483A33F93C00","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":3600.0},"EVID-238FF507E88B1AC45C97415F":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-238FF507E88B1AC45C97415F","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":260},"EVID-563CF3DD0B11F9EE318B64CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-563CF3DD0B11F9EE318B64CA","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":216.67},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-9B47E8DD6C50F547AD614266":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9B47E8DD6C50F547AD614266","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-D353A0904BB6A241CD4A8FCF":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-D353A0904BB6A241CD4A8FCF","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":60},"EVID-DD4AB7148F9EA2F96522D001":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DD4AB7148F9EA2F96522D001","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0},"EVID-E991D606CA5CF64A0BF34205":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-E991D606CA5CF64A0BF34205","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-F2F3E51797850FB6D31B3CE9":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-F2F3E51797850FB6D31B3CE9","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667}}</t>
+          <t>{"EVID-1C1403E5FDC40ADF27F58E2E":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-1C1403E5FDC40ADF27F58E2E","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":130000.0},"EVID-1F9B7F008085483A33F93C00":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1F9B7F008085483A33F93C00","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":3600.0},"EVID-238FF507E88B1AC45C97415F":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-238FF507E88B1AC45C97415F","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":260},"EVID-48AB665BCC0F78BDF2A9678D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48AB665BCC0F78BDF2A9678D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":64000.0},"EVID-563CF3DD0B11F9EE318B64CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-563CF3DD0B11F9EE318B64CA","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":216.67},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-9B47E8DD6C50F547AD614266":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9B47E8DD6C50F547AD614266","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-D353A0904BB6A241CD4A8FCF":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-D353A0904BB6A241CD4A8FCF","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":60},"EVID-E991D606CA5CF64A0BF34205":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-E991D606CA5CF64A0BF34205","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-F2F3E51797850FB6D31B3CE9":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-F2F3E51797850FB6D31B3CE9","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667}}</t>
         </is>
       </c>
       <c r="AV15" s="22" t="inlineStr">
@@ -16215,7 +16215,7 @@
       </c>
       <c r="AZ15" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-B31B08FCFCF16CF8C3ED3133","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-EB2C0C39F179860453FE1B76","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA15" s="22" t="inlineStr">
@@ -16227,12 +16227,12 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PKG-AF576EED00EE7686E958381E</t>
+          <t>PKG-7F257D02E028B13BE2486588</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>CAND-FBE101BD35EAD540544961F6</t>
+          <t>CAND-50DDBBB8A017E60563909CE4</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -16416,12 +16416,12 @@
       </c>
       <c r="AT16" s="22" t="inlineStr">
         <is>
-          <t>["EVID-E4B7509030D6AA1C7EE0DC48","EVID-D0A63A8CF2088FDE42703300","EVID-AD892CA77594BB00A48A1B37","EVID-3466FCD5ACCCF0CB40F076F6","EVID-5CA339D2D13816847797EB99","EVID-D36E9B4C473DB25466DABDB8","EVID-7F3FBCF285A330187414CCE9","EVID-6F5C81C659714CBD71F96903","EVID-6D57B4495F16EF2F1F11A058","EVID-7362CB175D2D3EE7F7FD836B","EVID-108CC2BBEE3480D859C1460C","EVID-BAA92FC68151FBCB7BAC6577","EVID-B2195A64E32504F7CA0F938B","EVID-798CAF1B6E59A5A6800BFDA6","EVID-DD4AB7148F9EA2F96522D001","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
+          <t>["EVID-E4B7509030D6AA1C7EE0DC48","EVID-D0A63A8CF2088FDE42703300","EVID-AD892CA77594BB00A48A1B37","EVID-3466FCD5ACCCF0CB40F076F6","EVID-5CA339D2D13816847797EB99","EVID-D36E9B4C473DB25466DABDB8","EVID-7F3FBCF285A330187414CCE9","EVID-6F5C81C659714CBD71F96903","EVID-6D57B4495F16EF2F1F11A058","EVID-7362CB175D2D3EE7F7FD836B","EVID-108CC2BBEE3480D859C1460C","EVID-BAA92FC68151FBCB7BAC6577","EVID-B2195A64E32504F7CA0F938B","EVID-798CAF1B6E59A5A6800BFDA6","EVID-48AB665BCC0F78BDF2A9678D","EVID-856AE353D873B76613562142","EVID-5FAA6569BBF4163B44E3BB5F"]</t>
         </is>
       </c>
       <c r="AU16" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-108CC2BBEE3480D859C1460C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-108CC2BBEE3480D859C1460C","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-3466FCD5ACCCF0CB40F076F6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3466FCD5ACCCF0CB40F076F6","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-5CA339D2D13816847797EB99":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5CA339D2D13816847797EB99","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":4875},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-6D57B4495F16EF2F1F11A058":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6D57B4495F16EF2F1F11A058","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":520},"EVID-6F5C81C659714CBD71F96903":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6F5C81C659714CBD71F96903","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-7362CB175D2D3EE7F7FD836B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7362CB175D2D3EE7F7FD836B","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-7F3FBCF285A330187414CCE9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7F3FBCF285A330187414CCE9","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-AD892CA77594BB00A48A1B37":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AD892CA77594BB00A48A1B37","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-B2195A64E32504F7CA0F938B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B2195A64E32504F7CA0F938B","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-BAA92FC68151FBCB7BAC6577":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA92FC68151FBCB7BAC6577","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-D0A63A8CF2088FDE42703300":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D0A63A8CF2088FDE42703300","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-D36E9B4C473DB25466DABDB8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D36E9B4C473DB25466DABDB8","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-DD4AB7148F9EA2F96522D001":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DD4AB7148F9EA2F96522D001","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":64000.0},"EVID-E4B7509030D6AA1C7EE0DC48":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E4B7509030D6AA1C7EE0DC48","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"}}</t>
+          <t>{"EVID-108CC2BBEE3480D859C1460C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-108CC2BBEE3480D859C1460C","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-3466FCD5ACCCF0CB40F076F6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3466FCD5ACCCF0CB40F076F6","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-48AB665BCC0F78BDF2A9678D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48AB665BCC0F78BDF2A9678D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":64000.0},"EVID-5CA339D2D13816847797EB99":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5CA339D2D13816847797EB99","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":4875},"EVID-5FAA6569BBF4163B44E3BB5F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5FAA6569BBF4163B44E3BB5F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":264},"EVID-6D57B4495F16EF2F1F11A058":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6D57B4495F16EF2F1F11A058","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":520},"EVID-6F5C81C659714CBD71F96903":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6F5C81C659714CBD71F96903","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-7362CB175D2D3EE7F7FD836B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7362CB175D2D3EE7F7FD836B","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-798CAF1B6E59A5A6800BFDA6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-798CAF1B6E59A5A6800BFDA6","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":56320.0},"EVID-7F3FBCF285A330187414CCE9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7F3FBCF285A330187414CCE9","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-856AE353D873B76613562142":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-856AE353D873B76613562142","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":74769.7},"EVID-AD892CA77594BB00A48A1B37":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AD892CA77594BB00A48A1B37","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-B2195A64E32504F7CA0F938B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B2195A64E32504F7CA0F938B","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-BAA92FC68151FBCB7BAC6577":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA92FC68151FBCB7BAC6577","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-D0A63A8CF2088FDE42703300":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D0A63A8CF2088FDE42703300","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-D36E9B4C473DB25466DABDB8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D36E9B4C473DB25466DABDB8","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-E4B7509030D6AA1C7EE0DC48":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E4B7509030D6AA1C7EE0DC48","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"}}</t>
         </is>
       </c>
       <c r="AV16" s="22" t="inlineStr">
@@ -16446,7 +16446,7 @@
       </c>
       <c r="AZ16" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-49F9E59C5DC51E8EA18565EB","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-BA79A1BAC0F873D6CDE9EC20","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA16" s="22" t="inlineStr">
@@ -16458,12 +16458,12 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>CAND-19114E8F568FBD08CD0E7342</t>
+          <t>CAND-470FD4CCBBE164E952753E39</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -16647,12 +16647,12 @@
       </c>
       <c r="AT17" s="22" t="inlineStr">
         <is>
-          <t>["EVID-C54D688D7F24665423F4E1C8","EVID-138DC2A3D2FA80EC64571C3B","EVID-70DB2AE41192F0BE08EDA0E4","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
+          <t>["EVID-C54D688D7F24665423F4E1C8","EVID-138DC2A3D2FA80EC64571C3B","EVID-4AE16179F3F066BEB4F4D971","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
         </is>
       </c>
       <c r="AU17" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-70DB2AE41192F0BE08EDA0E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-70DB2AE41192F0BE08EDA0E4","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-C54D688D7F24665423F4E1C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C54D688D7F24665423F4E1C8","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214}}</t>
+          <t>{"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-4AE16179F3F066BEB4F4D971":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AE16179F3F066BEB4F4D971","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-C54D688D7F24665423F4E1C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C54D688D7F24665423F4E1C8","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214}}</t>
         </is>
       </c>
       <c r="AV17" s="22" t="inlineStr">
@@ -16689,12 +16689,12 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>CAND-EB8642E918D1FD97EE3FA4E2</t>
+          <t>CAND-983E960CC6715CCFDAFC3353</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -16878,12 +16878,12 @@
       </c>
       <c r="AT18" s="22" t="inlineStr">
         <is>
-          <t>["EVID-ADBD9F5EF2B25F6F2301AC5D","EVID-BF740AE5AD36DB91FC871C3E","EVID-2BE6464F016F9F52AD9CB0A6","EVID-2F5A12215CC813683545D25C","EVID-634883B72B148A9943D89C0E","EVID-DCED59AF916F6BE35E271AE4","EVID-64A7680E004B2C425704B7E9","EVID-511D1D18D1235C9B3444A79E","EVID-3E1EFFF63FE150372B9DD4CB","EVID-138DC2A3D2FA80EC64571C3B","EVID-70DB2AE41192F0BE08EDA0E4","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
+          <t>["EVID-ADBD9F5EF2B25F6F2301AC5D","EVID-BF740AE5AD36DB91FC871C3E","EVID-2BE6464F016F9F52AD9CB0A6","EVID-2F5A12215CC813683545D25C","EVID-634883B72B148A9943D89C0E","EVID-DCED59AF916F6BE35E271AE4","EVID-64A7680E004B2C425704B7E9","EVID-511D1D18D1235C9B3444A79E","EVID-3E1EFFF63FE150372B9DD4CB","EVID-138DC2A3D2FA80EC64571C3B","EVID-4AE16179F3F066BEB4F4D971","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
         </is>
       </c>
       <c r="AU18" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-2BE6464F016F9F52AD9CB0A6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2BE6464F016F9F52AD9CB0A6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-2F5A12215CC813683545D25C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2F5A12215CC813683545D25C","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-3E1EFFF63FE150372B9DD4CB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3E1EFFF63FE150372B9DD4CB","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-511D1D18D1235C9B3444A79E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-511D1D18D1235C9B3444A79E","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6500},"EVID-634883B72B148A9943D89C0E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-634883B72B148A9943D89C0E","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-64A7680E004B2C425704B7E9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-64A7680E004B2C425704B7E9","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1900},"EVID-70DB2AE41192F0BE08EDA0E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-70DB2AE41192F0BE08EDA0E4","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-ADBD9F5EF2B25F6F2301AC5D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ADBD9F5EF2B25F6F2301AC5D","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-BF740AE5AD36DB91FC871C3E":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BF740AE5AD36DB91FC871C3E","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-DCED59AF916F6BE35E271AE4":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DCED59AF916F6BE35E271AE4","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
+          <t>{"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-2BE6464F016F9F52AD9CB0A6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2BE6464F016F9F52AD9CB0A6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-2F5A12215CC813683545D25C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2F5A12215CC813683545D25C","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-3E1EFFF63FE150372B9DD4CB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3E1EFFF63FE150372B9DD4CB","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-4AE16179F3F066BEB4F4D971":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AE16179F3F066BEB4F4D971","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":48000.0},"EVID-511D1D18D1235C9B3444A79E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-511D1D18D1235C9B3444A79E","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6500},"EVID-634883B72B148A9943D89C0E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-634883B72B148A9943D89C0E","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-64A7680E004B2C425704B7E9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-64A7680E004B2C425704B7E9","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1900},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-ADBD9F5EF2B25F6F2301AC5D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ADBD9F5EF2B25F6F2301AC5D","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-BF740AE5AD36DB91FC871C3E":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BF740AE5AD36DB91FC871C3E","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-DCED59AF916F6BE35E271AE4":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DCED59AF916F6BE35E271AE4","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3}}</t>
         </is>
       </c>
       <c r="AV18" s="22" t="inlineStr">
@@ -16908,7 +16908,7 @@
       </c>
       <c r="AZ18" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-9D2CE3A1C8DF6267C795DB02","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-26E77B55DE75D30BC7D94E62","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA18" s="22" t="inlineStr">
@@ -16920,12 +16920,12 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>CAND-40DECBD0C64F73A246651419</t>
+          <t>CAND-925E95E6BA6DA0ED59A9A733</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -17105,12 +17105,12 @@
       </c>
       <c r="AT19" s="22" t="inlineStr">
         <is>
-          <t>["EVID-0469DF8349DF92AE11B1D733","EVID-90FD7EC9CBD2C8836D6B0FFF","EVID-2B6F729499188E4516712DEF","EVID-528AF7AEAFDF42798FFAF40D","EVID-E5644C6E4E95CA9DFC6EA17E","EVID-CA4D7EC185EB84B896178975","EVID-138DC2A3D2FA80EC64571C3B","EVID-70DB2AE41192F0BE08EDA0E4","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
+          <t>["EVID-0469DF8349DF92AE11B1D733","EVID-90FD7EC9CBD2C8836D6B0FFF","EVID-2B6F729499188E4516712DEF","EVID-528AF7AEAFDF42798FFAF40D","EVID-E5644C6E4E95CA9DFC6EA17E","EVID-CA4D7EC185EB84B896178975","EVID-138DC2A3D2FA80EC64571C3B","EVID-4AE16179F3F066BEB4F4D971","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
         </is>
       </c>
       <c r="AU19" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0469DF8349DF92AE11B1D733":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0469DF8349DF92AE11B1D733","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":6},"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-2B6F729499188E4516712DEF":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-2B6F729499188E4516712DEF","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-528AF7AEAFDF42798FFAF40D":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-528AF7AEAFDF42798FFAF40D","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-70DB2AE41192F0BE08EDA0E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-70DB2AE41192F0BE08EDA0E4","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-90FD7EC9CBD2C8836D6B0FFF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-90FD7EC9CBD2C8836D6B0FFF","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":3},"EVID-CA4D7EC185EB84B896178975":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-CA4D7EC185EB84B896178975","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-E5644C6E4E95CA9DFC6EA17E":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-E5644C6E4E95CA9DFC6EA17E","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0}}</t>
+          <t>{"EVID-0469DF8349DF92AE11B1D733":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0469DF8349DF92AE11B1D733","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":6},"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-2B6F729499188E4516712DEF":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-2B6F729499188E4516712DEF","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-4AE16179F3F066BEB4F4D971":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AE16179F3F066BEB4F4D971","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":48000.0},"EVID-528AF7AEAFDF42798FFAF40D":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-528AF7AEAFDF42798FFAF40D","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-90FD7EC9CBD2C8836D6B0FFF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-90FD7EC9CBD2C8836D6B0FFF","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":3},"EVID-CA4D7EC185EB84B896178975":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-CA4D7EC185EB84B896178975","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-E5644C6E4E95CA9DFC6EA17E":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-E5644C6E4E95CA9DFC6EA17E","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV19" s="22" t="inlineStr">
@@ -17135,7 +17135,7 @@
       </c>
       <c r="AZ19" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-9D2CE3A1C8DF6267C795DB02","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-26E77B55DE75D30BC7D94E62","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA19" s="22" t="inlineStr">
@@ -17147,12 +17147,12 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>CAND-47C39CB54A496B16C7C5535D</t>
+          <t>CAND-C01B3B61787F253552AB5722</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
@@ -17332,12 +17332,12 @@
       </c>
       <c r="AT20" s="22" t="inlineStr">
         <is>
-          <t>["EVID-9C062F46FF3DD1C51BE0F5CF","EVID-28F961BADB1773C5BBE0E0FC","EVID-FCA7D73825895E13A667605E","EVID-962883EA791AE7B18476787C","EVID-18DEA81AF9B9B09E66190314","EVID-138DC2A3D2FA80EC64571C3B","EVID-70DB2AE41192F0BE08EDA0E4","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
+          <t>["EVID-9C062F46FF3DD1C51BE0F5CF","EVID-28F961BADB1773C5BBE0E0FC","EVID-FCA7D73825895E13A667605E","EVID-962883EA791AE7B18476787C","EVID-18DEA81AF9B9B09E66190314","EVID-138DC2A3D2FA80EC64571C3B","EVID-4AE16179F3F066BEB4F4D971","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
         </is>
       </c>
       <c r="AU20" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-18DEA81AF9B9B09E66190314":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-18DEA81AF9B9B09E66190314","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-28F961BADB1773C5BBE0E0FC":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-28F961BADB1773C5BBE0E0FC","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":88.0},"EVID-70DB2AE41192F0BE08EDA0E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-70DB2AE41192F0BE08EDA0E4","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-962883EA791AE7B18476787C":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-962883EA791AE7B18476787C","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-9C062F46FF3DD1C51BE0F5CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9C062F46FF3DD1C51BE0F5CF","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":3},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-FCA7D73825895E13A667605E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-FCA7D73825895E13A667605E","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0}}</t>
+          <t>{"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-18DEA81AF9B9B09E66190314":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-18DEA81AF9B9B09E66190314","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-28F961BADB1773C5BBE0E0FC":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-28F961BADB1773C5BBE0E0FC","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":88.0},"EVID-4AE16179F3F066BEB4F4D971":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AE16179F3F066BEB4F4D971","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-962883EA791AE7B18476787C":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-962883EA791AE7B18476787C","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-9C062F46FF3DD1C51BE0F5CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9C062F46FF3DD1C51BE0F5CF","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":3},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-FCA7D73825895E13A667605E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-FCA7D73825895E13A667605E","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0}}</t>
         </is>
       </c>
       <c r="AV20" s="22" t="inlineStr">
@@ -17362,7 +17362,7 @@
       </c>
       <c r="AZ20" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-9D2CE3A1C8DF6267C795DB02","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-26E77B55DE75D30BC7D94E62","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA20" s="22" t="inlineStr">
@@ -17374,12 +17374,12 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>CAND-7B32E8C35D19CC2C522779EC</t>
+          <t>CAND-014DD489DCA84594FA96ACC7</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -17559,12 +17559,12 @@
       </c>
       <c r="AT21" s="22" t="inlineStr">
         <is>
-          <t>["EVID-DFFE4AC535CD891824D51F47","EVID-AECADC84F1D8CBD06E73BED8","EVID-1E15FCB045036DE3E4936272","EVID-0E04A6B3AFE0680824E42A87","EVID-66A17A5BB4510C9DBCA2C477","EVID-3DF032BEFA85DB8FC552AEB3","EVID-CB02952CE3269D257AC973ED","EVID-D42D7396E4078F59ED71E357","EVID-138DC2A3D2FA80EC64571C3B","EVID-70DB2AE41192F0BE08EDA0E4","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
+          <t>["EVID-DFFE4AC535CD891824D51F47","EVID-AECADC84F1D8CBD06E73BED8","EVID-1E15FCB045036DE3E4936272","EVID-0E04A6B3AFE0680824E42A87","EVID-66A17A5BB4510C9DBCA2C477","EVID-3DF032BEFA85DB8FC552AEB3","EVID-CB02952CE3269D257AC973ED","EVID-D42D7396E4078F59ED71E357","EVID-138DC2A3D2FA80EC64571C3B","EVID-4AE16179F3F066BEB4F4D971","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
         </is>
       </c>
       <c r="AU21" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0E04A6B3AFE0680824E42A87":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-0E04A6B3AFE0680824E42A87","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":60000.0},"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-1E15FCB045036DE3E4936272":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-1E15FCB045036DE3E4936272","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":600},"EVID-3DF032BEFA85DB8FC552AEB3":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-3DF032BEFA85DB8FC552AEB3","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-66A17A5BB4510C9DBCA2C477":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-66A17A5BB4510C9DBCA2C477","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":6},"EVID-70DB2AE41192F0BE08EDA0E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-70DB2AE41192F0BE08EDA0E4","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-AECADC84F1D8CBD06E73BED8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AECADC84F1D8CBD06E73BED8","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":500.0},"EVID-CB02952CE3269D257AC973ED":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-CB02952CE3269D257AC973ED","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2},"EVID-D42D7396E4078F59ED71E357":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D42D7396E4078F59ED71E357","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":5500.0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-DFFE4AC535CD891824D51F47":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-DFFE4AC535CD891824D51F47","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":45,"unit":"minutes","value":120}}</t>
+          <t>{"EVID-0E04A6B3AFE0680824E42A87":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-0E04A6B3AFE0680824E42A87","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":60000.0},"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-1E15FCB045036DE3E4936272":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-1E15FCB045036DE3E4936272","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":600},"EVID-3DF032BEFA85DB8FC552AEB3":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-3DF032BEFA85DB8FC552AEB3","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-4AE16179F3F066BEB4F4D971":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AE16179F3F066BEB4F4D971","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":48000.0},"EVID-66A17A5BB4510C9DBCA2C477":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-66A17A5BB4510C9DBCA2C477","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":6},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-AECADC84F1D8CBD06E73BED8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AECADC84F1D8CBD06E73BED8","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":500.0},"EVID-CB02952CE3269D257AC973ED":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-CB02952CE3269D257AC973ED","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2},"EVID-D42D7396E4078F59ED71E357":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D42D7396E4078F59ED71E357","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":5500.0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-DFFE4AC535CD891824D51F47":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-DFFE4AC535CD891824D51F47","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":45,"unit":"minutes","value":120}}</t>
         </is>
       </c>
       <c r="AV21" s="22" t="inlineStr">
@@ -17589,7 +17589,7 @@
       </c>
       <c r="AZ21" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-9D2CE3A1C8DF6267C795DB02","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-26E77B55DE75D30BC7D94E62","scenario_name":"Plan A — Optimize current warehouse type","step":4}]</t>
         </is>
       </c>
       <c r="BA21" s="22" t="inlineStr">
@@ -17601,12 +17601,12 @@
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>PKG-00D335ABDE6268DF9BD34941</t>
+          <t>PKG-3A82B7A98C18CFAE14A8225C</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>CAND-1E5BC9641C5288D175C688E2</t>
+          <t>CAND-C8B00F2B86A8B7AF7549A783</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -17790,12 +17790,12 @@
       </c>
       <c r="AT22" s="22" t="inlineStr">
         <is>
-          <t>["EVID-7A3A3F9E60677F3A4138A318","EVID-5F47555F958537E30D6B43EB","EVID-0D4AD27CEF1BC4E014A366E0","EVID-9F97153165BA0D87B5E65DAB","EVID-83E6ACE6F898190CF078E276","EVID-AFA35C81985D592CA48145FD","EVID-F1CA50ECF9487421AC834976","EVID-C6C9F93AA2CBE86496C750A8","EVID-1A7EE4BB1C6CB7A9A2364274","EVID-1F30B9F5C01C5C2958401FB4","EVID-4B2FA824AF34D1756613D802","EVID-7D237D1142C76BF20FE66F78","EVID-06FC310FC9843E52C293EC95","EVID-138DC2A3D2FA80EC64571C3B","EVID-70DB2AE41192F0BE08EDA0E4","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
+          <t>["EVID-7A3A3F9E60677F3A4138A318","EVID-5F47555F958537E30D6B43EB","EVID-0D4AD27CEF1BC4E014A366E0","EVID-9F97153165BA0D87B5E65DAB","EVID-83E6ACE6F898190CF078E276","EVID-AFA35C81985D592CA48145FD","EVID-F1CA50ECF9487421AC834976","EVID-C6C9F93AA2CBE86496C750A8","EVID-1A7EE4BB1C6CB7A9A2364274","EVID-1F30B9F5C01C5C2958401FB4","EVID-4B2FA824AF34D1756613D802","EVID-7D237D1142C76BF20FE66F78","EVID-06FC310FC9843E52C293EC95","EVID-138DC2A3D2FA80EC64571C3B","EVID-4AE16179F3F066BEB4F4D971","EVID-843F72CCFB337DC9D837A0C8","EVID-D98ED418DDC55A2585D8D062"]</t>
         </is>
       </c>
       <c r="AU22" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-06FC310FC9843E52C293EC95":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-06FC310FC9843E52C293EC95","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-0D4AD27CEF1BC4E014A366E0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D4AD27CEF1BC4E014A366E0","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-1A7EE4BB1C6CB7A9A2364274":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1A7EE4BB1C6CB7A9A2364274","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1200},"EVID-1F30B9F5C01C5C2958401FB4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1F30B9F5C01C5C2958401FB4","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":3750},"EVID-4B2FA824AF34D1756613D802":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B2FA824AF34D1756613D802","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-5F47555F958537E30D6B43EB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5F47555F958537E30D6B43EB","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-70DB2AE41192F0BE08EDA0E4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-70DB2AE41192F0BE08EDA0E4","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":48000.0},"EVID-7A3A3F9E60677F3A4138A318":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A3A3F9E60677F3A4138A318","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-7D237D1142C76BF20FE66F78":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7D237D1142C76BF20FE66F78","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-83E6ACE6F898190CF078E276":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-83E6ACE6F898190CF078E276","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-9F97153165BA0D87B5E65DAB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9F97153165BA0D87B5E65DAB","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":11250},"EVID-AFA35C81985D592CA48145FD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AFA35C81985D592CA48145FD","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-C6C9F93AA2CBE86496C750A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C6C9F93AA2CBE86496C750A8","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-F1CA50ECF9487421AC834976":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F1CA50ECF9487421AC834976","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0}}</t>
+          <t>{"EVID-06FC310FC9843E52C293EC95":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-06FC310FC9843E52C293EC95","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-0D4AD27CEF1BC4E014A366E0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D4AD27CEF1BC4E014A366E0","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-138DC2A3D2FA80EC64571C3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-138DC2A3D2FA80EC64571C3B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":42240.0},"EVID-1A7EE4BB1C6CB7A9A2364274":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1A7EE4BB1C6CB7A9A2364274","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1200},"EVID-1F30B9F5C01C5C2958401FB4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1F30B9F5C01C5C2958401FB4","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":3750},"EVID-4AE16179F3F066BEB4F4D971":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4AE16179F3F066BEB4F4D971","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":48000.0},"EVID-4B2FA824AF34D1756613D802":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B2FA824AF34D1756613D802","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-5F47555F958537E30D6B43EB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5F47555F958537E30D6B43EB","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-7A3A3F9E60677F3A4138A318":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A3A3F9E60677F3A4138A318","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-7D237D1142C76BF20FE66F78":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7D237D1142C76BF20FE66F78","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-83E6ACE6F898190CF078E276":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-83E6ACE6F898190CF078E276","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-843F72CCFB337DC9D837A0C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-843F72CCFB337DC9D837A0C8","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":21285.98},"EVID-9F97153165BA0D87B5E65DAB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9F97153165BA0D87B5E65DAB","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":11250},"EVID-AFA35C81985D592CA48145FD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AFA35C81985D592CA48145FD","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-C6C9F93AA2CBE86496C750A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C6C9F93AA2CBE86496C750A8","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-D98ED418DDC55A2585D8D062":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D98ED418DDC55A2585D8D062","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":214},"EVID-F1CA50ECF9487421AC834976":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F1CA50ECF9487421AC834976","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV22" s="22" t="inlineStr">
@@ -17820,7 +17820,7 @@
       </c>
       <c r="AZ22" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-3E24BF4E2EB1FFD6BD97C5EF","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-DF356B65FC7D9469319D516C","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA22" s="22" t="inlineStr">
@@ -17832,12 +17832,12 @@
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>CAND-77B660B87F881D16821F65A4</t>
+          <t>CAND-A8E0C6C2514B7B2907081D31</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -18021,12 +18021,12 @@
       </c>
       <c r="AT23" s="22" t="inlineStr">
         <is>
-          <t>["EVID-6C649CEB38C11AD9F545A814","EVID-91E83CACE07F654C8375E91B","EVID-679B0BB84F874895FE357CF9","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
+          <t>["EVID-6C649CEB38C11AD9F545A814","EVID-91E83CACE07F654C8375E91B","EVID-120A7F0AFA3DF21C0BF51872","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
         </is>
       </c>
       <c r="AU23" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-679B0BB84F874895FE357CF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-679B0BB84F874895FE357CF9","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-6C649CEB38C11AD9F545A814":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6C649CEB38C11AD9F545A814","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254}}</t>
+          <t>{"EVID-120A7F0AFA3DF21C0BF51872":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-120A7F0AFA3DF21C0BF51872","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":36000.0},"EVID-6C649CEB38C11AD9F545A814":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6C649CEB38C11AD9F545A814","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254}}</t>
         </is>
       </c>
       <c r="AV23" s="22" t="inlineStr">
@@ -18063,12 +18063,12 @@
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>CAND-B2761F18473F72B19D49C194</t>
+          <t>CAND-6746672461AA4563E3A5F445</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -18270,12 +18270,12 @@
       </c>
       <c r="AT24" s="22" t="inlineStr">
         <is>
-          <t>["EVID-943CC5DA406961E6EB3068F0","EVID-A3FFF81B3A1797CA534E3F69","EVID-5559E287993BB07DE138FDF6","EVID-D5234CFF6B2C514C67CA7887","EVID-DCD165B1F77962F8297C7F4D","EVID-1A9FB4971218B885A774B43B","EVID-4CD8C8C1F0430C6A0156057C","EVID-DC3612A9EEBCACBD7708CC0E","EVID-3E3D4D117F217EA7DB1596CE","EVID-91E83CACE07F654C8375E91B","EVID-679B0BB84F874895FE357CF9","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
+          <t>["EVID-943CC5DA406961E6EB3068F0","EVID-A3FFF81B3A1797CA534E3F69","EVID-5559E287993BB07DE138FDF6","EVID-D5234CFF6B2C514C67CA7887","EVID-DCD165B1F77962F8297C7F4D","EVID-1A9FB4971218B885A774B43B","EVID-4CD8C8C1F0430C6A0156057C","EVID-DC3612A9EEBCACBD7708CC0E","EVID-3E3D4D117F217EA7DB1596CE","EVID-91E83CACE07F654C8375E91B","EVID-120A7F0AFA3DF21C0BF51872","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
         </is>
       </c>
       <c r="AU24" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1A9FB4971218B885A774B43B":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1A9FB4971218B885A774B43B","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-3E3D4D117F217EA7DB1596CE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3E3D4D117F217EA7DB1596CE","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-4CD8C8C1F0430C6A0156057C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4CD8C8C1F0430C6A0156057C","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3600},"EVID-5559E287993BB07DE138FDF6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-5559E287993BB07DE138FDF6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-679B0BB84F874895FE357CF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-679B0BB84F874895FE357CF9","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-943CC5DA406961E6EB3068F0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-943CC5DA406961E6EB3068F0","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-A3FFF81B3A1797CA534E3F69":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-A3FFF81B3A1797CA534E3F69","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-D5234CFF6B2C514C67CA7887":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-D5234CFF6B2C514C67CA7887","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-DC3612A9EEBCACBD7708CC0E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DC3612A9EEBCACBD7708CC0E","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":15000},"EVID-DCD165B1F77962F8297C7F4D":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DCD165B1F77962F8297C7F4D","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":12.0}}</t>
+          <t>{"EVID-120A7F0AFA3DF21C0BF51872":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-120A7F0AFA3DF21C0BF51872","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":36000.0},"EVID-1A9FB4971218B885A774B43B":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-1A9FB4971218B885A774B43B","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-3E3D4D117F217EA7DB1596CE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3E3D4D117F217EA7DB1596CE","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-4CD8C8C1F0430C6A0156057C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4CD8C8C1F0430C6A0156057C","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3600},"EVID-5559E287993BB07DE138FDF6":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-5559E287993BB07DE138FDF6","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-943CC5DA406961E6EB3068F0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-943CC5DA406961E6EB3068F0","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-A3FFF81B3A1797CA534E3F69":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-A3FFF81B3A1797CA534E3F69","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-D5234CFF6B2C514C67CA7887":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-D5234CFF6B2C514C67CA7887","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-DC3612A9EEBCACBD7708CC0E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DC3612A9EEBCACBD7708CC0E","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":15000},"EVID-DCD165B1F77962F8297C7F4D":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-DCD165B1F77962F8297C7F4D","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":12.0}}</t>
         </is>
       </c>
       <c r="AV24" s="22" t="inlineStr">
@@ -18312,12 +18312,12 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>CAND-2132EFA0CCC25A00B16EA2CF</t>
+          <t>CAND-6B2DDE23EC751D22DE4F7914</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -18497,12 +18497,12 @@
       </c>
       <c r="AT25" s="22" t="inlineStr">
         <is>
-          <t>["EVID-0CDFBA17157E22093D86EADE","EVID-B829726708E678EF6D0D4FFD","EVID-7C07E0575343482778154975","EVID-ED798F026DC7D4813C8D1BD7","EVID-CEF597117FDE03FC75D46082","EVID-C78D83012F1308C65615F356","EVID-91E83CACE07F654C8375E91B","EVID-679B0BB84F874895FE357CF9","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
+          <t>["EVID-0CDFBA17157E22093D86EADE","EVID-B829726708E678EF6D0D4FFD","EVID-7C07E0575343482778154975","EVID-ED798F026DC7D4813C8D1BD7","EVID-CEF597117FDE03FC75D46082","EVID-C78D83012F1308C65615F356","EVID-91E83CACE07F654C8375E91B","EVID-120A7F0AFA3DF21C0BF51872","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
         </is>
       </c>
       <c r="AU25" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0CDFBA17157E22093D86EADE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0CDFBA17157E22093D86EADE","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":2},"EVID-679B0BB84F874895FE357CF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-679B0BB84F874895FE357CF9","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-7C07E0575343482778154975":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-7C07E0575343482778154975","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":45.0},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-B829726708E678EF6D0D4FFD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B829726708E678EF6D0D4FFD","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C78D83012F1308C65615F356":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-C78D83012F1308C65615F356","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":65000},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-CEF597117FDE03FC75D46082":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-CEF597117FDE03FC75D46082","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":2160},"EVID-ED798F026DC7D4813C8D1BD7":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-ED798F026DC7D4813C8D1BD7","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":12.0}}</t>
+          <t>{"EVID-0CDFBA17157E22093D86EADE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0CDFBA17157E22093D86EADE","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":2},"EVID-120A7F0AFA3DF21C0BF51872":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-120A7F0AFA3DF21C0BF51872","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":36000.0},"EVID-7C07E0575343482778154975":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-7C07E0575343482778154975","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":45.0},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-B829726708E678EF6D0D4FFD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B829726708E678EF6D0D4FFD","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C78D83012F1308C65615F356":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-C78D83012F1308C65615F356","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":65000},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-CEF597117FDE03FC75D46082":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-CEF597117FDE03FC75D46082","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":2160},"EVID-ED798F026DC7D4813C8D1BD7":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-ED798F026DC7D4813C8D1BD7","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":12.0}}</t>
         </is>
       </c>
       <c r="AV25" s="22" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="AZ25" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY","scenario_id":"SCN-68E82895D5D2754159603420","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY","scenario_id":"SCN-268144CE4DBE7F2E116E140E","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA25" s="22" t="inlineStr">
@@ -18539,12 +18539,12 @@
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>CAND-8677BE4DC1B511B57B6B894C</t>
+          <t>CAND-73961AD4AD35D7CCF0FE42DD</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -18724,12 +18724,12 @@
       </c>
       <c r="AT26" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4D3A60329DCF7E143BD06023","EVID-4B254C8301F2AC01CC84CE76","EVID-CEB50ADB444DABFFABD2448A","EVID-8CF90399EB348CA2E57A41FC","EVID-E1011CEF886F3D479CF5E863","EVID-91E83CACE07F654C8375E91B","EVID-679B0BB84F874895FE357CF9","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
+          <t>["EVID-4D3A60329DCF7E143BD06023","EVID-4B254C8301F2AC01CC84CE76","EVID-CEB50ADB444DABFFABD2448A","EVID-8CF90399EB348CA2E57A41FC","EVID-E1011CEF886F3D479CF5E863","EVID-91E83CACE07F654C8375E91B","EVID-120A7F0AFA3DF21C0BF51872","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
         </is>
       </c>
       <c r="AU26" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-4B254C8301F2AC01CC84CE76":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-4B254C8301F2AC01CC84CE76","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":30.0},"EVID-4D3A60329DCF7E143BD06023":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4D3A60329DCF7E143BD06023","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-679B0BB84F874895FE357CF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-679B0BB84F874895FE357CF9","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-8CF90399EB348CA2E57A41FC":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-8CF90399EB348CA2E57A41FC","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":65000},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-CEB50ADB444DABFFABD2448A":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-CEB50ADB444DABFFABD2448A","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":12.0},"EVID-E1011CEF886F3D479CF5E863":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-E1011CEF886F3D479CF5E863","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":45.0}}</t>
+          <t>{"EVID-120A7F0AFA3DF21C0BF51872":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-120A7F0AFA3DF21C0BF51872","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":36000.0},"EVID-4B254C8301F2AC01CC84CE76":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-4B254C8301F2AC01CC84CE76","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":30.0},"EVID-4D3A60329DCF7E143BD06023":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4D3A60329DCF7E143BD06023","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-8CF90399EB348CA2E57A41FC":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-8CF90399EB348CA2E57A41FC","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":65000},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-CEB50ADB444DABFFABD2448A":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-CEB50ADB444DABFFABD2448A","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":12.0},"EVID-E1011CEF886F3D479CF5E863":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-E1011CEF886F3D479CF5E863","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":45.0}}</t>
         </is>
       </c>
       <c r="AV26" s="22" t="inlineStr">
@@ -18766,12 +18766,12 @@
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>CAND-E193BAA623F56B14C771BC33</t>
+          <t>CAND-FE18BD942E427F6BFF3FD25D</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -18951,12 +18951,12 @@
       </c>
       <c r="AT27" s="22" t="inlineStr">
         <is>
-          <t>["EVID-E14BE0884B6E34FCB998C395","EVID-E09FD1F994ABB868559DF515","EVID-E56F010E6353E5FD20061D06","EVID-753982E08475C2D3F33CAC84","EVID-A4F5DF730DDC736B98D2A1D2","EVID-947C133A7AF95BA119BCA9FF","EVID-8F4C40C92A48DE9D5B743C29","EVID-C5B21CB96D957B10D42BA42D","EVID-91E83CACE07F654C8375E91B","EVID-679B0BB84F874895FE357CF9","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
+          <t>["EVID-E14BE0884B6E34FCB998C395","EVID-E09FD1F994ABB868559DF515","EVID-E56F010E6353E5FD20061D06","EVID-753982E08475C2D3F33CAC84","EVID-A4F5DF730DDC736B98D2A1D2","EVID-947C133A7AF95BA119BCA9FF","EVID-8F4C40C92A48DE9D5B743C29","EVID-C5B21CB96D957B10D42BA42D","EVID-91E83CACE07F654C8375E91B","EVID-120A7F0AFA3DF21C0BF51872","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
         </is>
       </c>
       <c r="AU27" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-679B0BB84F874895FE357CF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-679B0BB84F874895FE357CF9","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-753982E08475C2D3F33CAC84":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-753982E08475C2D3F33CAC84","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-8F4C40C92A48DE9D5B743C29":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-8F4C40C92A48DE9D5B743C29","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1333},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-947C133A7AF95BA119BCA9FF":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-947C133A7AF95BA119BCA9FF","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-A4F5DF730DDC736B98D2A1D2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A4F5DF730DDC736B98D2A1D2","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":4},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C5B21CB96D957B10D42BA42D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C5B21CB96D957B10D42BA42D","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1200.0},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-E09FD1F994ABB868559DF515":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E09FD1F994ABB868559DF515","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":600.0},"EVID-E14BE0884B6E34FCB998C395":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-E14BE0884B6E34FCB998C395","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":45,"unit":"minutes","value":30},"EVID-E56F010E6353E5FD20061D06":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-E56F010E6353E5FD20061D06","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":720}}</t>
+          <t>{"EVID-120A7F0AFA3DF21C0BF51872":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-120A7F0AFA3DF21C0BF51872","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":36000.0},"EVID-753982E08475C2D3F33CAC84":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-753982E08475C2D3F33CAC84","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-8F4C40C92A48DE9D5B743C29":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-8F4C40C92A48DE9D5B743C29","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1333},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-947C133A7AF95BA119BCA9FF":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-947C133A7AF95BA119BCA9FF","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-A4F5DF730DDC736B98D2A1D2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A4F5DF730DDC736B98D2A1D2","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":4},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C5B21CB96D957B10D42BA42D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C5B21CB96D957B10D42BA42D","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1200.0},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-E09FD1F994ABB868559DF515":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E09FD1F994ABB868559DF515","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":600.0},"EVID-E14BE0884B6E34FCB998C395":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-E14BE0884B6E34FCB998C395","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":45,"unit":"minutes","value":30},"EVID-E56F010E6353E5FD20061D06":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-E56F010E6353E5FD20061D06","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":720}}</t>
         </is>
       </c>
       <c r="AV27" s="22" t="inlineStr">
@@ -18993,12 +18993,12 @@
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>PKG-4480611178CF570394C7DA7A</t>
+          <t>PKG-0B783AA69A5D8DC9AEACA574</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>CAND-A64CA3E68A669D150AAA07D6</t>
+          <t>CAND-05E76611FED4F59744C22AB8</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
@@ -19182,12 +19182,12 @@
       </c>
       <c r="AT28" s="22" t="inlineStr">
         <is>
-          <t>["EVID-33BB28CF6EC356A46BE6650D","EVID-35B29B2F02D863EAADFD08F3","EVID-11B2E705A613CE480286F6F3","EVID-57F17FFFCFEDA0A9A60A1FD8","EVID-358F61DFBB7111D4CFD58A1A","EVID-5427DFBFB88B9EBFC0C27786","EVID-081574EC86CCBD9D2F1F4CA7","EVID-57741F660C40486486D51EFB","EVID-28D2862523167B2FE81853B6","EVID-E9801B0191E0C020D4E6D167","EVID-F76F8313D068DA94D8D128E3","EVID-D8ED1DBE0C9CA9FD5031A804","EVID-A64BE1A219A5E17C9CF9589A","EVID-91E83CACE07F654C8375E91B","EVID-679B0BB84F874895FE357CF9","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
+          <t>["EVID-33BB28CF6EC356A46BE6650D","EVID-35B29B2F02D863EAADFD08F3","EVID-11B2E705A613CE480286F6F3","EVID-57F17FFFCFEDA0A9A60A1FD8","EVID-358F61DFBB7111D4CFD58A1A","EVID-5427DFBFB88B9EBFC0C27786","EVID-081574EC86CCBD9D2F1F4CA7","EVID-57741F660C40486486D51EFB","EVID-28D2862523167B2FE81853B6","EVID-E9801B0191E0C020D4E6D167","EVID-F76F8313D068DA94D8D128E3","EVID-D8ED1DBE0C9CA9FD5031A804","EVID-A64BE1A219A5E17C9CF9589A","EVID-91E83CACE07F654C8375E91B","EVID-120A7F0AFA3DF21C0BF51872","EVID-BC390FACE6BB107FDA76E438","EVID-C9561CB7C3F62405C4518E23"]</t>
         </is>
       </c>
       <c r="AU28" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-081574EC86CCBD9D2F1F4CA7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-081574EC86CCBD9D2F1F4CA7","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-11B2E705A613CE480286F6F3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-11B2E705A613CE480286F6F3","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-28D2862523167B2FE81853B6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-28D2862523167B2FE81853B6","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1440},"EVID-33BB28CF6EC356A46BE6650D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-33BB28CF6EC356A46BE6650D","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-358F61DFBB7111D4CFD58A1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-358F61DFBB7111D4CFD58A1A","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-35B29B2F02D863EAADFD08F3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-35B29B2F02D863EAADFD08F3","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-5427DFBFB88B9EBFC0C27786":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5427DFBFB88B9EBFC0C27786","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-57741F660C40486486D51EFB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-57741F660C40486486D51EFB","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-57F17FFFCFEDA0A9A60A1FD8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-57F17FFFCFEDA0A9A60A1FD8","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":13500},"EVID-679B0BB84F874895FE357CF9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-679B0BB84F874895FE357CF9","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":36000.0},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-A64BE1A219A5E17C9CF9589A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A64BE1A219A5E17C9CF9589A","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-D8ED1DBE0C9CA9FD5031A804":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D8ED1DBE0C9CA9FD5031A804","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-E9801B0191E0C020D4E6D167":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E9801B0191E0C020D4E6D167","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":4500},"EVID-F76F8313D068DA94D8D128E3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F76F8313D068DA94D8D128E3","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0}}</t>
+          <t>{"EVID-081574EC86CCBD9D2F1F4CA7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-081574EC86CCBD9D2F1F4CA7","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-11B2E705A613CE480286F6F3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-11B2E705A613CE480286F6F3","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-120A7F0AFA3DF21C0BF51872":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-120A7F0AFA3DF21C0BF51872","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":36000.0},"EVID-28D2862523167B2FE81853B6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-28D2862523167B2FE81853B6","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1440},"EVID-33BB28CF6EC356A46BE6650D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-33BB28CF6EC356A46BE6650D","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-358F61DFBB7111D4CFD58A1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-358F61DFBB7111D4CFD58A1A","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-35B29B2F02D863EAADFD08F3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-35B29B2F02D863EAADFD08F3","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-5427DFBFB88B9EBFC0C27786":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5427DFBFB88B9EBFC0C27786","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-57741F660C40486486D51EFB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-57741F660C40486486D51EFB","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-57F17FFFCFEDA0A9A60A1FD8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-57F17FFFCFEDA0A9A60A1FD8","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":13500},"EVID-91E83CACE07F654C8375E91B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91E83CACE07F654C8375E91B","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":31680.0},"EVID-A64BE1A219A5E17C9CF9589A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A64BE1A219A5E17C9CF9589A","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-BC390FACE6BB107FDA76E438":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC390FACE6BB107FDA76E438","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5380.16},"EVID-C9561CB7C3F62405C4518E23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C9561CB7C3F62405C4518E23","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":254},"EVID-D8ED1DBE0C9CA9FD5031A804":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D8ED1DBE0C9CA9FD5031A804","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-E9801B0191E0C020D4E6D167":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E9801B0191E0C020D4E6D167","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":4500},"EVID-F76F8313D068DA94D8D128E3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F76F8313D068DA94D8D128E3","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV28" s="22" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="AZ28" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-EC35EE7A8A459E1030386BDF","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-7541A4581D52616B7887204B","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA28" s="22" t="inlineStr">
@@ -19224,12 +19224,12 @@
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>CAND-2A21A45EFF69356D0EDB4F30</t>
+          <t>CAND-2DC77701D9463A039A4A3430</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -19413,12 +19413,12 @@
       </c>
       <c r="AT29" s="22" t="inlineStr">
         <is>
-          <t>["EVID-F06620CFA61363C1EB9B89DC","EVID-44397AB78F278179197384EA","EVID-673C5350CF07282A55EA50CF","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
+          <t>["EVID-F06620CFA61363C1EB9B89DC","EVID-44397AB78F278179197384EA","EVID-97CE51EBFF3652C229CC3237","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
         </is>
       </c>
       <c r="AU29" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-673C5350CF07282A55EA50CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-673C5350CF07282A55EA50CF","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-F06620CFA61363C1EB9B89DC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F06620CFA61363C1EB9B89DC","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
+          <t>{"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-97CE51EBFF3652C229CC3237":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-97CE51EBFF3652C229CC3237","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":18000.0},"EVID-F06620CFA61363C1EB9B89DC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F06620CFA61363C1EB9B89DC","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
         </is>
       </c>
       <c r="AV29" s="22" t="inlineStr">
@@ -19455,12 +19455,12 @@
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>CAND-AB3963A519CBBB85D39C5C32</t>
+          <t>CAND-BA05FACF1A2AF701F6188BBC</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -19644,12 +19644,12 @@
       </c>
       <c r="AT30" s="22" t="inlineStr">
         <is>
-          <t>["EVID-08358BCEEA08EE19FE1FBAA3","EVID-B566F403908A6960BED17E0C","EVID-197A8C457D558504B0E953FA","EVID-E84E8CD881597CF3498F5149","EVID-4CA277CD5E12D2564A4386D8","EVID-D4AA5B75F719775A0DE24274","EVID-0F38E2F7D06930B4B0B76120","EVID-01F71FB33E6FD6577DC5BBB0","EVID-49AC15C11B05FE0E025B4079","EVID-44397AB78F278179197384EA","EVID-673C5350CF07282A55EA50CF","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
+          <t>["EVID-08358BCEEA08EE19FE1FBAA3","EVID-B566F403908A6960BED17E0C","EVID-197A8C457D558504B0E953FA","EVID-E84E8CD881597CF3498F5149","EVID-4CA277CD5E12D2564A4386D8","EVID-D4AA5B75F719775A0DE24274","EVID-0F38E2F7D06930B4B0B76120","EVID-01F71FB33E6FD6577DC5BBB0","EVID-49AC15C11B05FE0E025B4079","EVID-44397AB78F278179197384EA","EVID-97CE51EBFF3652C229CC3237","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
         </is>
       </c>
       <c r="AU30" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-01F71FB33E6FD6577DC5BBB0":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-01F71FB33E6FD6577DC5BBB0","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7000},"EVID-08358BCEEA08EE19FE1FBAA3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-08358BCEEA08EE19FE1FBAA3","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-0F38E2F7D06930B4B0B76120":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0F38E2F7D06930B4B0B76120","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2200},"EVID-197A8C457D558504B0E953FA":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-197A8C457D558504B0E953FA","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-49AC15C11B05FE0E025B4079":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-49AC15C11B05FE0E025B4079","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-4CA277CD5E12D2564A4386D8":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4CA277CD5E12D2564A4386D8","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.2},"EVID-673C5350CF07282A55EA50CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-673C5350CF07282A55EA50CF","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-B566F403908A6960BED17E0C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-B566F403908A6960BED17E0C","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D4AA5B75F719775A0DE24274":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D4AA5B75F719775A0DE24274","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-E84E8CD881597CF3498F5149":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-E84E8CD881597CF3498F5149","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
+          <t>{"EVID-01F71FB33E6FD6577DC5BBB0":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-01F71FB33E6FD6577DC5BBB0","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7000},"EVID-08358BCEEA08EE19FE1FBAA3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-08358BCEEA08EE19FE1FBAA3","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-0F38E2F7D06930B4B0B76120":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0F38E2F7D06930B4B0B76120","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2200},"EVID-197A8C457D558504B0E953FA":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-197A8C457D558504B0E953FA","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-49AC15C11B05FE0E025B4079":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-49AC15C11B05FE0E025B4079","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-4CA277CD5E12D2564A4386D8":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-4CA277CD5E12D2564A4386D8","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.2},"EVID-97CE51EBFF3652C229CC3237":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-97CE51EBFF3652C229CC3237","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":18000.0},"EVID-B566F403908A6960BED17E0C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-B566F403908A6960BED17E0C","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D4AA5B75F719775A0DE24274":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D4AA5B75F719775A0DE24274","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-E84E8CD881597CF3498F5149":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-E84E8CD881597CF3498F5149","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
         </is>
       </c>
       <c r="AV30" s="22" t="inlineStr">
@@ -19674,7 +19674,7 @@
       </c>
       <c r="AZ30" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-819DAEDF07A8F0192D7A247C","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-434C077126B079E5142CDF8C","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA30" s="22" t="inlineStr">
@@ -19686,12 +19686,12 @@
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>CAND-04FD915BC6811A9ABF866B65</t>
+          <t>CAND-4701F5AB0B552D8BE3E4E34C</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -19871,12 +19871,12 @@
       </c>
       <c r="AT31" s="22" t="inlineStr">
         <is>
-          <t>["EVID-143518477975AC9C25611AB6","EVID-EEB8E13A0DB907A0E6067CAA","EVID-58AAD17D87FDB89D4BE902B2","EVID-8867C09103F24942A1655AA8","EVID-5B682EEE7197C853378411F5","EVID-7D4E39BC0F2BDAAF60D528F0","EVID-44397AB78F278179197384EA","EVID-673C5350CF07282A55EA50CF","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
+          <t>["EVID-143518477975AC9C25611AB6","EVID-EEB8E13A0DB907A0E6067CAA","EVID-58AAD17D87FDB89D4BE902B2","EVID-8867C09103F24942A1655AA8","EVID-5B682EEE7197C853378411F5","EVID-7D4E39BC0F2BDAAF60D528F0","EVID-44397AB78F278179197384EA","EVID-97CE51EBFF3652C229CC3237","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
         </is>
       </c>
       <c r="AU31" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-143518477975AC9C25611AB6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-143518477975AC9C25611AB6","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-58AAD17D87FDB89D4BE902B2":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-58AAD17D87FDB89D4BE902B2","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":1.0},"EVID-5B682EEE7197C853378411F5":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-5B682EEE7197C853378411F5","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":18},"EVID-673C5350CF07282A55EA50CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-673C5350CF07282A55EA50CF","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-7D4E39BC0F2BDAAF60D528F0":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-7D4E39BC0F2BDAAF60D528F0","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":1000},"EVID-8867C09103F24942A1655AA8":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-8867C09103F24942A1655AA8","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.2},"EVID-EEB8E13A0DB907A0E6067CAA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EEB8E13A0DB907A0E6067CAA","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
+          <t>{"EVID-143518477975AC9C25611AB6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-143518477975AC9C25611AB6","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-58AAD17D87FDB89D4BE902B2":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-58AAD17D87FDB89D4BE902B2","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":1.0},"EVID-5B682EEE7197C853378411F5":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-5B682EEE7197C853378411F5","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":18},"EVID-7D4E39BC0F2BDAAF60D528F0":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-7D4E39BC0F2BDAAF60D528F0","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":1000},"EVID-8867C09103F24942A1655AA8":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-8867C09103F24942A1655AA8","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.2},"EVID-97CE51EBFF3652C229CC3237":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-97CE51EBFF3652C229CC3237","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":18000.0},"EVID-EEB8E13A0DB907A0E6067CAA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EEB8E13A0DB907A0E6067CAA","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
         </is>
       </c>
       <c r="AV31" s="22" t="inlineStr">
@@ -19901,7 +19901,7 @@
       </c>
       <c r="AZ31" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-819DAEDF07A8F0192D7A247C","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-434C077126B079E5142CDF8C","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA31" s="22" t="inlineStr">
@@ -19913,12 +19913,12 @@
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>CAND-441EF1F7D10C5596117E1DEB</t>
+          <t>CAND-27600366920A82E7674E3D7A</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -20098,12 +20098,12 @@
       </c>
       <c r="AT32" s="22" t="inlineStr">
         <is>
-          <t>["EVID-604AC4779AD4C783C7EFA4CC","EVID-36F22BE2CCDB16F3AD7E178F","EVID-8F84F05872E6435005166D8D","EVID-BBD71C8135AF7545976EE916","EVID-8A99CBFA2631BA084AEDDF22","EVID-44397AB78F278179197384EA","EVID-673C5350CF07282A55EA50CF","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
+          <t>["EVID-604AC4779AD4C783C7EFA4CC","EVID-36F22BE2CCDB16F3AD7E178F","EVID-8F84F05872E6435005166D8D","EVID-BBD71C8135AF7545976EE916","EVID-8A99CBFA2631BA084AEDDF22","EVID-44397AB78F278179197384EA","EVID-97CE51EBFF3652C229CC3237","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
         </is>
       </c>
       <c r="AU32" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-36F22BE2CCDB16F3AD7E178F":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-36F22BE2CCDB16F3AD7E178F","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":62.0},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-604AC4779AD4C783C7EFA4CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-604AC4779AD4C783C7EFA4CC","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-673C5350CF07282A55EA50CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-673C5350CF07282A55EA50CF","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-8A99CBFA2631BA084AEDDF22":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-8A99CBFA2631BA084AEDDF22","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":1.0},"EVID-8F84F05872E6435005166D8D":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-8F84F05872E6435005166D8D","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.2},"EVID-BBD71C8135AF7545976EE916":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-BBD71C8135AF7545976EE916","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":1000},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
+          <t>{"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-36F22BE2CCDB16F3AD7E178F":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-36F22BE2CCDB16F3AD7E178F","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":62.0},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-604AC4779AD4C783C7EFA4CC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-604AC4779AD4C783C7EFA4CC","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-8A99CBFA2631BA084AEDDF22":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-8A99CBFA2631BA084AEDDF22","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":1.0},"EVID-8F84F05872E6435005166D8D":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-8F84F05872E6435005166D8D","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.2},"EVID-97CE51EBFF3652C229CC3237":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-97CE51EBFF3652C229CC3237","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":18000.0},"EVID-BBD71C8135AF7545976EE916":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-BBD71C8135AF7545976EE916","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":1000},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
         </is>
       </c>
       <c r="AV32" s="22" t="inlineStr">
@@ -20140,12 +20140,12 @@
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>CAND-94C56D19D728CCD8E36E75F2</t>
+          <t>CAND-8B9D97017D3CAA5DA66961BB</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -20325,12 +20325,12 @@
       </c>
       <c r="AT33" s="22" t="inlineStr">
         <is>
-          <t>["EVID-BFD933D03EDDB6B88F5B4CAF","EVID-7A6837724378711D474A758F","EVID-29E798CD3E14E9ED7476BC9B","EVID-95141085DD5DC4861990625B","EVID-62DB75214B161FAE24013595","EVID-8D939FBAAD70DE609CEEA32C","EVID-138128BA4272677A4B0AB7F4","EVID-00476B7B0F3D8275B2936132","EVID-44397AB78F278179197384EA","EVID-673C5350CF07282A55EA50CF","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
+          <t>["EVID-BFD933D03EDDB6B88F5B4CAF","EVID-7A6837724378711D474A758F","EVID-29E798CD3E14E9ED7476BC9B","EVID-95141085DD5DC4861990625B","EVID-62DB75214B161FAE24013595","EVID-8D939FBAAD70DE609CEEA32C","EVID-138128BA4272677A4B0AB7F4","EVID-00476B7B0F3D8275B2936132","EVID-44397AB78F278179197384EA","EVID-97CE51EBFF3652C229CC3237","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
         </is>
       </c>
       <c r="AU33" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00476B7B0F3D8275B2936132":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-00476B7B0F3D8275B2936132","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1728.0},"EVID-138128BA4272677A4B0AB7F4":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-138128BA4272677A4B0AB7F4","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2333},"EVID-29E798CD3E14E9ED7476BC9B":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-29E798CD3E14E9ED7476BC9B","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":360},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-62DB75214B161FAE24013595":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-62DB75214B161FAE24013595","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":7},"EVID-673C5350CF07282A55EA50CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-673C5350CF07282A55EA50CF","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-7A6837724378711D474A758F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A6837724378711D474A758F","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":300.0},"EVID-8D939FBAAD70DE609CEEA32C":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-8D939FBAAD70DE609CEEA32C","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-95141085DD5DC4861990625B":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-95141085DD5DC4861990625B","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-BFD933D03EDDB6B88F5B4CAF":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-BFD933D03EDDB6B88F5B4CAF","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":30},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
+          <t>{"EVID-00476B7B0F3D8275B2936132":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-00476B7B0F3D8275B2936132","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1728.0},"EVID-138128BA4272677A4B0AB7F4":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-138128BA4272677A4B0AB7F4","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2333},"EVID-29E798CD3E14E9ED7476BC9B":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-29E798CD3E14E9ED7476BC9B","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":360},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-62DB75214B161FAE24013595":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-62DB75214B161FAE24013595","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":7},"EVID-7A6837724378711D474A758F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A6837724378711D474A758F","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":300.0},"EVID-8D939FBAAD70DE609CEEA32C":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-8D939FBAAD70DE609CEEA32C","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-95141085DD5DC4861990625B":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-95141085DD5DC4861990625B","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-97CE51EBFF3652C229CC3237":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-97CE51EBFF3652C229CC3237","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":18000.0},"EVID-BFD933D03EDDB6B88F5B4CAF":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-BFD933D03EDDB6B88F5B4CAF","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":30},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242}}</t>
         </is>
       </c>
       <c r="AV33" s="22" t="inlineStr">
@@ -20367,12 +20367,12 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>PKG-C3150FAF84F8DD0C2EB22A52</t>
+          <t>PKG-6F21DD7A7F1C6FC940C8FC38</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>CAND-DBDB7630ED062E15E33B2B7A</t>
+          <t>CAND-2F116D492B169CDC7BFE4A4F</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -20556,12 +20556,12 @@
       </c>
       <c r="AT34" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4985D186823206E5659AD9FF","EVID-AFD7FB4C9DCB9C5F2EC567AE","EVID-2DF8660439C625CDBD529815","EVID-850D0D650424A506C00A22F9","EVID-623DCE1B20F50ED2CC8F4149","EVID-740D9017E7AC3B9814EF6F2B","EVID-0BA5CC7CA3B1F6049EB4670D","EVID-D1C799F1FF7272E4DA285A38","EVID-FE0CC0129747B52484AF90AA","EVID-AC243B02F6E32FEE516B7F1A","EVID-C7CC6C62FD487AC658763422","EVID-A8BFB204051100D76FD32275","EVID-7F91993E1D9D087F839A562B","EVID-44397AB78F278179197384EA","EVID-673C5350CF07282A55EA50CF","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
+          <t>["EVID-4985D186823206E5659AD9FF","EVID-AFD7FB4C9DCB9C5F2EC567AE","EVID-2DF8660439C625CDBD529815","EVID-850D0D650424A506C00A22F9","EVID-623DCE1B20F50ED2CC8F4149","EVID-740D9017E7AC3B9814EF6F2B","EVID-0BA5CC7CA3B1F6049EB4670D","EVID-D1C799F1FF7272E4DA285A38","EVID-FE0CC0129747B52484AF90AA","EVID-AC243B02F6E32FEE516B7F1A","EVID-C7CC6C62FD487AC658763422","EVID-A8BFB204051100D76FD32275","EVID-7F91993E1D9D087F839A562B","EVID-44397AB78F278179197384EA","EVID-97CE51EBFF3652C229CC3237","EVID-30E518A1606B6C1EDEC6D0A3","EVID-F7405E951F0792C6F09AD862"]</t>
         </is>
       </c>
       <c r="AU34" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0BA5CC7CA3B1F6049EB4670D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0BA5CC7CA3B1F6049EB4670D","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-2DF8660439C625CDBD529815":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2DF8660439C625CDBD529815","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-4985D186823206E5659AD9FF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4985D186823206E5659AD9FF","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-623DCE1B20F50ED2CC8F4149":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-623DCE1B20F50ED2CC8F4149","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-673C5350CF07282A55EA50CF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-673C5350CF07282A55EA50CF","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":18000.0},"EVID-740D9017E7AC3B9814EF6F2B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-740D9017E7AC3B9814EF6F2B","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-7F91993E1D9D087F839A562B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7F91993E1D9D087F839A562B","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-850D0D650424A506C00A22F9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-850D0D650424A506C00A22F9","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":6750},"EVID-A8BFB204051100D76FD32275":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A8BFB204051100D76FD32275","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-AC243B02F6E32FEE516B7F1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC243B02F6E32FEE516B7F1A","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":2250},"EVID-AFD7FB4C9DCB9C5F2EC567AE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AFD7FB4C9DCB9C5F2EC567AE","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-C7CC6C62FD487AC658763422":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C7CC6C62FD487AC658763422","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-D1C799F1FF7272E4DA285A38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D1C799F1FF7272E4DA285A38","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242},"EVID-FE0CC0129747B52484AF90AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FE0CC0129747B52484AF90AA","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":720}}</t>
+          <t>{"EVID-0BA5CC7CA3B1F6049EB4670D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0BA5CC7CA3B1F6049EB4670D","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-2DF8660439C625CDBD529815":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2DF8660439C625CDBD529815","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-30E518A1606B6C1EDEC6D0A3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30E518A1606B6C1EDEC6D0A3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5646.94},"EVID-44397AB78F278179197384EA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44397AB78F278179197384EA","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":15840.0},"EVID-4985D186823206E5659AD9FF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4985D186823206E5659AD9FF","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-623DCE1B20F50ED2CC8F4149":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-623DCE1B20F50ED2CC8F4149","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-740D9017E7AC3B9814EF6F2B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-740D9017E7AC3B9814EF6F2B","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-7F91993E1D9D087F839A562B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7F91993E1D9D087F839A562B","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-850D0D650424A506C00A22F9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-850D0D650424A506C00A22F9","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":6750},"EVID-97CE51EBFF3652C229CC3237":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-97CE51EBFF3652C229CC3237","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":18000.0},"EVID-A8BFB204051100D76FD32275":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A8BFB204051100D76FD32275","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-AC243B02F6E32FEE516B7F1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC243B02F6E32FEE516B7F1A","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":2250},"EVID-AFD7FB4C9DCB9C5F2EC567AE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AFD7FB4C9DCB9C5F2EC567AE","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-C7CC6C62FD487AC658763422":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C7CC6C62FD487AC658763422","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-D1C799F1FF7272E4DA285A38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D1C799F1FF7272E4DA285A38","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-F7405E951F0792C6F09AD862":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F7405E951F0792C6F09AD862","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":242},"EVID-FE0CC0129747B52484AF90AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FE0CC0129747B52484AF90AA","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":720}}</t>
         </is>
       </c>
       <c r="AV34" s="22" t="inlineStr">
@@ -20586,7 +20586,7 @@
       </c>
       <c r="AZ34" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-0C81CFCDAF78B26D6BFDAC1D","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-46131C6A05E4B40940D8714B","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA34" s="22" t="inlineStr">
@@ -20598,12 +20598,12 @@
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>CAND-539A61990AAE80EB5F7FEA28</t>
+          <t>CAND-4A1F51AB39038A7D21FFE467</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -20787,12 +20787,12 @@
       </c>
       <c r="AT35" s="22" t="inlineStr">
         <is>
-          <t>["EVID-BC2F2A3126DBAE90BE88DB4C","EVID-B5D676918ED2DA9FF88A6D1D","EVID-3423168674B585D72291AF40","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
+          <t>["EVID-BC2F2A3126DBAE90BE88DB4C","EVID-B5D676918ED2DA9FF88A6D1D","EVID-FDAAC0BC5E85652E7A547DED","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
         </is>
       </c>
       <c r="AU35" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-3423168674B585D72291AF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3423168674B585D72291AF40","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-BC2F2A3126DBAE90BE88DB4C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC2F2A3126DBAE90BE88DB4C","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"}}</t>
+          <t>{"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-BC2F2A3126DBAE90BE88DB4C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BC2F2A3126DBAE90BE88DB4C","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-FDAAC0BC5E85652E7A547DED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FDAAC0BC5E85652E7A547DED","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":14500.0}}</t>
         </is>
       </c>
       <c r="AV35" s="22" t="inlineStr">
@@ -20829,12 +20829,12 @@
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>CAND-91BB40F77CB18835E431CCE6</t>
+          <t>CAND-5021E6E6585A4FEE342CB4BB</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -21018,12 +21018,12 @@
       </c>
       <c r="AT36" s="22" t="inlineStr">
         <is>
-          <t>["EVID-45C4272AA3511B69A47B5B6A","EVID-C94B20B41C675AC388CC8348","EVID-2F27CB2083773BD3028BCFA7","EVID-3A74C56DDC296093EECF0652","EVID-32C2CD35574FD6E3A50F0D21","EVID-0D702A232EC127629AA49DFE","EVID-EF86C7A16AAF04754D43BD71","EVID-8C03476C65C1A1FCE93F5FB5","EVID-B21546F751C7C8A3A49A2CE3","EVID-B5D676918ED2DA9FF88A6D1D","EVID-3423168674B585D72291AF40","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
+          <t>["EVID-45C4272AA3511B69A47B5B6A","EVID-C94B20B41C675AC388CC8348","EVID-2F27CB2083773BD3028BCFA7","EVID-3A74C56DDC296093EECF0652","EVID-32C2CD35574FD6E3A50F0D21","EVID-0D702A232EC127629AA49DFE","EVID-EF86C7A16AAF04754D43BD71","EVID-8C03476C65C1A1FCE93F5FB5","EVID-B21546F751C7C8A3A49A2CE3","EVID-B5D676918ED2DA9FF88A6D1D","EVID-FDAAC0BC5E85652E7A547DED","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
         </is>
       </c>
       <c r="AU36" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0D702A232EC127629AA49DFE":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0D702A232EC127629AA49DFE","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-2F27CB2083773BD3028BCFA7":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2F27CB2083773BD3028BCFA7","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-32C2CD35574FD6E3A50F0D21":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-32C2CD35574FD6E3A50F0D21","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-3423168674B585D72291AF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3423168674B585D72291AF40","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-3A74C56DDC296093EECF0652":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-3A74C56DDC296093EECF0652","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-45C4272AA3511B69A47B5B6A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-45C4272AA3511B69A47B5B6A","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-8C03476C65C1A1FCE93F5FB5":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-8C03476C65C1A1FCE93F5FB5","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":11000},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B21546F751C7C8A3A49A2CE3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B21546F751C7C8A3A49A2CE3","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-C94B20B41C675AC388CC8348":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-C94B20B41C675AC388CC8348","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-EF86C7A16AAF04754D43BD71":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF86C7A16AAF04754D43BD71","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2800}}</t>
+          <t>{"EVID-0D702A232EC127629AA49DFE":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0D702A232EC127629AA49DFE","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-2F27CB2083773BD3028BCFA7":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-2F27CB2083773BD3028BCFA7","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-32C2CD35574FD6E3A50F0D21":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-32C2CD35574FD6E3A50F0D21","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-3A74C56DDC296093EECF0652":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-3A74C56DDC296093EECF0652","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-45C4272AA3511B69A47B5B6A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-45C4272AA3511B69A47B5B6A","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-8C03476C65C1A1FCE93F5FB5":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-8C03476C65C1A1FCE93F5FB5","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":11000},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B21546F751C7C8A3A49A2CE3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B21546F751C7C8A3A49A2CE3","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-C94B20B41C675AC388CC8348":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-C94B20B41C675AC388CC8348","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-EF86C7A16AAF04754D43BD71":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF86C7A16AAF04754D43BD71","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2800},"EVID-FDAAC0BC5E85652E7A547DED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FDAAC0BC5E85652E7A547DED","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":14500.0}}</t>
         </is>
       </c>
       <c r="AV36" s="22" t="inlineStr">
@@ -21048,7 +21048,7 @@
       </c>
       <c r="AZ36" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-FFA03F647640FAFA848CFDF5","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-C3C9758E12BA36251A7A8421","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA36" s="22" t="inlineStr">
@@ -21060,12 +21060,12 @@
     <row r="37" ht="32" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>CAND-9B652249BD980BF64F75C35A</t>
+          <t>CAND-3CDD1DCF71D56AF9C3F59C6F</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -21245,12 +21245,12 @@
       </c>
       <c r="AT37" s="22" t="inlineStr">
         <is>
-          <t>["EVID-F97697F36DAAB95BEA42DFBC","EVID-D89261AA21BB363F17428F63","EVID-086E9F10584C5D0E6D857229","EVID-7C54411923FB6D23463A13EC","EVID-3F89F4000A47FE9CCF922B1E","EVID-EBE1AA8740CF77C3D09FD892","EVID-B5D676918ED2DA9FF88A6D1D","EVID-3423168674B585D72291AF40","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
+          <t>["EVID-F97697F36DAAB95BEA42DFBC","EVID-D89261AA21BB363F17428F63","EVID-086E9F10584C5D0E6D857229","EVID-7C54411923FB6D23463A13EC","EVID-3F89F4000A47FE9CCF922B1E","EVID-EBE1AA8740CF77C3D09FD892","EVID-B5D676918ED2DA9FF88A6D1D","EVID-FDAAC0BC5E85652E7A547DED","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
         </is>
       </c>
       <c r="AU37" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-086E9F10584C5D0E6D857229":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-086E9F10584C5D0E6D857229","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-3423168674B585D72291AF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3423168674B585D72291AF40","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-3F89F4000A47FE9CCF922B1E":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-3F89F4000A47FE9CCF922B1E","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-7C54411923FB6D23463A13EC":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-7C54411923FB6D23463A13EC","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-D89261AA21BB363F17428F63":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D89261AA21BB363F17428F63","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":1},"EVID-EBE1AA8740CF77C3D09FD892":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-EBE1AA8740CF77C3D09FD892","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-F97697F36DAAB95BEA42DFBC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F97697F36DAAB95BEA42DFBC","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":3}}</t>
+          <t>{"EVID-086E9F10584C5D0E6D857229":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-086E9F10584C5D0E6D857229","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-3F89F4000A47FE9CCF922B1E":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-3F89F4000A47FE9CCF922B1E","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-7C54411923FB6D23463A13EC":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-7C54411923FB6D23463A13EC","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-D89261AA21BB363F17428F63":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D89261AA21BB363F17428F63","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":1},"EVID-EBE1AA8740CF77C3D09FD892":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-EBE1AA8740CF77C3D09FD892","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-F97697F36DAAB95BEA42DFBC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F97697F36DAAB95BEA42DFBC","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":3},"EVID-FDAAC0BC5E85652E7A547DED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FDAAC0BC5E85652E7A547DED","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":14500.0}}</t>
         </is>
       </c>
       <c r="AV37" s="22" t="inlineStr">
@@ -21275,7 +21275,7 @@
       </c>
       <c r="AZ37" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-FFA03F647640FAFA848CFDF5","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-C3C9758E12BA36251A7A8421","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA37" s="22" t="inlineStr">
@@ -21287,12 +21287,12 @@
     <row r="38" ht="32" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>CAND-941E7EE62D080D90E6C38505</t>
+          <t>CAND-70CACBDA2D7EC45AA36032AE</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -21472,12 +21472,12 @@
       </c>
       <c r="AT38" s="22" t="inlineStr">
         <is>
-          <t>["EVID-9223F725D7B62642F79C74BE","EVID-3119B00455317B76FC9BAA56","EVID-F60B902C091A7275F66D6800","EVID-FBE987F7046EE4D3FB3A43E3","EVID-3AEA4349F78415A6D5F2A5AF","EVID-B5D676918ED2DA9FF88A6D1D","EVID-3423168674B585D72291AF40","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
+          <t>["EVID-9223F725D7B62642F79C74BE","EVID-3119B00455317B76FC9BAA56","EVID-F60B902C091A7275F66D6800","EVID-FBE987F7046EE4D3FB3A43E3","EVID-3AEA4349F78415A6D5F2A5AF","EVID-B5D676918ED2DA9FF88A6D1D","EVID-FDAAC0BC5E85652E7A547DED","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
         </is>
       </c>
       <c r="AU38" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-3119B00455317B76FC9BAA56":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-3119B00455317B76FC9BAA56","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":55.0},"EVID-3423168674B585D72291AF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3423168674B585D72291AF40","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-3AEA4349F78415A6D5F2A5AF":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-3AEA4349F78415A6D5F2A5AF","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-9223F725D7B62642F79C74BE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9223F725D7B62642F79C74BE","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-F60B902C091A7275F66D6800":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-F60B902C091A7275F66D6800","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-FBE987F7046EE4D3FB3A43E3":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-FBE987F7046EE4D3FB3A43E3","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0}}</t>
+          <t>{"EVID-3119B00455317B76FC9BAA56":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-3119B00455317B76FC9BAA56","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":55.0},"EVID-3AEA4349F78415A6D5F2A5AF":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-3AEA4349F78415A6D5F2A5AF","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-9223F725D7B62642F79C74BE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9223F725D7B62642F79C74BE","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-F60B902C091A7275F66D6800":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-F60B902C091A7275F66D6800","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-FBE987F7046EE4D3FB3A43E3":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-FBE987F7046EE4D3FB3A43E3","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-FDAAC0BC5E85652E7A547DED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FDAAC0BC5E85652E7A547DED","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":14500.0}}</t>
         </is>
       </c>
       <c r="AV38" s="22" t="inlineStr">
@@ -21514,12 +21514,12 @@
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>CAND-912302CE7FA8ECEADF68A266</t>
+          <t>CAND-1CDA6A7761D3E39DAA39959D</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -21699,12 +21699,12 @@
       </c>
       <c r="AT39" s="22" t="inlineStr">
         <is>
-          <t>["EVID-E64F9D530A85A59E200D0361","EVID-69E5E89F43AFCABAB7C89422","EVID-5A333AAE306257AB660C6EF1","EVID-10DD8E20CFD0843967535C3D","EVID-F92148DD59D012DE5D45E077","EVID-C28DA97AA52F62A75E31930A","EVID-88E6B93132F288B55F9EB1C7","EVID-3AC8106EC1B53C26EA9AFFF3","EVID-B5D676918ED2DA9FF88A6D1D","EVID-3423168674B585D72291AF40","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
+          <t>["EVID-E64F9D530A85A59E200D0361","EVID-69E5E89F43AFCABAB7C89422","EVID-5A333AAE306257AB660C6EF1","EVID-10DD8E20CFD0843967535C3D","EVID-F92148DD59D012DE5D45E077","EVID-C28DA97AA52F62A75E31930A","EVID-88E6B93132F288B55F9EB1C7","EVID-3AC8106EC1B53C26EA9AFFF3","EVID-B5D676918ED2DA9FF88A6D1D","EVID-FDAAC0BC5E85652E7A547DED","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
         </is>
       </c>
       <c r="AU39" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-10DD8E20CFD0843967535C3D":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-10DD8E20CFD0843967535C3D","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":20000.0},"EVID-3423168674B585D72291AF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3423168674B585D72291AF40","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-3AC8106EC1B53C26EA9AFFF3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3AC8106EC1B53C26EA9AFFF3","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":10120.0},"EVID-5A333AAE306257AB660C6EF1":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-5A333AAE306257AB660C6EF1","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":36},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-69E5E89F43AFCABAB7C89422":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-69E5E89F43AFCABAB7C89422","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":30.0},"EVID-88E6B93132F288B55F9EB1C7":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-88E6B93132F288B55F9EB1C7","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-C28DA97AA52F62A75E31930A":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-C28DA97AA52F62A75E31930A","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-E64F9D530A85A59E200D0361":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-E64F9D530A85A59E200D0361","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":15,"unit":"minutes","value":120},"EVID-F92148DD59D012DE5D45E077":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F92148DD59D012DE5D45E077","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5}}</t>
+          <t>{"EVID-10DD8E20CFD0843967535C3D":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-10DD8E20CFD0843967535C3D","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":20000.0},"EVID-3AC8106EC1B53C26EA9AFFF3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3AC8106EC1B53C26EA9AFFF3","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":10120.0},"EVID-5A333AAE306257AB660C6EF1":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-5A333AAE306257AB660C6EF1","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":36},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-69E5E89F43AFCABAB7C89422":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-69E5E89F43AFCABAB7C89422","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":30.0},"EVID-88E6B93132F288B55F9EB1C7":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-88E6B93132F288B55F9EB1C7","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-C28DA97AA52F62A75E31930A":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-C28DA97AA52F62A75E31930A","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-E64F9D530A85A59E200D0361":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-E64F9D530A85A59E200D0361","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":15,"unit":"minutes","value":120},"EVID-F92148DD59D012DE5D45E077":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F92148DD59D012DE5D45E077","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-FDAAC0BC5E85652E7A547DED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FDAAC0BC5E85652E7A547DED","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":14500.0}}</t>
         </is>
       </c>
       <c r="AV39" s="22" t="inlineStr">
@@ -21729,7 +21729,7 @@
       </c>
       <c r="AZ39" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-FFA03F647640FAFA848CFDF5","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-C3C9758E12BA36251A7A8421","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA39" s="22" t="inlineStr">
@@ -21741,12 +21741,12 @@
     <row r="40" ht="32" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>PKG-D5BFB48E58D332977F8CE631</t>
+          <t>PKG-846B267BD2FF22780966979F</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>CAND-2CBB771D8661A0443D52D973</t>
+          <t>CAND-1FAD9418FB980278274923BD</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
@@ -21930,12 +21930,12 @@
       </c>
       <c r="AT40" s="22" t="inlineStr">
         <is>
-          <t>["EVID-E436F2B99029CFFC1A356400","EVID-7A0DB47C7FA59832F2B414AD","EVID-E32751AAF6F198EC3ABDE795","EVID-004F3A89FEF01598F8C11996","EVID-AE75973FFC8EE1632018BC85","EVID-C721CB58A713E142353C518C","EVID-932F65A95D13BD774AC110D4","EVID-088D18F498BE6F6075DD5EE7","EVID-2569CCF4C70D2EC05D37B00E","EVID-B91AB0D86D5DD19043793E83","EVID-AF646F8CF6ACFB35721CE7A5","EVID-AC85EC83EF0D7DA5FBE17B45","EVID-466B497A774CAF498A6BA9B6","EVID-B5D676918ED2DA9FF88A6D1D","EVID-3423168674B585D72291AF40","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
+          <t>["EVID-E436F2B99029CFFC1A356400","EVID-7A0DB47C7FA59832F2B414AD","EVID-E32751AAF6F198EC3ABDE795","EVID-004F3A89FEF01598F8C11996","EVID-AE75973FFC8EE1632018BC85","EVID-C721CB58A713E142353C518C","EVID-932F65A95D13BD774AC110D4","EVID-088D18F498BE6F6075DD5EE7","EVID-2569CCF4C70D2EC05D37B00E","EVID-B91AB0D86D5DD19043793E83","EVID-AF646F8CF6ACFB35721CE7A5","EVID-AC85EC83EF0D7DA5FBE17B45","EVID-466B497A774CAF498A6BA9B6","EVID-B5D676918ED2DA9FF88A6D1D","EVID-FDAAC0BC5E85652E7A547DED","EVID-95E864FEF55573BF9580AC47","EVID-68D1E890FA429A7A1DFE9334"]</t>
         </is>
       </c>
       <c r="AU40" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-004F3A89FEF01598F8C11996":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-004F3A89FEF01598F8C11996","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-088D18F498BE6F6075DD5EE7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-088D18F498BE6F6075DD5EE7","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-2569CCF4C70D2EC05D37B00E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2569CCF4C70D2EC05D37B00E","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":72},"EVID-3423168674B585D72291AF40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3423168674B585D72291AF40","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":14500.0},"EVID-466B497A774CAF498A6BA9B6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-466B497A774CAF498A6BA9B6","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-7A0DB47C7FA59832F2B414AD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A0DB47C7FA59832F2B414AD","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-932F65A95D13BD774AC110D4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-932F65A95D13BD774AC110D4","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-AC85EC83EF0D7DA5FBE17B45":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC85EC83EF0D7DA5FBE17B45","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-AE75973FFC8EE1632018BC85":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AE75973FFC8EE1632018BC85","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-AF646F8CF6ACFB35721CE7A5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AF646F8CF6ACFB35721CE7A5","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-B91AB0D86D5DD19043793E83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B91AB0D86D5DD19043793E83","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-C721CB58A713E142353C518C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C721CB58A713E142353C518C","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":675},"EVID-E32751AAF6F198EC3ABDE795":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E32751AAF6F198EC3ABDE795","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-E436F2B99029CFFC1A356400":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E436F2B99029CFFC1A356400","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"}}</t>
+          <t>{"EVID-004F3A89FEF01598F8C11996":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-004F3A89FEF01598F8C11996","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-088D18F498BE6F6075DD5EE7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-088D18F498BE6F6075DD5EE7","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-2569CCF4C70D2EC05D37B00E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2569CCF4C70D2EC05D37B00E","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":72},"EVID-466B497A774CAF498A6BA9B6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-466B497A774CAF498A6BA9B6","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-68D1E890FA429A7A1DFE9334":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68D1E890FA429A7A1DFE9334","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":228},"EVID-7A0DB47C7FA59832F2B414AD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7A0DB47C7FA59832F2B414AD","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-932F65A95D13BD774AC110D4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-932F65A95D13BD774AC110D4","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-95E864FEF55573BF9580AC47":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E864FEF55573BF9580AC47","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":6659.65},"EVID-AC85EC83EF0D7DA5FBE17B45":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC85EC83EF0D7DA5FBE17B45","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-AE75973FFC8EE1632018BC85":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AE75973FFC8EE1632018BC85","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-AF646F8CF6ACFB35721CE7A5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AF646F8CF6ACFB35721CE7A5","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-B5D676918ED2DA9FF88A6D1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B5D676918ED2DA9FF88A6D1D","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":12760.0},"EVID-B91AB0D86D5DD19043793E83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B91AB0D86D5DD19043793E83","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-C721CB58A713E142353C518C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C721CB58A713E142353C518C","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":675},"EVID-E32751AAF6F198EC3ABDE795":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E32751AAF6F198EC3ABDE795","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-E436F2B99029CFFC1A356400":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E436F2B99029CFFC1A356400","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-FDAAC0BC5E85652E7A547DED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FDAAC0BC5E85652E7A547DED","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":14500.0}}</t>
         </is>
       </c>
       <c r="AV40" s="22" t="inlineStr">
@@ -21960,7 +21960,7 @@
       </c>
       <c r="AZ40" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-B9518765A9CBB3B850E61ABC","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-582CD070FCA0E22EFE63E1A6","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA40" s="22" t="inlineStr">
@@ -21972,12 +21972,12 @@
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>CAND-D02211BBD5905FD5780AB565</t>
+          <t>CAND-2AB73E156C1AAF3CDDA0CA86</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -22161,12 +22161,12 @@
       </c>
       <c r="AT41" s="22" t="inlineStr">
         <is>
-          <t>["EVID-2FCC248C10E9F48BD4D77F54","EVID-75644FA33C29D8ED513B803F","EVID-D3EEA70AC8B32F968D671AC3","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
+          <t>["EVID-2FCC248C10E9F48BD4D77F54","EVID-75644FA33C29D8ED513B803F","EVID-E051999032917A838DDCD461","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
         </is>
       </c>
       <c r="AU41" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-2FCC248C10E9F48BD4D77F54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2FCC248C10E9F48BD4D77F54","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-D3EEA70AC8B32F968D671AC3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3EEA70AC8B32F968D671AC3","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0}}</t>
+          <t>{"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-2FCC248C10E9F48BD4D77F54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2FCC248C10E9F48BD4D77F54","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-E051999032917A838DDCD461":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E051999032917A838DDCD461","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":12000.0}}</t>
         </is>
       </c>
       <c r="AV41" s="22" t="inlineStr">
@@ -22203,12 +22203,12 @@
     <row r="42" ht="32" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>CAND-7D5805D2FF2492BB3634AF1C</t>
+          <t>CAND-332EED83B1AA249101A44265</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
@@ -22410,12 +22410,12 @@
       </c>
       <c r="AT42" s="22" t="inlineStr">
         <is>
-          <t>["EVID-B13D8C673679E8D15718908E","EVID-166A67EED614A58D24276B2F","EVID-F6216CA683B090EFED8D549C","EVID-64D30D4AB8C6E6421AD90719","EVID-E3F075A72C222D8EBDE27B38","EVID-D856366644C3446CA8C9738B","EVID-6F897904B230528E289C4123","EVID-03B05DA96489C34CE2110208","EVID-089CD33D495CC6061EFF7764","EVID-75644FA33C29D8ED513B803F","EVID-D3EEA70AC8B32F968D671AC3","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
+          <t>["EVID-B13D8C673679E8D15718908E","EVID-166A67EED614A58D24276B2F","EVID-F6216CA683B090EFED8D549C","EVID-64D30D4AB8C6E6421AD90719","EVID-E3F075A72C222D8EBDE27B38","EVID-D856366644C3446CA8C9738B","EVID-6F897904B230528E289C4123","EVID-03B05DA96489C34CE2110208","EVID-089CD33D495CC6061EFF7764","EVID-75644FA33C29D8ED513B803F","EVID-E051999032917A838DDCD461","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
         </is>
       </c>
       <c r="AU42" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03B05DA96489C34CE2110208":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-03B05DA96489C34CE2110208","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":8000},"EVID-089CD33D495CC6061EFF7764":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-089CD33D495CC6061EFF7764","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-166A67EED614A58D24276B2F":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-166A67EED614A58D24276B2F","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-64D30D4AB8C6E6421AD90719":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-64D30D4AB8C6E6421AD90719","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-6F897904B230528E289C4123":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6F897904B230528E289C4123","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2400},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-B13D8C673679E8D15718908E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B13D8C673679E8D15718908E","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-D3EEA70AC8B32F968D671AC3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3EEA70AC8B32F968D671AC3","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0},"EVID-D856366644C3446CA8C9738B":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D856366644C3446CA8C9738B","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-E3F075A72C222D8EBDE27B38":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E3F075A72C222D8EBDE27B38","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-F6216CA683B090EFED8D549C":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-F6216CA683B090EFED8D549C","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0}}</t>
+          <t>{"EVID-03B05DA96489C34CE2110208":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-03B05DA96489C34CE2110208","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":8000},"EVID-089CD33D495CC6061EFF7764":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-089CD33D495CC6061EFF7764","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-166A67EED614A58D24276B2F":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-166A67EED614A58D24276B2F","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-64D30D4AB8C6E6421AD90719":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-64D30D4AB8C6E6421AD90719","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-6F897904B230528E289C4123":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6F897904B230528E289C4123","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2400},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-B13D8C673679E8D15718908E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B13D8C673679E8D15718908E","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-D856366644C3446CA8C9738B":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D856366644C3446CA8C9738B","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-E051999032917A838DDCD461":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E051999032917A838DDCD461","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":12000.0},"EVID-E3F075A72C222D8EBDE27B38":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E3F075A72C222D8EBDE27B38","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-F6216CA683B090EFED8D549C":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-F6216CA683B090EFED8D549C","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV42" s="22" t="inlineStr">
@@ -22452,12 +22452,12 @@
     <row r="43" ht="32" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>CAND-4345B5FAFDB5E955A5FD97F9</t>
+          <t>CAND-75CB5E15D22B4E0E72A3CCBC</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr">
@@ -22637,12 +22637,12 @@
       </c>
       <c r="AT43" s="22" t="inlineStr">
         <is>
-          <t>["EVID-91B8D540E9B7FD033C34AA62","EVID-E3969B0FEA1EC3E2953E6635","EVID-EF6BEBBCCBDCFF649C090BB2","EVID-330787B0D67DADCBF273B64B","EVID-FEA1593579C33BD7E3F5E803","EVID-686AD89E86CEBC94CB6BED6C","EVID-75644FA33C29D8ED513B803F","EVID-D3EEA70AC8B32F968D671AC3","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
+          <t>["EVID-91B8D540E9B7FD033C34AA62","EVID-E3969B0FEA1EC3E2953E6635","EVID-EF6BEBBCCBDCFF649C090BB2","EVID-330787B0D67DADCBF273B64B","EVID-FEA1593579C33BD7E3F5E803","EVID-686AD89E86CEBC94CB6BED6C","EVID-75644FA33C29D8ED513B803F","EVID-E051999032917A838DDCD461","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
         </is>
       </c>
       <c r="AU43" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-330787B0D67DADCBF273B64B":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-330787B0D67DADCBF273B64B","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-686AD89E86CEBC94CB6BED6C":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-686AD89E86CEBC94CB6BED6C","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-91B8D540E9B7FD033C34AA62":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91B8D540E9B7FD033C34AA62","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":2},"EVID-D3EEA70AC8B32F968D671AC3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3EEA70AC8B32F968D671AC3","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0},"EVID-E3969B0FEA1EC3E2953E6635":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E3969B0FEA1EC3E2953E6635","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":1},"EVID-EF6BEBBCCBDCFF649C090BB2":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF6BEBBCCBDCFF649C090BB2","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-FEA1593579C33BD7E3F5E803":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-FEA1593579C33BD7E3F5E803","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0}}</t>
+          <t>{"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-330787B0D67DADCBF273B64B":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-330787B0D67DADCBF273B64B","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-686AD89E86CEBC94CB6BED6C":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-686AD89E86CEBC94CB6BED6C","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-91B8D540E9B7FD033C34AA62":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-91B8D540E9B7FD033C34AA62","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":2},"EVID-E051999032917A838DDCD461":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E051999032917A838DDCD461","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":12000.0},"EVID-E3969B0FEA1EC3E2953E6635":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E3969B0FEA1EC3E2953E6635","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":1},"EVID-EF6BEBBCCBDCFF649C090BB2":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-EF6BEBBCCBDCFF649C090BB2","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-FEA1593579C33BD7E3F5E803":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-FEA1593579C33BD7E3F5E803","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV43" s="22" t="inlineStr">
@@ -22679,12 +22679,12 @@
     <row r="44" ht="32" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>CAND-411A0364EF7BDE3A2D8A1FC4</t>
+          <t>CAND-2A0FC9335E57A3C9B7F9C7B8</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
@@ -22864,12 +22864,12 @@
       </c>
       <c r="AT44" s="22" t="inlineStr">
         <is>
-          <t>["EVID-FD23561554D253F349F128BD","EVID-56715B4903BFF401AF13B22C","EVID-E868B02D7C51E1D2B2C65B3E","EVID-DD24119637B30D9234FEEA1B","EVID-DC8EDE09C90729113AE9AB54","EVID-75644FA33C29D8ED513B803F","EVID-D3EEA70AC8B32F968D671AC3","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
+          <t>["EVID-FD23561554D253F349F128BD","EVID-56715B4903BFF401AF13B22C","EVID-E868B02D7C51E1D2B2C65B3E","EVID-DD24119637B30D9234FEEA1B","EVID-DC8EDE09C90729113AE9AB54","EVID-75644FA33C29D8ED513B803F","EVID-E051999032917A838DDCD461","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
         </is>
       </c>
       <c r="AU44" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-56715B4903BFF401AF13B22C":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-56715B4903BFF401AF13B22C","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":60.0},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-D3EEA70AC8B32F968D671AC3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3EEA70AC8B32F968D671AC3","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0},"EVID-DC8EDE09C90729113AE9AB54":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-DC8EDE09C90729113AE9AB54","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-DD24119637B30D9234FEEA1B":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-DD24119637B30D9234FEEA1B","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-E868B02D7C51E1D2B2C65B3E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-E868B02D7C51E1D2B2C65B3E","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-FD23561554D253F349F128BD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FD23561554D253F349F128BD","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1}}</t>
+          <t>{"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-56715B4903BFF401AF13B22C":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-56715B4903BFF401AF13B22C","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":60.0},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-DC8EDE09C90729113AE9AB54":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-DC8EDE09C90729113AE9AB54","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-DD24119637B30D9234FEEA1B":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-DD24119637B30D9234FEEA1B","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-E051999032917A838DDCD461":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E051999032917A838DDCD461","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":12000.0},"EVID-E868B02D7C51E1D2B2C65B3E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-E868B02D7C51E1D2B2C65B3E","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-FD23561554D253F349F128BD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-FD23561554D253F349F128BD","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1}}</t>
         </is>
       </c>
       <c r="AV44" s="22" t="inlineStr">
@@ -22906,12 +22906,12 @@
     <row r="45" ht="32" customHeight="1">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>CAND-687CCF977D322BBD979CD3F1</t>
+          <t>CAND-9E9049ADCEEB150F7DAC6289</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr">
@@ -23115,12 +23115,12 @@
       </c>
       <c r="AT45" s="22" t="inlineStr">
         <is>
-          <t>["EVID-17967E4F367F91174E4DD90A","EVID-CC158A559E6C492D009CC048","EVID-03B043795BC8E94DD967C7AF","EVID-DB69FA385B9B0EC01CC13C6E","EVID-B733CE4EA148EA8A95C45B40","EVID-B6AB0F518D240C586B6A9BAA","EVID-3138604EBCD528E08EA037B3","EVID-BB0C712245F54E1792FB4DFF","EVID-75644FA33C29D8ED513B803F","EVID-D3EEA70AC8B32F968D671AC3","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
+          <t>["EVID-17967E4F367F91174E4DD90A","EVID-CC158A559E6C492D009CC048","EVID-03B043795BC8E94DD967C7AF","EVID-DB69FA385B9B0EC01CC13C6E","EVID-B733CE4EA148EA8A95C45B40","EVID-B6AB0F518D240C586B6A9BAA","EVID-3138604EBCD528E08EA037B3","EVID-BB0C712245F54E1792FB4DFF","EVID-75644FA33C29D8ED513B803F","EVID-E051999032917A838DDCD461","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
         </is>
       </c>
       <c r="AU45" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03B043795BC8E94DD967C7AF":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-03B043795BC8E94DD967C7AF","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":96},"EVID-17967E4F367F91174E4DD90A":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-17967E4F367F91174E4DD90A","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-3138604EBCD528E08EA037B3":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-3138604EBCD528E08EA037B3","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-B6AB0F518D240C586B6A9BAA":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-B6AB0F518D240C586B6A9BAA","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-B733CE4EA148EA8A95C45B40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B733CE4EA148EA8A95C45B40","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":3},"EVID-BB0C712245F54E1792FB4DFF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BB0C712245F54E1792FB4DFF","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-CC158A559E6C492D009CC048":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CC158A559E6C492D009CC048","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":80.0},"EVID-D3EEA70AC8B32F968D671AC3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3EEA70AC8B32F968D671AC3","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0},"EVID-DB69FA385B9B0EC01CC13C6E":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-DB69FA385B9B0EC01CC13C6E","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":20000.0}}</t>
+          <t>{"EVID-03B043795BC8E94DD967C7AF":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-03B043795BC8E94DD967C7AF","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":96},"EVID-17967E4F367F91174E4DD90A":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-17967E4F367F91174E4DD90A","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-3138604EBCD528E08EA037B3":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-3138604EBCD528E08EA037B3","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-B6AB0F518D240C586B6A9BAA":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-B6AB0F518D240C586B6A9BAA","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-B733CE4EA148EA8A95C45B40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B733CE4EA148EA8A95C45B40","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":3},"EVID-BB0C712245F54E1792FB4DFF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BB0C712245F54E1792FB4DFF","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-CC158A559E6C492D009CC048":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CC158A559E6C492D009CC048","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":80.0},"EVID-DB69FA385B9B0EC01CC13C6E":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-DB69FA385B9B0EC01CC13C6E","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":20000.0},"EVID-E051999032917A838DDCD461":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E051999032917A838DDCD461","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":12000.0}}</t>
         </is>
       </c>
       <c r="AV45" s="22" t="inlineStr">
@@ -23157,12 +23157,12 @@
     <row r="46" ht="32" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>PKG-923A8D0FA3F713D5EB831F6B</t>
+          <t>PKG-96324620A070F31DA32A2F41</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>CAND-66E8F8CE41F453720A81BDE7</t>
+          <t>CAND-7E49B030E1FF3BD2B17E40BF</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr">
@@ -23370,12 +23370,12 @@
       </c>
       <c r="AT46" s="22" t="inlineStr">
         <is>
-          <t>["EVID-BD604BDEFD4EA94581027C35","EVID-ED313069E9F61EFA0C5EFD56","EVID-CD5D8CB70FA3A41B08E180E2","EVID-81CFE973454DD11FB7E57FAD","EVID-1E8EDA23B2F72B36B1D93744","EVID-87899198CD3D28F8AF6A0665","EVID-260136938BF8F30C964EF511","EVID-DFFC77E0EA06DD119782A5C8","EVID-DED90243F1C5B80CE20CDB44","EVID-46F28580C58548862BD2A95B","EVID-1F147A54A4B903EA9FF757E1","EVID-E7592E31B8FF567DFD8C4BAC","EVID-9EBEB2F65E2632EC2AE72129","EVID-75644FA33C29D8ED513B803F","EVID-D3EEA70AC8B32F968D671AC3","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
+          <t>["EVID-BD604BDEFD4EA94581027C35","EVID-ED313069E9F61EFA0C5EFD56","EVID-CD5D8CB70FA3A41B08E180E2","EVID-81CFE973454DD11FB7E57FAD","EVID-1E8EDA23B2F72B36B1D93744","EVID-87899198CD3D28F8AF6A0665","EVID-260136938BF8F30C964EF511","EVID-DFFC77E0EA06DD119782A5C8","EVID-DED90243F1C5B80CE20CDB44","EVID-46F28580C58548862BD2A95B","EVID-1F147A54A4B903EA9FF757E1","EVID-E7592E31B8FF567DFD8C4BAC","EVID-9EBEB2F65E2632EC2AE72129","EVID-75644FA33C29D8ED513B803F","EVID-E051999032917A838DDCD461","EVID-58EC282F7FC8A787ECCBF4CA","EVID-22737B2A74C73AA4C040BE38"]</t>
         </is>
       </c>
       <c r="AU46" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1E8EDA23B2F72B36B1D93744":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1E8EDA23B2F72B36B1D93744","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-1F147A54A4B903EA9FF757E1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1F147A54A4B903EA9FF757E1","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-260136938BF8F30C964EF511":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-260136938BF8F30C964EF511","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-46F28580C58548862BD2A95B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-46F28580C58548862BD2A95B","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":600},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-81CFE973454DD11FB7E57FAD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-81CFE973454DD11FB7E57FAD","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":1800},"EVID-87899198CD3D28F8AF6A0665":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-87899198CD3D28F8AF6A0665","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-9EBEB2F65E2632EC2AE72129":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9EBEB2F65E2632EC2AE72129","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-BD604BDEFD4EA94581027C35":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BD604BDEFD4EA94581027C35","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-CD5D8CB70FA3A41B08E180E2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD5D8CB70FA3A41B08E180E2","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-D3EEA70AC8B32F968D671AC3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D3EEA70AC8B32F968D671AC3","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":12000.0},"EVID-DED90243F1C5B80CE20CDB44":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DED90243F1C5B80CE20CDB44","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":192},"EVID-DFFC77E0EA06DD119782A5C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DFFC77E0EA06DD119782A5C8","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-E7592E31B8FF567DFD8C4BAC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7592E31B8FF567DFD8C4BAC","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-ED313069E9F61EFA0C5EFD56":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ED313069E9F61EFA0C5EFD56","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0}}</t>
+          <t>{"EVID-1E8EDA23B2F72B36B1D93744":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1E8EDA23B2F72B36B1D93744","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-1F147A54A4B903EA9FF757E1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1F147A54A4B903EA9FF757E1","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-22737B2A74C73AA4C040BE38":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22737B2A74C73AA4C040BE38","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":3},"EVID-260136938BF8F30C964EF511":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-260136938BF8F30C964EF511","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-46F28580C58548862BD2A95B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-46F28580C58548862BD2A95B","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":600},"EVID-58EC282F7FC8A787ECCBF4CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-58EC282F7FC8A787ECCBF4CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":151840.0},"EVID-75644FA33C29D8ED513B803F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75644FA33C29D8ED513B803F","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":10560.0},"EVID-81CFE973454DD11FB7E57FAD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-81CFE973454DD11FB7E57FAD","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":1800},"EVID-87899198CD3D28F8AF6A0665":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-87899198CD3D28F8AF6A0665","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-9EBEB2F65E2632EC2AE72129":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9EBEB2F65E2632EC2AE72129","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-BD604BDEFD4EA94581027C35":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BD604BDEFD4EA94581027C35","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-CD5D8CB70FA3A41B08E180E2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD5D8CB70FA3A41B08E180E2","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-DED90243F1C5B80CE20CDB44":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DED90243F1C5B80CE20CDB44","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":192},"EVID-DFFC77E0EA06DD119782A5C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DFFC77E0EA06DD119782A5C8","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-E051999032917A838DDCD461":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E051999032917A838DDCD461","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":12000.0},"EVID-E7592E31B8FF567DFD8C4BAC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7592E31B8FF567DFD8C4BAC","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-ED313069E9F61EFA0C5EFD56":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ED313069E9F61EFA0C5EFD56","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0}}</t>
         </is>
       </c>
       <c r="AV46" s="22" t="inlineStr">
@@ -23412,12 +23412,12 @@
     <row r="47" ht="32" customHeight="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>CAND-00CB68D319FAA492A409545D</t>
+          <t>CAND-D701CCAADA13C792A1F2ABC4</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">
@@ -23601,12 +23601,12 @@
       </c>
       <c r="AT47" s="22" t="inlineStr">
         <is>
-          <t>["EVID-DB2D727300A84DFD591BEA88","EVID-0D2577F99A78F966A66B9B75","EVID-9AAC252ACF6900D791D2AD26","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
+          <t>["EVID-DB2D727300A84DFD591BEA88","EVID-0D2577F99A78F966A66B9B75","EVID-DA09F55E9B9D4B9E274D1724","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
         </is>
       </c>
       <c r="AU47" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-9AAC252ACF6900D791D2AD26":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9AAC252ACF6900D791D2AD26","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0},"EVID-DB2D727300A84DFD591BEA88":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DB2D727300A84DFD591BEA88","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0}}</t>
+          <t>{"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-DA09F55E9B9D4B9E274D1724":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DA09F55E9B9D4B9E274D1724","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":52000.0},"EVID-DB2D727300A84DFD591BEA88":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DB2D727300A84DFD591BEA88","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0}}</t>
         </is>
       </c>
       <c r="AV47" s="22" t="inlineStr">
@@ -23643,12 +23643,12 @@
     <row r="48" ht="32" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>CAND-EDB08C1E32CD5DFD2B45A9F1</t>
+          <t>CAND-0B53B1CF89A1FF45576E8ACD</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
@@ -23832,12 +23832,12 @@
       </c>
       <c r="AT48" s="22" t="inlineStr">
         <is>
-          <t>["EVID-8AFB6F95D7C42F5401483897","EVID-BEB268DC8C1FCAFB79C58653","EVID-FA9EDB53BA7E51763A168D86","EVID-A86918C3CB8E0352D71F4318","EVID-30BE7B268EBCA2C565E734CE","EVID-9747F4CBC71901286891D2E9","EVID-E8A374E6704F50307F8F7829","EVID-6B7CC2A9F0FE053CF03DFB5E","EVID-D6A49DE19AB0D51EE2C9E21C","EVID-0D2577F99A78F966A66B9B75","EVID-9AAC252ACF6900D791D2AD26","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
+          <t>["EVID-8AFB6F95D7C42F5401483897","EVID-BEB268DC8C1FCAFB79C58653","EVID-FA9EDB53BA7E51763A168D86","EVID-A86918C3CB8E0352D71F4318","EVID-30BE7B268EBCA2C565E734CE","EVID-9747F4CBC71901286891D2E9","EVID-E8A374E6704F50307F8F7829","EVID-6B7CC2A9F0FE053CF03DFB5E","EVID-D6A49DE19AB0D51EE2C9E21C","EVID-0D2577F99A78F966A66B9B75","EVID-DA09F55E9B9D4B9E274D1724","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
         </is>
       </c>
       <c r="AU48" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-30BE7B268EBCA2C565E734CE":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-30BE7B268EBCA2C565E734CE","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-6B7CC2A9F0FE053CF03DFB5E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6B7CC2A9F0FE053CF03DFB5E","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":5500},"EVID-8AFB6F95D7C42F5401483897":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8AFB6F95D7C42F5401483897","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-9747F4CBC71901286891D2E9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9747F4CBC71901286891D2E9","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-9AAC252ACF6900D791D2AD26":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9AAC252ACF6900D791D2AD26","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0},"EVID-A86918C3CB8E0352D71F4318":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-A86918C3CB8E0352D71F4318","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-BEB268DC8C1FCAFB79C58653":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BEB268DC8C1FCAFB79C58653","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D6A49DE19AB0D51EE2C9E21C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D6A49DE19AB0D51EE2C9E21C","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-E8A374E6704F50307F8F7829":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E8A374E6704F50307F8F7829","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1800},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-FA9EDB53BA7E51763A168D86":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-FA9EDB53BA7E51763A168D86","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0}}</t>
+          <t>{"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-30BE7B268EBCA2C565E734CE":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-30BE7B268EBCA2C565E734CE","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-6B7CC2A9F0FE053CF03DFB5E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6B7CC2A9F0FE053CF03DFB5E","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":5500},"EVID-8AFB6F95D7C42F5401483897":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8AFB6F95D7C42F5401483897","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-9747F4CBC71901286891D2E9":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-9747F4CBC71901286891D2E9","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-A86918C3CB8E0352D71F4318":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-A86918C3CB8E0352D71F4318","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-BEB268DC8C1FCAFB79C58653":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-BEB268DC8C1FCAFB79C58653","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D6A49DE19AB0D51EE2C9E21C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D6A49DE19AB0D51EE2C9E21C","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-DA09F55E9B9D4B9E274D1724":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DA09F55E9B9D4B9E274D1724","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":52000.0},"EVID-E8A374E6704F50307F8F7829":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E8A374E6704F50307F8F7829","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":1800},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-FA9EDB53BA7E51763A168D86":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-FA9EDB53BA7E51763A168D86","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV48" s="22" t="inlineStr">
@@ -23862,7 +23862,7 @@
       </c>
       <c r="AZ48" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-25C50A8B284AD6025A2723EA","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-69D437D3D8FDDFE6F953315B","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA48" s="22" t="inlineStr">
@@ -23874,12 +23874,12 @@
     <row r="49" ht="32" customHeight="1">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>CAND-064DD3A175BE92BD9C658F7C</t>
+          <t>CAND-F867AC6F987F34C1567B71E4</t>
         </is>
       </c>
       <c r="C49" s="14" t="inlineStr">
@@ -24059,12 +24059,12 @@
       </c>
       <c r="AT49" s="22" t="inlineStr">
         <is>
-          <t>["EVID-D6CDBCF2AF4AE9D6F8CE9653","EVID-CF8BA68C57BA71F1BDD694FC","EVID-F832B6C7EEAD59A8276C0A30","EVID-08C70D3F461AA8C9C1E94646","EVID-D194EDED7F6F327969D292B4","EVID-85BF82D6ECB297978551A196","EVID-0D2577F99A78F966A66B9B75","EVID-9AAC252ACF6900D791D2AD26","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
+          <t>["EVID-D6CDBCF2AF4AE9D6F8CE9653","EVID-CF8BA68C57BA71F1BDD694FC","EVID-F832B6C7EEAD59A8276C0A30","EVID-08C70D3F461AA8C9C1E94646","EVID-D194EDED7F6F327969D292B4","EVID-85BF82D6ECB297978551A196","EVID-0D2577F99A78F966A66B9B75","EVID-DA09F55E9B9D4B9E274D1724","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
         </is>
       </c>
       <c r="AU49" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-08C70D3F461AA8C9C1E94646":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-08C70D3F461AA8C9C1E94646","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-85BF82D6ECB297978551A196":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-85BF82D6ECB297978551A196","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-9AAC252ACF6900D791D2AD26":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9AAC252ACF6900D791D2AD26","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0},"EVID-CF8BA68C57BA71F1BDD694FC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CF8BA68C57BA71F1BDD694FC","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":4},"EVID-D194EDED7F6F327969D292B4":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-D194EDED7F6F327969D292B4","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-D6CDBCF2AF4AE9D6F8CE9653":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D6CDBCF2AF4AE9D6F8CE9653","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":10},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-F832B6C7EEAD59A8276C0A30":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F832B6C7EEAD59A8276C0A30","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0}}</t>
+          <t>{"EVID-08C70D3F461AA8C9C1E94646":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-08C70D3F461AA8C9C1E94646","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-85BF82D6ECB297978551A196":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-85BF82D6ECB297978551A196","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-CF8BA68C57BA71F1BDD694FC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CF8BA68C57BA71F1BDD694FC","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":4},"EVID-D194EDED7F6F327969D292B4":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-D194EDED7F6F327969D292B4","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-D6CDBCF2AF4AE9D6F8CE9653":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D6CDBCF2AF4AE9D6F8CE9653","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":10},"EVID-DA09F55E9B9D4B9E274D1724":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DA09F55E9B9D4B9E274D1724","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":52000.0},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-F832B6C7EEAD59A8276C0A30":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F832B6C7EEAD59A8276C0A30","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0}}</t>
         </is>
       </c>
       <c r="AV49" s="22" t="inlineStr">
@@ -24089,7 +24089,7 @@
       </c>
       <c r="AZ49" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-25C50A8B284AD6025A2723EA","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-69D437D3D8FDDFE6F953315B","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA49" s="22" t="inlineStr">
@@ -24101,12 +24101,12 @@
     <row r="50" ht="32" customHeight="1">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>CAND-66F4CCF16FDA6E5ED2780272</t>
+          <t>CAND-91319B61F24C51743453ED64</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
@@ -24286,12 +24286,12 @@
       </c>
       <c r="AT50" s="22" t="inlineStr">
         <is>
-          <t>["EVID-EF9DF359F0ABC4B35E372381","EVID-7DD72E73E5027A86095C5BAF","EVID-00F687C1E6EEFA91E74B77BC","EVID-95322770660C5432BDE5C66B","EVID-ADC407565C55B500C48F5ED2","EVID-0D2577F99A78F966A66B9B75","EVID-9AAC252ACF6900D791D2AD26","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
+          <t>["EVID-EF9DF359F0ABC4B35E372381","EVID-7DD72E73E5027A86095C5BAF","EVID-00F687C1E6EEFA91E74B77BC","EVID-95322770660C5432BDE5C66B","EVID-ADC407565C55B500C48F5ED2","EVID-0D2577F99A78F966A66B9B75","EVID-DA09F55E9B9D4B9E274D1724","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
         </is>
       </c>
       <c r="AU50" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00F687C1E6EEFA91E74B77BC":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-00F687C1E6EEFA91E74B77BC","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-7DD72E73E5027A86095C5BAF":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-7DD72E73E5027A86095C5BAF","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":0.0},"EVID-95322770660C5432BDE5C66B":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-95322770660C5432BDE5C66B","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-9AAC252ACF6900D791D2AD26":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9AAC252ACF6900D791D2AD26","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0},"EVID-ADC407565C55B500C48F5ED2":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-ADC407565C55B500C48F5ED2","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-EF9DF359F0ABC4B35E372381":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EF9DF359F0ABC4B35E372381","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1}}</t>
+          <t>{"EVID-00F687C1E6EEFA91E74B77BC":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-00F687C1E6EEFA91E74B77BC","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-7DD72E73E5027A86095C5BAF":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-7DD72E73E5027A86095C5BAF","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":0.0},"EVID-95322770660C5432BDE5C66B":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-95322770660C5432BDE5C66B","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-ADC407565C55B500C48F5ED2":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-ADC407565C55B500C48F5ED2","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-DA09F55E9B9D4B9E274D1724":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DA09F55E9B9D4B9E274D1724","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":52000.0},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-EF9DF359F0ABC4B35E372381":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EF9DF359F0ABC4B35E372381","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1}}</t>
         </is>
       </c>
       <c r="AV50" s="22" t="inlineStr">
@@ -24328,12 +24328,12 @@
     <row r="51" ht="32" customHeight="1">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>CAND-F4D441B77DA39A68A9B6983C</t>
+          <t>CAND-D955E2B2473C8669E75F5A3E</t>
         </is>
       </c>
       <c r="C51" s="14" t="inlineStr">
@@ -24513,12 +24513,12 @@
       </c>
       <c r="AT51" s="22" t="inlineStr">
         <is>
-          <t>["EVID-01C10C33A653913CBECF537E","EVID-126B0066E8ED9BC396AF90F5","EVID-B277B645978A6DDE26F31849","EVID-A151021739E107AC0765F6ED","EVID-44095FB79A7F7BEF72DA46ED","EVID-F41A422F78611D9A8DBC6C9F","EVID-9ABB987739ABEE5C6E537210","EVID-AC4441B3F007D44D4E87FF73","EVID-0D2577F99A78F966A66B9B75","EVID-9AAC252ACF6900D791D2AD26","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
+          <t>["EVID-01C10C33A653913CBECF537E","EVID-126B0066E8ED9BC396AF90F5","EVID-B277B645978A6DDE26F31849","EVID-A151021739E107AC0765F6ED","EVID-44095FB79A7F7BEF72DA46ED","EVID-F41A422F78611D9A8DBC6C9F","EVID-9ABB987739ABEE5C6E537210","EVID-AC4441B3F007D44D4E87FF73","EVID-0D2577F99A78F966A66B9B75","EVID-DA09F55E9B9D4B9E274D1724","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
         </is>
       </c>
       <c r="AU51" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-01C10C33A653913CBECF537E":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-01C10C33A653913CBECF537E","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":10,"unit":"minutes","value":10},"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-126B0066E8ED9BC396AF90F5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-126B0066E8ED9BC396AF90F5","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":733.33},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-44095FB79A7F7BEF72DA46ED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44095FB79A7F7BEF72DA46ED","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":0},"EVID-9AAC252ACF6900D791D2AD26":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9AAC252ACF6900D791D2AD26","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0},"EVID-9ABB987739ABEE5C6E537210":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-9ABB987739ABEE5C6E537210","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.0},"EVID-A151021739E107AC0765F6ED":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-A151021739E107AC0765F6ED","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":56000.0},"EVID-AC4441B3F007D44D4E87FF73":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC4441B3F007D44D4E87FF73","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1920.0},"EVID-B277B645978A6DDE26F31849":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-B277B645978A6DDE26F31849","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":880},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-F41A422F78611D9A8DBC6C9F":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-F41A422F78611D9A8DBC6C9F","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":0}}</t>
+          <t>{"EVID-01C10C33A653913CBECF537E":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-01C10C33A653913CBECF537E","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":10,"unit":"minutes","value":10},"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-126B0066E8ED9BC396AF90F5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-126B0066E8ED9BC396AF90F5","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":733.33},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-44095FB79A7F7BEF72DA46ED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-44095FB79A7F7BEF72DA46ED","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":0},"EVID-9ABB987739ABEE5C6E537210":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-9ABB987739ABEE5C6E537210","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.0},"EVID-A151021739E107AC0765F6ED":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-A151021739E107AC0765F6ED","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":56000.0},"EVID-AC4441B3F007D44D4E87FF73":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AC4441B3F007D44D4E87FF73","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1920.0},"EVID-B277B645978A6DDE26F31849":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-B277B645978A6DDE26F31849","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":880},"EVID-DA09F55E9B9D4B9E274D1724":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DA09F55E9B9D4B9E274D1724","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":52000.0},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-F41A422F78611D9A8DBC6C9F":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-F41A422F78611D9A8DBC6C9F","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":0}}</t>
         </is>
       </c>
       <c r="AV51" s="22" t="inlineStr">
@@ -24555,12 +24555,12 @@
     <row r="52" ht="32" customHeight="1">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>PKG-39A0046BADA47CAB1AF59FD5</t>
+          <t>PKG-E17FC65E6367642C810E4562</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>CAND-1F3EBDB3DFBB20D0B1CD4658</t>
+          <t>CAND-09EB817A3591B59B95A5BDA5</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
@@ -24744,12 +24744,12 @@
       </c>
       <c r="AT52" s="22" t="inlineStr">
         <is>
-          <t>["EVID-0DFBE3E1D8CA16638D34ABF6","EVID-48E87CEE6D354F7DE92B8533","EVID-A75FAB3134E0BBD8EC73EEB4","EVID-4266ECEA017A21660614C087","EVID-6FCA127FE42DCA1BFEA9DCDD","EVID-6CF2C562A97DB25CEDFBA2E1","EVID-ADA7AC1BCB3C988A132932FF","EVID-2276D86FAB7C2B5BC1B741C8","EVID-F5753F549769D56D0A75DE45","EVID-51E1C6FB4D6767553EA80848","EVID-A97EBA544AC3955018A16D3B","EVID-43CAB2D4F8BAA15A8A9A3F70","EVID-59FD4115ACB0EBCC2B63BCA7","EVID-0D2577F99A78F966A66B9B75","EVID-9AAC252ACF6900D791D2AD26","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
+          <t>["EVID-0DFBE3E1D8CA16638D34ABF6","EVID-48E87CEE6D354F7DE92B8533","EVID-A75FAB3134E0BBD8EC73EEB4","EVID-4266ECEA017A21660614C087","EVID-6FCA127FE42DCA1BFEA9DCDD","EVID-6CF2C562A97DB25CEDFBA2E1","EVID-ADA7AC1BCB3C988A132932FF","EVID-2276D86FAB7C2B5BC1B741C8","EVID-F5753F549769D56D0A75DE45","EVID-51E1C6FB4D6767553EA80848","EVID-A97EBA544AC3955018A16D3B","EVID-43CAB2D4F8BAA15A8A9A3F70","EVID-59FD4115ACB0EBCC2B63BCA7","EVID-0D2577F99A78F966A66B9B75","EVID-DA09F55E9B9D4B9E274D1724","EVID-EAC3FD6CB132DD4EC094D307","EVID-22BC61EE8E8120AFBAD301A8"]</t>
         </is>
       </c>
       <c r="AU52" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-0DFBE3E1D8CA16638D34ABF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0DFBE3E1D8CA16638D34ABF6","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"SERVERLESS"},"EVID-2276D86FAB7C2B5BC1B741C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2276D86FAB7C2B5BC1B741C8","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-4266ECEA017A21660614C087":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4266ECEA017A21660614C087","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":16500},"EVID-43CAB2D4F8BAA15A8A9A3F70":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-43CAB2D4F8BAA15A8A9A3F70","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-48E87CEE6D354F7DE92B8533":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48E87CEE6D354F7DE92B8533","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":100.0},"EVID-51E1C6FB4D6767553EA80848":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-51E1C6FB4D6767553EA80848","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":5500},"EVID-59FD4115ACB0EBCC2B63BCA7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-59FD4115ACB0EBCC2B63BCA7","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-6CF2C562A97DB25CEDFBA2E1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6CF2C562A97DB25CEDFBA2E1","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-6FCA127FE42DCA1BFEA9DCDD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6FCA127FE42DCA1BFEA9DCDD","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-9AAC252ACF6900D791D2AD26":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9AAC252ACF6900D791D2AD26","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":52000.0},"EVID-A75FAB3134E0BBD8EC73EEB4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A75FAB3134E0BBD8EC73EEB4","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-A97EBA544AC3955018A16D3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A97EBA544AC3955018A16D3B","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-ADA7AC1BCB3C988A132932FF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ADA7AC1BCB3C988A132932FF","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-F5753F549769D56D0A75DE45":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F5753F549769D56D0A75DE45","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1760}}</t>
+          <t>{"EVID-0D2577F99A78F966A66B9B75":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0D2577F99A78F966A66B9B75","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":45760.0},"EVID-0DFBE3E1D8CA16638D34ABF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0DFBE3E1D8CA16638D34ABF6","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"SERVERLESS"},"EVID-2276D86FAB7C2B5BC1B741C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2276D86FAB7C2B5BC1B741C8","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-22BC61EE8E8120AFBAD301A8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-22BC61EE8E8120AFBAD301A8","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":269},"EVID-4266ECEA017A21660614C087":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4266ECEA017A21660614C087","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":16500},"EVID-43CAB2D4F8BAA15A8A9A3F70":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-43CAB2D4F8BAA15A8A9A3F70","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-48E87CEE6D354F7DE92B8533":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-48E87CEE6D354F7DE92B8533","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":100.0},"EVID-51E1C6FB4D6767553EA80848":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-51E1C6FB4D6767553EA80848","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":5500},"EVID-59FD4115ACB0EBCC2B63BCA7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-59FD4115ACB0EBCC2B63BCA7","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-6CF2C562A97DB25CEDFBA2E1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6CF2C562A97DB25CEDFBA2E1","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-6FCA127FE42DCA1BFEA9DCDD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6FCA127FE42DCA1BFEA9DCDD","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-A75FAB3134E0BBD8EC73EEB4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A75FAB3134E0BBD8EC73EEB4","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-A97EBA544AC3955018A16D3B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A97EBA544AC3955018A16D3B","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-ADA7AC1BCB3C988A132932FF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ADA7AC1BCB3C988A132932FF","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-DA09F55E9B9D4B9E274D1724":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DA09F55E9B9D4B9E274D1724","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":52000.0},"EVID-EAC3FD6CB132DD4EC094D307":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EAC3FD6CB132DD4EC094D307","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":0.0},"EVID-F5753F549769D56D0A75DE45":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F5753F549769D56D0A75DE45","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1760}}</t>
         </is>
       </c>
       <c r="AV52" s="22" t="inlineStr">
@@ -24774,7 +24774,7 @@
       </c>
       <c r="AZ52" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-BF14FB572683C696D02CD7EA","scenario_name":"Plan B — Pro migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-27D656892CFF54E7DE80A40B","scenario_name":"Plan B — Pro migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA52" s="22" t="inlineStr">
@@ -24786,12 +24786,12 @@
     <row r="53" ht="32" customHeight="1">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>CAND-F68319AE1BD26F3AE3D7C206</t>
+          <t>CAND-328B32A3406D831E36A10996</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
@@ -24975,12 +24975,12 @@
       </c>
       <c r="AT53" s="22" t="inlineStr">
         <is>
-          <t>["EVID-B0ADC3F9BBD9ECB4740C747D","EVID-6665943F60B0947FC1DB72B0","EVID-98CAA6224EA61D09431C73D8","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
+          <t>["EVID-B0ADC3F9BBD9ECB4740C747D","EVID-6665943F60B0947FC1DB72B0","EVID-6AD0AE822DC4491A8A6E59A2","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
         </is>
       </c>
       <c r="AU53" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-98CAA6224EA61D09431C73D8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98CAA6224EA61D09431C73D8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-B0ADC3F9BBD9ECB4740C747D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B0ADC3F9BBD9ECB4740C747D","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249}}</t>
+          <t>{"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6AD0AE822DC4491A8A6E59A2","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":17000.0},"EVID-B0ADC3F9BBD9ECB4740C747D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B0ADC3F9BBD9ECB4740C747D","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249}}</t>
         </is>
       </c>
       <c r="AV53" s="22" t="inlineStr">
@@ -25017,12 +25017,12 @@
     <row r="54" ht="32" customHeight="1">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>CAND-51124DC4FB8ADD3865AA63DB</t>
+          <t>CAND-9D796F49F0E013A31CC9883D</t>
         </is>
       </c>
       <c r="C54" s="14" t="inlineStr">
@@ -25206,12 +25206,12 @@
       </c>
       <c r="AT54" s="22" t="inlineStr">
         <is>
-          <t>["EVID-ED7225D949D2C454A0AF5F1D","EVID-9FD6DEBD0F2C18B06B0371E9","EVID-8CF968FBF50B177B3FEDC10A","EVID-35D1AC26AEE944960C554D47","EVID-059FE4330A15AD87E55A2739","EVID-57FF2359E7551FE22742D506","EVID-F589EAB431C557C66AD277CE","EVID-84308FE592F273E313559071","EVID-157609D059EE617240F34DBA","EVID-6665943F60B0947FC1DB72B0","EVID-98CAA6224EA61D09431C73D8","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
+          <t>["EVID-ED7225D949D2C454A0AF5F1D","EVID-9FD6DEBD0F2C18B06B0371E9","EVID-8CF968FBF50B177B3FEDC10A","EVID-35D1AC26AEE944960C554D47","EVID-059FE4330A15AD87E55A2739","EVID-57FF2359E7551FE22742D506","EVID-F589EAB431C557C66AD277CE","EVID-84308FE592F273E313559071","EVID-157609D059EE617240F34DBA","EVID-6665943F60B0947FC1DB72B0","EVID-6AD0AE822DC4491A8A6E59A2","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
         </is>
       </c>
       <c r="AU54" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-059FE4330A15AD87E55A2739":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-059FE4330A15AD87E55A2739","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-157609D059EE617240F34DBA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-157609D059EE617240F34DBA","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-35D1AC26AEE944960C554D47":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-35D1AC26AEE944960C554D47","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-57FF2359E7551FE22742D506":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-57FF2359E7551FE22742D506","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-84308FE592F273E313559071":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-84308FE592F273E313559071","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":9000},"EVID-8CF968FBF50B177B3FEDC10A":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-8CF968FBF50B177B3FEDC10A","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-98CAA6224EA61D09431C73D8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98CAA6224EA61D09431C73D8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-9FD6DEBD0F2C18B06B0371E9":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-9FD6DEBD0F2C18B06B0371E9","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-ED7225D949D2C454A0AF5F1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ED7225D949D2C454A0AF5F1D","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-F589EAB431C557C66AD277CE":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F589EAB431C557C66AD277CE","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3000}}</t>
+          <t>{"EVID-059FE4330A15AD87E55A2739":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-059FE4330A15AD87E55A2739","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-157609D059EE617240F34DBA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-157609D059EE617240F34DBA","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-35D1AC26AEE944960C554D47":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-35D1AC26AEE944960C554D47","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-57FF2359E7551FE22742D506":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-57FF2359E7551FE22742D506","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6AD0AE822DC4491A8A6E59A2","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":17000.0},"EVID-84308FE592F273E313559071":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-84308FE592F273E313559071","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":9000},"EVID-8CF968FBF50B177B3FEDC10A":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-8CF968FBF50B177B3FEDC10A","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-9FD6DEBD0F2C18B06B0371E9":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-9FD6DEBD0F2C18B06B0371E9","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-ED7225D949D2C454A0AF5F1D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-ED7225D949D2C454A0AF5F1D","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-F589EAB431C557C66AD277CE":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-F589EAB431C557C66AD277CE","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":3000}}</t>
         </is>
       </c>
       <c r="AV54" s="22" t="inlineStr">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="AZ54" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-7999EC8BC5B2A2F2A072C81B","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-2CC0626945850CA914D1FE52","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA54" s="22" t="inlineStr">
@@ -25248,12 +25248,12 @@
     <row r="55" ht="32" customHeight="1">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>CAND-A61DE0B24632CFBA54001A80</t>
+          <t>CAND-577A4357DFAC3AC2FC120CCC</t>
         </is>
       </c>
       <c r="C55" s="14" t="inlineStr">
@@ -25433,12 +25433,12 @@
       </c>
       <c r="AT55" s="22" t="inlineStr">
         <is>
-          <t>["EVID-A8402360CEDF0C2D631CA71B","EVID-3DCE404051777C9BAEF8B72E","EVID-34F5EEC65A083C997173A336","EVID-B4303033D02B81F9FB9A34FB","EVID-8B9D2E503AD6756D35F0BAB9","EVID-B475BD587CAF88BFD454BCEE","EVID-6665943F60B0947FC1DB72B0","EVID-98CAA6224EA61D09431C73D8","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
+          <t>["EVID-A8402360CEDF0C2D631CA71B","EVID-3DCE404051777C9BAEF8B72E","EVID-34F5EEC65A083C997173A336","EVID-B4303033D02B81F9FB9A34FB","EVID-8B9D2E503AD6756D35F0BAB9","EVID-B475BD587CAF88BFD454BCEE","EVID-6665943F60B0947FC1DB72B0","EVID-6AD0AE822DC4491A8A6E59A2","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
         </is>
       </c>
       <c r="AU55" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-34F5EEC65A083C997173A336":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-34F5EEC65A083C997173A336","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-3DCE404051777C9BAEF8B72E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3DCE404051777C9BAEF8B72E","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-8B9D2E503AD6756D35F0BAB9":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-8B9D2E503AD6756D35F0BAB9","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-98CAA6224EA61D09431C73D8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98CAA6224EA61D09431C73D8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-A8402360CEDF0C2D631CA71B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A8402360CEDF0C2D631CA71B","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-B4303033D02B81F9FB9A34FB":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-B4303033D02B81F9FB9A34FB","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-B475BD587CAF88BFD454BCEE":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-B475BD587CAF88BFD454BCEE","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249}}</t>
+          <t>{"EVID-34F5EEC65A083C997173A336":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-34F5EEC65A083C997173A336","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-3DCE404051777C9BAEF8B72E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3DCE404051777C9BAEF8B72E","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6AD0AE822DC4491A8A6E59A2","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":17000.0},"EVID-8B9D2E503AD6756D35F0BAB9":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-8B9D2E503AD6756D35F0BAB9","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-A8402360CEDF0C2D631CA71B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A8402360CEDF0C2D631CA71B","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-B4303033D02B81F9FB9A34FB":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-B4303033D02B81F9FB9A34FB","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-B475BD587CAF88BFD454BCEE":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-B475BD587CAF88BFD454BCEE","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249}}</t>
         </is>
       </c>
       <c r="AV55" s="22" t="inlineStr">
@@ -25463,7 +25463,7 @@
       </c>
       <c r="AZ55" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-7999EC8BC5B2A2F2A072C81B","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-2CC0626945850CA914D1FE52","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA55" s="22" t="inlineStr">
@@ -25475,12 +25475,12 @@
     <row r="56" ht="32" customHeight="1">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>CAND-B374D8D47EA49C8263B110B4</t>
+          <t>CAND-0158D968DBF1312B9426F514</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
@@ -25660,12 +25660,12 @@
       </c>
       <c r="AT56" s="22" t="inlineStr">
         <is>
-          <t>["EVID-30873B9A166C94B785F6DD9E","EVID-DC5EA1E87EB0CD581FE95A54","EVID-81A596AD7DC138D8FF017479","EVID-91F2C85163E9C268917948AE","EVID-6836034413538E0247BCD39C","EVID-6665943F60B0947FC1DB72B0","EVID-98CAA6224EA61D09431C73D8","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
+          <t>["EVID-30873B9A166C94B785F6DD9E","EVID-DC5EA1E87EB0CD581FE95A54","EVID-81A596AD7DC138D8FF017479","EVID-91F2C85163E9C268917948AE","EVID-6836034413538E0247BCD39C","EVID-6665943F60B0947FC1DB72B0","EVID-6AD0AE822DC4491A8A6E59A2","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
         </is>
       </c>
       <c r="AU56" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-30873B9A166C94B785F6DD9E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30873B9A166C94B785F6DD9E","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6836034413538E0247BCD39C":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-6836034413538E0247BCD39C","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-81A596AD7DC138D8FF017479":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-81A596AD7DC138D8FF017479","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-91F2C85163E9C268917948AE":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-91F2C85163E9C268917948AE","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-98CAA6224EA61D09431C73D8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98CAA6224EA61D09431C73D8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-DC5EA1E87EB0CD581FE95A54":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-DC5EA1E87EB0CD581FE95A54","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":60.0}}</t>
+          <t>{"EVID-30873B9A166C94B785F6DD9E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-30873B9A166C94B785F6DD9E","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6836034413538E0247BCD39C":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-6836034413538E0247BCD39C","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6AD0AE822DC4491A8A6E59A2","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":17000.0},"EVID-81A596AD7DC138D8FF017479":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-81A596AD7DC138D8FF017479","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-91F2C85163E9C268917948AE":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-91F2C85163E9C268917948AE","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-DC5EA1E87EB0CD581FE95A54":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-DC5EA1E87EB0CD581FE95A54","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":60.0}}</t>
         </is>
       </c>
       <c r="AV56" s="22" t="inlineStr">
@@ -25702,12 +25702,12 @@
     <row r="57" ht="32" customHeight="1">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>CAND-2FBBF83290400F68817DBC65</t>
+          <t>CAND-D698FAAC1DCEDE4698BD76F8</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -25911,12 +25911,12 @@
       </c>
       <c r="AT57" s="22" t="inlineStr">
         <is>
-          <t>["EVID-92DAC2328781D259CBBFBB85","EVID-E264F0D7C3BF2400A7542F09","EVID-BBF9DD673AEF81FA3C8AA061","EVID-503B61DBFF6F18290B1D0B98","EVID-65D3B2971A671665ED696DAB","EVID-FA63F69E827870908D19759E","EVID-1FE0A1D231A62E4C4F11DCD0","EVID-D7DBB679528E173F5E5E7B67","EVID-6665943F60B0947FC1DB72B0","EVID-98CAA6224EA61D09431C73D8","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
+          <t>["EVID-92DAC2328781D259CBBFBB85","EVID-E264F0D7C3BF2400A7542F09","EVID-BBF9DD673AEF81FA3C8AA061","EVID-503B61DBFF6F18290B1D0B98","EVID-65D3B2971A671665ED696DAB","EVID-FA63F69E827870908D19759E","EVID-1FE0A1D231A62E4C4F11DCD0","EVID-D7DBB679528E173F5E5E7B67","EVID-6665943F60B0947FC1DB72B0","EVID-6AD0AE822DC4491A8A6E59A2","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
         </is>
       </c>
       <c r="AU57" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1FE0A1D231A62E4C4F11DCD0":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-1FE0A1D231A62E4C4F11DCD0","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.8},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-503B61DBFF6F18290B1D0B98":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-503B61DBFF6F18290B1D0B98","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-65D3B2971A671665ED696DAB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-65D3B2971A671665ED696DAB","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":24},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-92DAC2328781D259CBBFBB85":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-92DAC2328781D259CBBFBB85","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-98CAA6224EA61D09431C73D8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98CAA6224EA61D09431C73D8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-BBF9DD673AEF81FA3C8AA061":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-BBF9DD673AEF81FA3C8AA061","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":192},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-D7DBB679528E173F5E5E7B67":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D7DBB679528E173F5E5E7B67","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-E264F0D7C3BF2400A7542F09":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E264F0D7C3BF2400A7542F09","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":160.0},"EVID-FA63F69E827870908D19759E":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-FA63F69E827870908D19759E","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":85000}}</t>
+          <t>{"EVID-1FE0A1D231A62E4C4F11DCD0":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-1FE0A1D231A62E4C4F11DCD0","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.8},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-503B61DBFF6F18290B1D0B98":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-503B61DBFF6F18290B1D0B98","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-65D3B2971A671665ED696DAB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-65D3B2971A671665ED696DAB","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":24},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6AD0AE822DC4491A8A6E59A2","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":17000.0},"EVID-92DAC2328781D259CBBFBB85":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-92DAC2328781D259CBBFBB85","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-BBF9DD673AEF81FA3C8AA061":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-BBF9DD673AEF81FA3C8AA061","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":192},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-D7DBB679528E173F5E5E7B67":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D7DBB679528E173F5E5E7B67","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-E264F0D7C3BF2400A7542F09":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E264F0D7C3BF2400A7542F09","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":160.0},"EVID-FA63F69E827870908D19759E":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-FA63F69E827870908D19759E","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":85000}}</t>
         </is>
       </c>
       <c r="AV57" s="22" t="inlineStr">
@@ -25953,12 +25953,12 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>PKG-32BFFEC26AF4B55BB7C90095</t>
+          <t>PKG-81ABFCC9AC0BE0CB18010B22</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>CAND-FF15B75DF3EB05354881F56F</t>
+          <t>CAND-113EE95F32D6329E0F3A4C61</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
@@ -26142,12 +26142,12 @@
       </c>
       <c r="AT58" s="22" t="inlineStr">
         <is>
-          <t>["EVID-AEBD7278AEA481239BF5900E","EVID-98004CC96788E8AD51027C2D","EVID-40AB8EEB573EBBC490AC80C3","EVID-9907A30A1D61046BB3CED706","EVID-15CF0A5DC41DD4B62D3D9890","EVID-E7E44A13571351BB72C59DF7","EVID-C1375153ED8F081F94960AD2","EVID-3FA7FA11988FE0E694F141BC","EVID-61F35E8FA5A8996603C62417","EVID-709D8A90FB2DAC2E837F6CC4","EVID-42094F6FB6165ECA71933317","EVID-3B99677A5BA12CD929F685C8","EVID-DAE8F937EC8E2BC926FB7373","EVID-6665943F60B0947FC1DB72B0","EVID-98CAA6224EA61D09431C73D8","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
+          <t>["EVID-AEBD7278AEA481239BF5900E","EVID-98004CC96788E8AD51027C2D","EVID-40AB8EEB573EBBC490AC80C3","EVID-9907A30A1D61046BB3CED706","EVID-15CF0A5DC41DD4B62D3D9890","EVID-E7E44A13571351BB72C59DF7","EVID-C1375153ED8F081F94960AD2","EVID-3FA7FA11988FE0E694F141BC","EVID-61F35E8FA5A8996603C62417","EVID-709D8A90FB2DAC2E837F6CC4","EVID-42094F6FB6165ECA71933317","EVID-3B99677A5BA12CD929F685C8","EVID-DAE8F937EC8E2BC926FB7373","EVID-6665943F60B0947FC1DB72B0","EVID-6AD0AE822DC4491A8A6E59A2","EVID-3C64C89ED2B7A4B580E2C9CA","EVID-D517C647FD60879252972C6F"]</t>
         </is>
       </c>
       <c r="AU58" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-15CF0A5DC41DD4B62D3D9890":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-15CF0A5DC41DD4B62D3D9890","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-3B99677A5BA12CD929F685C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3B99677A5BA12CD929F685C8","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-3FA7FA11988FE0E694F141BC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3FA7FA11988FE0E694F141BC","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-40AB8EEB573EBBC490AC80C3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-40AB8EEB573EBBC490AC80C3","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-42094F6FB6165ECA71933317":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-42094F6FB6165ECA71933317","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-61F35E8FA5A8996603C62417":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-61F35E8FA5A8996603C62417","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":384},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-709D8A90FB2DAC2E837F6CC4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-709D8A90FB2DAC2E837F6CC4","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":1200},"EVID-98004CC96788E8AD51027C2D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98004CC96788E8AD51027C2D","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-98CAA6224EA61D09431C73D8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98CAA6224EA61D09431C73D8","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":17000.0},"EVID-9907A30A1D61046BB3CED706":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9907A30A1D61046BB3CED706","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":3600},"EVID-AEBD7278AEA481239BF5900E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AEBD7278AEA481239BF5900E","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-C1375153ED8F081F94960AD2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C1375153ED8F081F94960AD2","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-DAE8F937EC8E2BC926FB7373":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DAE8F937EC8E2BC926FB7373","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-E7E44A13571351BB72C59DF7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7E44A13571351BB72C59DF7","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0}}</t>
+          <t>{"EVID-15CF0A5DC41DD4B62D3D9890":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-15CF0A5DC41DD4B62D3D9890","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-3B99677A5BA12CD929F685C8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3B99677A5BA12CD929F685C8","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-3C64C89ED2B7A4B580E2C9CA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3C64C89ED2B7A4B580E2C9CA","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5488.19},"EVID-3FA7FA11988FE0E694F141BC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3FA7FA11988FE0E694F141BC","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-40AB8EEB573EBBC490AC80C3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-40AB8EEB573EBBC490AC80C3","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-42094F6FB6165ECA71933317":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-42094F6FB6165ECA71933317","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-61F35E8FA5A8996603C62417":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-61F35E8FA5A8996603C62417","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":384},"EVID-6665943F60B0947FC1DB72B0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6665943F60B0947FC1DB72B0","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":14960.0},"EVID-6AD0AE822DC4491A8A6E59A2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6AD0AE822DC4491A8A6E59A2","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":17000.0},"EVID-709D8A90FB2DAC2E837F6CC4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-709D8A90FB2DAC2E837F6CC4","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":1200},"EVID-98004CC96788E8AD51027C2D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-98004CC96788E8AD51027C2D","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-9907A30A1D61046BB3CED706":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9907A30A1D61046BB3CED706","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":3600},"EVID-AEBD7278AEA481239BF5900E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AEBD7278AEA481239BF5900E","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-C1375153ED8F081F94960AD2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C1375153ED8F081F94960AD2","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-D517C647FD60879252972C6F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D517C647FD60879252972C6F","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":249},"EVID-DAE8F937EC8E2BC926FB7373":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-DAE8F937EC8E2BC926FB7373","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-E7E44A13571351BB72C59DF7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7E44A13571351BB72C59DF7","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV58" s="22" t="inlineStr">
@@ -26172,7 +26172,7 @@
       </c>
       <c r="AZ58" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-2CF9865BFB2C9E9FFFB1F087","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-1A607722905F5626F2592F39","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA58" s="22" t="inlineStr">
@@ -26184,12 +26184,12 @@
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>CAND-1E085EA645EBFB2349B07E26</t>
+          <t>CAND-72B9F4A05D77B11C4A04BA02</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -26373,12 +26373,12 @@
       </c>
       <c r="AT59" s="22" t="inlineStr">
         <is>
-          <t>["EVID-8FDDF71E8ED766014CAF3614","EVID-EE90BBAB0C3D69CFB2392B54","EVID-1484D2B86288BD9635B50252","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
+          <t>["EVID-8FDDF71E8ED766014CAF3614","EVID-EE90BBAB0C3D69CFB2392B54","EVID-CD777A9CADB66005FD36878A","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
         </is>
       </c>
       <c r="AU59" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1484D2B86288BD9635B50252":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1484D2B86288BD9635B50252","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-8FDDF71E8ED766014CAF3614":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8FDDF71E8ED766014CAF3614","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
+          <t>{"EVID-8FDDF71E8ED766014CAF3614":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8FDDF71E8ED766014CAF3614","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-CD777A9CADB66005FD36878A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD777A9CADB66005FD36878A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":58000.0},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
         </is>
       </c>
       <c r="AV59" s="22" t="inlineStr">
@@ -26415,12 +26415,12 @@
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>CAND-0E877A6745803DC5EB83DB93</t>
+          <t>CAND-B6EB43F303C4E8EE0A6DFB03</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
@@ -26604,12 +26604,12 @@
       </c>
       <c r="AT60" s="22" t="inlineStr">
         <is>
-          <t>["EVID-A344FF415E43ADC4B5D305F8","EVID-2A056D89F1674EA69954505E","EVID-173D30F30D973D96C190D660","EVID-13DE1277A3F214D8F8E7400C","EVID-AFA585D0E5C1CA1B67E2DDE8","EVID-B3729CEB99342E73AC28D761","EVID-78C22D80D0216E511EF28D8C","EVID-03A258EE64A16BEDB5966773","EVID-4B874828C8EF72E08DEA0F30","EVID-EE90BBAB0C3D69CFB2392B54","EVID-1484D2B86288BD9635B50252","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
+          <t>["EVID-A344FF415E43ADC4B5D305F8","EVID-2A056D89F1674EA69954505E","EVID-173D30F30D973D96C190D660","EVID-13DE1277A3F214D8F8E7400C","EVID-AFA585D0E5C1CA1B67E2DDE8","EVID-B3729CEB99342E73AC28D761","EVID-78C22D80D0216E511EF28D8C","EVID-03A258EE64A16BEDB5966773","EVID-4B874828C8EF72E08DEA0F30","EVID-EE90BBAB0C3D69CFB2392B54","EVID-CD777A9CADB66005FD36878A","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
         </is>
       </c>
       <c r="AU60" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-03A258EE64A16BEDB5966773":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-03A258EE64A16BEDB5966773","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":36000},"EVID-13DE1277A3F214D8F8E7400C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-13DE1277A3F214D8F8E7400C","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":2147483648},"EVID-1484D2B86288BD9635B50252":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1484D2B86288BD9635B50252","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-173D30F30D973D96C190D660":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-173D30F30D973D96C190D660","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":412},"EVID-2A056D89F1674EA69954505E":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2A056D89F1674EA69954505E","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":4.2},"EVID-4B874828C8EF72E08DEA0F30":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B874828C8EF72E08DEA0F30","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-78C22D80D0216E511EF28D8C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-78C22D80D0216E511EF28D8C","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":11000},"EVID-A344FF415E43ADC4B5D305F8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A344FF415E43ADC4B5D305F8","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-AFA585D0E5C1CA1B67E2DDE8":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-AFA585D0E5C1CA1B67E2DDE8","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":1.0},"EVID-B3729CEB99342E73AC28D761":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-B3729CEB99342E73AC28D761","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
+          <t>{"EVID-03A258EE64A16BEDB5966773":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-03A258EE64A16BEDB5966773","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":36000},"EVID-13DE1277A3F214D8F8E7400C":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-13DE1277A3F214D8F8E7400C","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":2147483648},"EVID-173D30F30D973D96C190D660":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-173D30F30D973D96C190D660","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":412},"EVID-2A056D89F1674EA69954505E":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-2A056D89F1674EA69954505E","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":4.2},"EVID-4B874828C8EF72E08DEA0F30":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B874828C8EF72E08DEA0F30","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-78C22D80D0216E511EF28D8C":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-78C22D80D0216E511EF28D8C","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":11000},"EVID-A344FF415E43ADC4B5D305F8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A344FF415E43ADC4B5D305F8","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"LARGE"},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-AFA585D0E5C1CA1B67E2DDE8":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-AFA585D0E5C1CA1B67E2DDE8","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":1.0},"EVID-B3729CEB99342E73AC28D761":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-B3729CEB99342E73AC28D761","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-CD777A9CADB66005FD36878A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD777A9CADB66005FD36878A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":58000.0},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
         </is>
       </c>
       <c r="AV60" s="22" t="inlineStr">
@@ -26634,7 +26634,7 @@
       </c>
       <c r="AZ60" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY","scenario_id":"SCN-6034F47F88FE870BCBD38A83","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY","scenario_id":"SCN-AC27CF4B8FF664CD14E343AA","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA60" s="22" t="inlineStr">
@@ -26646,12 +26646,12 @@
     <row r="61" ht="32" customHeight="1">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>CAND-3E3533A2458836277B998E86</t>
+          <t>CAND-AEF82F4F82A158C8B6DEE7FC</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
@@ -26831,12 +26831,12 @@
       </c>
       <c r="AT61" s="22" t="inlineStr">
         <is>
-          <t>["EVID-D187DFEAE1763FDDD86483AA","EVID-9F221DC63C2B232A5A2F6CEA","EVID-5C92297D19DABFC0D44936CE","EVID-8AACAEEF28E431476CC1B4D7","EVID-F772EC513A5C2299BF08C8D9","EVID-C59B9CC24DF2F6B383FBBDD7","EVID-EE90BBAB0C3D69CFB2392B54","EVID-1484D2B86288BD9635B50252","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
+          <t>["EVID-D187DFEAE1763FDDD86483AA","EVID-9F221DC63C2B232A5A2F6CEA","EVID-5C92297D19DABFC0D44936CE","EVID-8AACAEEF28E431476CC1B4D7","EVID-F772EC513A5C2299BF08C8D9","EVID-C59B9CC24DF2F6B383FBBDD7","EVID-EE90BBAB0C3D69CFB2392B54","EVID-CD777A9CADB66005FD36878A","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
         </is>
       </c>
       <c r="AU61" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1484D2B86288BD9635B50252":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1484D2B86288BD9635B50252","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-5C92297D19DABFC0D44936CE":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5C92297D19DABFC0D44936CE","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":15.0},"EVID-8AACAEEF28E431476CC1B4D7":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-8AACAEEF28E431476CC1B4D7","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":1.0},"EVID-9F221DC63C2B232A5A2F6CEA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9F221DC63C2B232A5A2F6CEA","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":7},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-C59B9CC24DF2F6B383FBBDD7":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-C59B9CC24DF2F6B383FBBDD7","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":9000},"EVID-D187DFEAE1763FDDD86483AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D187DFEAE1763FDDD86483AA","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":8},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0},"EVID-F772EC513A5C2299BF08C8D9":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-F772EC513A5C2299BF08C8D9","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":98}}</t>
+          <t>{"EVID-5C92297D19DABFC0D44936CE":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5C92297D19DABFC0D44936CE","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":15.0},"EVID-8AACAEEF28E431476CC1B4D7":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-8AACAEEF28E431476CC1B4D7","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":1.0},"EVID-9F221DC63C2B232A5A2F6CEA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9F221DC63C2B232A5A2F6CEA","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":7},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-C59B9CC24DF2F6B383FBBDD7":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-C59B9CC24DF2F6B383FBBDD7","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":9000},"EVID-CD777A9CADB66005FD36878A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD777A9CADB66005FD36878A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":58000.0},"EVID-D187DFEAE1763FDDD86483AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D187DFEAE1763FDDD86483AA","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":8},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0},"EVID-F772EC513A5C2299BF08C8D9":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-F772EC513A5C2299BF08C8D9","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":98}}</t>
         </is>
       </c>
       <c r="AV61" s="22" t="inlineStr">
@@ -26873,12 +26873,12 @@
     <row r="62" ht="32" customHeight="1">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>CAND-A3DE947D6AF269F223F3E0EF</t>
+          <t>CAND-E7EBDE9C9950918CFE5D7D41</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
@@ -27058,12 +27058,12 @@
       </c>
       <c r="AT62" s="22" t="inlineStr">
         <is>
-          <t>["EVID-6F22403CC3615114ACF5B618","EVID-BF41760B14372497E2F416C7","EVID-BCF06BC5C9ABBA23587D9AAD","EVID-6F6A8539FD4499A3F56C3D3E","EVID-0E17892A53D58AB0E3D81DA9","EVID-EE90BBAB0C3D69CFB2392B54","EVID-1484D2B86288BD9635B50252","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
+          <t>["EVID-6F22403CC3615114ACF5B618","EVID-BF41760B14372497E2F416C7","EVID-BCF06BC5C9ABBA23587D9AAD","EVID-6F6A8539FD4499A3F56C3D3E","EVID-0E17892A53D58AB0E3D81DA9","EVID-EE90BBAB0C3D69CFB2392B54","EVID-CD777A9CADB66005FD36878A","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
         </is>
       </c>
       <c r="AU62" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0E17892A53D58AB0E3D81DA9":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-0E17892A53D58AB0E3D81DA9","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":15.0},"EVID-1484D2B86288BD9635B50252":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1484D2B86288BD9635B50252","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-6F22403CC3615114ACF5B618":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6F22403CC3615114ACF5B618","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2},"EVID-6F6A8539FD4499A3F56C3D3E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-6F6A8539FD4499A3F56C3D3E","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":9000},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-BCF06BC5C9ABBA23587D9AAD":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-BCF06BC5C9ABBA23587D9AAD","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":1.0},"EVID-BF41760B14372497E2F416C7":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-BF41760B14372497E2F416C7","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":35.0},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
+          <t>{"EVID-0E17892A53D58AB0E3D81DA9":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-0E17892A53D58AB0E3D81DA9","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":15.0},"EVID-6F22403CC3615114ACF5B618":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6F22403CC3615114ACF5B618","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2},"EVID-6F6A8539FD4499A3F56C3D3E":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-6F6A8539FD4499A3F56C3D3E","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":9000},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-BCF06BC5C9ABBA23587D9AAD":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-BCF06BC5C9ABBA23587D9AAD","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":1.0},"EVID-BF41760B14372497E2F416C7":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-BF41760B14372497E2F416C7","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":35.0},"EVID-CD777A9CADB66005FD36878A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD777A9CADB66005FD36878A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":58000.0},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
         </is>
       </c>
       <c r="AV62" s="22" t="inlineStr">
@@ -27100,12 +27100,12 @@
     <row r="63" ht="32" customHeight="1">
       <c r="A63" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>CAND-497F0500B2853FDB8B49F0E2</t>
+          <t>CAND-347FA9E6410390B0FEC735D0</t>
         </is>
       </c>
       <c r="C63" s="14" t="inlineStr">
@@ -27285,12 +27285,12 @@
       </c>
       <c r="AT63" s="22" t="inlineStr">
         <is>
-          <t>["EVID-6AAE5CF1ECE6878C2CF26D21","EVID-E7D093253C03B8E31471B2A1","EVID-44B03B2E73C720355A16DDE9","EVID-5F409B008B651F25022FB9F1","EVID-425B9A2FF4A64BAA904964D0","EVID-17090E3CB43BF9A4A57ABFE7","EVID-7162B5A4A2E75540071E6568","EVID-713796EA239C1695235EF207","EVID-EE90BBAB0C3D69CFB2392B54","EVID-1484D2B86288BD9635B50252","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
+          <t>["EVID-6AAE5CF1ECE6878C2CF26D21","EVID-E7D093253C03B8E31471B2A1","EVID-44B03B2E73C720355A16DDE9","EVID-5F409B008B651F25022FB9F1","EVID-425B9A2FF4A64BAA904964D0","EVID-17090E3CB43BF9A4A57ABFE7","EVID-7162B5A4A2E75540071E6568","EVID-713796EA239C1695235EF207","EVID-EE90BBAB0C3D69CFB2392B54","EVID-CD777A9CADB66005FD36878A","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
         </is>
       </c>
       <c r="AU63" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1484D2B86288BD9635B50252":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1484D2B86288BD9635B50252","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-17090E3CB43BF9A4A57ABFE7":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-17090E3CB43BF9A4A57ABFE7","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-425B9A2FF4A64BAA904964D0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-425B9A2FF4A64BAA904964D0","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-44B03B2E73C720355A16DDE9":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-44B03B2E73C720355A16DDE9","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":392},"EVID-5F409B008B651F25022FB9F1":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-5F409B008B651F25022FB9F1","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":130000.0},"EVID-6AAE5CF1ECE6878C2CF26D21":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-6AAE5CF1ECE6878C2CF26D21","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":45},"EVID-713796EA239C1695235EF207":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-713796EA239C1695235EF207","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1728.0},"EVID-7162B5A4A2E75540071E6568":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-7162B5A4A2E75540071E6568","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-E7D093253C03B8E31471B2A1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7D093253C03B8E31471B2A1","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":326.67},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
+          <t>{"EVID-17090E3CB43BF9A4A57ABFE7":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-17090E3CB43BF9A4A57ABFE7","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-425B9A2FF4A64BAA904964D0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-425B9A2FF4A64BAA904964D0","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-44B03B2E73C720355A16DDE9":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-44B03B2E73C720355A16DDE9","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":392},"EVID-5F409B008B651F25022FB9F1":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-5F409B008B651F25022FB9F1","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":130000.0},"EVID-6AAE5CF1ECE6878C2CF26D21":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-6AAE5CF1ECE6878C2CF26D21","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":45},"EVID-713796EA239C1695235EF207":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-713796EA239C1695235EF207","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1728.0},"EVID-7162B5A4A2E75540071E6568":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-7162B5A4A2E75540071E6568","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-CD777A9CADB66005FD36878A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD777A9CADB66005FD36878A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":58000.0},"EVID-E7D093253C03B8E31471B2A1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E7D093253C03B8E31471B2A1","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":326.67},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0}}</t>
         </is>
       </c>
       <c r="AV63" s="22" t="inlineStr">
@@ -27315,7 +27315,7 @@
       </c>
       <c r="AZ63" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-6034F47F88FE870BCBD38A83","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-AC27CF4B8FF664CD14E343AA","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA63" s="22" t="inlineStr">
@@ -27327,12 +27327,12 @@
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>PKG-293F70C0D8CCCD1D7E5449C8</t>
+          <t>PKG-72B28A1A84F29D0A01B3AC5F</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>CAND-3588FD08E2C2D20AB63356BE</t>
+          <t>CAND-EDC5DB36F0D1AC83E7D2D87F</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
@@ -27516,12 +27516,12 @@
       </c>
       <c r="AT64" s="22" t="inlineStr">
         <is>
-          <t>["EVID-86AA6C5EC99B8A9212BEB2BC","EVID-D120D5D150026DD0020186ED","EVID-6E448D71588E95147EFF2F88","EVID-E96DF29A15DA7414D3724B94","EVID-C81F08A5E6EFA115692E37D1","EVID-C54ADBED5D740B08A9ABDE1A","EVID-77561C963E48CE1FD39A2EF6","EVID-EB97E31584CD7C2D55ED8084","EVID-F92EDAAB3D1B901B5682377E","EVID-8D442199D3A610D39837FACC","EVID-86A54913D98871BFD62DA3D6","EVID-90948AD02E9D2F3CDA3FCC77","EVID-6463CC8FB6187D01932BF793","EVID-EE90BBAB0C3D69CFB2392B54","EVID-1484D2B86288BD9635B50252","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
+          <t>["EVID-86AA6C5EC99B8A9212BEB2BC","EVID-D120D5D150026DD0020186ED","EVID-6E448D71588E95147EFF2F88","EVID-E96DF29A15DA7414D3724B94","EVID-C81F08A5E6EFA115692E37D1","EVID-C54ADBED5D740B08A9ABDE1A","EVID-77561C963E48CE1FD39A2EF6","EVID-EB97E31584CD7C2D55ED8084","EVID-F92EDAAB3D1B901B5682377E","EVID-8D442199D3A610D39837FACC","EVID-86A54913D98871BFD62DA3D6","EVID-90948AD02E9D2F3CDA3FCC77","EVID-6463CC8FB6187D01932BF793","EVID-EE90BBAB0C3D69CFB2392B54","EVID-CD777A9CADB66005FD36878A","EVID-B60E411C1121A2E587066DF4","EVID-AB2B7562E0C8B11CCC0C5784"]</t>
         </is>
       </c>
       <c r="AU64" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1484D2B86288BD9635B50252":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1484D2B86288BD9635B50252","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":58000.0},"EVID-6463CC8FB6187D01932BF793":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6463CC8FB6187D01932BF793","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-6E448D71588E95147EFF2F88":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6E448D71588E95147EFF2F88","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-77561C963E48CE1FD39A2EF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-77561C963E48CE1FD39A2EF6","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-86A54913D98871BFD62DA3D6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-86A54913D98871BFD62DA3D6","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-86AA6C5EC99B8A9212BEB2BC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-86AA6C5EC99B8A9212BEB2BC","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-8D442199D3A610D39837FACC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8D442199D3A610D39837FACC","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-90948AD02E9D2F3CDA3FCC77":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-90948AD02E9D2F3CDA3FCC77","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-C54ADBED5D740B08A9ABDE1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C54ADBED5D740B08A9ABDE1A","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-C81F08A5E6EFA115692E37D1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C81F08A5E6EFA115692E37D1","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":7350},"EVID-D120D5D150026DD0020186ED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D120D5D150026DD0020186ED","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-E96DF29A15DA7414D3724B94":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E96DF29A15DA7414D3724B94","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-EB97E31584CD7C2D55ED8084":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EB97E31584CD7C2D55ED8084","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0},"EVID-F92EDAAB3D1B901B5682377E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F92EDAAB3D1B901B5682377E","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":784}}</t>
+          <t>{"EVID-6463CC8FB6187D01932BF793":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6463CC8FB6187D01932BF793","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-6E448D71588E95147EFF2F88":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6E448D71588E95147EFF2F88","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-77561C963E48CE1FD39A2EF6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-77561C963E48CE1FD39A2EF6","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-86A54913D98871BFD62DA3D6":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-86A54913D98871BFD62DA3D6","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-86AA6C5EC99B8A9212BEB2BC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-86AA6C5EC99B8A9212BEB2BC","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-8D442199D3A610D39837FACC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8D442199D3A610D39837FACC","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-90948AD02E9D2F3CDA3FCC77":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-90948AD02E9D2F3CDA3FCC77","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-AB2B7562E0C8B11CCC0C5784":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB2B7562E0C8B11CCC0C5784","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":262},"EVID-B60E411C1121A2E587066DF4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B60E411C1121A2E587066DF4","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":37670.23},"EVID-C54ADBED5D740B08A9ABDE1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C54ADBED5D740B08A9ABDE1A","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-C81F08A5E6EFA115692E37D1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C81F08A5E6EFA115692E37D1","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":7350},"EVID-CD777A9CADB66005FD36878A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CD777A9CADB66005FD36878A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":58000.0},"EVID-D120D5D150026DD0020186ED":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D120D5D150026DD0020186ED","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-E96DF29A15DA7414D3724B94":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E96DF29A15DA7414D3724B94","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-EB97E31584CD7C2D55ED8084":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EB97E31584CD7C2D55ED8084","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-EE90BBAB0C3D69CFB2392B54":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EE90BBAB0C3D69CFB2392B54","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":51040.0},"EVID-F92EDAAB3D1B901B5682377E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F92EDAAB3D1B901B5682377E","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":784}}</t>
         </is>
       </c>
       <c r="AV64" s="22" t="inlineStr">
@@ -27546,7 +27546,7 @@
       </c>
       <c r="AZ64" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-60E6E4CF8B3C2E2611EA9BFA","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-7DA4C286CAFA46529A941D00","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA64" s="22" t="inlineStr">
@@ -27558,12 +27558,12 @@
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>CAND-129F67319BADFA2CE089FF64</t>
+          <t>CAND-8805373F493C9312FE14B270</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
@@ -27747,12 +27747,12 @@
       </c>
       <c r="AT65" s="22" t="inlineStr">
         <is>
-          <t>["EVID-5E2B2F90F6A7FB35A3F53418","EVID-50F616330E5AB32E27962258","EVID-99EACDD52661CD8933464BA5","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
+          <t>["EVID-5E2B2F90F6A7FB35A3F53418","EVID-50F616330E5AB32E27962258","EVID-68034385A85814CE5E9D431D","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
         </is>
       </c>
       <c r="AU65" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-5E2B2F90F6A7FB35A3F53418":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5E2B2F90F6A7FB35A3F53418","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-99EACDD52661CD8933464BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-99EACDD52661CD8933464BA5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252}}</t>
+          <t>{"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-5E2B2F90F6A7FB35A3F53418":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5E2B2F90F6A7FB35A3F53418","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-68034385A85814CE5E9D431D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68034385A85814CE5E9D431D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":15500.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252}}</t>
         </is>
       </c>
       <c r="AV65" s="22" t="inlineStr">
@@ -27789,12 +27789,12 @@
     <row r="66" ht="32" customHeight="1">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>CAND-7ADCC0E72B9FC08857017FB5</t>
+          <t>CAND-4C2622B3D4EF1E9ED54322C7</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
@@ -27978,12 +27978,12 @@
       </c>
       <c r="AT66" s="22" t="inlineStr">
         <is>
-          <t>["EVID-20B43961F3C6C1A2EE95A29D","EVID-070F7AF4873DD67819657684","EVID-AD888A128A52C49972FDD70D","EVID-8DEEE675FDE9D16D0002AF87","EVID-BE35B69390609AEABE70E371","EVID-0226BD31F1B474314ECB9FDD","EVID-E027D765B3EFD2171CC0F0E5","EVID-B8BA520171E53FD0595019DF","EVID-07DD446F0342AA9E5EE9CD19","EVID-50F616330E5AB32E27962258","EVID-99EACDD52661CD8933464BA5","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
+          <t>["EVID-20B43961F3C6C1A2EE95A29D","EVID-070F7AF4873DD67819657684","EVID-AD888A128A52C49972FDD70D","EVID-8DEEE675FDE9D16D0002AF87","EVID-BE35B69390609AEABE70E371","EVID-0226BD31F1B474314ECB9FDD","EVID-E027D765B3EFD2171CC0F0E5","EVID-B8BA520171E53FD0595019DF","EVID-07DD446F0342AA9E5EE9CD19","EVID-50F616330E5AB32E27962258","EVID-68034385A85814CE5E9D431D","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
         </is>
       </c>
       <c r="AU66" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0226BD31F1B474314ECB9FDD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0226BD31F1B474314ECB9FDD","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-070F7AF4873DD67819657684":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-070F7AF4873DD67819657684","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-07DD446F0342AA9E5EE9CD19":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-07DD446F0342AA9E5EE9CD19","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-20B43961F3C6C1A2EE95A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-20B43961F3C6C1A2EE95A29D","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-8DEEE675FDE9D16D0002AF87":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8DEEE675FDE9D16D0002AF87","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-99EACDD52661CD8933464BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-99EACDD52661CD8933464BA5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-AD888A128A52C49972FDD70D":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-AD888A128A52C49972FDD70D","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-B8BA520171E53FD0595019DF":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-B8BA520171E53FD0595019DF","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6000},"EVID-BE35B69390609AEABE70E371":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-BE35B69390609AEABE70E371","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-E027D765B3EFD2171CC0F0E5":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E027D765B3EFD2171CC0F0E5","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2000},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252}}</t>
+          <t>{"EVID-0226BD31F1B474314ECB9FDD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0226BD31F1B474314ECB9FDD","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-070F7AF4873DD67819657684":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-070F7AF4873DD67819657684","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-07DD446F0342AA9E5EE9CD19":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-07DD446F0342AA9E5EE9CD19","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-20B43961F3C6C1A2EE95A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-20B43961F3C6C1A2EE95A29D","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-68034385A85814CE5E9D431D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68034385A85814CE5E9D431D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":15500.0},"EVID-8DEEE675FDE9D16D0002AF87":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8DEEE675FDE9D16D0002AF87","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-AD888A128A52C49972FDD70D":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-AD888A128A52C49972FDD70D","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-B8BA520171E53FD0595019DF":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-B8BA520171E53FD0595019DF","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":6000},"EVID-BE35B69390609AEABE70E371":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-BE35B69390609AEABE70E371","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-E027D765B3EFD2171CC0F0E5":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-E027D765B3EFD2171CC0F0E5","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2000},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252}}</t>
         </is>
       </c>
       <c r="AV66" s="22" t="inlineStr">
@@ -28008,7 +28008,7 @@
       </c>
       <c r="AZ66" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-F8D0AE11F3CFA07D7DFBD032","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-578A1D1819D737E19D5DEDBE","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA66" s="22" t="inlineStr">
@@ -28020,12 +28020,12 @@
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>CAND-55B90A7F8AD84F5FFABA5BD2</t>
+          <t>CAND-6A4B2951E2A605857E3D99F2</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
@@ -28205,12 +28205,12 @@
       </c>
       <c r="AT67" s="22" t="inlineStr">
         <is>
-          <t>["EVID-39EADFD6CF9C66CE5165ED62","EVID-5066EABB27208C07CAC1039A","EVID-01425C0BD47160649D9BDBF9","EVID-24D506A8E7E2AEB695EA147B","EVID-B0FA3283F415F95E654D23E0","EVID-8B7E04D0182B235AA7CA4455","EVID-50F616330E5AB32E27962258","EVID-99EACDD52661CD8933464BA5","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
+          <t>["EVID-39EADFD6CF9C66CE5165ED62","EVID-5066EABB27208C07CAC1039A","EVID-01425C0BD47160649D9BDBF9","EVID-24D506A8E7E2AEB695EA147B","EVID-B0FA3283F415F95E654D23E0","EVID-8B7E04D0182B235AA7CA4455","EVID-50F616330E5AB32E27962258","EVID-68034385A85814CE5E9D431D","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
         </is>
       </c>
       <c r="AU67" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-01425C0BD47160649D9BDBF9":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-01425C0BD47160649D9BDBF9","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-24D506A8E7E2AEB695EA147B":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-24D506A8E7E2AEB695EA147B","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-39EADFD6CF9C66CE5165ED62":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-39EADFD6CF9C66CE5165ED62","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":2},"EVID-5066EABB27208C07CAC1039A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5066EABB27208C07CAC1039A","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-8B7E04D0182B235AA7CA4455":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-8B7E04D0182B235AA7CA4455","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-99EACDD52661CD8933464BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-99EACDD52661CD8933464BA5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-B0FA3283F415F95E654D23E0":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-B0FA3283F415F95E654D23E0","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252}}</t>
+          <t>{"EVID-01425C0BD47160649D9BDBF9":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-01425C0BD47160649D9BDBF9","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-24D506A8E7E2AEB695EA147B":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-24D506A8E7E2AEB695EA147B","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-39EADFD6CF9C66CE5165ED62":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-39EADFD6CF9C66CE5165ED62","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":2},"EVID-5066EABB27208C07CAC1039A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5066EABB27208C07CAC1039A","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-68034385A85814CE5E9D431D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68034385A85814CE5E9D431D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":15500.0},"EVID-8B7E04D0182B235AA7CA4455":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-8B7E04D0182B235AA7CA4455","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-B0FA3283F415F95E654D23E0":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-B0FA3283F415F95E654D23E0","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252}}</t>
         </is>
       </c>
       <c r="AV67" s="22" t="inlineStr">
@@ -28247,12 +28247,12 @@
     <row r="68" ht="32" customHeight="1">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>CAND-76FF89D1C033A3CA62741ACF</t>
+          <t>CAND-016EDFB75AF0AF6A2C07E315</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
@@ -28432,12 +28432,12 @@
       </c>
       <c r="AT68" s="22" t="inlineStr">
         <is>
-          <t>["EVID-9F434CDB24D2A3FE3556080D","EVID-82066A1F9E22BA891367ABC2","EVID-FB48096C1335A2562EDE03B0","EVID-D3FEC6D7C214B8D3BF551FE2","EVID-AF75DEF9DB7D574EDF91EC64","EVID-50F616330E5AB32E27962258","EVID-99EACDD52661CD8933464BA5","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
+          <t>["EVID-9F434CDB24D2A3FE3556080D","EVID-82066A1F9E22BA891367ABC2","EVID-FB48096C1335A2562EDE03B0","EVID-D3FEC6D7C214B8D3BF551FE2","EVID-AF75DEF9DB7D574EDF91EC64","EVID-50F616330E5AB32E27962258","EVID-68034385A85814CE5E9D431D","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
         </is>
       </c>
       <c r="AU68" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-82066A1F9E22BA891367ABC2":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-82066A1F9E22BA891367ABC2","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":90.0},"EVID-99EACDD52661CD8933464BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-99EACDD52661CD8933464BA5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-9F434CDB24D2A3FE3556080D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9F434CDB24D2A3FE3556080D","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2},"EVID-AF75DEF9DB7D574EDF91EC64":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-AF75DEF9DB7D574EDF91EC64","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-D3FEC6D7C214B8D3BF551FE2":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-D3FEC6D7C214B8D3BF551FE2","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-FB48096C1335A2562EDE03B0":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-FB48096C1335A2562EDE03B0","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0}}</t>
+          <t>{"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-68034385A85814CE5E9D431D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68034385A85814CE5E9D431D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":15500.0},"EVID-82066A1F9E22BA891367ABC2":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-82066A1F9E22BA891367ABC2","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":90.0},"EVID-9F434CDB24D2A3FE3556080D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9F434CDB24D2A3FE3556080D","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":2},"EVID-AF75DEF9DB7D574EDF91EC64":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-AF75DEF9DB7D574EDF91EC64","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-D3FEC6D7C214B8D3BF551FE2":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-D3FEC6D7C214B8D3BF551FE2","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-FB48096C1335A2562EDE03B0":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-FB48096C1335A2562EDE03B0","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0}}</t>
         </is>
       </c>
       <c r="AV68" s="22" t="inlineStr">
@@ -28462,7 +28462,7 @@
       </c>
       <c r="AZ68" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F8D0AE11F3CFA07D7DFBD032","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-578A1D1819D737E19D5DEDBE","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA68" s="22" t="inlineStr">
@@ -28474,12 +28474,12 @@
     <row r="69" ht="32" customHeight="1">
       <c r="A69" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>CAND-5763B8095F259B3EEED222B0</t>
+          <t>CAND-4C891B8A1136F219041C9F4E</t>
         </is>
       </c>
       <c r="C69" s="14" t="inlineStr">
@@ -28659,12 +28659,12 @@
       </c>
       <c r="AT69" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4E38AC87147767827FFDF2EC","EVID-964D24D8B7D84854CFE55FA8","EVID-0DADE24E847363DC78BF885D","EVID-F13795802F91F9228B6FFB67","EVID-43592DE0B8462712436545A5","EVID-C182DDECD19F750F8D25FA15","EVID-2C3474A5C11EEF4B849349EF","EVID-5B407641EEE5BA93D851431E","EVID-50F616330E5AB32E27962258","EVID-99EACDD52661CD8933464BA5","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
+          <t>["EVID-4E38AC87147767827FFDF2EC","EVID-964D24D8B7D84854CFE55FA8","EVID-0DADE24E847363DC78BF885D","EVID-F13795802F91F9228B6FFB67","EVID-43592DE0B8462712436545A5","EVID-C182DDECD19F750F8D25FA15","EVID-2C3474A5C11EEF4B849349EF","EVID-5B407641EEE5BA93D851431E","EVID-50F616330E5AB32E27962258","EVID-68034385A85814CE5E9D431D","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
         </is>
       </c>
       <c r="AU69" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0DADE24E847363DC78BF885D":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-0DADE24E847363DC78BF885D","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":128},"EVID-2C3474A5C11EEF4B849349EF":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-2C3474A5C11EEF4B849349EF","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1333},"EVID-43592DE0B8462712436545A5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-43592DE0B8462712436545A5","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":4},"EVID-4E38AC87147767827FFDF2EC":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-4E38AC87147767827FFDF2EC","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-5B407641EEE5BA93D851431E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5B407641EEE5BA93D851431E","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-964D24D8B7D84854CFE55FA8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-964D24D8B7D84854CFE55FA8","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":106.67},"EVID-99EACDD52661CD8933464BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-99EACDD52661CD8933464BA5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-C182DDECD19F750F8D25FA15":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-C182DDECD19F750F8D25FA15","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-F13795802F91F9228B6FFB67":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-F13795802F91F9228B6FFB67","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":40000.0}}</t>
+          <t>{"EVID-0DADE24E847363DC78BF885D":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-0DADE24E847363DC78BF885D","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":128},"EVID-2C3474A5C11EEF4B849349EF":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-2C3474A5C11EEF4B849349EF","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1333},"EVID-43592DE0B8462712436545A5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-43592DE0B8462712436545A5","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":4},"EVID-4E38AC87147767827FFDF2EC":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-4E38AC87147767827FFDF2EC","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":120},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-5B407641EEE5BA93D851431E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-5B407641EEE5BA93D851431E","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":7920.0},"EVID-68034385A85814CE5E9D431D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68034385A85814CE5E9D431D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":15500.0},"EVID-964D24D8B7D84854CFE55FA8":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-964D24D8B7D84854CFE55FA8","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":106.67},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-C182DDECD19F750F8D25FA15":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-C182DDECD19F750F8D25FA15","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-F13795802F91F9228B6FFB67":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-F13795802F91F9228B6FFB67","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":40000.0}}</t>
         </is>
       </c>
       <c r="AV69" s="22" t="inlineStr">
@@ -28689,7 +28689,7 @@
       </c>
       <c r="AZ69" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-F8D0AE11F3CFA07D7DFBD032","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-578A1D1819D737E19D5DEDBE","scenario_name":"Plan A — Optimize current warehouse type","step":3}]</t>
         </is>
       </c>
       <c r="BA69" s="22" t="inlineStr">
@@ -28701,12 +28701,12 @@
     <row r="70" ht="32" customHeight="1">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>PKG-4379CF0AEFE42673A832518C</t>
+          <t>PKG-AB5BA2CB27FA33C4F2BE7A85</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>CAND-AC5879A21066084E08E49997</t>
+          <t>CAND-C1507494ED1BA885FBF9071F</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
@@ -28890,12 +28890,12 @@
       </c>
       <c r="AT70" s="22" t="inlineStr">
         <is>
-          <t>["EVID-EC39084808469B0496A22797","EVID-E06323EF562817A561795FDA","EVID-8C522E311D367BAF61F3E85A","EVID-4093408BEE57005F6E49D35A","EVID-A9B9E90D64D9BB66A374C8AA","EVID-979658122CEE3DF38426CB8E","EVID-CB205C7DCDC2DCF82E6A039B","EVID-F00D55756F8FD6C9CF89C2AF","EVID-D29573C2C46F89F85FAB8045","EVID-4A2C03CEA6A05D220F7D2277","EVID-EBECC6E7D3E86EC9BF696CBC","EVID-AF4D3B48D369F40E23E3E9BD","EVID-0DAD979C2237FD3233FFDBB7","EVID-50F616330E5AB32E27962258","EVID-99EACDD52661CD8933464BA5","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
+          <t>["EVID-EC39084808469B0496A22797","EVID-E06323EF562817A561795FDA","EVID-8C522E311D367BAF61F3E85A","EVID-4093408BEE57005F6E49D35A","EVID-A9B9E90D64D9BB66A374C8AA","EVID-979658122CEE3DF38426CB8E","EVID-CB205C7DCDC2DCF82E6A039B","EVID-F00D55756F8FD6C9CF89C2AF","EVID-D29573C2C46F89F85FAB8045","EVID-4A2C03CEA6A05D220F7D2277","EVID-EBECC6E7D3E86EC9BF696CBC","EVID-AF4D3B48D369F40E23E3E9BD","EVID-0DAD979C2237FD3233FFDBB7","EVID-50F616330E5AB32E27962258","EVID-68034385A85814CE5E9D431D","EVID-BECB952FE23A55CFA5BADC5E","EVID-E1D312A511027E48D5E88AB0"]</t>
         </is>
       </c>
       <c r="AU70" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0DAD979C2237FD3233FFDBB7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0DAD979C2237FD3233FFDBB7","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-4093408BEE57005F6E49D35A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4093408BEE57005F6E49D35A","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":2400},"EVID-4A2C03CEA6A05D220F7D2277":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4A2C03CEA6A05D220F7D2277","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":800},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-8C522E311D367BAF61F3E85A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8C522E311D367BAF61F3E85A","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-979658122CEE3DF38426CB8E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-979658122CEE3DF38426CB8E","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-99EACDD52661CD8933464BA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-99EACDD52661CD8933464BA5","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":15500.0},"EVID-A9B9E90D64D9BB66A374C8AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A9B9E90D64D9BB66A374C8AA","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-AF4D3B48D369F40E23E3E9BD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AF4D3B48D369F40E23E3E9BD","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-CB205C7DCDC2DCF82E6A039B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CB205C7DCDC2DCF82E6A039B","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-D29573C2C46F89F85FAB8045":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D29573C2C46F89F85FAB8045","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":256},"EVID-E06323EF562817A561795FDA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E06323EF562817A561795FDA","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-EBECC6E7D3E86EC9BF696CBC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EBECC6E7D3E86EC9BF696CBC","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-EC39084808469B0496A22797":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EC39084808469B0496A22797","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-F00D55756F8FD6C9CF89C2AF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F00D55756F8FD6C9CF89C2AF","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0}}</t>
+          <t>{"EVID-0DAD979C2237FD3233FFDBB7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0DAD979C2237FD3233FFDBB7","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-4093408BEE57005F6E49D35A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4093408BEE57005F6E49D35A","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":2400},"EVID-4A2C03CEA6A05D220F7D2277":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4A2C03CEA6A05D220F7D2277","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":800},"EVID-50F616330E5AB32E27962258":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-50F616330E5AB32E27962258","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":13640.0},"EVID-68034385A85814CE5E9D431D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-68034385A85814CE5E9D431D","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":15500.0},"EVID-8C522E311D367BAF61F3E85A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8C522E311D367BAF61F3E85A","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-979658122CEE3DF38426CB8E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-979658122CEE3DF38426CB8E","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-A9B9E90D64D9BB66A374C8AA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-A9B9E90D64D9BB66A374C8AA","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-AF4D3B48D369F40E23E3E9BD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AF4D3B48D369F40E23E3E9BD","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-BECB952FE23A55CFA5BADC5E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BECB952FE23A55CFA5BADC5E","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3615.24},"EVID-CB205C7DCDC2DCF82E6A039B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CB205C7DCDC2DCF82E6A039B","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-D29573C2C46F89F85FAB8045":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D29573C2C46F89F85FAB8045","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":256},"EVID-E06323EF562817A561795FDA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E06323EF562817A561795FDA","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-E1D312A511027E48D5E88AB0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1D312A511027E48D5E88AB0","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":252},"EVID-EBECC6E7D3E86EC9BF696CBC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EBECC6E7D3E86EC9BF696CBC","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-EC39084808469B0496A22797":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-EC39084808469B0496A22797","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-F00D55756F8FD6C9CF89C2AF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F00D55756F8FD6C9CF89C2AF","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV70" s="22" t="inlineStr">
@@ -28920,7 +28920,7 @@
       </c>
       <c r="AZ70" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-80FA6497D1269DF9BC6CDAC9","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-D3A3FAD11AC31FEC9D1A2AB5","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA70" s="22" t="inlineStr">
@@ -28932,12 +28932,12 @@
     <row r="71" ht="32" customHeight="1">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>CAND-244B6A9BF1597473726DCECE</t>
+          <t>CAND-69FB4749B4D73D743D4C0864</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
@@ -29121,12 +29121,12 @@
       </c>
       <c r="AT71" s="22" t="inlineStr">
         <is>
-          <t>["EVID-45924CB6AA2E38CA92267128","EVID-34C490032C237ACC89D87EC2","EVID-CA272E3BD0899A1D187BF510","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
+          <t>["EVID-45924CB6AA2E38CA92267128","EVID-34C490032C237ACC89D87EC2","EVID-8866BAE17752BA680D35AD9A","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
         </is>
       </c>
       <c r="AU71" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-45924CB6AA2E38CA92267128":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-45924CB6AA2E38CA92267128","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-CA272E3BD0899A1D187BF510":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CA272E3BD0899A1D187BF510","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0}}</t>
+          <t>{"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-45924CB6AA2E38CA92267128":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-45924CB6AA2E38CA92267128","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-8866BAE17752BA680D35AD9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8866BAE17752BA680D35AD9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":26000.0}}</t>
         </is>
       </c>
       <c r="AV71" s="22" t="inlineStr">
@@ -29163,12 +29163,12 @@
     <row r="72" ht="32" customHeight="1">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>CAND-CD04AB68BD52CC1E1EB78D67</t>
+          <t>CAND-0E0C39CCFED2B26094B35BC6</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
@@ -29352,12 +29352,12 @@
       </c>
       <c r="AT72" s="22" t="inlineStr">
         <is>
-          <t>["EVID-E62E849BC0654AAF5D85EAB7","EVID-3DAFFB80935B845D569F18C4","EVID-B2D7C2EE2968246DB663D751","EVID-10240CC6FE1740F33E7065A9","EVID-FE0A8787D4FE7A85E7328F2A","EVID-6231DA309B2890FEE5630D9F","EVID-5CB0B7A8854907E8F5396E26","EVID-D1B0E499E69AFDB6F3002005","EVID-C132BD268C13FF70511A4C23","EVID-34C490032C237ACC89D87EC2","EVID-CA272E3BD0899A1D187BF510","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
+          <t>["EVID-E62E849BC0654AAF5D85EAB7","EVID-3DAFFB80935B845D569F18C4","EVID-B2D7C2EE2968246DB663D751","EVID-10240CC6FE1740F33E7065A9","EVID-FE0A8787D4FE7A85E7328F2A","EVID-6231DA309B2890FEE5630D9F","EVID-5CB0B7A8854907E8F5396E26","EVID-D1B0E499E69AFDB6F3002005","EVID-C132BD268C13FF70511A4C23","EVID-34C490032C237ACC89D87EC2","EVID-8866BAE17752BA680D35AD9A","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
         </is>
       </c>
       <c r="AU72" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-10240CC6FE1740F33E7065A9":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-10240CC6FE1740F33E7065A9","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-3DAFFB80935B845D569F18C4":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-3DAFFB80935B845D569F18C4","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-5CB0B7A8854907E8F5396E26":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5CB0B7A8854907E8F5396E26","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2100},"EVID-6231DA309B2890FEE5630D9F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6231DA309B2890FEE5630D9F","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-B2D7C2EE2968246DB663D751":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-B2D7C2EE2968246DB663D751","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-C132BD268C13FF70511A4C23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C132BD268C13FF70511A4C23","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-CA272E3BD0899A1D187BF510":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CA272E3BD0899A1D187BF510","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0},"EVID-D1B0E499E69AFDB6F3002005":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D1B0E499E69AFDB6F3002005","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7200},"EVID-E62E849BC0654AAF5D85EAB7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E62E849BC0654AAF5D85EAB7","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-FE0A8787D4FE7A85E7328F2A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FE0A8787D4FE7A85E7328F2A","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0}}</t>
+          <t>{"EVID-10240CC6FE1740F33E7065A9":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-10240CC6FE1740F33E7065A9","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-3DAFFB80935B845D569F18C4":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-3DAFFB80935B845D569F18C4","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-5CB0B7A8854907E8F5396E26":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-5CB0B7A8854907E8F5396E26","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":2100},"EVID-6231DA309B2890FEE5630D9F":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-6231DA309B2890FEE5630D9F","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-8866BAE17752BA680D35AD9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8866BAE17752BA680D35AD9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":26000.0},"EVID-B2D7C2EE2968246DB663D751":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-B2D7C2EE2968246DB663D751","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-C132BD268C13FF70511A4C23":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C132BD268C13FF70511A4C23","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0},"EVID-D1B0E499E69AFDB6F3002005":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-D1B0E499E69AFDB6F3002005","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":7200},"EVID-E62E849BC0654AAF5D85EAB7":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E62E849BC0654AAF5D85EAB7","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"MEDIUM"},"EVID-FE0A8787D4FE7A85E7328F2A":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-FE0A8787D4FE7A85E7328F2A","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0}}</t>
         </is>
       </c>
       <c r="AV72" s="22" t="inlineStr">
@@ -29382,7 +29382,7 @@
       </c>
       <c r="AZ72" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-6AF109497D3D72C350D1DB24","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-523803CD1056F839B5F4CF5A","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA72" s="22" t="inlineStr">
@@ -29394,12 +29394,12 @@
     <row r="73" ht="32" customHeight="1">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>CAND-4D1C8BB67AC3293C91608AA1</t>
+          <t>CAND-16C467F705AC450DD5FB6F3F</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
@@ -29579,12 +29579,12 @@
       </c>
       <c r="AT73" s="22" t="inlineStr">
         <is>
-          <t>["EVID-BA7BE08DA2BEE2DBBB5B7266","EVID-2EEE40F816BC1314FC6D6794","EVID-252BD3F3682258C790F28B6B","EVID-B53D17514F2583F70618DF69","EVID-88F5112E71B1CC7681FAE85F","EVID-9919C3953E1E5DF2D700BD47","EVID-34C490032C237ACC89D87EC2","EVID-CA272E3BD0899A1D187BF510","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
+          <t>["EVID-BA7BE08DA2BEE2DBBB5B7266","EVID-2EEE40F816BC1314FC6D6794","EVID-252BD3F3682258C790F28B6B","EVID-B53D17514F2583F70618DF69","EVID-88F5112E71B1CC7681FAE85F","EVID-9919C3953E1E5DF2D700BD47","EVID-34C490032C237ACC89D87EC2","EVID-8866BAE17752BA680D35AD9A","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
         </is>
       </c>
       <c r="AU73" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-252BD3F3682258C790F28B6B":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-252BD3F3682258C790F28B6B","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-2EEE40F816BC1314FC6D6794":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2EEE40F816BC1314FC6D6794","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-88F5112E71B1CC7681FAE85F":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-88F5112E71B1CC7681FAE85F","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-9919C3953E1E5DF2D700BD47":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-9919C3953E1E5DF2D700BD47","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-B53D17514F2583F70618DF69":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-B53D17514F2583F70618DF69","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-BA7BE08DA2BEE2DBBB5B7266":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BA7BE08DA2BEE2DBBB5B7266","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":8},"EVID-CA272E3BD0899A1D187BF510":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CA272E3BD0899A1D187BF510","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0}}</t>
+          <t>{"EVID-252BD3F3682258C790F28B6B":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-252BD3F3682258C790F28B6B","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":0.0},"EVID-2EEE40F816BC1314FC6D6794":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2EEE40F816BC1314FC6D6794","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-8866BAE17752BA680D35AD9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8866BAE17752BA680D35AD9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":26000.0},"EVID-88F5112E71B1CC7681FAE85F":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-88F5112E71B1CC7681FAE85F","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":0},"EVID-9919C3953E1E5DF2D700BD47":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-9919C3953E1E5DF2D700BD47","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":0},"EVID-B53D17514F2583F70618DF69":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-B53D17514F2583F70618DF69","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.0},"EVID-BA7BE08DA2BEE2DBBB5B7266":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BA7BE08DA2BEE2DBBB5B7266","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":8}}</t>
         </is>
       </c>
       <c r="AV73" s="22" t="inlineStr">
@@ -29609,7 +29609,7 @@
       </c>
       <c r="AZ73" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-6AF109497D3D72C350D1DB24","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-523803CD1056F839B5F4CF5A","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA73" s="22" t="inlineStr">
@@ -29621,12 +29621,12 @@
     <row r="74" ht="32" customHeight="1">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>CAND-911B8170B602DC4F576083D1</t>
+          <t>CAND-17A18E302E55C3A7875CBEE5</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
@@ -29806,12 +29806,12 @@
       </c>
       <c r="AT74" s="22" t="inlineStr">
         <is>
-          <t>["EVID-0B9354DFC8337B7FF4FBFEDD","EVID-8AE0144C4CD3EFAA8C1FEDD6","EVID-5BA30663403D70E972E0FD56","EVID-64C8C669F3D65EB7D6DBE41D","EVID-61FD8CB671DF85EFF00A4198","EVID-34C490032C237ACC89D87EC2","EVID-CA272E3BD0899A1D187BF510","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
+          <t>["EVID-0B9354DFC8337B7FF4FBFEDD","EVID-8AE0144C4CD3EFAA8C1FEDD6","EVID-5BA30663403D70E972E0FD56","EVID-64C8C669F3D65EB7D6DBE41D","EVID-61FD8CB671DF85EFF00A4198","EVID-34C490032C237ACC89D87EC2","EVID-8866BAE17752BA680D35AD9A","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
         </is>
       </c>
       <c r="AU74" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0B9354DFC8337B7FF4FBFEDD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0B9354DFC8337B7FF4FBFEDD","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-5BA30663403D70E972E0FD56":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-5BA30663403D70E972E0FD56","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-61FD8CB671DF85EFF00A4198":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-61FD8CB671DF85EFF00A4198","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-64C8C669F3D65EB7D6DBE41D":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-64C8C669F3D65EB7D6DBE41D","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-8AE0144C4CD3EFAA8C1FEDD6":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-8AE0144C4CD3EFAA8C1FEDD6","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":58.0},"EVID-CA272E3BD0899A1D187BF510":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CA272E3BD0899A1D187BF510","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0}}</t>
+          <t>{"EVID-0B9354DFC8337B7FF4FBFEDD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0B9354DFC8337B7FF4FBFEDD","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-5BA30663403D70E972E0FD56":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-5BA30663403D70E972E0FD56","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.0},"EVID-61FD8CB671DF85EFF00A4198":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-61FD8CB671DF85EFF00A4198","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":0.0},"EVID-64C8C669F3D65EB7D6DBE41D":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-64C8C669F3D65EB7D6DBE41D","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":0},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-8866BAE17752BA680D35AD9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8866BAE17752BA680D35AD9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":26000.0},"EVID-8AE0144C4CD3EFAA8C1FEDD6":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-8AE0144C4CD3EFAA8C1FEDD6","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":58.0}}</t>
         </is>
       </c>
       <c r="AV74" s="22" t="inlineStr">
@@ -29848,12 +29848,12 @@
     <row r="75" ht="32" customHeight="1">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>CAND-21808FD63999AEC86B578E0F</t>
+          <t>CAND-26A61CADCADBE0C78C5ED6CC</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
@@ -30033,12 +30033,12 @@
       </c>
       <c r="AT75" s="22" t="inlineStr">
         <is>
-          <t>["EVID-2184712B5D074BB210FB51B7","EVID-20AE8FF8C49B268F1050ADCD","EVID-00A3773856382E51F32E0890","EVID-2E143851B2321E5658F0CAC4","EVID-71B1F5AA54FCF16B3FE8EDBA","EVID-49901827FD730943673C522F","EVID-9E2A0ACE00349FC117E45E89","EVID-751B770717B686A49D65471D","EVID-34C490032C237ACC89D87EC2","EVID-CA272E3BD0899A1D187BF510","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
+          <t>["EVID-2184712B5D074BB210FB51B7","EVID-20AE8FF8C49B268F1050ADCD","EVID-00A3773856382E51F32E0890","EVID-2E143851B2321E5658F0CAC4","EVID-71B1F5AA54FCF16B3FE8EDBA","EVID-49901827FD730943673C522F","EVID-9E2A0ACE00349FC117E45E89","EVID-751B770717B686A49D65471D","EVID-34C490032C237ACC89D87EC2","EVID-8866BAE17752BA680D35AD9A","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
         </is>
       </c>
       <c r="AU75" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00A3773856382E51F32E0890":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-00A3773856382E51F32E0890","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":520},"EVID-20AE8FF8C49B268F1050ADCD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-20AE8FF8C49B268F1050ADCD","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":433.33},"EVID-2184712B5D074BB210FB51B7":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-2184712B5D074BB210FB51B7","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":30},"EVID-2E143851B2321E5658F0CAC4":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-2E143851B2321E5658F0CAC4","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-49901827FD730943673C522F":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-49901827FD730943673C522F","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-71B1F5AA54FCF16B3FE8EDBA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-71B1F5AA54FCF16B3FE8EDBA","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":6},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-751B770717B686A49D65471D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-751B770717B686A49D65471D","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1728.0},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-9E2A0ACE00349FC117E45E89":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-9E2A0ACE00349FC117E45E89","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2},"EVID-CA272E3BD0899A1D187BF510":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CA272E3BD0899A1D187BF510","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0}}</t>
+          <t>{"EVID-00A3773856382E51F32E0890":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-00A3773856382E51F32E0890","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":520},"EVID-20AE8FF8C49B268F1050ADCD":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-20AE8FF8C49B268F1050ADCD","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":433.33},"EVID-2184712B5D074BB210FB51B7":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-2184712B5D074BB210FB51B7","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":30},"EVID-2E143851B2321E5658F0CAC4":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-2E143851B2321E5658F0CAC4","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-49901827FD730943673C522F":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-49901827FD730943673C522F","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-71B1F5AA54FCF16B3FE8EDBA":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-71B1F5AA54FCF16B3FE8EDBA","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":6},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-751B770717B686A49D65471D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-751B770717B686A49D65471D","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":1728.0},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-8866BAE17752BA680D35AD9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8866BAE17752BA680D35AD9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":26000.0},"EVID-9E2A0ACE00349FC117E45E89":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-9E2A0ACE00349FC117E45E89","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.2}}</t>
         </is>
       </c>
       <c r="AV75" s="22" t="inlineStr">
@@ -30075,12 +30075,12 @@
     <row r="76" ht="32" customHeight="1">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>PKG-2B1D4DABAB31B9C98B678CAB</t>
+          <t>PKG-DBEE3B8CE61661460AF22184</t>
         </is>
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>CAND-8DAE20517B39B4C87C5DB0F9</t>
+          <t>CAND-3533B4E4348CE8BBC3CD27A3</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
@@ -30264,12 +30264,12 @@
       </c>
       <c r="AT76" s="22" t="inlineStr">
         <is>
-          <t>["EVID-9A7629DAFB1FBA68EA7CC011","EVID-0273418DF08CF77E8FEA19EC","EVID-B8F35C06BEA4E6B4653B2CA5","EVID-67937AF881DA47B4E7F6F58F","EVID-3CD13C8C8685F803F84E6C0C","EVID-75A390A72C67FC229F633E03","EVID-2D058786FA5DD49B24F1B760","EVID-D0676180FFB706041DF59124","EVID-233AA44D11F809A7348519BE","EVID-E90DF6D21AF730E06ED07EF2","EVID-0B673BFB80ED7BCA73AD9E28","EVID-804BAA58EAAF38FFE577161F","EVID-94A46684F527C403627646A4","EVID-34C490032C237ACC89D87EC2","EVID-CA272E3BD0899A1D187BF510","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
+          <t>["EVID-9A7629DAFB1FBA68EA7CC011","EVID-0273418DF08CF77E8FEA19EC","EVID-B8F35C06BEA4E6B4653B2CA5","EVID-67937AF881DA47B4E7F6F58F","EVID-3CD13C8C8685F803F84E6C0C","EVID-75A390A72C67FC229F633E03","EVID-2D058786FA5DD49B24F1B760","EVID-D0676180FFB706041DF59124","EVID-233AA44D11F809A7348519BE","EVID-E90DF6D21AF730E06ED07EF2","EVID-0B673BFB80ED7BCA73AD9E28","EVID-804BAA58EAAF38FFE577161F","EVID-94A46684F527C403627646A4","EVID-34C490032C237ACC89D87EC2","EVID-8866BAE17752BA680D35AD9A","EVID-74FF3187C068E27FFD83A29D","EVID-7E5A58CA120115D1E2ED5C61"]</t>
         </is>
       </c>
       <c r="AU76" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0273418DF08CF77E8FEA19EC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0273418DF08CF77E8FEA19EC","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-0B673BFB80ED7BCA73AD9E28":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0B673BFB80ED7BCA73AD9E28","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-233AA44D11F809A7348519BE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-233AA44D11F809A7348519BE","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1040},"EVID-2D058786FA5DD49B24F1B760":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2D058786FA5DD49B24F1B760","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-3CD13C8C8685F803F84E6C0C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3CD13C8C8685F803F84E6C0C","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-67937AF881DA47B4E7F6F58F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-67937AF881DA47B4E7F6F58F","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":9750},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-75A390A72C67FC229F633E03":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75A390A72C67FC229F633E03","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-804BAA58EAAF38FFE577161F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-804BAA58EAAF38FFE577161F","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-94A46684F527C403627646A4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-94A46684F527C403627646A4","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-9A7629DAFB1FBA68EA7CC011":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7629DAFB1FBA68EA7CC011","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-B8F35C06BEA4E6B4653B2CA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B8F35C06BEA4E6B4653B2CA5","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-CA272E3BD0899A1D187BF510":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-CA272E3BD0899A1D187BF510","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":26000.0},"EVID-D0676180FFB706041DF59124":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D0676180FFB706041DF59124","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-E90DF6D21AF730E06ED07EF2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E90DF6D21AF730E06ED07EF2","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":3250}}</t>
+          <t>{"EVID-0273418DF08CF77E8FEA19EC":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0273418DF08CF77E8FEA19EC","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-0B673BFB80ED7BCA73AD9E28":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0B673BFB80ED7BCA73AD9E28","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-233AA44D11F809A7348519BE":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-233AA44D11F809A7348519BE","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":1040},"EVID-2D058786FA5DD49B24F1B760":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-2D058786FA5DD49B24F1B760","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-34C490032C237ACC89D87EC2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-34C490032C237ACC89D87EC2","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":22880.0},"EVID-3CD13C8C8685F803F84E6C0C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-3CD13C8C8685F803F84E6C0C","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-67937AF881DA47B4E7F6F58F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-67937AF881DA47B4E7F6F58F","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":9750},"EVID-74FF3187C068E27FFD83A29D":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-74FF3187C068E27FFD83A29D","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":5338.12},"EVID-75A390A72C67FC229F633E03":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-75A390A72C67FC229F633E03","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":0},"EVID-7E5A58CA120115D1E2ED5C61":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7E5A58CA120115D1E2ED5C61","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":256},"EVID-804BAA58EAAF38FFE577161F":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-804BAA58EAAF38FFE577161F","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-8866BAE17752BA680D35AD9A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-8866BAE17752BA680D35AD9A","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":26000.0},"EVID-94A46684F527C403627646A4":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-94A46684F527C403627646A4","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-9A7629DAFB1FBA68EA7CC011":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9A7629DAFB1FBA68EA7CC011","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-B8F35C06BEA4E6B4653B2CA5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B8F35C06BEA4E6B4653B2CA5","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-D0676180FFB706041DF59124":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-D0676180FFB706041DF59124","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-E90DF6D21AF730E06ED07EF2":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E90DF6D21AF730E06ED07EF2","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":3250}}</t>
         </is>
       </c>
       <c r="AV76" s="22" t="inlineStr">
@@ -30294,7 +30294,7 @@
       </c>
       <c r="AZ76" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-1A718415E777F8AF64EDE335","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-79199C03A3C215D8409EAD4B","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA76" s="22" t="inlineStr">
@@ -30306,12 +30306,12 @@
     <row r="77" ht="32" customHeight="1">
       <c r="A77" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>CAND-AAB5D0F8604AAE069E7BB81F</t>
+          <t>CAND-209F8112923FB7D955D9E642</t>
         </is>
       </c>
       <c r="C77" s="14" t="inlineStr">
@@ -30495,12 +30495,12 @@
       </c>
       <c r="AT77" s="22" t="inlineStr">
         <is>
-          <t>["EVID-23708F72EC5B59C135E02F34","EVID-1EC6339D5DE6445CE509F960","EVID-BAA119A401A590AC412ABE46","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
+          <t>["EVID-23708F72EC5B59C135E02F34","EVID-1EC6339D5DE6445CE509F960","EVID-0A3918300145A810E01D7505","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
         </is>
       </c>
       <c r="AU77" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-23708F72EC5B59C135E02F34":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-23708F72EC5B59C135E02F34","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-BAA119A401A590AC412ABE46":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA119A401A590AC412ABE46","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0}}</t>
+          <t>{"EVID-0A3918300145A810E01D7505":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0A3918300145A810E01D7505","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":21000.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-23708F72EC5B59C135E02F34":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-23708F72EC5B59C135E02F34","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53}}</t>
         </is>
       </c>
       <c r="AV77" s="22" t="inlineStr">
@@ -30537,12 +30537,12 @@
     <row r="78" ht="32" customHeight="1">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>CAND-CB50137D13AA86B1380E9225</t>
+          <t>CAND-428D7886836325C1957B2FC7</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
@@ -30726,12 +30726,12 @@
       </c>
       <c r="AT78" s="22" t="inlineStr">
         <is>
-          <t>["EVID-1C4C5F2DD86D5D02CEEC8DDF","EVID-6DB47127905826426728EB23","EVID-37879E4CC18FB3E3DD0B4326","EVID-8E66F44EED7CB4EABFC52575","EVID-64535252D2DA01A6AA9B32FD","EVID-36A7BD1B9906F3FAC507CA6E","EVID-19C6EC9C89DF11542B23C017","EVID-7788ACC9A8B33D87E56CB271","EVID-F181CC0538E3C28FAA841E28","EVID-1EC6339D5DE6445CE509F960","EVID-BAA119A401A590AC412ABE46","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
+          <t>["EVID-1C4C5F2DD86D5D02CEEC8DDF","EVID-6DB47127905826426728EB23","EVID-37879E4CC18FB3E3DD0B4326","EVID-8E66F44EED7CB4EABFC52575","EVID-64535252D2DA01A6AA9B32FD","EVID-36A7BD1B9906F3FAC507CA6E","EVID-19C6EC9C89DF11542B23C017","EVID-7788ACC9A8B33D87E56CB271","EVID-F181CC0538E3C28FAA841E28","EVID-1EC6339D5DE6445CE509F960","EVID-0A3918300145A810E01D7505","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
         </is>
       </c>
       <c r="AU78" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-19C6EC9C89DF11542B23C017":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-19C6EC9C89DF11542B23C017","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":4200},"EVID-1C4C5F2DD86D5D02CEEC8DDF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1C4C5F2DD86D5D02CEEC8DDF","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-36A7BD1B9906F3FAC507CA6E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-36A7BD1B9906F3FAC507CA6E","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-37879E4CC18FB3E3DD0B4326":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-37879E4CC18FB3E3DD0B4326","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-64535252D2DA01A6AA9B32FD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-64535252D2DA01A6AA9B32FD","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-6DB47127905826426728EB23":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-6DB47127905826426728EB23","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-7788ACC9A8B33D87E56CB271":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-7788ACC9A8B33D87E56CB271","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":16000},"EVID-8E66F44EED7CB4EABFC52575":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8E66F44EED7CB4EABFC52575","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-BAA119A401A590AC412ABE46":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA119A401A590AC412ABE46","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0},"EVID-F181CC0538E3C28FAA841E28":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F181CC0538E3C28FAA841E28","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0}}</t>
+          <t>{"EVID-0A3918300145A810E01D7505":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0A3918300145A810E01D7505","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":21000.0},"EVID-19C6EC9C89DF11542B23C017":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-19C6EC9C89DF11542B23C017","interpretation":"Tail execution latency guardrail.","metric":"p95_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":5000,"unit":"ms","value":4200},"EVID-1C4C5F2DD86D5D02CEEC8DDF":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1C4C5F2DD86D5D02CEEC8DDF","interpretation":"Current warehouse size.","metric":"warehouse_size","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_size","threshold":null,"unit":"value","value":"SMALL"},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-36A7BD1B9906F3FAC507CA6E":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-36A7BD1B9906F3FAC507CA6E","interpretation":"Failed or cancelled query share; a high rate undermines the no-pressure evidence a downsize relies on.","metric":"failure_cancel_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_status","threshold":5.0,"unit":"%","value":0.3},"EVID-37879E4CC18FB3E3DD0B4326":{"comparator":"&gt;= evidence minimum for upsize","epoch_scope":"CURRENT","evidence_id":"EVID-37879E4CC18FB3E3DD0B4326","interpretation":"Queries that spilled; the spill severity percentile is computed over these queries only.","metric":"spill_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":20,"unit":"queries","value":0},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-64535252D2DA01A6AA9B32FD":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-64535252D2DA01A6AA9B32FD","interpretation":"Concurrency pressure during the decision window.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-6DB47127905826426728EB23":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-6DB47127905826426728EB23","interpretation":"Frequency of queries spilling to local storage.","metric":"spill_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":2.0,"unit":"%","value":0.0},"EVID-7788ACC9A8B33D87E56CB271":{"comparator":"&lt;= downsize-safe","epoch_scope":"CURRENT","evidence_id":"EVID-7788ACC9A8B33D87E56CB271","interpretation":"Extreme tail execution latency guardrail.","metric":"p99_execution_ms_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"execution_duration_ms","threshold":30000,"unit":"ms","value":16000},"EVID-8E66F44EED7CB4EABFC52575":{"comparator":"&gt;= upsize signal","epoch_scope":"CURRENT","evidence_id":"EVID-8E66F44EED7CB4EABFC52575","interpretation":"Severity of spill at p95 among queries that spilled.","metric":"p95_spill_bytes_when_spilled_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"spilled_local_bytes","threshold":1073741824,"unit":"bytes","value":0},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-F181CC0538E3C28FAA841E28":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F181CC0538E3C28FAA841E28","interpretation":"I/O cache evidence for HITL context; not a v2 size decision threshold.","metric":"avg_read_io_cache_percent_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"read_io_cache_percent","threshold":null,"unit":"%","value":35.0}}</t>
         </is>
       </c>
       <c r="AV78" s="22" t="inlineStr">
@@ -30756,7 +30756,7 @@
       </c>
       <c r="AZ78" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-3C4F23823E7323060F7D590E","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-66A9ACF16F67715AEDE3DD1E","scenario_name":"Plan A — Optimize current warehouse type","step":1}]</t>
         </is>
       </c>
       <c r="BA78" s="22" t="inlineStr">
@@ -30768,12 +30768,12 @@
     <row r="79" ht="32" customHeight="1">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>CAND-55C42C4CB74E0DDB5E248AD5</t>
+          <t>CAND-5D881068EC81653BFBAE9057</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
@@ -30953,12 +30953,12 @@
       </c>
       <c r="AT79" s="22" t="inlineStr">
         <is>
-          <t>["EVID-4B4458954444D6D1761F2B97","EVID-95AE888C192E87C9600B841A","EVID-0B74F9AC5B2FB5BA3961B896","EVID-0AF4AC4CC2EFE0D7B0D04C7D","EVID-D3229EED878B4951211AF5C1","EVID-ADA47AE99362347459714D8A","EVID-1EC6339D5DE6445CE509F960","EVID-BAA119A401A590AC412ABE46","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
+          <t>["EVID-4B4458954444D6D1761F2B97","EVID-95AE888C192E87C9600B841A","EVID-0B74F9AC5B2FB5BA3961B896","EVID-0AF4AC4CC2EFE0D7B0D04C7D","EVID-D3229EED878B4951211AF5C1","EVID-ADA47AE99362347459714D8A","EVID-1EC6339D5DE6445CE509F960","EVID-0A3918300145A810E01D7505","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
         </is>
       </c>
       <c r="AU79" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0AF4AC4CC2EFE0D7B0D04C7D":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-0AF4AC4CC2EFE0D7B0D04C7D","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.1},"EVID-0B74F9AC5B2FB5BA3961B896":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0B74F9AC5B2FB5BA3961B896","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":2.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-4B4458954444D6D1761F2B97":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B4458954444D6D1761F2B97","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-95AE888C192E87C9600B841A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95AE888C192E87C9600B841A","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-ADA47AE99362347459714D8A":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-ADA47AE99362347459714D8A","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":1000},"EVID-BAA119A401A590AC412ABE46":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA119A401A590AC412ABE46","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0},"EVID-D3229EED878B4951211AF5C1":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-D3229EED878B4951211AF5C1","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":7}}</t>
+          <t>{"EVID-0A3918300145A810E01D7505":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0A3918300145A810E01D7505","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":21000.0},"EVID-0AF4AC4CC2EFE0D7B0D04C7D":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-0AF4AC4CC2EFE0D7B0D04C7D","interpretation":"Frequency of capacity queueing.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5.0,"unit":"%","value":0.1},"EVID-0B74F9AC5B2FB5BA3961B896":{"comparator":"&lt;= reduce-safe","epoch_scope":"CURRENT","evidence_id":"EVID-0B74F9AC5B2FB5BA3961B896","interpretation":"Fraction of running time at configured maximum.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":1.0,"unit":"%","value":2.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-4B4458954444D6D1761F2B97":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4B4458954444D6D1761F2B97","interpretation":"Configured concurrency ceiling.","metric":"max_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"max_clusters","threshold":null,"unit":"value","value":4},"EVID-95AE888C192E87C9600B841A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95AE888C192E87C9600B841A","interpretation":"Highest observed scale level.","metric":"max_observed_clusters","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":null,"unit":"clusters","value":2},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-ADA47AE99362347459714D8A":{"comparator":"&gt;= increase signal","epoch_scope":"CURRENT","evidence_id":"EVID-ADA47AE99362347459714D8A","interpretation":"Severity of capacity queueing at p95 among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":30000,"unit":"ms","value":1000},"EVID-D3229EED878B4951211AF5C1":{"comparator":"&gt;= evidence minimum for increase","epoch_scope":"CURRENT","evidence_id":"EVID-D3229EED878B4951211AF5C1","interpretation":"Queries that queued at capacity; the wait percentile is computed over these queries only.","metric":"queued_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":20,"unit":"queries","value":7}}</t>
         </is>
       </c>
       <c r="AV79" s="22" t="inlineStr">
@@ -30995,12 +30995,12 @@
     <row r="80" ht="32" customHeight="1">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>CAND-065AC8BFFA6CD2F35B884972</t>
+          <t>CAND-E4E81DFEE63DC47048502757</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
@@ -31180,12 +31180,12 @@
       </c>
       <c r="AT80" s="22" t="inlineStr">
         <is>
-          <t>["EVID-40AD09E7303B8B2EDD979703","EVID-6BD6044B2F8274556325FEA5","EVID-6ECF76708502117135458415","EVID-4403DA2AD6FBF575B1913672","EVID-49DDC09967250A39DC8AA8E3","EVID-1EC6339D5DE6445CE509F960","EVID-BAA119A401A590AC412ABE46","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
+          <t>["EVID-40AD09E7303B8B2EDD979703","EVID-6BD6044B2F8274556325FEA5","EVID-6ECF76708502117135458415","EVID-4403DA2AD6FBF575B1913672","EVID-49DDC09967250A39DC8AA8E3","EVID-1EC6339D5DE6445CE509F960","EVID-0A3918300145A810E01D7505","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
         </is>
       </c>
       <c r="AU80" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-40AD09E7303B8B2EDD979703":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-40AD09E7303B8B2EDD979703","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-4403DA2AD6FBF575B1913672":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-4403DA2AD6FBF575B1913672","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":1000},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-49DDC09967250A39DC8AA8E3":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-49DDC09967250A39DC8AA8E3","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":2.0},"EVID-6BD6044B2F8274556325FEA5":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-6BD6044B2F8274556325FEA5","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":55.0},"EVID-6ECF76708502117135458415":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-6ECF76708502117135458415","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-BAA119A401A590AC412ABE46":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA119A401A590AC412ABE46","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0}}</t>
+          <t>{"EVID-0A3918300145A810E01D7505":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0A3918300145A810E01D7505","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":21000.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-40AD09E7303B8B2EDD979703":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-40AD09E7303B8B2EDD979703","interpretation":"Configured minimum scale.","metric":"min_clusters","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"min_clusters","threshold":null,"unit":"value","value":1},"EVID-4403DA2AD6FBF575B1913672":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-4403DA2AD6FBF575B1913672","interpretation":"Queue latency guardrail among queued queries.","metric":"p95_wait_capacity_ms_when_queued_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":5000,"unit":"ms","value":1000},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-49DDC09967250A39DC8AA8E3":{"comparator":"&gt;= blocker","epoch_scope":"CURRENT","evidence_id":"EVID-49DDC09967250A39DC8AA8E3","interpretation":"Sustained scale pressure blocks minimum reduction.","metric":"time_at_max_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":20.0,"unit":"%","value":2.0},"EVID-6BD6044B2F8274556325FEA5":{"comparator":"&gt;= reduction signal","epoch_scope":"CURRENT","evidence_id":"EVID-6BD6044B2F8274556325FEA5","interpretation":"How often the warehouse sits at its minimum.","metric":"time_at_min_pct","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count","threshold":25.0,"unit":"%","value":55.0},"EVID-6ECF76708502117135458415":{"comparator":"&lt;= safe","epoch_scope":"CURRENT","evidence_id":"EVID-6ECF76708502117135458415","interpretation":"Queue guardrail before reducing baseline capacity.","metric":"queued_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_at_capacity_duration_ms","threshold":0.5,"unit":"%","value":0.1},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53}}</t>
         </is>
       </c>
       <c r="AV80" s="22" t="inlineStr">
@@ -31222,12 +31222,12 @@
     <row r="81" ht="32" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>CAND-ACD999430C8A059DFB38EBAC</t>
+          <t>CAND-6B0ACEABD2495B5A3B07846B</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
@@ -31407,12 +31407,12 @@
       </c>
       <c r="AT81" s="22" t="inlineStr">
         <is>
-          <t>["EVID-2E939D43F5BB323DF22E4026","EVID-346B866635D3784872770C40","EVID-C6D7693171830636FB13018B","EVID-D53E2EF13F1E733634CCCD78","EVID-466AA6DFF5D422053A0304C3","EVID-2C012211C1C911F47F72090F","EVID-60FEA6406889613BF7D0D7B2","EVID-180293A6D9DB38441576C299","EVID-1EC6339D5DE6445CE509F960","EVID-BAA119A401A590AC412ABE46","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
+          <t>["EVID-2E939D43F5BB323DF22E4026","EVID-346B866635D3784872770C40","EVID-C6D7693171830636FB13018B","EVID-D53E2EF13F1E733634CCCD78","EVID-466AA6DFF5D422053A0304C3","EVID-2C012211C1C911F47F72090F","EVID-60FEA6406889613BF7D0D7B2","EVID-180293A6D9DB38441576C299","EVID-1EC6339D5DE6445CE509F960","EVID-0A3918300145A810E01D7505","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
         </is>
       </c>
       <c r="AU81" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-180293A6D9DB38441576C299":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-180293A6D9DB38441576C299","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":3600.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-2C012211C1C911F47F72090F":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-2C012211C1C911F47F72090F","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-2E939D43F5BB323DF22E4026":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-2E939D43F5BB323DF22E4026","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":60},"EVID-346B866635D3784872770C40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-346B866635D3784872770C40","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":240.0},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-466AA6DFF5D422053A0304C3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-466AA6DFF5D422053A0304C3","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-60FEA6406889613BF7D0D7B2":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-60FEA6406889613BF7D0D7B2","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-BAA119A401A590AC412ABE46":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA119A401A590AC412ABE46","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0},"EVID-C6D7693171830636FB13018B":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-C6D7693171830636FB13018B","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":288},"EVID-D53E2EF13F1E733634CCCD78":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-D53E2EF13F1E733634CCCD78","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0}}</t>
+          <t>{"EVID-0A3918300145A810E01D7505":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0A3918300145A810E01D7505","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":21000.0},"EVID-180293A6D9DB38441576C299":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-180293A6D9DB38441576C299","interpretation":"Estimated additional off-time at the candidate target.","metric":"estimated_additional_off_minutes","observation_window":"current epoch","source":"system.query.history","source_field":"inter-query gap","threshold":null,"unit":"minutes","value":3600.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-2C012211C1C911F47F72090F":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-2C012211C1C911F47F72090F","interpretation":"Cold-start sensitivity guardrail at p95 among queries that waited for compute.","metric":"p95_wait_compute_ms_when_waited_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":60000,"unit":"ms","value":3500},"EVID-2E939D43F5BB323DF22E4026":{"comparator":"&gt; target","epoch_scope":"CURRENT","evidence_id":"EVID-2E939D43F5BB323DF22E4026","interpretation":"Current idle termination setting versus deterministic policy target.","metric":"auto_stop_minutes","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"auto_stop_minutes","threshold":30,"unit":"minutes","value":60},"EVID-346B866635D3784872770C40":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-346B866635D3784872770C40","interpretation":"Activity density selects the auto-stop target.","metric":"queries_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"start_time","threshold":null,"unit":"queries/day","value":240.0},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-466AA6DFF5D422053A0304C3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-466AA6DFF5D422053A0304C3","interpretation":"Queries that waited for compute; the wait percentile is computed over these queries only.","metric":"compute_wait_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"waiting_for_compute_duration_ms","threshold":null,"unit":"queries","value":5},"EVID-60FEA6406889613BF7D0D7B2":{"comparator":"&gt;= cold-start blocker","epoch_scope":"CURRENT","evidence_id":"EVID-60FEA6406889613BF7D0D7B2","interpretation":"Restart frequency guardrail.","metric":"starts_per_active_day_30","observation_window":"last 30 days within current epoch","source":"system.compute.warehouse_events","source_field":"event_type=STARTING","threshold":0.5,"unit":"starts/day","value":0.1667},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-C6D7693171830636FB13018B":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-C6D7693171830636FB13018B","interpretation":"Non-overlapping inter-query gap sample supporting the auto-stop counterfactual.","metric":"idle_gap_count","observation_window":"current epoch","source":"system.query.history","source_field":"start_time/end_time","threshold":30,"unit":"gaps","value":288},"EVID-D53E2EF13F1E733634CCCD78":{"comparator":"&gt;= evidence minimum","epoch_scope":"CURRENT","evidence_id":"EVID-D53E2EF13F1E733634CCCD78","interpretation":"Observed resource-time basis used to convert idle time into cost effect.","metric":"cluster_minutes","observation_window":"current epoch","source":"system.compute.warehouse_events","source_field":"cluster_count/event_time","threshold":1.0,"unit":"cluster-minutes","value":30000.0}}</t>
         </is>
       </c>
       <c r="AV81" s="22" t="inlineStr">
@@ -31437,7 +31437,7 @@
       </c>
       <c r="AZ81" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-3C4F23823E7323060F7D590E","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
+          <t>[{"execution_state":"PENDING_REEVALUATION","scenario_id":"SCN-66A9ACF16F67715AEDE3DD1E","scenario_name":"Plan A — Optimize current warehouse type","step":2}]</t>
         </is>
       </c>
       <c r="BA81" s="22" t="inlineStr">
@@ -31449,12 +31449,12 @@
     <row r="82" ht="32" customHeight="1">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>PKG-D4236B52C79354C1BD221E9A</t>
+          <t>PKG-8157B13DCBA4F6D10AAD35EE</t>
         </is>
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>CAND-32DF6FED0478FEF9963854FF</t>
+          <t>CAND-B9A432AC45556AC42F2CDE81</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
@@ -31638,12 +31638,12 @@
       </c>
       <c r="AT82" s="22" t="inlineStr">
         <is>
-          <t>["EVID-6877D38EED61AEE41EC2E4C9","EVID-B779811345CC9113D2D9A1EB","EVID-00BD6F78F73E54B4ED6BBBD0","EVID-E1B10E4FB81AFD2B35E43242","EVID-B4CF1A6ABE4A98216DB749FB","EVID-7799CCE95E17579305B3C541","EVID-0164D6D29E0EA5CF4E8AB303","EVID-95E2FB2242901BE5827CAF65","EVID-363203EBE91A6BA8FE765D72","EVID-F15353EC12D6ACAD2E076C5B","EVID-C48F43336C1B2F7A7A8B6E1A","EVID-82B45567DA4A70CD40CCBF6C","EVID-4D3BC0C4CD326B137F0E6E65","EVID-1EC6339D5DE6445CE509F960","EVID-BAA119A401A590AC412ABE46","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
+          <t>["EVID-6877D38EED61AEE41EC2E4C9","EVID-B779811345CC9113D2D9A1EB","EVID-00BD6F78F73E54B4ED6BBBD0","EVID-E1B10E4FB81AFD2B35E43242","EVID-B4CF1A6ABE4A98216DB749FB","EVID-7799CCE95E17579305B3C541","EVID-0164D6D29E0EA5CF4E8AB303","EVID-95E2FB2242901BE5827CAF65","EVID-363203EBE91A6BA8FE765D72","EVID-F15353EC12D6ACAD2E076C5B","EVID-C48F43336C1B2F7A7A8B6E1A","EVID-82B45567DA4A70CD40CCBF6C","EVID-4D3BC0C4CD326B137F0E6E65","EVID-1EC6339D5DE6445CE509F960","EVID-0A3918300145A810E01D7505","EVID-AB85741601676CEF4EC99624","EVID-4651F04F55F5093F44CEAF83"]</t>
         </is>
       </c>
       <c r="AU82" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-00BD6F78F73E54B4ED6BBBD0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-00BD6F78F73E54B4ED6BBBD0","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-0164D6D29E0EA5CF4E8AB303":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0164D6D29E0EA5CF4E8AB303","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-363203EBE91A6BA8FE765D72":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-363203EBE91A6BA8FE765D72","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":576},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-4D3BC0C4CD326B137F0E6E65":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4D3BC0C4CD326B137F0E6E65","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-6877D38EED61AEE41EC2E4C9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6877D38EED61AEE41EC2E4C9","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-7799CCE95E17579305B3C541":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7799CCE95E17579305B3C541","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":5400},"EVID-82B45567DA4A70CD40CCBF6C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-82B45567DA4A70CD40CCBF6C","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-95E2FB2242901BE5827CAF65":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E2FB2242901BE5827CAF65","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-B4CF1A6ABE4A98216DB749FB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B4CF1A6ABE4A98216DB749FB","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-B779811345CC9113D2D9A1EB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B779811345CC9113D2D9A1EB","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-BAA119A401A590AC412ABE46":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-BAA119A401A590AC412ABE46","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":21000.0},"EVID-C48F43336C1B2F7A7A8B6E1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C48F43336C1B2F7A7A8B6E1A","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-E1B10E4FB81AFD2B35E43242":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1B10E4FB81AFD2B35E43242","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-F15353EC12D6ACAD2E076C5B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F15353EC12D6ACAD2E076C5B","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0}}</t>
+          <t>{"EVID-00BD6F78F73E54B4ED6BBBD0":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-00BD6F78F73E54B4ED6BBBD0","interpretation":"Query-tag coverage supplied to HITL for workload attribution and migration validation.","metric":"tagged_query_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_tags","threshold":null,"unit":"%","value":70.0},"EVID-0164D6D29E0EA5CF4E8AB303":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0164D6D29E0EA5CF4E8AB303","interpretation":"Genie workload mix context.","metric":"genie_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.genie_space_id","threshold":null,"unit":"queries","value":0},"EVID-0A3918300145A810E01D7505":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0A3918300145A810E01D7505","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":21000.0},"EVID-1EC6339D5DE6445CE509F960":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1EC6339D5DE6445CE509F960","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":18480.0},"EVID-363203EBE91A6BA8FE765D72":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-363203EBE91A6BA8FE765D72","interpretation":"Databricks SQL editor/query workload mix context.","metric":"sql_editor_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.sql_query_id","threshold":null,"unit":"queries","value":576},"EVID-4651F04F55F5093F44CEAF83":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4651F04F55F5093F44CEAF83","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":233},"EVID-4D3BC0C4CD326B137F0E6E65":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-4D3BC0C4CD326B137F0E6E65","interpretation":"Potential migration-review signal only; this does not prove an external legacy Hive metastore is configured.","metric":"hive_metastore_reference_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text (aggregated pattern only)","threshold":null,"unit":"queries","value":0},"EVID-6877D38EED61AEE41EC2E4C9":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6877D38EED61AEE41EC2E4C9","interpretation":"Current warehouse type.","metric":"warehouse_type","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_type","threshold":null,"unit":"value","value":"PRO"},"EVID-7799CCE95E17579305B3C541":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-7799CCE95E17579305B3C541","interpretation":"Notebook workload mix context.","metric":"notebook_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.notebook_id","threshold":null,"unit":"queries","value":5400},"EVID-82B45567DA4A70CD40CCBF6C":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-82B45567DA4A70CD40CCBF6C","interpretation":"Coverage available for deterministic pattern checks. Raw SQL text is not exported.","metric":"statement_text_visible_pct_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"statement_text","threshold":null,"unit":"%","value":100.0},"EVID-95E2FB2242901BE5827CAF65":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-95E2FB2242901BE5827CAF65","interpretation":"Alert workload mix context.","metric":"alert_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.alert_id","threshold":null,"unit":"queries","value":0},"EVID-AB85741601676CEF4EC99624":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-AB85741601676CEF4EC99624","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":2932.53},"EVID-B4CF1A6ABE4A98216DB749FB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B4CF1A6ABE4A98216DB749FB","interpretation":"Job workload mix context.","metric":"job_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.job_info.job_id","threshold":null,"unit":"queries","value":0},"EVID-B779811345CC9113D2D9A1EB":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-B779811345CC9113D2D9A1EB","interpretation":"Observed billing evidence; not used as current configuration source.","metric":"serverless_usage_pct_365","observation_window":"trailing 365 days","source":"system.billing.usage","source_field":"product_features.is_serverless","threshold":null,"unit":"%","value":0.0},"EVID-C48F43336C1B2F7A7A8B6E1A":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-C48F43336C1B2F7A7A8B6E1A","interpretation":"Tableau client workload mix context.","metric":"tableau_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0},"EVID-E1B10E4FB81AFD2B35E43242":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-E1B10E4FB81AFD2B35E43242","interpretation":"Dashboard workload mix context.","metric":"dashboard_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"query_source.dashboard_id","threshold":null,"unit":"queries","value":0},"EVID-F15353EC12D6ACAD2E076C5B":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F15353EC12D6ACAD2E076C5B","interpretation":"Power BI client workload mix context.","metric":"power_bi_queries_30","observation_window":"last 30 days within current epoch","source":"system.query.history","source_field":"client_application","threshold":null,"unit":"queries","value":0}}</t>
         </is>
       </c>
       <c r="AV82" s="22" t="inlineStr">
@@ -31668,7 +31668,7 @@
       </c>
       <c r="AZ82" s="22" t="inlineStr">
         <is>
-          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-1B5457B19E85EA205F9057D6","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
+          <t>[{"execution_state":"READY_FOR_CANARY","scenario_id":"SCN-EEA1172BA764560AD0C5776C","scenario_name":"Plan B — Serverless migration experiment","step":2}]</t>
         </is>
       </c>
       <c r="BA82" s="22" t="inlineStr">
@@ -31680,12 +31680,12 @@
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>PKG-02C2A3390BC1C4114197FDAD</t>
+          <t>PKG-664E535A61AEB69185D775A9</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>CAND-DF495D633D84F3AE8A813276</t>
+          <t>CAND-186FCE93391AFC4EF35A6CBC</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
@@ -31869,12 +31869,12 @@
       </c>
       <c r="AT83" s="22" t="inlineStr">
         <is>
-          <t>["EVID-76CE682449BA3088A5EBB4E1","EVID-1FDA0700A45761E2E0DC6B81","EVID-0E39BB07A52CCA2264264F50","EVID-6DD782A2BB5F89EE62C99CA3","EVID-9349C4F74710189DF28D26E5"]</t>
+          <t>["EVID-76CE682449BA3088A5EBB4E1","EVID-1FDA0700A45761E2E0DC6B81","EVID-F9AD519DB03E1D0381CB098E","EVID-6DD782A2BB5F89EE62C99CA3","EVID-9349C4F74710189DF28D26E5"]</t>
         </is>
       </c>
       <c r="AU83" s="22" t="inlineStr">
         <is>
-          <t>{"EVID-0E39BB07A52CCA2264264F50":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-0E39BB07A52CCA2264264F50","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.7","threshold":null,"unit":"USD","value":3200.0},"EVID-1FDA0700A45761E2E0DC6B81":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1FDA0700A45761E2E0DC6B81","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":2816.0},"EVID-6DD782A2BB5F89EE62C99CA3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6DD782A2BB5F89EE62C99CA3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3733.77},"EVID-76CE682449BA3088A5EBB4E1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-76CE682449BA3088A5EBB4E1","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-9349C4F74710189DF28D26E5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9349C4F74710189DF28D26E5","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":122}}</t>
+          <t>{"EVID-1FDA0700A45761E2E0DC6B81":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-1FDA0700A45761E2E0DC6B81","interpretation":"Observed trailing-365-day Databricks SQL list cost attributed to the warehouse.","metric":"actual_dbu_cost_365d","observation_window":"trailing_365d","source":"system.billing.usage","source_field":"usage_quantity × historical effective list price","threshold":null,"unit":"USD","value":2816.0},"EVID-6DD782A2BB5F89EE62C99CA3":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-6DD782A2BB5F89EE62C99CA3","interpretation":"Forward customer AWS infrastructure cost model for the current configuration epoch; null when unavailable.","metric":"forward_aws_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"aws_current_epoch_cost_model","threshold":null,"unit":"USD","value":3733.77},"EVID-76CE682449BA3088A5EBB4E1":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-76CE682449BA3088A5EBB4E1","interpretation":"Current release channel from the current configuration epoch.","metric":"warehouse_channel","observation_window":"current epoch","source":"system.compute.warehouses","source_field":"warehouse_channel","threshold":null,"unit":"value","value":"CURRENT"},"EVID-9349C4F74710189DF28D26E5":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-9349C4F74710189DF28D26E5","interpretation":"Calendar-day coverage available to the forward cost model.","metric":"cost_history_days","observation_window":"current_epoch","source":"system.billing.usage","source_field":"usage_date","threshold":null,"unit":"days","value":122},"EVID-F9AD519DB03E1D0381CB098E":{"comparator":"","epoch_scope":"CURRENT","evidence_id":"EVID-F9AD519DB03E1D0381CB098E","interpretation":"No-change forward DBU cost forecast anchored to the current configuration epoch.","metric":"forward_dbu_cost_365d","observation_window":"forward_365d","source":"derived","source_field":"epoch-runrate-v2.10.0","threshold":null,"unit":"USD","value":3200.0}}</t>
         </is>
       </c>
       <c r="AV83" s="22" t="inlineStr">
@@ -31911,12 +31911,12 @@
     <row r="84" ht="32" customHeight="1">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>PKG-02C2A3390BC1C4114197FDAD</t>
+          <t>PKG-664E535A61AEB69185D775A9</t>
         </is>
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>CAND-B1ED2C3FFE321E66E70DDEA3</t>
+          <t>CAND-B53760F75B53442716A3FA4F</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
@@ -32118,12 +32118,12 @@
       </c>
       <c r="AT84" s="22" t="inlineStr">
         <is>
-          <t>["EVID-D13BA07AC4F2B2109C2C45B7","EVID-738C19E56B6084DC96E07DFC","EVID-C8DD5554A816A72AA6BFADCE","EVID-160E49D36662E0D31042F51A","EVID-89B2E15FC06474BF301B094E","EVID-616B75581FAF5783E6529E1D","EVID-34F1847BE68B6EBBFA915B95","EVID-9C5A7D28B4BA43DE7C3220CD","EVID-9520A9F3745C6B42827B881A","EVID-1FDA0700A45761E2E0DC6B81","EVID-0E39BB07A52CCA2264264F50","EVID-6DD782A2BB5F89EE62C99CA3","EVID-9349C4F74710189DF28D26E5"]</t>
+          <t>["EVID-D13BA07AC4F2B2109C2C45B7","EVID-738C19E56B6084DC96E07DFC","EVID-C8DD5554A816A72AA6BFADCE","EVID-160E49